<commit_message>
Updates after cleaning objectives
</commit_message>
<xml_diff>
--- a/www/LENS_INDICATORS_DB.xlsx
+++ b/www/LENS_INDICATORS_DB.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L228"/>
+  <dimension ref="A1:L226"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -655,16 +655,6 @@
           <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Consumer protection</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Impact</t>
-        </is>
-      </c>
       <c r="L6" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Channel type; Financial service provider (FSP) type</t>
@@ -1682,12 +1672,12 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Consumer protection; Market development</t>
+          <t>Market development</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Impact, Capital markets development</t>
+          <t>Capital markets development</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
@@ -1743,12 +1733,12 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Consumer protection; Market development</t>
+          <t>Market development</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Impact, Capital markets development</t>
+          <t>Capital markets development</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -2688,16 +2678,6 @@
           <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>Consumer protection</t>
-        </is>
-      </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>Impact</t>
-        </is>
-      </c>
       <c r="L44" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
@@ -2798,16 +2778,6 @@
           <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>Consumer protection</t>
-        </is>
-      </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>Impact</t>
-        </is>
-      </c>
       <c r="L46" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
@@ -3053,16 +3023,6 @@
           <t>Are there gender disparities in the likelihood of engaging in e-commerce transactions, including for MSMEs based on the gender of the owner? Do transaction patterns—such as frequency and average ticket size—differ by gender, and how do these vary across income groups, age brackets, and locations? Are e-commerce transactions concentrated within specific financial service providers (FSPs) or market segments, and does this concentration reflect gender imbalances? Could differences in transaction volumes by gender indicate limited access to e-commerce payment channels or the unsuitability of available solutions for certain groups? Are FSPs with higher levels of gender diversity more likely to support inclusive e-commerce participation across genders?</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>Consumer protection</t>
-        </is>
-      </c>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>Impact</t>
-        </is>
-      </c>
       <c r="L51" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
@@ -3299,16 +3259,6 @@
           <t>What are the gender dynamics in remittance transactions? Is there a gender that is the predominant recipient of international remittances? What are the gender differences in the size and frequency of remittances? Are remittances concentrated in certain geographical areas, FSP types, and account types? Which channels are mostly used to receive remittances? Are these areas considered low-income locations or locations with low cash access point density? Comparing with indicators on transaction channel locations, how do they compare with remittance reception? Are remittance recipients particularly underserved by access points? Is there any correlation between the gender of recipients and FSP gender diversity? Which countries originate the most remittances to low-income locations and populations? Do these coincide with countries with higher remittance costs?</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>Other; Consumer protection</t>
-        </is>
-      </c>
-      <c r="K56" t="inlineStr">
-        <is>
-          <t>Statistics and research, Impact</t>
-        </is>
-      </c>
       <c r="L56" t="inlineStr">
         <is>
           <t>Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Channel type; Transaction type</t>
@@ -3354,16 +3304,6 @@
           <t>What are the gender dynamics in remittance transactions? Is there a gender that is the predominant recipient of international remittances? What are the gender differences in the size and frequency of remittances? Are remittances concentrated in certain geographical areas, FSP types, and account types? Which channels are mostly used to receive remittances? Are these areas considered low-income locations or locations with low cash access point density? Comparing with indicators on transaction channel locations, how do they compare with remittance reception? Are remittance recipients particularly underserved by access points? Is there any correlation between the gender of recipients and FSP gender diversity? Which countries originate the most remittances to low-income locations and populations? Do these coincide with countries with higher remittance costs?</t>
         </is>
       </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>Other; Consumer protection</t>
-        </is>
-      </c>
-      <c r="K57" t="inlineStr">
-        <is>
-          <t>Statistics and research, Impact</t>
-        </is>
-      </c>
       <c r="L57" t="inlineStr">
         <is>
           <t>Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Channel type; Transaction type</t>
@@ -3409,16 +3349,6 @@
           <t>How do genders differ in how much and how often they transact through different channels (cash, ATM, digital, agents, mobile, etc.), by transaction value and frequency? Are there gender differences in the choice of channels associated with high‐value vs low‐value transactions? How have channel usage patterns for different genders evolved over time, especially for younger, lower‐income, or rural women? Do providers who are more gender‐inclusive tend to offer or promote more equitable access and usage across channels?</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>Consumer protection</t>
-        </is>
-      </c>
-      <c r="K58" t="inlineStr">
-        <is>
-          <t>Impact</t>
-        </is>
-      </c>
       <c r="L58" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Financial service provider (FSP) type; Product type; Transaction type</t>
@@ -3464,16 +3394,6 @@
           <t>How do genders differ in how much and how often they transact through different channels (cash, ATM, digital, agents, mobile, etc.)? How have channel usage patterns for different genders evolved over time, especially for younger, lower‐income, or rural women? Do providers who are more gender‐inclusive tend to offer or promote more equitable access and usage across channels?</t>
         </is>
       </c>
-      <c r="J59" t="inlineStr">
-        <is>
-          <t>Consumer protection</t>
-        </is>
-      </c>
-      <c r="K59" t="inlineStr">
-        <is>
-          <t>Impact</t>
-        </is>
-      </c>
       <c r="L59" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Financial service provider (FSP) type; Product type; Transaction type</t>
@@ -3744,16 +3664,6 @@
           <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
         </is>
       </c>
-      <c r="J64" t="inlineStr">
-        <is>
-          <t>Consumer protection</t>
-        </is>
-      </c>
-      <c r="K64" t="inlineStr">
-        <is>
-          <t>Impact</t>
-        </is>
-      </c>
       <c r="L64" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
@@ -4186,12 +4096,12 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Total outstanding balances in active deposit accounts</t>
+          <t>Total balances in active deposit accounts</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Measures the total outstanding balance in all active deposit accounts at the end of the reporting period. It represents the aggregate value of deposits held in accounts that are actively used, distinguishing them from dormant or inactive balances. Captures the volume of mobilized deposits that are linked to active financial relationships, providing insight into financial depth, liquidity, and the stability of deposit funding within the banking system. Tracking the balance of active accounts helps regulators and analysts: Evaluate effective deposit mobilization and financial intermediation; Identify the share of deposits that are transactionally relevant versus idle; Monitor liquidity risks and customer engagement in deposit markets; Assess financial inclusion quality and trust in the formal system. Higher balances indicate stronger deposit mobilization and customer trust in institutions. Declining balances may reflect economic stress, withdrawals, or shift toward alternative financial instruments. Stable ratios of active to total balances indicate healthy engagement and liquidity management. !- Definitions and concepts: Active deposit account: An account with at least one transaction or a positive balance during the reporting period. Outstanding balance: The total value of deposits held in those accounts as of the reference date. !- Derivable indicators: Average balance per active account = (Total active deposit balances / Number of active deposit accounts); Weighted deposit activity rate = (Active deposit balances / Total deposit balances) × 100</t>
+          <t>Measures the total balance in all active deposit accounts at the end of the reporting period. It represents the aggregate value of deposits held in accounts that are actively used, distinguishing them from dormant or inactive balances. Captures the volume of mobilized deposits that are linked to active financial relationships, providing insight into financial depth, liquidity, and the stability of deposit funding within the banking system. Tracking the balance of active accounts helps regulators and analysts: Evaluate effective deposit mobilization and financial intermediation; Identify the share of deposits that are transactionally relevant versus idle; Monitor liquidity risks and customer engagement in deposit markets; Assess financial inclusion quality and trust in the formal system. Higher balances indicate stronger deposit mobilization and customer trust in institutions. Declining balances may reflect economic stress, withdrawals, or shift toward alternative financial instruments. Stable ratios of active to total balances indicate healthy engagement and liquidity management. !- Definitions and concepts: Active deposit account: An account with at least one transaction or a positive balance during the reporting period. Balance: The total value of deposits held in those accounts as of the reference date. !- Derivable indicators: Average balance per active account = (Total active deposit balances / Number of active deposit accounts); Weighted deposit activity rate = (Active deposit balances / Total deposit balances) × 100</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -4523,17 +4433,17 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>E-money accounts (outstanding balance)</t>
+          <t>E-money accounts (balance)</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Outstanding balances in e-money accounts</t>
+          <t>Balances in e-money accounts</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Measures the total outstanding value of e-money issued and held in customer accounts at a given point in time. It represents the monetary value of customer funds stored electronically and redeemable on demand. Captures the stock of e-money in circulation, serving as an indicator of digital liquidity, trust in electronic value storage, and systemic importance of e-money issuers within the payments landscape. The total e-money float helps supervisors monitor: System-wide liquidity exposure of e-money issuers, customer fund safeguarding and segregation compliance, the role of e-money in monetary aggregates and financial stability. It is also a key input to assessing digital financial inclusion and payment ecosystem growth. Higher balances indicate increased usage and confidence in e-money as a store of value. Rapid increases may reflect accelerating digital adoption or limited conversion to cash; Declines could signal withdrawals or regulatory tightening. !- Definitions and concepts: E-money is prepaid value stored electronically, which represents a liability of the e-money issuer (a bank, an e-money institution or any other entity authorised or allowed to issue e-money in the local jurisdiction) and which is denominated in a currency backed by an authority. Outstanding balance: The monetary value of all e-money not yet redeemed or withdrawn by customers. E-money float: The total value of customer funds corresponding to issued e-money liabilities, typically held in trust or custodial accounts with regulated financial institutions. !- Data requirements: Sum of all outstanding e-money balances across customer accounts at the end of the reference period, based on account-level data from licensed e-money issuers with additional disaggregation for segmentation analysis (e.g. age, gender, location of customer). !- Derivable indicators: Average balance per account = (Total e-money balances / Number of e-money accounts); Average balance per account holder = (Total e-money balances / Number of e-money account holders).</t>
+          <t>Measures the total value (balance) of e-money issued and held in customer accounts at a given point in time. It represents the monetary value of customer funds stored electronically and redeemable on demand. Captures the stock of e-money in circulation, serving as an indicator of digital liquidity, trust in electronic value storage, and systemic importance of e-money issuers within the payments landscape. The total e-money float helps supervisors monitor: System-wide liquidity exposure of e-money issuers, customer fund safeguarding and segregation compliance, the role of e-money in monetary aggregates and financial stability. It is also a key input to assessing digital financial inclusion and payment ecosystem growth. Higher balances indicate increased usage and confidence in e-money as a store of value. Rapid increases may reflect accelerating digital adoption or limited conversion to cash; Declines could signal withdrawals or regulatory tightening. !- Definitions and concepts: E-money is prepaid value stored electronically, which represents a liability of the e-money issuer (a bank, an e-money institution or any other entity authorised or allowed to issue e-money in the local jurisdiction) and which is denominated in a currency backed by an authority. Balance: The monetary value of all e-money not yet redeemed or withdrawn by customers. E-money float: The total value of customer funds corresponding to issued e-money liabilities, typically held in trust or custodial accounts with regulated financial institutions. !- Data requirements: Sum of all e-money balances across customer accounts at the end of the reference period, based on account-level data from licensed e-money issuers with additional disaggregation for segmentation analysis (e.g. age, gender, location of customer). !- Derivable indicators: Average balance per account = (Total e-money balances / Number of e-money accounts); Average balance per account holder = (Total e-money balances / Number of e-money account holders).</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -4569,17 +4479,17 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Mobile money accounts (outstanding balance)</t>
+          <t>Mobile money accounts (balance)</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Outstanding balances in mobile money accounts</t>
+          <t>Balances in mobile money accounts</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Measures the total outstanding value of mobile-money issued and held in customer accounts at a given point in time. It represents the monetary value of customer funds stored electronically and redeemable on demand. Captures the stock of mobile money in circulation, serving as an indicator of digital liquidity, trust in electronic value storage, and systemic importance of mobile money issuers within the payments landscape. The total mobile money float helps supervisors monitor: System-wide liquidity exposure of mobile money issuers, customer fund safeguarding and segregation compliance, the role of mobile money in monetary aggregates and financial stability. It is also a key input to assessing digital financial inclusion and payment ecosystem growth. Higher balances indicate increased usage and confidence in mobile money as a store of value. Rapid increases may reflect accelerating digital adoption or limited conversion to cash; Declines could signal withdrawals or regulatory tightening. !- Definitions and concepts: Mobile money accounts are a type of e-money account. Mobile money refers to a form of e-money where funds are stored in a mobile money account linked to a phone number accessible through a mobile phone, or any SIM-enabled device, and facilitated by a network of mobile money agents (IMF FAS). It is a financial service offered to its clients by a mobile network operator or another entity that partners with mobile network operators, independent of the traditional banking network. Outstanding balance: The monetary value of all mobile money not yet redeemed or withdrawn by customers. !- Data requirements: Sum of all outstanding mobile money balances across customer accounts at the end of the reference period, based on account-level data from licensed mobile money issuers with additional disaggregation for segmentation analysis (e.g. age, gender, location of customer). !- Derivable indicators: Average balance per account = (Total mobile money balances / Number of mobile money accounts); Average balance per account holder = (Total mobile money balances / Number of mobile money account holders).</t>
+          <t>Measures the total outstanding value of mobile-money issued and held in customer accounts at a given point in time. It represents the monetary value of customer funds stored electronically and redeemable on demand. Captures the stock of mobile money in circulation, serving as an indicator of digital liquidity, trust in electronic value storage, and systemic importance of mobile money issuers within the payments landscape. The total mobile money float helps supervisors monitor: System-wide liquidity exposure of mobile money issuers, customer fund safeguarding and segregation compliance, the role of mobile money in monetary aggregates and financial stability. It is also a key input to assessing digital financial inclusion and payment ecosystem growth. Higher balances indicate increased usage and confidence in mobile money as a store of value. Rapid increases may reflect accelerating digital adoption or limited conversion to cash; Declines could signal withdrawals or regulatory tightening. !- Definitions and concepts: Mobile money accounts are a type of e-money account. Mobile money refers to a form of e-money where funds are stored in a mobile money account linked to a phone number accessible through a mobile phone, or any SIM-enabled device, and facilitated by a network of mobile money agents (IMF FAS). It is a financial service offered to its clients by a mobile network operator or another entity that partners with mobile network operators, independent of the traditional banking network. Outstanding balance: The monetary value of all mobile money not yet redeemed or withdrawn by customers. !- Data requirements: Sum of all mobile money balances across customer accounts at the end of the reference period, based on account-level data from licensed mobile money issuers with additional disaggregation for segmentation analysis (e.g. age, gender, location of customer). !- Derivable indicators: Average balance per account = (Total mobile money balances / Number of mobile money accounts); Average balance per account holder = (Total mobile money balances / Number of mobile money account holders).</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -4590,7 +4500,7 @@
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t>Customer type; Account type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Account type</t>
         </is>
       </c>
     </row>
@@ -4699,7 +4609,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Impact</t>
+          <t>Usage</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -4742,7 +4652,7 @@
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>Uptake (account ownership)</t>
+          <t>Usage</t>
         </is>
       </c>
       <c r="L84" t="inlineStr">
@@ -4832,17 +4742,17 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Investment accounts (outstanding balance)</t>
+          <t>Investment accounts (balance)</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Outstanding balance in investment accounts</t>
+          <t>Balance in investment accounts</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Measures the total value of financial assets held by individuals in all investment accounts at the end of the reference period. Captures the aggregate stock of investment wealth intermediated through formal financial channels, reflecting financial market depth, asset accumulation, and portfolio diversification. The outstanding balance in investment accounts provides insights into: The size and composition of retail investments; Trends in wealth accumulation and capital-market development; The contribution of investment activity to domestic financial stability and savings mobilization. For supervisory analysis, it informs monitoring of asset-price exposure, systemic linkages, and investor concentration. Higher values indicate growing household and institutional asset holdings and deepening financial markets. Volatility may reflect market valuation changes or shifts in investor behavior. Persistent growth signals increasing intermediation through formal channels. !- Definitions and concepts: Investment accounts: An account used to hold, trade, or manage financial assets through a licensed intermediary and can include securities trading accounts, collective investment scheme accounts, mutual fund accounts, retirement investment sub-accounts, and other regulated investment products. They can be held in banks, brokerage firms, asset managers, investment platforms and other financial institutions. They are different from deposit accounts, as their returns are not guaranteed and their value can fluctuate. Outstanding balance (investment accounts): The total market value of financial assets held in investment accounts at the reporting date, net of withdrawals or redemptions. Financial assets: Tradable or redeemable instruments such as equities, bonds, units in mutual funds, ETFs, or money-market funds. !- Data requirements: Sum of all balanes in investment accounts (market value of assets held) at the end of the reference period. Aggregated balance-sheet or custodial data from brokers, asset managers, fund administrators, and investment platforms. Disaggregation by product type (equities, fixed income, mutual funds, etc.). !- Derivable indicators: Average investment account balance = (Total investment account balances / Number of investment accounts)</t>
+          <t>Measures the total value (balance) of financial assets held by individuals in all investment accounts at the end of the reference period. Captures the aggregate stock of investment wealth intermediated through formal financial channels, reflecting financial market depth, asset accumulation, and portfolio diversification. The balance in investment accounts provides insights into: The size and composition of retail investments; Trends in wealth accumulation and capital-market development; The contribution of investment activity to domestic financial stability and savings mobilization. For supervisory analysis, it informs monitoring of asset-price exposure, systemic linkages, and investor concentration. Higher values indicate growing household and institutional asset holdings and deepening financial markets. Volatility may reflect market valuation changes or shifts in investor behavior. Persistent growth signals increasing intermediation through formal channels. !- Definitions and concepts: Investment accounts: An account used to hold, trade, or manage financial assets through a licensed intermediary and can include securities trading accounts, collective investment scheme accounts, mutual fund accounts, retirement investment sub-accounts, and other regulated investment products. They can be held in banks, brokerage firms, asset managers, investment platforms and other financial institutions. They are different from deposit accounts, as their returns are not guaranteed and their value can fluctuate. Balance (investment accounts): The total market value of financial assets held in investment accounts at the reporting date, net of withdrawals or redemptions. Financial assets: Tradable or redeemable instruments such as equities, bonds, units in mutual funds, ETFs, or money-market funds. !- Data requirements: Sum of all balances in investment accounts (market value of assets held) at the end of the reference period. Aggregated balance-sheet or custodial data from brokers, asset managers, fund administrators, and investment platforms. Disaggregation by product type (equities, fixed income, mutual funds, etc.). !- Derivable indicators: Average investment account balance = (Total investment account balances / Number of investment accounts)</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -4857,17 +4767,17 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>Consumer protection; Market development</t>
+          <t>Market development</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>Impact, Capital markets development</t>
+          <t>Capital markets development</t>
         </is>
       </c>
       <c r="L86" t="inlineStr">
         <is>
-          <t>Customer type; Account type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Account type</t>
         </is>
       </c>
     </row>
@@ -4912,12 +4822,12 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>Consumer protection; Stability, safety and soundness</t>
+          <t>Stability, safety and soundness</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>Impact, Operational risk</t>
+          <t>Operational risk</t>
         </is>
       </c>
       <c r="L87" t="inlineStr">
@@ -5044,7 +4954,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Usage</t>
+          <t>Usage, Outcomes</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -5087,7 +4997,7 @@
       </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t>Suitability,</t>
+          <t>Suitability, Stability</t>
         </is>
       </c>
       <c r="L90" t="inlineStr">
@@ -5262,12 +5172,12 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>Other; Consumer protection</t>
+          <t>Consumer protection</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>Statistics and research, Suitability</t>
+          <t>Suitability</t>
         </is>
       </c>
       <c r="L93" t="inlineStr">
@@ -5322,12 +5232,12 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>Other; Consumer protection</t>
+          <t>Consumer protection</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
         <is>
-          <t>Statistics and research, Quality</t>
+          <t>Suitability</t>
         </is>
       </c>
       <c r="L94" t="inlineStr">
@@ -5438,16 +5348,6 @@
       <c r="I96" t="inlineStr">
         <is>
           <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J96" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="K96" t="inlineStr">
-        <is>
-          <t>Statistics and research</t>
         </is>
       </c>
       <c r="L96" t="inlineStr">
@@ -5763,7 +5663,7 @@
       </c>
       <c r="K102" t="inlineStr">
         <is>
-          <t>Fair treatment</t>
+          <t>Fair treatment, Complaints handling</t>
         </is>
       </c>
       <c r="L102" t="inlineStr">
@@ -5823,7 +5723,7 @@
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>Fair treatment</t>
+          <t>Fair treatment, Complaints handling</t>
         </is>
       </c>
       <c r="L103" t="inlineStr">
@@ -5840,35 +5740,35 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Quality</t>
+          <t>Outcomes</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Payments, Savings, Credit, Insurance, Pensions, Investments</t>
+          <t>Savings</t>
         </is>
       </c>
       <c r="D104">
-        <v>322</v>
+        <v>164</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Fraud prevalence in complaints</t>
+          <t>Early extraction of term deposits</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>Portion and volume of complaints received by providers, regulators, and ombuds that are fraud-related.</t>
+          <t>% of term deposit account holders who extracted funds before reaching maturity</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>Tracks how much of the complaint landscape is driven by fraud—both the count (volume) and the share (portion) of total complaints. Rising prevalence of frauds signals elevated customer harm, control weaknesses (KYC/AML, authentication, data security), or new attack vectors (social engineering). It helps guide supervision, consumer protection responses, reimbursement policies, and investment in fraud controls. !- Definitions and concepts: Fraud-related complaint: a case alleging unauthorised or deceptive activity resulting in loss or attempted loss—e.g., account takeover, card-not-present, phishing/SMiShing, SIM-swap, mule accounts, synthetic identity, merchant fraud, insider abuse, and authorised push payment (APP) scams. Volume: number of fraud-related complaints received in the period. Share: [# of fraud complaints / # of all complaints] x 100%. Intensity companions: fraud complaints per 1,000 customers or per 1 million transactions, value lens using claimed or confirmed loss amounts. Outcome cuts: upheld rate, reimbursement rate, median loss, time-to-resolution. A standard taxonomy for fraud types is needed, including the differentiation between fraud and disputed transaction. !- Limitations and considerations:  Under-reporting: many victims never complain or only contact the bank—triangulate with dispute/chargeback data and incident logs.</t>
+          <t>A measure of unplanned demand for liquidity, potentially indicating financial distress. !- Definitions and concepts: Term deposit accounts (such as certificates of deposit) are interest-bearing accounts whose funds can be withdrawn (without penalty) at the maturity date. !- Data requirements: Transaction level information or system flag that can produce a list of term deposit accounts with an early, full extraction of funds over a specific period. To the extent that for a given reporting institution customers can open more than one term-deposit account, unique customer IDs can de-duplicate account-level records to produce a list of unique term-deposit customers that extracted funds before maturity. In addition, the total number of term-deposit accounts (or unique account-holders) is required to compute the percentage.</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>Are there gender differences in the proportion of fraud-related complaints submitted to providers, regulators, or ombuds services?  Do individuals of different genders tend to report different types of fraud, such as identity theft, phishing, or agent misconduct, and are specific delivery channels more commonly associated with these complaints? Is the volume of fraud-related complaints disproportionately high among certain gender groups when compared to their levels of account ownership or usage? Do complaint resolution rates and timeframes differ by gender across various FSP or reporting channels?</t>
+          <t>Are there gender disparities in savings discipline, particularly in whether term deposits are retained until maturity or withdrawn early? Is there evidence that term deposit savings serve as coping mechanisms differently by gender? How do term deposit savings behaviors differ among more vulnerable or underserved individuals by gender?</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -5876,19 +5776,9 @@
           <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
         </is>
       </c>
-      <c r="J104" t="inlineStr">
-        <is>
-          <t>Consumer protection</t>
-        </is>
-      </c>
-      <c r="K104" t="inlineStr">
-        <is>
-          <t>Fair treatment</t>
-        </is>
-      </c>
       <c r="L104" t="inlineStr">
         <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Complaints resolution outcome; Complaints resolution time</t>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
         </is>
       </c>
     </row>
@@ -5909,26 +5799,26 @@
         </is>
       </c>
       <c r="D105">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Early extraction of term deposits</t>
+          <t>Resumption of savings after early extraction from term deposits</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>% of term deposit account holders who extracted funds before reaching maturity</t>
+          <t>% of term deposit account holders who resumed savings after extracting funds prior to maturity</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>A measure of unplanned demand for liquidity, potentially indicating financial distress. !- Definitions and concepts: Term deposit accounts (such as certificates of deposit) are interest-bearing accounts whose funds can be withdrawn (without penalty) at the maturity date. !- Data requirements: Transaction level information or system flag that can produce a list of term deposit accounts with an early, full extraction of funds over a specific period. To the extent that for a given reporting institution customers can open more than one term-deposit account, unique customer IDs can de-duplicate account-level records to produce a list of unique term-deposit customers that extracted funds before maturity. In addition, the total number of term-deposit accounts (or unique account-holders) is required to compute the percentage.</t>
+          <t>A measure of financial resilience or the ability to bounce back after an unplanned use of committed resources.  !- Definitions and concepts: Term deposit accounts (such as certificates of deposit) are interest-bearing accounts whose funds can be withdrawn (without penalty) at the maturity date. !- Data requirements: Transaction level information or system flag that can produce a list of term deposit accounts that had an early, full extraction of funds over a specific period, and of those, the number that made subsquent repleneshing deposits to the account. To the extent that for a given reporting institution customers can open more than one term-deposit account, unique customer IDs can de-duplicate account-level records to produce a list of unique term-deposit customers that extracted funds before maturity. In addition, the total number of term-deposit accounts (or unique account-holders) is required as the denominator to compute the percentage.</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>Are there gender disparities in savings discipline, particularly in whether term deposits are retained until maturity or withdrawn early? Is there evidence that term deposit savings serve as coping mechanisms differently by gender? How do term deposit savings behaviors differ among more vulnerable or underserved individuals by gender?</t>
+          <t>Are there gender disparities in the likelihood of resuming term deposit savings after withdrawing them before maturity? What are the characteristics of individuals who resume term deposit savings by gender? Which FSPs rank highest and lowest in the resumption of term deposit savings, and does this ranking change when analyzed by gender?</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -5959,26 +5849,26 @@
         </is>
       </c>
       <c r="D106">
-        <v>165</v>
+        <v>148</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Resumption of savings after early extraction from term deposits</t>
+          <t>Deposit and payment account holders who also hold term deposits</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>% of term deposit account holders who resumed savings after extracting funds prior to maturity</t>
+          <t>% of deposit and payment account holders who also have term deposits</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>A measure of financial resilience or the ability to bounce back after an unplanned use of committed resources.  !- Definitions and concepts: Term deposit accounts (such as certificates of deposit) are interest-bearing accounts whose funds can be withdrawn (without penalty) at the maturity date. !- Data requirements: Transaction level information or system flag that can produce a list of term deposit accounts that had an early, full extraction of funds over a specific period, and of those, the number that made subsquent repleneshing deposits to the account. To the extent that for a given reporting institution customers can open more than one term-deposit account, unique customer IDs can de-duplicate account-level records to produce a list of unique term-deposit customers that extracted funds before maturity. In addition, the total number of term-deposit accounts (or unique account-holders) is required as the denominator to compute the percentage.</t>
+          <t>A measure of the demand for long-term savings instruments among account holders. !- Data requirements: List of customers with deposit or payment accounts over a specific period of time, List of customers with time or term-deposit accounts over a specific period of time. Both lists should be linkable with a unique customer ID. When the lists are merged, the number of unique customers with both a deposit or payment account and a term deposit account can be counted and reported. For a system-wide count, the number of unique customers with both a deposit or payment account and term account across all reporting institutions can be summed up  and divided by the total number of unique customers and multiplied by 100 to obtain a percentage.  At the system level, there is a risk of counting individuals more than once in the numerator and denominator, unless national IDs can be used to de-duplicate records across FSPs.</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the likelihood of resuming term deposit savings after withdrawing them before maturity? What are the characteristics of individuals who resume term deposit savings by gender? Which FSPs rank highest and lowest in the resumption of term deposit savings, and does this ranking change when analyzed by gender?</t>
+          <t>How common is it for individuals holding transaction accounts to also maintain interest-bearing term deposit accounts? Are there gender disparities in the multiple ownership and distribution of these different account types across age groups and location types, both at the total market level and by relevant FSP/type? How prevalent is the cross-sell of term deposit accounts among vulnerable customer segments, and are there gender disparities within these segments? How do average balances differ between transaction and term deposit accounts across gender, age groups, and location types, both at the total market level and by relevant FSP/type? Are there gender disparities in average balances across these account types? How do average balances vary among vulnerable customer segments, and are there gender disparities within these segments? What are the gender disparities in cross-selling and average balances of transaction accounts and term deposit accounts across age groups and location types, both at the total market level and by relevant FSP/type?</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -6005,35 +5895,45 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Savings</t>
+          <t>Savings, Credit</t>
         </is>
       </c>
       <c r="D107">
-        <v>148</v>
+        <v>173</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Deposit and payment account holders who also hold term deposits</t>
+          <t>Depositors-borrowers ratio</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>% of deposit and payment account holders who also have term deposits</t>
+          <t>% of unsecured borrowers who also have a deposit account</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>A measure of the demand for long-term savings instruments among account holders. !- Data requirements: List of customers with deposit or payment accounts over a specific period of time, List of customers with time or term-deposit accounts over a specific period of time. Both lists should be linkable with a unique customer ID. When the lists are merged, the number of unique customers with both a deposit or payment account and a term deposit account can be counted and reported. For a system-wide count, the number of unique customers with both a deposit or payment account and term account across all reporting institutions can be summed up  and divided by the total number of unique customers and multiplied by 100 to obtain a percentage.  At the system level, there is a risk of counting individuals more than once in the numerator and denominator, unless national IDs can be used to de-duplicate records across FSPs.</t>
+          <t>A measure of cross-selling additional financial services to borrowers (alternatively, a measure of the demand for deposit accounts among short-term borrowers). !- Data requirements: Granular data or data systems that can produce (1) A list of unique customers of any (at least one) unsecured loan or line of credit (e.g. credit card, personal loan) and (2) A list of unique customers of any (at least one) type of deposit account (e.g. current/checking, savings, time deposit). A unique customer ID to identify customers that are in both list (1) AND list (2). The total number of unique borrowers meeting this condition (also having a deposit account) is then divided by the total number of borrowers and multiplied by 100 to obtain the ratio.</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>How common is it for individuals holding transaction accounts to also maintain interest-bearing term deposit accounts? Are there gender disparities in the multiple ownership and distribution of these different account types across age groups and location types, both at the total market level and by relevant FSP/type? How prevalent is the cross-sell of term deposit accounts among vulnerable customer segments, and are there gender disparities within these segments? How do average balances differ between transaction and term deposit accounts across gender, age groups, and location types, both at the total market level and by relevant FSP/type? Are there gender disparities in average balances across these account types? How do average balances vary among vulnerable customer segments, and are there gender disparities within these segments? What are the gender disparities in cross-selling and average balances of transaction accounts and term deposit accounts across age groups and location types, both at the total market level and by relevant FSP/type?</t>
+          <t>Are there sociodemographic (gender, age, location, income) disparities in borrowers' cross-sell ratios of deposit accounts and in the likelihood of being a stand-alone borrower? Have gender disparities in cross-sell ratios changed over time, particularly for underserved borrowers?</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
         <is>
           <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>Consumer protection</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>Suitability</t>
         </is>
       </c>
       <c r="L107" t="inlineStr">
@@ -6059,41 +5959,31 @@
         </is>
       </c>
       <c r="D108">
-        <v>173</v>
+        <v>261</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Depositors-borrowers ratio</t>
+          <t>Savings to borrowings ratio</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>% of unsecured borrowers who also have a deposit account</t>
+          <t>% of outstanding balances of unsecured credit in relation to savings balances, for borrowers who also have a savings account</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>A measure of cross-selling additional financial services to borrowers (alternatively, a measure of the demand for deposit accounts among short-term borrowers). !- Data requirements: Granular data or data systems that can produce (1) A list of unique customers of any (at least one) unsecured loan or line of credit (e.g. credit card, personal loan) and (2) A list of unique customers of any (at least one) type of deposit account (e.g. current/checking, savings, time deposit). A unique customer ID to identify customers that are in both list (1) AND list (2). The total number of unique borrowers meeting this condition (also having a deposit account) is then divided by the total number of borrowers and multiplied by 100 to obtain the ratio.</t>
+          <t>This indicator measures the degree to which outstanding balances on unsecured loans or lines of credit (such as credit card debt, digital loans or other personal loans) can be covered with savings balances at a specific point in time, potentially providing insights on the financial health of the borrower. !- Data requirements: Granular data that can enable identifiction of (1) list of unique borrowers using any unsecured credit product AND a savings account, (2) total outstanding balances across all unsecured credit products at a specific point in time (e.g. end of quarter) by unique borrower, (3) total balances in savings accounts at a specific point in time by unique borrower. Among the borrowers who meet the conditions in (1) the indicator can be computed by taking the sum of total outstanding debt divided by the sum of total savings balances.</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>Are there sociodemographic (gender, age, location, income) disparities in borrowers' cross-sell ratios of deposit accounts and in the likelihood of being a stand-alone borrower? Have gender disparities in cross-sell ratios changed over time, particularly for underserved borrowers?</t>
+          <t>Are there disparities in borrowers' cross-sell ratios of deposit accounts by gender, and/or age, location or income?? And in the likelihood of being a stand-alone borrower? Have gender disparities in cross-sell ratios changed over time, particularly for underserved borrowers?</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
         <is>
           <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J108" t="inlineStr">
-        <is>
-          <t>Consumer protection</t>
-        </is>
-      </c>
-      <c r="K108" t="inlineStr">
-        <is>
-          <t>Suitability</t>
         </is>
       </c>
       <c r="L108" t="inlineStr">
@@ -6110,35 +6000,36 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Outcomes</t>
+          <t>Uptake (account ownership)</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Savings, Credit</t>
+          <t>Credit</t>
         </is>
       </c>
       <c r="D109">
-        <v>261</v>
+        <v>172</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Savings to borrowings ratio</t>
+          <t>First-time borrowers</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>% of outstanding balances of unsecured credit in relation to savings balances, for borrowers who also have a savings account</t>
+          <t>% of borrowers who are first-time borrowers with the FSP (or in the financial system)</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>This indicator measures the degree to which outstanding balances on unsecured loans or lines of credit (such as credit card debt, digital loans or other personal loans) can be covered with savings balances at a specific point in time, potentially providing insights on the financial health of the borrower. !- Data requirements: Granular data that can enable identifiction of (1) list of unique borrowers using any unsecured credit product AND a savings account, (2) total outstanding balances across all unsecured credit products at a specific point in time (e.g. end of quarter) by unique borrower, (3) total balances in savings accounts at a specific point in time by unique borrower. Among the borrowers who meet the conditions in (1) the indicator can be computed by taking the sum of total outstanding debt divided by the sum of total savings balances.</t>
+          <t>This indicator shows the share of active borrowing retail customers who are new to the lender (new-to-bank/FSP) or new to formal credit altogether (new-to-credit, NTC). It is a direct barometer of financial inclusion and retail credit growth. A higher share can signal effective onboarding and market expansion, but it also shifts portfolio risk: NTC borrowers may lack repayment histories, making underwriting more model-driven and subject to greater uncertainty. Supervisors and lenders can monitor this metric to balance inclusion objectives with prudent risk management and to evaluate the effectiveness of credit-bureau coverage. !- Definitions and concepts: First-time borrower (FSP scope): a customer with no prior loan or credit line ever booked by the FSP before the reference period. First-time borrower (system scope / NTC): a customer with no prior loan or credit line reported to the national credit registry/bureau within a defined historical look-back (commonly “ever,” or a long horizon such as 5–10 years). This indicator is obtained by dividing the number of first-time borrowers by the total number of borrowers. Variants of this indicator include: value-weighted (by origination amount), new originations only (versus the entire active book), and cohort-based analysis (by origination month or quarter). !- Data requirements: Customer master records with unique, reliable identifiers (national ID/tax ID; deduplicated across branches). Loan-booking history from the FSP’s core systems. Credit-bureau/registry match results (for system-wide NTC status). Product taxonomy (include/exclude credit cards, overdrafts, BNPL) and reference dates. Limitaitons and considerations: Coverage gaps: thin or partial bureau coverage, informal lenders, or non-reporting segments can misclassify NTC status.
+Identifier quality: name changes, multiple IDs, or data-entry errors cause false “first-time” flags; robust deduplication is essential. Look-back window choice: shorter windows inflate “first-time” shares; disclose methodology. Product scope: excluding revolving credit or microloans biases results.</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>Are there disparities in borrowers' cross-sell ratios of deposit accounts by gender, and/or age, location or income?? And in the likelihood of being a stand-alone borrower? Have gender disparities in cross-sell ratios changed over time, particularly for underserved borrowers?</t>
+          <t>Do first-time borrowers reflect a balanced gender representation, or are there gender disparities? How do FSPs rank in onboarding typically underserved borrowers, and does this ranking change when analyzed by gender?</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -6160,7 +6051,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Suitability</t>
+          <t>Usage</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -6196,16 +6087,6 @@
           <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
         </is>
       </c>
-      <c r="J110" t="inlineStr">
-        <is>
-          <t>Central banking</t>
-        </is>
-      </c>
-      <c r="K110" t="inlineStr">
-        <is>
-          <t>Currency management and cash handling</t>
-        </is>
-      </c>
       <c r="L110" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
@@ -6220,28 +6101,88 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
+          <t>Outcomes</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Savings</t>
+        </is>
+      </c>
+      <c r="D111">
+        <v>156</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Depositors who actively close deposit accounts</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>% of retail depositors who actively closed a deposit account</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>A measure of the incidence of account closing among depositors, if the measure is high, it could potentially signal issues with the quality of accounts or concerns about the safety of funds. !- Definitions and concepts: Deposit accounts include transaction and non-transaction deposit accounts, for example: Checking/demand, savings, time/term deposit accounts, pensions. 'Active' closure of an account refers to cases where the closure is initiated at the request of the customer, and not due to inactivity or dormancy. !- Data requirements: List of unique deposit account holders (i.e. an individual  must be counted as one depositor irrespective of the number of deposit accounts held) who actively close any of their accounts over a specified period of time (e.g. quarter or year); Total number of unique depositors at the beginning of the specified period.</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>How do active closure rates compare by gender? Which types of accounts are most frequently closed by each gender? How do FSPs rank in active account closures, and does this ranking change when analyzed by gender?</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>Consumer protection; Stability, safety and soundness</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>Fair treatment, Stability</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Financial inclusion</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
           <t>Access</t>
         </is>
       </c>
-      <c r="C111" t="inlineStr">
+      <c r="C112" t="inlineStr">
         <is>
           <t>Insurance</t>
         </is>
       </c>
-      <c r="D111">
+      <c r="D112">
         <v>393</v>
       </c>
-      <c r="E111" t="inlineStr">
+      <c r="E112" t="inlineStr">
         <is>
           <t>Access to inclusive insurance products</t>
         </is>
       </c>
-      <c r="F111" t="inlineStr">
+      <c r="F112" t="inlineStr">
         <is>
           <t>% of financial service providers offering inclusive or micro insurance products</t>
         </is>
       </c>
-      <c r="G111" t="inlineStr">
+      <c r="G112" t="inlineStr">
         <is>
           <t>This indicator measures the proportion of licensed insurance providers (or other entities authorized to underwrite insurance) that offer inclusive insurance or microinsurance products. It provides a supply-side measure of the extent to which the insurance market is serving un- or underserved populations, including low-income individuals and communities that face specific risks but have traditionally been excluded from formal insurance coverage. Tracking this indicator over time allows financial sector authorities to assess whether regulatory frameworks and market conditions are effectively encouraging providers to develop and distribute products that address the protection gap. It is particularly relevant for supervisors pursuing financial inclusion objectives and for evaluating the impact of proportionate regulatory approaches, such as dedicated microinsurance licensing frameworks or regulatory sandboxes, on the breadth of product offerings in the market.
 !-Definitions and concepts: Inclusive insurance, as defined in the IAIS Issues Paper on Conduct of Business in Inclusive Insurance (2015), refers broadly to all insurance products aimed at the excluded or underserved market, rather than only those targeted at the poor or a narrow conception of the low-income population. Microinsurance is a subset of inclusive insurance, defined by the IAIS (2007) as insurance that is accessed by the low-income population, provided by a variety of different entities, but run in accordance with generally accepted insurance practices and funded by premiums. Each jurisdiction should adapt this definition to its own context, considering national regulatory frameworks, market characteristics, and the specific populations identified as underserved. The formula is: Access to inclusive insurance products (%) = (Number of FSPs offering at least one inclusive or microinsurance product / Total number of licensed insurance providers) × 100.
@@ -6249,120 +6190,60 @@
 !-Limitations and considerations: The meaningfulness of this indicator depends heavily on how inclusive insurance or microinsurance is defined in each jurisdiction. In countries without a dedicated regulatory framework or formal product classification, identifying which providers offer qualifying products may require subjective judgments or additional data collection efforts. The indicator captures the share of providers offering inclusive products but does not measure the depth, quality, or uptake of those products; a provider may offer a single inclusive product with very limited reach. Complementary indicators such as the number of inclusive insurance policies in force, premiums written, or claims settlement ratios for inclusive products would provide a fuller picture of market development. The indicator also does not distinguish between providers for whom inclusive insurance is a core business versus those for whom it is a marginal product line. Cross-country comparisons should be made cautiously due to differences in regulatory definitions, market structures, and the types of entities authorized to offer insurance. Finally, because this indicator focuses on the supply side, it should be interpreted alongside demand-side measures to understand whether available products are actually reaching and benefiting the intended populations.</t>
         </is>
       </c>
-      <c r="L111" t="inlineStr">
+      <c r="L112" t="inlineStr">
         <is>
           <t>Financial service provider (FSP) type</t>
         </is>
       </c>
     </row>
-    <row r="112">
-      <c r="A112" t="inlineStr">
-        <is>
-          <t>Financial inclusion</t>
-        </is>
-      </c>
-      <c r="B112" t="inlineStr">
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Financial inclusion</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
         <is>
           <t>Uptake (account ownership)</t>
         </is>
       </c>
-      <c r="C112" t="inlineStr">
+      <c r="C113" t="inlineStr">
         <is>
           <t>Insurance</t>
         </is>
       </c>
-      <c r="D112">
+      <c r="D113">
         <v>395</v>
       </c>
-      <c r="E112" t="inlineStr">
+      <c r="E113" t="inlineStr">
         <is>
           <t>Insured or lives covered</t>
         </is>
       </c>
-      <c r="F112" t="inlineStr">
+      <c r="F113" t="inlineStr">
         <is>
           <t>Number of insured persons or lives covered by insurance</t>
         </is>
       </c>
-      <c r="G112" t="inlineStr">
+      <c r="G113" t="inlineStr">
         <is>
           <t>Refers to the total count of people covered by insurance, a key metric of coverage breadth and insurance uptake, complementary to the number of insurance policyholders. The policyholder and the insured can be different people -for example, if someone takes out a policy on another individual, the latter is the insured because the policy covers them, and the former is the policyholder, who purchases and owns the policy, and holds the right to make changes. An insurance policy can also cover several people, such as in member-owned schemes, group plans, and other variations. 
 When expressed as a share of the population or in per capita terms, it is a measure of the prevalence of insurance adoption and facilitates comparison with other countries. For microinsurance, a coverage ratio can reflect the number of lives covered expressed as a share of the target market or population participating in microinsurance programs  !- Definitions and concepts: Lives covered by insurance refers to the total number of people covered by life and non-life insurance policies. A customer covered by more than one (life or non-life) insurance policy should be counted as one life covered. !- Data requirements: Number of lives insured at the end of a specific period (e.g. quarter or year);  Total adult population (official counts from recent census or estimates from national statistics agency); Target population (number of people targeted by microinsurance, which may include segments of a community or clients from an MFI). !- Limitations and considerations: If an individual is covered by multiple insurers, they may be counted more than once in aggregations of lives covered across institutions, unless a national ID can be used . !- Derivable indicators: Lives covered by insurance per 1,000 adults; Lives covered by insurance as a share of the target population.</t>
         </is>
       </c>
-      <c r="H112" t="inlineStr">
+      <c r="H113" t="inlineStr">
         <is>
           <t>Are there gender differences in the total number of lives covered by insurance, including across product types and providers? How do multiple insurance coverages and coverage amounts vary by gender, age, income, and location? To what extent do providers with higher gender diversity attract more gender-balanced portfolios of lives covered? Are gender disparities consistent or do they vary across life and non-life insurance within the overall market?</t>
         </is>
       </c>
-      <c r="I112" t="inlineStr">
+      <c r="I113" t="inlineStr">
         <is>
           <t>For analyses with a primary focus on financial inclusion, for this indicator, it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered.</t>
         </is>
       </c>
-      <c r="L112" t="inlineStr">
+      <c r="L113" t="inlineStr">
         <is>
           <t>Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Insurance type</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" t="inlineStr">
-        <is>
-          <t>Consumer protection</t>
-        </is>
-      </c>
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>Suitability</t>
-        </is>
-      </c>
-      <c r="C113" t="inlineStr">
-        <is>
-          <t>Credit</t>
-        </is>
-      </c>
-      <c r="D113">
-        <v>103</v>
-      </c>
-      <c r="E113" t="inlineStr">
-        <is>
-          <t>Borrowers whose collateral was seized</t>
-        </is>
-      </c>
-      <c r="F113" t="inlineStr">
-        <is>
-          <t>% of borrowers whose collateral was seized</t>
-        </is>
-      </c>
-      <c r="G113" t="inlineStr">
-        <is>
-          <t>A measure of loan portfolio/credit risk assessment quality or financial distress among borrowers. !- Data requirements: Granular data that can yield (1) A count of unique borrowers of secured loans (those with collateral requirements) who subsequently had collateral seized by lender due to default over a specific period of time (e.g. past quarter or past year), (2) Total unique borrowers of secured loans over a specific period of time.</t>
-        </is>
-      </c>
-      <c r="H113" t="inlineStr">
-        <is>
-          <t>How does the share of customers whose collateral was seized due to default vary by gender and othe rkey sociodemographics? Are women more or less likely than men to have their collateral seized following loan default? How does the share differ by gender across different loan sizes, loan products,  types of financial service providers (FSP), collateral type (e.g., movable, immovable, alternative)? And how do any of these differences relate to seizure rates? Are women more likely to be subject to stricter collateral requirements or less flexible repayment terms that increase the likelihood of asset seizure?</t>
-        </is>
-      </c>
-      <c r="I113" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J113" t="inlineStr">
-        <is>
-          <t>Financial inclusion; Stability, safety and soundness</t>
-        </is>
-      </c>
-      <c r="K113" t="inlineStr">
-        <is>
-          <t>Outcomes, Credit risk</t>
-        </is>
-      </c>
-      <c r="L113" t="inlineStr">
-        <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Loan type; Collateral type; Loan size; Loan term; Interest rate category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
         </is>
       </c>
     </row>
@@ -6374,7 +6255,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Complaints handling</t>
+          <t>Complaints handling, Safety and security</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -6383,26 +6264,26 @@
         </is>
       </c>
       <c r="D114">
-        <v>239</v>
+        <v>322</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Customer complaints (number)</t>
+          <t>Fraud prevalence in complaints</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>Number of customer complaints (including processing status, channels, type)</t>
+          <t>Portion and volume of complaints received by providers, regulators, and ombuds that are fraud-related.</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>This indicator tallies the formal expressions of dissatisfaction that retail or MSME clients lodge with a financial-service provider (or an external ombudsman) about products, services, or staff conduct over a specified period and can be normalized by dividing by the customer basis to obtain an intensity metric (e.g. complaints per 1,000 active customers). A rising complaint count can signal service-quality gaps, mis-selling, opaque fees, or inadequate disclosure—issues that erode trust and may escalate into regulatory sanctions or litigation. Supervisors can track both the absolute number and complaint-to-account ratios to test consumer-protection frameworks, prioritise thematic reviews, and assess whether rapid product roll-outs (e.g., digital lending, mobile wallets) are being matched by robust after-sales support. Where granular data or more detailed reporting templates permit, customer complaints can be disaggregated by processing status (e.g. received, accepted/rejected, in process, resolved, escalated/disputed, withdrawn), product (e.g. consumer loan, deposit account, etc), channel (e.g. digital, phone, in-person), issue category (e.g. fraudulent or unauthorized transactions, unfair treatment, unexpected fees, errors on statements,  etc.), resolution status (open, resolved with monetary compensation, resolved without compensation, escalated to ombudsman/regulator, other). Combined with resolution-time, compensation and other metrics, the number of customer complaints provides a critical, early-warning lens on conduct risk and customer-experience health. !- Definitions and concepts:  Complaints are expressions of dissatisfaction by (or on behalf of) customers that are related to their experiences with FSPs and can include any written, digital or recorded verbal statement made through any available channel, such as a branch, call-centre, email, social media, chatbots and other portals. Complaints may relate to the quality of a product or service, treatment by an FSP (including its agents and other third parties), or suspected wrongdoing. Complaints are different from general inquiries (e.g., where can I find an ATM?) or legal disputes between parties that may require formal dispute resolution. For more information, see for example CGAP's toolkit on using complaints data for market conduct supervision: https://www.cgap.org/research/publication/market-monitoring-tool-analysis-complaints-data and the Alliance for Financial Inclusion's framework on 'Complaint handling in Central Banks': https://www.afi-global.org/sites/default/files/publications/2020-04/AFI_CEMC_framework_AW_digital%20v2.pdf. !- Data requirements:  Database or log of customer complaints, detailing date of complaint and additional information, such as channel through which complaint was lodged, associated product or account, details or brief description of the complaint, and resolution status. !- Limitations and considerations: Complaints processes differ across FSPs in terms of steps/levels for routing, hand-over, escalations to higher management levels and to external ombudsman. Customer details and demographics of complainants are not always capture/stored on FSPs' systems, or may be stored in fragmented data bases. Complaints logged at aggregator sites/portals may not request customer demographics. Limited to officially logged complaints and/or maintaining records of inbound customer communications. Dependent on having electronic complaints management system.  Reporting culture: firms with easy‐to‐use channels may record more complaints than peers, even if service quality is similar—benchmark using severity and uphold rates. Under-reporting bias: vulnerable customers may forgo formal complaints; mystery-shopping and survey data can complement administrative counts. Duplicate cases: the same issue voiced through multiple channels can inflate totals unless robust deduplication exists. Product mix effects: complaint propensity varies—e.g., complex investments draw more grievances than basic savings; segment analysis is essential. Regulatory divergence: definitions and mandatory reporting thresholds differ across jurisdictions, complicating cross-border comparisons.</t>
+          <t>Tracks how much of the complaint landscape is driven by fraud—both the count (volume) and the share (portion) of total complaints. Rising prevalence of frauds signals elevated customer harm, control weaknesses (KYC/AML, authentication, data security), or new attack vectors (social engineering). It helps guide supervision, consumer protection responses, reimbursement policies, and investment in fraud controls. !- Definitions and concepts: Fraud-related complaint: a case alleging unauthorised or deceptive activity resulting in loss or attempted loss—e.g., account takeover, card-not-present, phishing/SMiShing, SIM-swap, mule accounts, synthetic identity, merchant fraud, insider abuse, and authorised push payment (APP) scams. Volume: number of fraud-related complaints received in the period. Share: [# of fraud complaints / # of all complaints] x 100%. Intensity companions: fraud complaints per 1,000 customers or per 1 million transactions, value lens using claimed or confirmed loss amounts. Outcome cuts: upheld rate, reimbursement rate, median loss, time-to-resolution. A standard taxonomy for fraud types is needed, including the differentiation between fraud and disputed transaction. !- Limitations and considerations:  Under-reporting: many victims never complain or only contact the bank—triangulate with dispute/chargeback data and incident logs.</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>How does the number of complaints at each processing stage vary by gender? Are complaints disproportionately concentrated at certain processing stages for any gender? How do FSPs compare to market averages in the number of complaints at each processing stage?"</t>
+          <t>Are there gender differences in the proportion of fraud-related complaints submitted to providers, regulators, or ombuds services?  Do individuals of different genders tend to report different types of fraud, such as identity theft, phishing, or agent misconduct, and are specific delivery channels more commonly associated with these complaints? Is the volume of fraud-related complaints disproportionately high among certain gender groups when compared to their levels of account ownership or usage? Do complaint resolution rates and timeframes differ by gender across various FSP or reporting channels?</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -6412,17 +6293,17 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>Financial inclusion; Stability, safety and soundness</t>
+          <t>Financial inclusion</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>Quality,</t>
+          <t>Quality</t>
         </is>
       </c>
       <c r="L114" t="inlineStr">
         <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Complaints filing channel; Complaints issue category; Complaints processing status; Complaints resolution outcome; Complaints resolution time</t>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Complaints resolution outcome; Complaints resolution time</t>
         </is>
       </c>
     </row>
@@ -6434,35 +6315,35 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Complaints handling</t>
+          <t>Suitability</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Payments, Savings, Credit, Insurance, Pensions, Investments</t>
+          <t>Credit</t>
         </is>
       </c>
       <c r="D115">
-        <v>243</v>
+        <v>103</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Customer complaints resolved in the customer's favor</t>
+          <t>Borrowers whose collateral was seized</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>% of customer complaints that were solved in the customer's favor in the most recent period</t>
+          <t>% of borrowers whose collateral was seized</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>This indicator shows the share of complaints closed in the reference period that were resolved in the customer’s favor. It is a direct outcome metric for fair treatment and service quality. A higher “uphold rate” can indicate strong remediation and customer-centric policies; a very low rate may suggest poor triage, overly narrow eligibility rules, or weak guidance to customers on evidence requirements. Supervisors use it to benchmark conduct outcomes across firms and products; boards track it alongside complaint volumes and resolution times to target root-cause fixes. Tracked with complaint volume, resolution time, and compensation totals, this indicator provides a balanced view of consumer outcomes and conduct risk. !- Definitions and concepts: Resolved in the customer’s favor (upheld): final decision grants redress—monetary (refund/compensation/fee reversal) or non-monetary (policy correction, contract change, apology with tangible remedy). Many firms also count partially upheld cases; disclose whether partials are included. Denominator: all complaints closed in the period. Segment results by product, channel, and severtiy to avoid masking problem areas. !- Data requirements: Central complaint-management records with unique IDs, receipt date, closure date, product, channel, allegation type, decision outcome (upheld/partially/declined), and compensation amount. Deduplication logic across channels; linkages to ombudsman/regulator portals for escalations and reversals. Customer-base denominator (for intensity metrics) and service level agreement (SLA) timestamps for parallel monitoring* (see note below). !- Limitations and considerations: Classification discretion: definitions of “partial uphold” vary; publish inclusion rules. Case mix effects: a surge in low-merit mass claims can depress the percentage; report severity-adjusted or line-of-business cuts. Gaming risk: chasing high uphold rates may encourage paying weak claims; pair with fraud flags, root-cause fixes, and cost-per-case. Timing bias: complex cases close later and differ in uphold propensity; use rolling averages and track median resolution time. External outcomes: include overturned-on-appeal adjustments to reflect true customer outcome. *With granular time-stamped complaints data, timeliness of key milestones in the complaints resolution process can be tracked, for example time to acknowledge complaint, time to first response, time to resolution. With this data, supervisors can track not just outcomes, but also whether providers are meeting required timeframes per their own SLA.</t>
+          <t>A measure of loan portfolio/credit risk assessment quality or financial distress among borrowers. !- Data requirements: Granular data that can yield (1) A count of unique borrowers of secured loans (those with collateral requirements) who subsequently had collateral seized by lender due to default over a specific period of time (e.g. past quarter or past year), (2) Total unique borrowers of secured loans over a specific period of time.</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>How do the percentages of complaints resolved in favor of customers vary by gender? Are any genders more likely to receive favorable resolutions? How do FSPs rank in terms of favorable resolutions by gender?</t>
+          <t>How does the share of customers whose collateral was seized due to default vary by gender and othe rkey sociodemographics? Are women more or less likely than men to have their collateral seized following loan default? How does the share differ by gender across different loan sizes, loan products,  types of financial service providers (FSP), collateral type (e.g., movable, immovable, alternative)? And how do any of these differences relate to seizure rates? Are women more likely to be subject to stricter collateral requirements or less flexible repayment terms that increase the likelihood of asset seizure?</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -6477,12 +6358,12 @@
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>Quality,</t>
+          <t>Outcomes, Credit risk</t>
         </is>
       </c>
       <c r="L115" t="inlineStr">
         <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Complaints filing channel; Complaints issue category; Complaints processing status; Complaints resolution outcome; Complaints resolution time</t>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Loan type; Collateral type; Loan size; Loan term; Interest rate category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
         </is>
       </c>
     </row>
@@ -6494,7 +6375,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Data privacy and protection</t>
+          <t>Complaints handling</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -6503,26 +6384,26 @@
         </is>
       </c>
       <c r="D116">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Consent rate for FSP contact</t>
+          <t>Customer complaints (number)</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>% of customers who provide consent to be contacted in the future by the FSP for sales, awareness and new offerings</t>
+          <t>Number of customer complaints (including processing status, channels, type)</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>Measures the percentage of customers who have provided explicit consent to be contacted in the future by their financial service provider (FSP) for purposes such as product marketing, customer awareness campaigns, or information on new offerings. This indicator reflects how institutions manage customer permissions for communication under applicable data privacy and marketing regulations. Captures the extent of customer consent and data-use transparency in the financial system, serving as a proxy for compliance with consent-based communication standards and the balance between customer engagement and data protection. Tracking customer contact consents helps regulators and providers: Monitor compliance with data protection and privacy laws (e.g., GDPR-like frameworks, data protection acts); Assess ethical marketing practices and responsible customer engagement; Evaluate trust and willingness of customers to maintain open communication with FSPs; Understand customer attitudes toward data sharing and digital outreach. For supervisors, it provides a measurable view of market conduct, customer empowerment, and institutional transparency. High consent rates suggest strong customer trust and engagement, but may require close monitoring to ensure non-coercive consent collection and ethical marketing practices. Low consent rates may reflect privacy concerns, limited digital literacy, or overly complex consent processes. Changes over time can signal shifts in consumer sentiment or compliance practices following new regulations. !- Definitions and concepts: Consent: A freely given, informed, and specific agreement by a customer allowing the FSP to contact them for defined purposes. Data privacy regulation: Legal framework governing the collection, storage, and use of personal data, including consent requirements for marketing communications. !- Data requirements: Administrative data from FSP customer relationship management (CRM) or consent-management systems to obtain the number of customers who provided consent to be contact and the total number of customers.</t>
+          <t>This indicator tallies the formal expressions of dissatisfaction that retail or MSME clients lodge with a financial-service provider (or an external ombudsman) about products, services, or staff conduct over a specified period and can be normalized by dividing by the customer basis to obtain an intensity metric (e.g. complaints per 1,000 active customers). A rising complaint count can signal service-quality gaps, mis-selling, opaque fees, or inadequate disclosure—issues that erode trust and may escalate into regulatory sanctions or litigation. Supervisors can track both the absolute number and complaint-to-account ratios to test consumer-protection frameworks, prioritise thematic reviews, and assess whether rapid product roll-outs (e.g., digital lending, mobile wallets) are being matched by robust after-sales support. Where granular data or more detailed reporting templates permit, customer complaints can be disaggregated by processing status (e.g. received, accepted/rejected, in process, resolved, escalated/disputed, withdrawn), product (e.g. consumer loan, deposit account, etc), channel (e.g. digital, phone, in-person), issue category (e.g. fraudulent or unauthorized transactions, unfair treatment, unexpected fees, errors on statements,  etc.), resolution status (open, resolved with monetary compensation, resolved without compensation, escalated to ombudsman/regulator, other). Combined with resolution-time, compensation and other metrics, the number of customer complaints provides a critical, early-warning lens on conduct risk and customer-experience health. !- Definitions and concepts:  Complaints are expressions of dissatisfaction by (or on behalf of) customers that are related to their experiences with FSPs and can include any written, digital or recorded verbal statement made through any available channel, such as a branch, call-centre, email, social media, chatbots and other portals. Complaints may relate to the quality of a product or service, treatment by an FSP (including its agents and other third parties), or suspected wrongdoing. Complaints are different from general inquiries (e.g., where can I find an ATM?) or legal disputes between parties that may require formal dispute resolution. For more information, see for example CGAP's toolkit on using complaints data for market conduct supervision: https://www.cgap.org/research/publication/market-monitoring-tool-analysis-complaints-data and the Alliance for Financial Inclusion's framework on 'Complaint handling in Central Banks': https://www.afi-global.org/sites/default/files/publications/2020-04/AFI_CEMC_framework_AW_digital%20v2.pdf. !- Data requirements:  Database or log of customer complaints, detailing date of complaint and additional information, such as channel through which complaint was lodged, associated product or account, details or brief description of the complaint, and resolution status. !- Limitations and considerations: Complaints processes differ across FSPs in terms of steps/levels for routing, hand-over, escalations to higher management levels and to external ombudsman. Customer details and demographics of complainants are not always capture/stored on FSPs' systems, or may be stored in fragmented data bases. Complaints logged at aggregator sites/portals may not request customer demographics. Limited to officially logged complaints and/or maintaining records of inbound customer communications. Dependent on having electronic complaints management system.  Reporting culture: firms with easy‐to‐use channels may record more complaints than peers, even if service quality is similar—benchmark using severity and uphold rates. Under-reporting bias: vulnerable customers may forgo formal complaints; mystery-shopping and survey data can complement administrative counts. Duplicate cases: the same issue voiced through multiple channels can inflate totals unless robust deduplication exists. Product mix effects: complaint propensity varies—e.g., complex investments draw more grievances than basic savings; segment analysis is essential. Regulatory divergence: definitions and mandatory reporting thresholds differ across jurisdictions, complicating cross-border comparisons.</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>How do consent rates for customer contact vary by gender? Are any genders more likely to provide consent to be contacted? How do FSPs rank in terms of consent rates by gender?</t>
+          <t>How does the number of complaints at each processing stage vary by gender? Are complaints disproportionately concentrated at certain processing stages for any gender? How do FSPs compare to market averages in the number of complaints at each processing stage?"</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -6542,7 +6423,7 @@
       </c>
       <c r="L116" t="inlineStr">
         <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Complaints filing channel; Complaints issue category; Complaints processing status; Complaints resolution outcome; Complaints resolution time</t>
         </is>
       </c>
     </row>
@@ -6554,28 +6435,148 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
+          <t>Complaints handling</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Payments, Savings, Credit, Insurance, Pensions, Investments</t>
+        </is>
+      </c>
+      <c r="D117">
+        <v>243</v>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Customer complaints resolved in the customer's favor</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>% of customer complaints that were solved in the customer's favor in the most recent period</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>This indicator shows the share of complaints closed in the reference period that were resolved in the customer’s favor. It is a direct outcome metric for fair treatment and service quality. A higher “uphold rate” can indicate strong remediation and customer-centric policies; a very low rate may suggest poor triage, overly narrow eligibility rules, or weak guidance to customers on evidence requirements. Supervisors use it to benchmark conduct outcomes across firms and products; boards track it alongside complaint volumes and resolution times to target root-cause fixes. Tracked with complaint volume, resolution time, and compensation totals, this indicator provides a balanced view of consumer outcomes and conduct risk. !- Definitions and concepts: Resolved in the customer’s favor (upheld): final decision grants redress—monetary (refund/compensation/fee reversal) or non-monetary (policy correction, contract change, apology with tangible remedy). Many firms also count partially upheld cases; disclose whether partials are included. Denominator: all complaints closed in the period. Segment results by product, channel, and severtiy to avoid masking problem areas. !- Data requirements: Central complaint-management records with unique IDs, receipt date, closure date, product, channel, allegation type, decision outcome (upheld/partially/declined), and compensation amount. Deduplication logic across channels; linkages to ombudsman/regulator portals for escalations and reversals. Customer-base denominator (for intensity metrics) and service level agreement (SLA) timestamps for parallel monitoring* (see note below). !- Limitations and considerations: Classification discretion: definitions of “partial uphold” vary; publish inclusion rules. Case mix effects: a surge in low-merit mass claims can depress the percentage; report severity-adjusted or line-of-business cuts. Gaming risk: chasing high uphold rates may encourage paying weak claims; pair with fraud flags, root-cause fixes, and cost-per-case. Timing bias: complex cases close later and differ in uphold propensity; use rolling averages and track median resolution time. External outcomes: include overturned-on-appeal adjustments to reflect true customer outcome. *With granular time-stamped complaints data, timeliness of key milestones in the complaints resolution process can be tracked, for example time to acknowledge complaint, time to first response, time to resolution. With this data, supervisors can track not just outcomes, but also whether providers are meeting required timeframes per their own SLA.</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>How do the percentages of complaints resolved in favor of customers vary by gender? Are any genders more likely to receive favorable resolutions? How do FSPs rank in terms of favorable resolutions by gender?</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>Financial inclusion</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Complaints filing channel; Complaints issue category; Complaints processing status; Complaints resolution outcome; Complaints resolution time</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Consumer protection</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Data privacy and protection</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Payments, Savings, Credit, Insurance, Pensions, Investments</t>
+        </is>
+      </c>
+      <c r="D118">
+        <v>234</v>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Consent rate for FSP contact</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>% of customers who provide consent to be contacted in the future by the FSP for sales, awareness and new offerings</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>Measures the percentage of customers who have provided explicit consent to be contacted in the future by their financial service provider (FSP) for purposes such as product marketing, customer awareness campaigns, or information on new offerings. This indicator reflects how institutions manage customer permissions for communication under applicable data privacy and marketing regulations. Captures the extent of customer consent and data-use transparency in the financial system, serving as a proxy for compliance with consent-based communication standards and the balance between customer engagement and data protection. Tracking customer contact consents helps regulators and providers: Monitor compliance with data protection and privacy laws (e.g., GDPR-like frameworks, data protection acts); Assess ethical marketing practices and responsible customer engagement; Evaluate trust and willingness of customers to maintain open communication with FSPs; Understand customer attitudes toward data sharing and digital outreach. For supervisors, it provides a measurable view of market conduct, customer empowerment, and institutional transparency. High consent rates suggest strong customer trust and engagement, but may require close monitoring to ensure non-coercive consent collection and ethical marketing practices. Low consent rates may reflect privacy concerns, limited digital literacy, or overly complex consent processes. Changes over time can signal shifts in consumer sentiment or compliance practices following new regulations. !- Definitions and concepts: Consent: A freely given, informed, and specific agreement by a customer allowing the FSP to contact them for defined purposes. Data privacy regulation: Legal framework governing the collection, storage, and use of personal data, including consent requirements for marketing communications. !- Data requirements: Administrative data from FSP customer relationship management (CRM) or consent-management systems to obtain the number of customers who provided consent to be contact and the total number of customers.</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>How do consent rates for customer contact vary by gender? Are any genders more likely to provide consent to be contacted? How do FSPs rank in terms of consent rates by gender?</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>Financial inclusion</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Consumer protection</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
           <t>Fair treatment</t>
         </is>
       </c>
-      <c r="C117" t="inlineStr">
+      <c r="C119" t="inlineStr">
         <is>
           <t>Credit</t>
         </is>
       </c>
-      <c r="D117">
+      <c r="D119">
         <v>284</v>
       </c>
-      <c r="E117" t="inlineStr">
+      <c r="E119" t="inlineStr">
         <is>
           <t>Annual percentage rate (APR) for retail credit</t>
         </is>
       </c>
-      <c r="F117" t="inlineStr">
+      <c r="F119" t="inlineStr">
         <is>
           <t>Average cost of borrowing money, including fees to get the loan, as a% of the loan principal (except for credit cards)</t>
         </is>
       </c>
-      <c r="G117" t="inlineStr">
+      <c r="G119" t="inlineStr">
         <is>
           <t>APR is the standardized annualized cost of borrowing that incorporates the contractual interest rate plus certain up-front or periodic fees required to obtain and maintain the credit. It lets consumers compare offers across lenders and products on a like-for-like basis, and helps supervisors monitor pricing fairness and market competitiveness. Unlike a simple “nominal” rate, APR reflects timing of cash flows and required charges, so it better approximates the true price of credit. !- Definitions and concepts: Installment credit APR (actuarial method): the internal rate of return (IRR) that equates the amount advanced to the borrower with the present value of all required payments (principal, interest, and included fees), expressed on an annual basis.
 Revolving credit APR (cards/overdrafts): the periodic rate applied to the average daily balance, annualized (e.g., daily rate × 365 or monthly rate × 12), plus disclosure of any mandatory fees as prescribed. Scope of fees: typically includes origination/processing fees and compulsory charges; excludes penalty fees and optional add-ons (unless mandated). APR vs. EIR: APR is a consumer disclosure metric (jurisdiction-specific rules); EIR is an accounting yield used to recognize interest income.!- Data requirements: Contract terms: principal advanced, repayment schedule (dates/amounts), nominal rate, compounding frequency, and variable-rate index/margins. Included fees: origination/processing, mandatory maintenance or platform fees, financed vs. paid-in-cash. For revolving products: periodic rate(s), balance computation method (average daily balance), mandatory annual fees, grace-period rules, promotional/teaser rates.
@@ -6583,149 +6584,29 @@
 Promotions &amp; step-ups: teaser or deferred-interest offers can make snapshot APRs unrepresentative—show lifetime-effective examples when possible. Variable rates: APR at origination may understate future cost if reference rates rise. Loan term effects: fixed fees loom larger on short tenors; present both APR and the fee share of cost for transparency.</t>
         </is>
       </c>
-      <c r="H117" t="inlineStr">
+      <c r="H119" t="inlineStr">
         <is>
           <t>Are there gender disparities in the APR applied to loans disbursed to women and men, including MSMEs by gender of ownership? Do women borrowers systematically face higher average APRs than men within the same loan type, amount range, or provider category? Are higher APRs for women associated with smaller loan sizes, shorter maturities, or higher perceived credit risk? Do FSPs with greater gender diversity or stronger inclusion policies show smaller gender gaps in average APRs? How do APR differences relate to borrower profiles and do they suggest the presence of gender-based pricing bias or structural credit segmentation?</t>
         </is>
       </c>
-      <c r="I117" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J117" t="inlineStr">
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
         <is>
           <t>Financial inclusion; Market development</t>
         </is>
       </c>
-      <c r="K117" t="inlineStr">
+      <c r="K119" t="inlineStr">
         <is>
           <t>Quality, Competition</t>
         </is>
       </c>
-      <c r="L117" t="inlineStr">
+      <c r="L119" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" t="inlineStr">
-        <is>
-          <t>Consumer protection</t>
-        </is>
-      </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>Data privacy and protection</t>
-        </is>
-      </c>
-      <c r="C118" t="inlineStr">
-        <is>
-          <t>Payments, Savings, Credit, Insurance, Pensions, Investments</t>
-        </is>
-      </c>
-      <c r="D118">
-        <v>235</v>
-      </c>
-      <c r="E118" t="inlineStr">
-        <is>
-          <t>Consents for sharing data with third-parties</t>
-        </is>
-      </c>
-      <c r="F118" t="inlineStr">
-        <is>
-          <t>% of customers who have given explicit consent for their data to be shared by FSPs with third parties, for various purposes</t>
-        </is>
-      </c>
-      <c r="G118" t="inlineStr">
-        <is>
-          <t>This indicator shows how many customers have actively opted in to let a financial service provider (FSP) share their data with external parties—for open-banking/aggregation, credit scoring, fraud prevention, marketing, analytics, etc. A higher share can reflect strong digital adoption and trust; low or falling rates may signal poor consent UX, unclear value propositions, or privacy concerns. It helps compliance teams evidence lawfulness, product teams gauge partner-integration reach, and supervisors assess the maturity of consent-based data-sharing ecosystems. !- Definitions and concepts: Explicit consent: a clear, affirmative action (e.g., checked box, strong-customer-authenticated authorization) tied to a specific purpose, with intelligible notice and the ability to withdraw at any time. Active consent: consent that is valid as of the reference date (not expired, not withdrawn, not superseded). Purpose taxonomy: e.g., account information services (AIS), payment initiation services (PIS), credit decisioning/bureau pulls, fraud/AML tools, personalised marketing, data portability. Metric: % of customer with active consent for purpose p = [# of unique customers with at least 1 active consent for p / # of active customers] x 100%. Indicator companions: Any-purpose consent, consents per consenting customer and revocation rate. !- Data requirements: Consent ledger that includes: customer ID, purpose(s) granted, third-party identity, channel, timestamp, expiry/refresh cycle, version of the privacy notice, proof of consent (hash, audit trail, SCA event). Status events: withdrawals, expiries, scope changes, third-party disconnects. Reference universe: deduplicated active-customer list (define “active”: e.g., ≥1 product in force or ≥1 login/transaction in last 12 months). !- Limitations and considerations: Granularity &amp; fragmentation: a customer may consent per app, per account, and per purpose; avoid double counting by using unique customers and report purpose-level cuts. Expiry &amp; refresh: open-banking tokens often have short authorizations; snapshot dates vs. rolling windows will yield different figures—disclose method. Consumer protection risk: high opt-ins driven by coercive UX can backfire (complaints, revocations); pair with revocation rate, time-to-revocation, and complaints about data sharing. Coverage gaps: legacy channels without digital capture may under-record historical consents; backfill or disclose limitations.</t>
-        </is>
-      </c>
-      <c r="H118" t="inlineStr">
-        <is>
-          <t>How do consent rates for data sharing with third parties vary by gender? Are any genders more likely to provide consent for data sharing? How do FSPs rank in terms of consent rates for data sharing by gender?</t>
-        </is>
-      </c>
-      <c r="I118" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J118" t="inlineStr">
-        <is>
-          <t>Market development</t>
-        </is>
-      </c>
-      <c r="K118" t="inlineStr">
-        <is>
-          <t>Competition</t>
-        </is>
-      </c>
-      <c r="L118" t="inlineStr">
-        <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t>Consumer protection</t>
-        </is>
-      </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>Fair treatment</t>
-        </is>
-      </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>Credit</t>
-        </is>
-      </c>
-      <c r="D119">
-        <v>260</v>
-      </c>
-      <c r="E119" t="inlineStr">
-        <is>
-          <t>Late penalty charges/fees on retail credit</t>
-        </is>
-      </c>
-      <c r="F119" t="inlineStr">
-        <is>
-          <t>Income from penalty fees as % of total net interest income</t>
-        </is>
-      </c>
-      <c r="G119" t="inlineStr">
-        <is>
-          <t>This indicator shows how much of a lender is relying on penalty fees for income. Revenue from penalty fees and other charges applied when a loan payment is late is compared with the total gross interest income. A high share could signal borrower stress and potential conduct risk (reliance on punitive pricing). Boards and supervisors use the metric to assess earnings quality, pricing fairness. !- Definitions and concepts: Penalty/default fees and charges: the fees and costs charged once a loan  is past due. Numerator (preferred “incremental” view): Penalty actually recognized as income on retail loans during the period. Denominator: Gross interest income. !- Data requirements: General-ledger mapping that identifies penalty income at product level. Period interest income totals for the denominator.  !- Limitations and considerations: Mix effects: card-heavy books show higher shares of penalty income; segment by product. Conduct lens: pair with % customers incurring penalty charges, related complaints.</t>
-        </is>
-      </c>
-      <c r="H119" t="inlineStr">
-        <is>
-          <t>What percentages of net interest income are attributable to penalties and other punitive charges earned from borrowers of unsecured loans/lines of credit, and how do these vary by gender across age bands and location types, at a total market level and by relevant FSP/type? How do these percentages compare across relevant FSPs/types and against market norms across age bands and location types? How do gender disparities manifest in these percentages at a total market level and by relevant FSP/type?</t>
-        </is>
-      </c>
-      <c r="I119" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J119" t="inlineStr">
-        <is>
-          <t>Financial inclusion</t>
-        </is>
-      </c>
-      <c r="K119" t="inlineStr">
-        <is>
-          <t>Quality</t>
-        </is>
-      </c>
-      <c r="L119" t="inlineStr">
-        <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Loan type</t>
         </is>
       </c>
     </row>
@@ -6737,177 +6618,177 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
+          <t>Data privacy and protection</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Payments, Savings, Credit, Insurance, Pensions, Investments</t>
+        </is>
+      </c>
+      <c r="D120">
+        <v>235</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Consents for sharing data with third-parties</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>% of customers who have given explicit consent for their data to be shared by FSPs with third parties, for various purposes</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>This indicator shows how many customers have actively opted in to let a financial service provider (FSP) share their data with external parties—for open-banking/aggregation, credit scoring, fraud prevention, marketing, analytics, etc. A higher share can reflect strong digital adoption and trust; low or falling rates may signal poor consent UX, unclear value propositions, or privacy concerns. It helps compliance teams evidence lawfulness, product teams gauge partner-integration reach, and supervisors assess the maturity of consent-based data-sharing ecosystems. !- Definitions and concepts: Explicit consent: a clear, affirmative action (e.g., checked box, strong-customer-authenticated authorization) tied to a specific purpose, with intelligible notice and the ability to withdraw at any time. Active consent: consent that is valid as of the reference date (not expired, not withdrawn, not superseded). Purpose taxonomy: e.g., account information services (AIS), payment initiation services (PIS), credit decisioning/bureau pulls, fraud/AML tools, personalised marketing, data portability. Metric: % of customer with active consent for purpose p = [# of unique customers with at least 1 active consent for p / # of active customers] x 100%. Indicator companions: Any-purpose consent, consents per consenting customer and revocation rate. !- Data requirements: Consent ledger that includes: customer ID, purpose(s) granted, third-party identity, channel, timestamp, expiry/refresh cycle, version of the privacy notice, proof of consent (hash, audit trail, SCA event). Status events: withdrawals, expiries, scope changes, third-party disconnects. Reference universe: deduplicated active-customer list (define “active”: e.g., ≥1 product in force or ≥1 login/transaction in last 12 months). !- Limitations and considerations: Granularity &amp; fragmentation: a customer may consent per app, per account, and per purpose; avoid double counting by using unique customers and report purpose-level cuts. Expiry &amp; refresh: open-banking tokens often have short authorizations; snapshot dates vs. rolling windows will yield different figures—disclose method. Consumer protection risk: high opt-ins driven by coercive UX can backfire (complaints, revocations); pair with revocation rate, time-to-revocation, and complaints about data sharing. Coverage gaps: legacy channels without digital capture may under-record historical consents; backfill or disclose limitations.</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>How do consent rates for data sharing with third parties vary by gender? Are any genders more likely to provide consent for data sharing? How do FSPs rank in terms of consent rates for data sharing by gender?</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>Market development</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>Competition</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Consumer protection</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
           <t>Fair treatment</t>
         </is>
       </c>
-      <c r="C120" t="inlineStr">
+      <c r="C121" t="inlineStr">
         <is>
           <t>Credit</t>
         </is>
       </c>
-      <c r="D120">
+      <c r="D121">
+        <v>260</v>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Late penalty charges/fees on retail credit</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>Income from penalty fees as % of total net interest income</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>This indicator shows how much of a lender is relying on penalty fees for income. Revenue from penalty fees and other charges applied when a loan payment is late is compared with the total gross interest income. A high share could signal borrower stress and potential conduct risk (reliance on punitive pricing). Boards and supervisors use the metric to assess earnings quality, pricing fairness. !- Definitions and concepts: Penalty/default fees and charges: the fees and costs charged once a loan  is past due. Numerator (preferred “incremental” view): Penalty actually recognized as income on retail loans during the period. Denominator: Gross interest income. !- Data requirements: General-ledger mapping that identifies penalty income at product level. Period interest income totals for the denominator.  !- Limitations and considerations: Mix effects: card-heavy books show higher shares of penalty income; segment by product. Conduct lens: pair with % customers incurring penalty charges, related complaints.</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>What percentages of net interest income are attributable to penalties and other punitive charges earned from borrowers of unsecured loans/lines of credit, and how do these vary by gender across age bands and location types, at a total market level and by relevant FSP/type? How do these percentages compare across relevant FSPs/types and against market norms across age bands and location types? How do gender disparities manifest in these percentages at a total market level and by relevant FSP/type?</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>Financial inclusion</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Loan type</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Consumer protection</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Fair treatment</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="D122">
         <v>185</v>
       </c>
-      <c r="E120" t="inlineStr">
+      <c r="E122" t="inlineStr">
         <is>
           <t>Processing and application fees or PAF (as % of loan principal)</t>
         </is>
       </c>
-      <c r="F120" t="inlineStr">
+      <c r="F122" t="inlineStr">
         <is>
           <t>PAF as % of loan principal in unsecured credit operations</t>
         </is>
       </c>
-      <c r="G120" t="inlineStr">
+      <c r="G122" t="inlineStr">
         <is>
           <t>This indicator expresses the total up-front charges borrowers pay to originate an unsecured loan—processing fees, application fees, documentation charges—as a percentage of the loan’s principal amount. Because unsecured credit often targets price-sensitive segments and carries higher risk-based interest rates, excessive PAFs can materially raise the all-in cost of borrowing, undermine affordability tests, and trigger consumer-protection scrutiny. Tracking the ratio helps regulators detect predatory pricing, compare lenders’ transparency practices, and gauge competition in loan-origination services. For lenders, it is a barometer of non-interest revenue reliance and a lever for recouping acquisition costs. Processing &amp; Application Fees (PAF): any non-refundable charge levied at or before disbursement for administrative tasks (credit checks, KYC, documentation, platform usage). Late-payment or insurance fees are excluded.
 PAF ratio (simple): [Total PAF charged/Gross loan principal]×100%
 Where multiple partial disbursements occur, use the aggregate principal amount. Annualised impact: when PAFs are capitalised into the Effective Annual Percentage Rate (APR), their weight declines as term length rises—monitor both absolute and APR-embedded views. !- Data requirements: Loan-level records capturing principal, disbursement date, PAF amount, and any rebates for cancellations. Product codes distinguishing personal instalment loans, credit-card cash advances, payday/BNPL equivalents. Borrower demographics and channel identifiers (branch, mobile app, marketplace) for segmentation. Accounting entries showing whether fees are recognised up-front (IFRS 15 “contract costs”) or amortised via the effective-interest-rate (EIR) method. !- Limitations and considerations: Amortisation differences: Lenders using EIR spread PAFs over the loan’s life; comparing ratios on a cash basis versus amortised income can mislead. Bundled products: Cross-selling (e.g., credit-life insurance) may shift income from PAF to commissions, understating the ratio. Regulatory caps &amp; disclosures: Jurisdictions with fee ceilings or mandatory APR disclosures compress PAF ratios; cross-country benchmarking must control for such rules. Loan term effects: Short-tenor payday or BNPL loans show high PAF percentages even when absolute fees are small; interpret in context of maturity profile and APR. Waivers &amp; promotions: Temporary fee holidays for marketing campaigns can distort time-series trends—flag promotional periods separately. Should FSPs not be allowed/willing to share sensitive revenue data, ratios/percentages can be performed in-house and then shared with regulator.</t>
         </is>
       </c>
-      <c r="H120" t="inlineStr">
+      <c r="H122" t="inlineStr">
         <is>
           <t>What are the origination fee percentages as a share of loan principal by gender? Are there gender disparities in the origination fee percentages incurred? How do FSPs rank in terms of origination fee percentages by gender?</t>
         </is>
       </c>
-      <c r="I120" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J120" t="inlineStr">
-        <is>
-          <t>Financial inclusion</t>
-        </is>
-      </c>
-      <c r="K120" t="inlineStr">
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>Financial inclusion</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
         <is>
           <t>Quality</t>
         </is>
       </c>
-      <c r="L120" t="inlineStr">
+      <c r="L122" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Product type</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" t="inlineStr">
-        <is>
-          <t>Consumer protection</t>
-        </is>
-      </c>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t>Data privacy and protection</t>
-        </is>
-      </c>
-      <c r="C121" t="inlineStr">
-        <is>
-          <t>Payments, Savings, Credit, Insurance, Pensions, Investments</t>
-        </is>
-      </c>
-      <c r="D121">
-        <v>232</v>
-      </c>
-      <c r="E121" t="inlineStr">
-        <is>
-          <t>Data breaches</t>
-        </is>
-      </c>
-      <c r="F121" t="inlineStr">
-        <is>
-          <t>% of customers affected by data breaches</t>
-        </is>
-      </c>
-      <c r="G121" t="inlineStr">
-        <is>
-          <t>A measure of the depth of cyberattacks or other data security breach that result in unauthorized access to customer data. Definitions and concept: A data breach is any security incident in which unauthorized parties access sensitive or confidential information, including personal data (tax numbers, ID information, bank account numbers, healthcare data) and corporate data (customer records, intellectual property, financial information). Data requirement: Number of customers whose data was accessed without authorization during a specified period of time (e.g. quarter or year); Total number of customers at the beginning of the specified period (e.g. quarter or year).</t>
-        </is>
-      </c>
-      <c r="H121" t="inlineStr">
-        <is>
-          <t>How does the percentage of customers affected by data breaches vary by gender? Are any genders disproportionately affected by data breaches? Are data breaches more frequent in certain types of FSPs? Are data breaches more common in specific channels or interfaces?"</t>
-        </is>
-      </c>
-      <c r="I121" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J121" t="inlineStr">
-        <is>
-          <t>Financial inclusion; Stability, safety and soundness</t>
-        </is>
-      </c>
-      <c r="K121" t="inlineStr">
-        <is>
-          <t>Quality, Operational risk</t>
-        </is>
-      </c>
-      <c r="L121" t="inlineStr">
-        <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" t="inlineStr">
-        <is>
-          <t>Consumer protection</t>
-        </is>
-      </c>
-      <c r="B122" t="inlineStr">
-        <is>
-          <t>Depositor protection</t>
-        </is>
-      </c>
-      <c r="C122" t="inlineStr">
-        <is>
-          <t>Savings</t>
-        </is>
-      </c>
-      <c r="D122">
-        <v>15</v>
-      </c>
-      <c r="E122" t="inlineStr">
-        <is>
-          <t>Deposit accounts covered by direct deposit insurance</t>
-        </is>
-      </c>
-      <c r="F122" t="inlineStr">
-        <is>
-          <t>Volume and value (balances) of deposit accounts covered by direct deposit insurance</t>
-        </is>
-      </c>
-      <c r="G122" t="inlineStr">
-        <is>
-          <t>This indicator counts (or expresses as a percentage) the deposit accounts that fall within the scope of an explicit, statutory deposit insurance scheme (DIS) or deposit guarantee fund. It helps supervisors gauge how much of the retail/MSME funding base is protected against bank failure. This is key for financial stability monitoring, payout readiness, and for calibrating the deposit insurance/guarantee fund. High coverage supports confidence and can dampen run dynamics. Source: https://www.iadi.org/uploads/cprevised2014nov.pdf. !- Definitions and concepts: Covered (eligible) account: a deposit type included by law. Fully insured vs. partially insured: “Fully insured” balances are ≤ the coverage limit per depositor, per bank, per ownership category; “covered/eligible” may include accounts whose balances exceed the cap (partially insured). Ownership categories: individual, joint, trust/fiduciary, retirement—rules vary by jurisdiction and affect aggregation across accounts. Indicator variants: % Eligible accounts = eligible deposit accounts ÷ total deposit accounts. Insured balance share = insured amounts in eligible accounts ÷ total deposit balances in eligible accounts. Dormancy: dormant accounts may be treated differently in coverage statistics.</t>
-        </is>
-      </c>
-      <c r="H122" t="inlineStr">
-        <is>
-          <t>Are there gender disparities in the number of deposit accounts covered by direct deposit insurance? How do these disparities vary by age, income level, and geographic location? Are certain gender groups, especially within vulnerable or low-income populations, less likely to hold insured deposit accounts? How do the average insured deposit account balances differ across genders, and what might this indicate about savings behavior, access to financial protection, or economic security? Do financial service providers with higher levels of gender diversity in leadership or staff tend to offer more equitable access to insured deposit accounts and balanced coverage across genders? Additionally, how do gender differences in insured deposit accounts relate to broader financial inclusion and resilience against financial shocks?</t>
-        </is>
-      </c>
-      <c r="I122" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J122" t="inlineStr">
-        <is>
-          <t>Financial inclusion; Consumer protection; Stability, safety and soundness</t>
-        </is>
-      </c>
-      <c r="K122" t="inlineStr">
-        <is>
-          <t>Quality, Suitability,</t>
-        </is>
-      </c>
-      <c r="L122" t="inlineStr">
-        <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Deposit account type</t>
         </is>
       </c>
     </row>
@@ -6919,28 +6800,148 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
+          <t>Data privacy and protection</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Payments, Savings, Credit, Insurance, Pensions, Investments</t>
+        </is>
+      </c>
+      <c r="D123">
+        <v>232</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Data breaches</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>% of customers affected by data breaches</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>A measure of the depth of cyberattacks or other data security breach that result in unauthorized access to customer data. Definitions and concept: A data breach is any security incident in which unauthorized parties access sensitive or confidential information, including personal data (tax numbers, ID information, bank account numbers, healthcare data) and corporate data (customer records, intellectual property, financial information). Data requirement: Number of customers whose data was accessed without authorization during a specified period of time (e.g. quarter or year); Total number of customers at the beginning of the specified period (e.g. quarter or year).</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>How does the percentage of customers affected by data breaches vary by gender? Are any genders disproportionately affected by data breaches? Are data breaches more frequent in certain types of FSPs? Are data breaches more common in specific channels or interfaces?"</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>Financial inclusion; Stability, safety and soundness</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>Quality, Operational risk</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Consumer protection</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
           <t>Depositor protection</t>
         </is>
       </c>
-      <c r="C123" t="inlineStr">
+      <c r="C124" t="inlineStr">
         <is>
           <t>Savings</t>
         </is>
       </c>
-      <c r="D123">
+      <c r="D124">
+        <v>15</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Deposit accounts covered by direct deposit insurance</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>Volume and value (balances) of deposit accounts covered by direct deposit insurance</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>This indicator counts (or expresses as a percentage) the deposit accounts that fall within the scope of an explicit, statutory deposit insurance scheme (DIS) or deposit guarantee fund. It helps supervisors gauge how much of the retail/MSME funding base is protected against bank failure. This is key for financial stability monitoring, payout readiness, and for calibrating the deposit insurance/guarantee fund. High coverage supports confidence and can dampen run dynamics. Source: https://www.iadi.org/uploads/cprevised2014nov.pdf. !- Definitions and concepts: Covered (eligible) account: a deposit type included by law. Fully insured vs. partially insured: “Fully insured” balances are ≤ the coverage limit per depositor, per bank, per ownership category; “covered/eligible” may include accounts whose balances exceed the cap (partially insured). Ownership categories: individual, joint, trust/fiduciary, retirement—rules vary by jurisdiction and affect aggregation across accounts. Indicator variants: % Eligible accounts = eligible deposit accounts ÷ total deposit accounts. Insured balance share = insured amounts in eligible accounts ÷ total deposit balances in eligible accounts. Dormancy: dormant accounts may be treated differently in coverage statistics.</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>Are there gender disparities in the number of deposit accounts covered by direct deposit insurance? How do these disparities vary by age, income level, and geographic location? Are certain gender groups, especially within vulnerable or low-income populations, less likely to hold insured deposit accounts? How do the average insured deposit account balances differ across genders, and what might this indicate about savings behavior, access to financial protection, or economic security? Do financial service providers with higher levels of gender diversity in leadership or staff tend to offer more equitable access to insured deposit accounts and balanced coverage across genders? Additionally, how do gender differences in insured deposit accounts relate to broader financial inclusion and resilience against financial shocks?</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>Financial inclusion; Consumer protection</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>Quality, Suitability</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Deposit account type</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Consumer protection</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Depositor protection</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Savings</t>
+        </is>
+      </c>
+      <c r="D125">
         <v>16</v>
       </c>
-      <c r="E123" t="inlineStr">
+      <c r="E125" t="inlineStr">
         <is>
           <t>G2P accounts covered by deposit insurance</t>
         </is>
       </c>
-      <c r="F123" t="inlineStr">
+      <c r="F125" t="inlineStr">
         <is>
           <t>% of all accounts receiving G2P payments that are covered by deposit protection</t>
         </is>
       </c>
-      <c r="G123" t="inlineStr">
+      <c r="G125" t="inlineStr">
         <is>
           <t>This indicator helps analyze the extent to which low-value accounts are covered by deposit insurance or other protection. It focuses on account holders who are recipients of G2P programs. It quantifies how many of the government-to-person (G2P) payments recipients are protected by an explicit deposit insurance scheme or guarantee fund. It can be shown as (a) the share of G2P accounts that are eligible/fully insured and/or (b) the insured share of G2P balances. This indicator informs strategies for insurance/coverage payouts and the calibration of the deposit insurance fund. Definitions  and concepts: G2P account: an account that receives social transfers, government pensions, subsidies, or cash-benefit programs.
 Covered (eligible) vs. fully insured: “Eligible” products fall within the deposit insurance scope; “fully insured” means the balance per beneficiary per insured bank does not exceed the coverage cap. 
@@ -6949,664 +6950,549 @@
 Core-banking (and, where applicable, e-money) extracts: product code, ownership category, end-of-day balance, currency. Rules engine encoding national deposit-insurance scope, limits, and aggregation logic (per depositor—per bank). Sub-ledger data for pooled/FBO accounts to support pass-through eligibility. Timing sensitivity: balances spike on disbursement days; define the snapshot (e.g., month-end vs. T+2 after payout).</t>
         </is>
       </c>
-      <c r="H123" t="inlineStr">
+      <c r="H125" t="inlineStr">
         <is>
           <t>Are there gender disparities in the number of G2P accounts covered by deposit insurance? How do these disparities vary across different age groups, income levels, and geographic locations? Are women and other gender groups within vulnerable populations less likely to have G2P accounts that are insured, potentially affecting their financial security? How do the average balances of insured G2P accounts compare across genders, and what does this imply about economic empowerment and financial resilience? Do government programs and financial service providers with greater gender diversity in design or delivery show more equitable insurance coverage of G2P accounts? Additionally, how do gender differences in insured G2P accounts influence overall inclusion and access to social safety nets?</t>
         </is>
       </c>
-      <c r="I123" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J123" t="inlineStr">
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
         <is>
           <t>Financial inclusion; Consumer protection; Stability, safety and soundness</t>
         </is>
       </c>
-      <c r="K123" t="inlineStr">
-        <is>
-          <t>Quality, Suitability, Depositor protection</t>
-        </is>
-      </c>
-      <c r="L123" t="inlineStr">
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>Quality, Suitability, Stability</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
         </is>
       </c>
     </row>
-    <row r="124">
-      <c r="A124" t="inlineStr">
+    <row r="126">
+      <c r="A126" t="inlineStr">
         <is>
           <t>Consumer protection</t>
         </is>
       </c>
-      <c r="B124" t="inlineStr">
+      <c r="B126" t="inlineStr">
         <is>
           <t>Fair treatment</t>
         </is>
       </c>
-      <c r="C124" t="inlineStr">
+      <c r="C126" t="inlineStr">
         <is>
           <t>Credit</t>
         </is>
       </c>
-      <c r="D124">
+      <c r="D126">
         <v>183</v>
       </c>
-      <c r="E124" t="inlineStr">
+      <c r="E126" t="inlineStr">
         <is>
           <t>Average cost-to-borrower for unsecured retail lending</t>
         </is>
       </c>
-      <c r="F124" t="inlineStr">
+      <c r="F126" t="inlineStr">
         <is>
           <t>Average topline revenue earned from unsecured retail credit operations (as percentage of the average outstanding unsecured credit)</t>
         </is>
       </c>
-      <c r="G124" t="inlineStr">
+      <c r="G126" t="inlineStr">
         <is>
           <t>This indicator is a portfolio-level proxy for the all-in price actually paid by customers on unsecured retail credit during the period. It answers: How many currency units of revenue did the lender earn for each 100 units of average unpaid balance? Rising values may reflect higher base rates, heavier fee reliance (e.g., late/over-limit charges), or a shift toward shorter-tenor/high-yield products; falling values can indicate competitive pressure, promotional pricing, or relief programs. Boards, supervisors, and consumer-protection teams use it to benchmark pricing fairness, earnings quality, and sensitivity to interest-rate cycles. !- Definitions and concepts: Recommended numerator (topline revenue, P&amp;L-recognized): Interest income (EIR basis) + contractual fees (origination, servicing) + penalty/default interest actually recognized + punitive fees (late, over-limit, returned-payment) − waivers/reversals. Denominator: Average outstanding unsecured retail balances (use Average Daily Balance - ADB). Formula: Cost-to-customer yield = Topline revenue from unsecured retail credit divded by Average outstanding unsecured retail balances. This indicator can be reported separately for interest, contractual fees and penalities if the data is available and when the period is less than 12 months, report an annualized figure. !- Data requirements: General ledger and product-level revenue broken into interest, contractual fees, penalty interest, punitive fees; flags for waivers/reversals and non-accrual. Loan/card-level balances to compute ADB, segmented by product (cards, instalment, overdraft, BNPL), channel, and risk bucket. Accounting policies: EIR vs. cash, Stage-3/non-accrual treatment, capitalization rules.
 FX mapping for multi-currency portfolios. !- Limitations and considerations: Comparability: EIR vs. cash accounting and non-accrual practices differ; disclose methodology. Mix effects: more revolving/short-tenor loans inflate yields; always segment. Penalty bias: high ratios may be driven by a small cohort repeatedly paying fees—track % customers incurring penalties. Promotions/teasers: intro 0% and fee holidays distort short periods—show trailing-12-month and cohort views. Scope creep: exclude bundled insurance premiums or merchant discounts (BNPL) unless consistently included and disclosed.</t>
         </is>
       </c>
-      <c r="H124" t="inlineStr">
+      <c r="H126" t="inlineStr">
         <is>
           <t>Are there gender disparities in the percentage of topline revenue relative to outstanding loan balances? Is there any gender paying comparatively more than market percentages for the same account types? How do FSPs rank in terms of these percentages by gender?</t>
         </is>
       </c>
-      <c r="J124" t="inlineStr">
-        <is>
-          <t>Financial inclusion</t>
-        </is>
-      </c>
-      <c r="K124" t="inlineStr">
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>Financial inclusion</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
         <is>
           <t>Quality</t>
         </is>
       </c>
-      <c r="L124" t="inlineStr">
+      <c r="L126" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Loan type</t>
         </is>
       </c>
     </row>
-    <row r="125">
-      <c r="A125" t="inlineStr">
+    <row r="127">
+      <c r="A127" t="inlineStr">
         <is>
           <t>Consumer protection</t>
         </is>
       </c>
-      <c r="B125" t="inlineStr">
+      <c r="B127" t="inlineStr">
         <is>
           <t>Fair treatment</t>
         </is>
       </c>
-      <c r="C125" t="inlineStr">
+      <c r="C127" t="inlineStr">
         <is>
           <t>Credit</t>
         </is>
       </c>
-      <c r="D125">
+      <c r="D127">
         <v>181</v>
       </c>
-      <c r="E125" t="inlineStr">
+      <c r="E127" t="inlineStr">
         <is>
           <t>Revenue generated by unsecured credit</t>
         </is>
       </c>
-      <c r="F125" t="inlineStr">
+      <c r="F127" t="inlineStr">
         <is>
           <t>% of total topline revenue attributable to unsecured credit operations and interest and non-interest revenue proportions</t>
         </is>
       </c>
-      <c r="G125" t="inlineStr">
+      <c r="G127" t="inlineStr">
         <is>
           <t>This indicator captures the total income that a lending institution earns from unsecured credit products—credit cards, personal instalment loans, overdrafts, payday and buy-now-pay-later (BNPL) facilities—over a reporting period. Because unsecured lending is typically high-yield and high-risk, tracking its revenue helps supervisors and management understand how much of the institution’s top line depends on products that are more sensitive to economic downturns, job-market shocks and aggressive competition. A rising share can boost short-term profitability, but it may also presage higher future credit losses and conduct-risk concerns if underwriting standards slip. !- Definitions and concepts: Unsecured credit – loans that are not backed by collateral; repayment relies on the borrower’s cash flow and creditworthiness.
 Revenue components – Interest income (accrued and collected) from outstanding balances. Fee income: annual fees, origination fees, late-payment charges, interchange on card transactions, BNPL merchant discount rates. Net insurance or payment-protection premiums (if bundled) may be included subject to local accounting rules.
 Revenue share metric: Unsecured-credit revenue ÷ Total lending revenue expresses concentration risk. Risk-adjusted yield – revenue net of credit-loss provisions gives a clearer view of economic profitability. !- Data requirements: Product-level general-ledger extracts segregating interest, fees and other income. Loan-level flags identifying collateral status (secured vs. unsecured). Average daily or month-end balances to compute effective yields. Associated credit-loss provisions and write-offs for risk-adjusted analysis. !- Limitations and considerations: Mixed products: Some personal loans are partially secured (e.g., salary-linked) or carry optional collateral; clear taxonomy is essential. Fee recognition rules: Capitalised origination fees amortised under effective-interest-rate (EIR) accounting may blur timing comparisons across banks or jurisdictions. Regulatory caps: Interest-rate or fee ceilings (e.g., usury limits) affect revenue potential and comparability. Promotional pricing: Introductory 0 % card offers or BNPL “pay-in-4” models generate deferred revenue; headline figures may understate future income. Economic cyclicality: Unsecured-credit revenue can fall sharply in recessions as balances contract and charge-offs rise; pairing with delinquency and provision metrics is crucial for a full risk-return picture.</t>
         </is>
       </c>
-      <c r="H125" t="inlineStr">
+      <c r="H127" t="inlineStr">
         <is>
           <t>What proportion of total topline revenue comes from unsecured credit operations, and are there gender disparities in this distribution? How do FSPs rank in their reliance on unsecured credit revenue by gender?</t>
         </is>
       </c>
-      <c r="I125" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="L125" t="inlineStr">
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Loan type</t>
         </is>
       </c>
     </row>
-    <row r="126">
-      <c r="A126" t="inlineStr">
+    <row r="128">
+      <c r="A128" t="inlineStr">
         <is>
           <t>Consumer protection</t>
         </is>
       </c>
-      <c r="B126" t="inlineStr">
+      <c r="B128" t="inlineStr">
         <is>
           <t>Fair treatment</t>
         </is>
       </c>
-      <c r="C126" t="inlineStr">
+      <c r="C128" t="inlineStr">
         <is>
           <t>Insurance</t>
         </is>
       </c>
-      <c r="D126">
+      <c r="D128">
         <v>198</v>
       </c>
-      <c r="E126" t="inlineStr">
+      <c r="E128" t="inlineStr">
         <is>
           <t>Insurance approved claims not paid</t>
         </is>
       </c>
-      <c r="F126" t="inlineStr">
+      <c r="F128" t="inlineStr">
         <is>
           <t>% of approved/accepted claims that remain unpaid to customers</t>
         </is>
       </c>
-      <c r="G126" t="inlineStr">
+      <c r="G128" t="inlineStr">
         <is>
           <t>This indicator shows the share of claims that have been approved (final liability accepted) but not yet disbursed to the claimant. A high rate flags operational bottlenecks or weak payout controls, directly impacting customer outcomes. Track alongside claims turnaround time, claims rejection rates, and complaints, to get a full picture of payout effectiveness and customer fairness. !- Definitions and concepts: Approved / accepted claim: a claim with a final decision to pay (post-analysis), a recorded payable, and no outstanding dispute. Unpaid status: no successful settlement to the beneficiary by period end. Formula: Amount weighted (unpaid approved amount ÷ approved amount) reveal economic impact. Count basis (# approved claims not paid by cut-off ÷ # claims approved in teh period). SLA variant: % not paid within X days of approval (e.g., 5/10/30 days) to neutralize end-period timing bias. Treatment of partial payments: disclose whether partially paid claims are counted as unpaid or excluded. The indicator may also track the reasons for non-payment, if these are standardized for reporting. !- Limitations and considerations: Cut-off effects: approvals late in the period will naturally be unpaid—use the SLA variant and report both snapshot and flow views. Reopened claims / appeals: specify whether reversals after approval are removed from both numerator and denominator. Segmentation: monitor by line of business, payment method, channel, and claim size to target fixes.</t>
         </is>
       </c>
-      <c r="H126" t="inlineStr">
+      <c r="H128" t="inlineStr">
         <is>
           <t>How do the average values of outstanding insurance claims compare by gender? Is there a gender group with consistently higher average unpaid claims? How do different FSPs rank in terms of outstanding claims by gender? Are vulnerable gender groups disproportionately affected by delayed or unpaid claims?</t>
         </is>
       </c>
-      <c r="I126" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J126" t="inlineStr">
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
         <is>
           <t>Financial inclusion; Stability, safety and soundness</t>
         </is>
       </c>
-      <c r="K126" t="inlineStr">
+      <c r="K128" t="inlineStr">
         <is>
           <t>Quality, Reputational and legal risk</t>
         </is>
       </c>
-      <c r="L126" t="inlineStr">
+      <c r="L128" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Insurance type</t>
         </is>
       </c>
     </row>
-    <row r="127">
-      <c r="A127" t="inlineStr">
+    <row r="129">
+      <c r="A129" t="inlineStr">
         <is>
           <t>Consumer protection</t>
         </is>
       </c>
-      <c r="B127" t="inlineStr">
+      <c r="B129" t="inlineStr">
         <is>
           <t>Fair treatment</t>
         </is>
       </c>
-      <c r="C127" t="inlineStr">
+      <c r="C129" t="inlineStr">
         <is>
           <t>Insurance</t>
         </is>
       </c>
-      <c r="D127">
+      <c r="D129">
         <v>256</v>
       </c>
-      <c r="E127" t="inlineStr">
+      <c r="E129" t="inlineStr">
         <is>
           <t>Insurance claims declined</t>
         </is>
       </c>
-      <c r="F127" t="inlineStr">
+      <c r="F129" t="inlineStr">
         <is>
           <t>% of claims logged by policyholders that are declined prior to substantive analysis</t>
         </is>
       </c>
-      <c r="G127" t="inlineStr">
+      <c r="G129" t="inlineStr">
         <is>
           <t>This indicator captures the share of claim notifications the insurer does not accept for assessment at the front door—typically during first notice of loss (FNOL)/triage—because they are ineligible or incomplete. A high intake-decline rate can point to unclear policy wording, poor customer guidance, data-capture frictions, or overly strict gatekeeping. It is a key conduct-risk and customer-experience signal and, operationally, helps size avoidable workload versus genuinely assessable claims. Claim logged / FNOL: the moment a policyholder submits a claim or loss notice. Declined at intake (non-acceptance): the insurer refuses to open an assessable claim before investigation (e.g., policy not in force, peril not covered, waiting period, duplicate claim, claim below deductible/threshold, incomplete mandatory data not cured within a set window). Indicator formula (count basis): # claims declined at intake in period divided by # claim notifications received in period . Variants: exclude cured cases later resubmitted; report by product/channel. !- Data requirements: Claims-intake system fields: FNOL timestamp, policy ID/status at loss date, coverage/peril checks, deductible, mandatory-document checklist, triage outcome. Standardised reason codes (e.g., not covered, lapsed, duplicate, below excess, incomplete info). Deduplication logic (policyholder ID + incident date + peril). Linkage to resubmissions/appeals and to complaint records for outcome tracking. !- Limitations and considerations: Definition variance: what counts as “prior to analysis” differs; some firms place incomplete cases in “pending info” instead of “declined,” affecting comparability.
 Gaming risk: shifting cases to “withdrawn” or “pending” to improve this metric; require audit trails and age-off rules. Mix effects: products with low deductibles or mandatory documents (e.g., health) have different baseline rates—segment results. Customer fairness: high early declines may reflect confusing onboarding or exclusion wording; monitor alongside claims rejection rate (post-assessment), turnaround time, and complaints upheld. Resubmission policy: disclose whether cured resubmissions are excluded from the numerator to avoid double counting.</t>
         </is>
       </c>
-      <c r="H127" t="inlineStr">
+      <c r="H129" t="inlineStr">
         <is>
           <t>What percentage of claims logged by policyholders are declined, disaggregated by gender? How do these decline rates vary across FSPs, policy types, age groups, and locations? Are there notable gender disparities in claim declines at the market level or within specific providers? Are women or other gender groups more likely to face claim denial?</t>
         </is>
       </c>
-      <c r="I127" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J127" t="inlineStr">
-        <is>
-          <t>Financial inclusion; Stability, safety and soundness</t>
-        </is>
-      </c>
-      <c r="K127" t="inlineStr">
-        <is>
-          <t>Quality,</t>
-        </is>
-      </c>
-      <c r="L127" t="inlineStr">
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>Financial inclusion</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Insurance type</t>
         </is>
       </c>
     </row>
-    <row r="128">
-      <c r="A128" t="inlineStr">
+    <row r="130">
+      <c r="A130" t="inlineStr">
         <is>
           <t>Consumer protection</t>
         </is>
       </c>
-      <c r="B128" t="inlineStr">
+      <c r="B130" t="inlineStr">
         <is>
           <t>Fair treatment</t>
         </is>
       </c>
-      <c r="C128" t="inlineStr">
+      <c r="C130" t="inlineStr">
         <is>
           <t>Insurance</t>
         </is>
       </c>
-      <c r="D128">
+      <c r="D130">
         <v>60</v>
       </c>
-      <c r="E128" t="inlineStr">
+      <c r="E130" t="inlineStr">
         <is>
           <t>Insurance claims rejection rate</t>
         </is>
       </c>
-      <c r="F128" t="inlineStr">
+      <c r="F130" t="inlineStr">
         <is>
           <t>% of all insurance claims that are rejected by insurers (post-analysis)</t>
         </is>
       </c>
-      <c r="G128" t="inlineStr">
+      <c r="G130" t="inlineStr">
         <is>
           <t>The claims rejection rate shows the share of claims that an insurer declines to pay—fully or partially—relative to the total number (or value) of claims submitted in a period. Because denial directly affects customer trust, supervisors use the metric to monitor fair treatment outcomes, detect aggressive underwriting or opaque policy wording, and flag operational shortcomings. A sudden rise may presage reputational damage, regulatory sanctions, or litigation costs, while an unusually low rate can hint at lax fraud controls or inadequate claims processing. !- Definitions and concepts: Claims rejected (denied): claims for which the insurer issues a final communication refusing payment on contractual grounds (e.g., policy exclusions, lapsed cover, misrepresentation) or on fraud findings. !- Limitations and considerations: Definition divergence: Some regimes class “claims closed without payment” (due to missing documents) as rejections; others record them as pending, complicating cross-market comparison. Fraud vs. technical denial: Combining fraud rejections with contractual exclusions can blur very different issues. Separate reporting is best practice. Volume vs. value: A single large, legitimately denied loss can distort amount-based ratios; analysts should monitor both count and value metrics.
 Appeals and reversals: Denials overturned on review lower true rejection rates; timely data updates are essential.
 Incentive effects: Over-emphasis on low rejection rates may weaken fraud vigilance, whereas strict targets can push staff toward technical denials—pair the indicator with complaint ratios, turnaround times, and fraud-detection statistics for balanced oversight.</t>
         </is>
       </c>
-      <c r="H128" t="inlineStr">
+      <c r="H130" t="inlineStr">
         <is>
           <t>Are there gender disparities in the rejection rates of insurance claims, including for MSMEs by owner gender? Which types of policies or claims see higher rejection rates, and do these differ by gender? How does claim rejection relate to coverage levels and turnaround times? Do FSPs with higher gender diversity have lower rejection rates for vulnerable gender groups?</t>
         </is>
       </c>
-      <c r="I128" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J128" t="inlineStr">
-        <is>
-          <t>Financial inclusion</t>
-        </is>
-      </c>
-      <c r="K128" t="inlineStr">
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>Financial inclusion</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
         <is>
           <t>Quality</t>
         </is>
       </c>
-      <c r="L128" t="inlineStr">
+      <c r="L130" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Insurance type</t>
         </is>
       </c>
     </row>
-    <row r="129">
-      <c r="A129" t="inlineStr">
+    <row r="131">
+      <c r="A131" t="inlineStr">
         <is>
           <t>Consumer protection</t>
         </is>
       </c>
-      <c r="B129" t="inlineStr">
+      <c r="B131" t="inlineStr">
         <is>
           <t>Fair treatment</t>
         </is>
       </c>
-      <c r="C129" t="inlineStr">
+      <c r="C131" t="inlineStr">
         <is>
           <t>Insurance</t>
         </is>
       </c>
-      <c r="D129">
+      <c r="D131">
         <v>201</v>
       </c>
-      <c r="E129" t="inlineStr">
+      <c r="E131" t="inlineStr">
         <is>
           <t>Insurance claims settlement ratio</t>
         </is>
       </c>
-      <c r="F129" t="inlineStr">
+      <c r="F131" t="inlineStr">
         <is>
           <t>% of insurance claims logged by policyholders that have been paid by insurers</t>
         </is>
       </c>
-      <c r="G129" t="inlineStr">
+      <c r="G131" t="inlineStr">
         <is>
           <t>Measures the percentage of insurance claims settled by an insurer out of the total claims it receives. It is a direct measure of an insurer's reliability and its commitment to fulfilling its primary promise to policyholders. This indicator is a cornerstone of conduct supervision, as it provides a quantitative view of how an insurer treats its customers at their most critical moment of need. For prudential supervisors, it could help analysis of operational and reputational risk. This indicator should be used together with other indicators on the performance of the claims process in the insurance sector.</t>
         </is>
       </c>
-      <c r="H129" t="inlineStr">
+      <c r="H131" t="inlineStr">
         <is>
           <t>How do claim settlement ratios vary by gender? Are any gender groups receiving lower settlement ratios compared to the market average? Are there FSPs with particularly low or high settlement ratios for certain genders? How do these ratios intersect with policy type and customer demographics?</t>
         </is>
       </c>
-      <c r="I129" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J129" t="inlineStr">
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
         <is>
           <t>Financial inclusion; Stability, safety and soundness</t>
         </is>
       </c>
-      <c r="K129" t="inlineStr">
+      <c r="K131" t="inlineStr">
         <is>
           <t>Outcomes, Reputational and legal risk</t>
         </is>
       </c>
-      <c r="L129" t="inlineStr">
+      <c r="L131" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Insurance type</t>
         </is>
       </c>
     </row>
-    <row r="130">
-      <c r="A130" t="inlineStr">
+    <row r="132">
+      <c r="A132" t="inlineStr">
         <is>
           <t>Consumer protection</t>
         </is>
       </c>
-      <c r="B130" t="inlineStr">
+      <c r="B132" t="inlineStr">
         <is>
           <t>Fair treatment</t>
         </is>
       </c>
-      <c r="C130" t="inlineStr">
+      <c r="C132" t="inlineStr">
         <is>
           <t>Insurance</t>
         </is>
       </c>
-      <c r="D130">
+      <c r="D132">
         <v>59</v>
       </c>
-      <c r="E130" t="inlineStr">
+      <c r="E132" t="inlineStr">
         <is>
           <t>Insurance claims turnaround time</t>
         </is>
       </c>
-      <c r="F130" t="inlineStr">
+      <c r="F132" t="inlineStr">
         <is>
           <t>Average number of days to process insurance claims</t>
         </is>
       </c>
-      <c r="G130" t="inlineStr">
+      <c r="G132" t="inlineStr">
         <is>
           <t>This indicator captures the average calendar days an insurer takes to settle a claim—from the claim filing date to the final payment or formal denial. It is a direct yard-stick of operational efficiency and customer experience. Shorter turnaround times (TATs) enhance policy-holder trust, limit reputational risk, and can lower claims handling expenses. Supervisors use the metric to enforce fair-treatment rules, while actuaries and underwriters link it to reserving accuracy—prolonged settlement can signal documentation bottlenecks, fraud investigations, policy transparency issues, or catastrophic complexity that may keep outstanding reserves elevated. !- Definitions and concepts:  Start point – the timestamp when the insurer first receives the claim request. End point – the date the insurer issues full payment, partial final payment, or a written denial. Average turnaround time (TAT) – arithmetic mean; many firms also monitor median and 90th-percentile to limit outlier masking.
 Segmented TATs – tracked by line of business, claim severity band, and distribution channel to isolate problem areas.
 !- Limitations and considerations: Partial settlements: Recording the date of first partial payment can understate full-and-final completion time. Dispute and litigation pauses: Regulatory or court‐mandated suspensions inflate TAT yet lie outside managerial control.</t>
         </is>
       </c>
-      <c r="H130" t="inlineStr">
+      <c r="H132" t="inlineStr">
         <is>
           <t>Are there gender disparities in the average time taken to process and settle insurance claims? How does processing time vary by policy type, premium, claim amount, and customer demographics? Are insurers with lower gender diversity more likely to have longer turnaround times? Are vulnerable gender groups disproportionately affected by delays?</t>
         </is>
       </c>
-      <c r="J130" t="inlineStr">
-        <is>
-          <t>Financial inclusion</t>
-        </is>
-      </c>
-      <c r="K130" t="inlineStr">
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>Financial inclusion</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
         <is>
           <t>Quality</t>
         </is>
       </c>
-      <c r="L130" t="inlineStr">
+      <c r="L132" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Insurance type</t>
         </is>
       </c>
     </row>
-    <row r="131">
-      <c r="A131" t="inlineStr">
+    <row r="133">
+      <c r="A133" t="inlineStr">
         <is>
           <t>Consumer protection</t>
         </is>
       </c>
-      <c r="B131" t="inlineStr">
+      <c r="B133" t="inlineStr">
         <is>
           <t>Fair treatment</t>
         </is>
       </c>
-      <c r="C131" t="inlineStr">
+      <c r="C133" t="inlineStr">
         <is>
           <t>Investments</t>
         </is>
       </c>
-      <c r="D131">
+      <c r="D133">
         <v>207</v>
       </c>
-      <c r="E131" t="inlineStr">
+      <c r="E133" t="inlineStr">
         <is>
           <t>Net rate of return on investments</t>
         </is>
       </c>
-      <c r="F131" t="inlineStr">
+      <c r="F133" t="inlineStr">
         <is>
           <t>% point differential between the average rates of returns on investments and the average performance/administration fees charged</t>
         </is>
       </c>
-      <c r="G131" t="inlineStr">
+      <c r="G133" t="inlineStr">
         <is>
           <t>Measures the profitability of a financial institution's own investment portfolio after accounting for all associated costs. It reveals the actual, bottom-line gain or loss generated by the institution's securities, real estate, or other investments. This is a fundamental indicator of an institution's ability to effectively manage its own capital and generate profit from non-lending activities, of particular importance to prudential supervisors, including supervisors of insurance and pension administrators. Net Rate of Return (%)= 
 [(Market Value final-Market Value initial+Income−Expenses)/Market Value initial]×100</t>
         </is>
       </c>
-      <c r="H131" t="inlineStr">
+      <c r="H133" t="inlineStr">
         <is>
           <t>How do net returns (% returns minus % performance fees and charges) on longer-term investments compare by gender? Do net returns for any gender differ from the overall market average for similar investment products? How do FSPs compare in terms of net returns earned by gender?</t>
         </is>
       </c>
-      <c r="J131" t="inlineStr">
+      <c r="J133" t="inlineStr">
         <is>
           <t>Market development</t>
         </is>
       </c>
-      <c r="K131" t="inlineStr">
+      <c r="K133" t="inlineStr">
         <is>
           <t>Capital markets development</t>
         </is>
       </c>
-      <c r="L131" t="inlineStr">
+      <c r="L133" t="inlineStr">
         <is>
           <t>Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
         </is>
       </c>
     </row>
-    <row r="132">
-      <c r="A132" t="inlineStr">
+    <row r="134">
+      <c r="A134" t="inlineStr">
         <is>
           <t>Consumer protection</t>
         </is>
       </c>
-      <c r="B132" t="inlineStr">
+      <c r="B134" t="inlineStr">
         <is>
           <t>Fair treatment</t>
         </is>
       </c>
-      <c r="C132" t="inlineStr">
+      <c r="C134" t="inlineStr">
         <is>
           <t>Savings</t>
         </is>
       </c>
-      <c r="D132">
+      <c r="D134">
         <v>159</v>
       </c>
-      <c r="E132" t="inlineStr">
+      <c r="E134" t="inlineStr">
         <is>
           <t>Average cost-to-customer for transaction accounts</t>
         </is>
       </c>
-      <c r="F132" t="inlineStr">
+      <c r="F134" t="inlineStr">
         <is>
           <t>Average topline revenue earned per account holder as % of average account balances</t>
         </is>
       </c>
-      <c r="G132" t="inlineStr">
+      <c r="G134" t="inlineStr">
         <is>
           <t>This indicator estimates the effective price of holding and using a transaction account, expressed as a yield on the customer’s average balance. By computing it for each account type (e.g., basic/no-frills, standard retail, premium, SME, e-money wallet), it reveals where pricing and usage frictions are highest. It helps supervisors assess fairness, inclusion quality, and reliance on fee income. !- Definitions and concepts: Non-interest fees: maintenance/inactivity, ATM/network, FX/transfer, statement/card fees, overdraft &amp; returned-payment fees tied to the account. 
 Per account-holder basis: aggregate all accounts of the same type per customer, then average (also show balance-weighted results). !- Data requirements: Core-banking data: customer ID, account type tags, average daily balance by customer for each account type, interest credited, revenue by fee code linked to accounts; flags for waivers/refunds/chargebacks. Channel/product hierarchies (basic vs. premium, retail vs. SME, wallet vs. bank account) and currency/FX mapping. Optional: usage indicators (transactions per month) to explain differences across types.</t>
         </is>
       </c>
-      <c r="H132" t="inlineStr">
+      <c r="H134" t="inlineStr">
         <is>
           <t>Are there gender disparities in the costs (fees, charges) borne by account holders of transaction accounts? Do women tend to hold transaction accounts with higher fee burdens (relative to income or transaction frequency) than men, particularly in certain regions or among lower‐income groups? How do costs compare across FSPs with different levels of gender diversity? Is fee structure or cost‐to‐customer a barrier to transaction usage for some gender/age/income cohorts?</t>
         </is>
       </c>
-      <c r="J132" t="inlineStr">
-        <is>
-          <t>Financial inclusion</t>
-        </is>
-      </c>
-      <c r="K132" t="inlineStr">
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>Financial inclusion</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
         <is>
           <t>Quality</t>
         </is>
       </c>
-      <c r="L132" t="inlineStr">
+      <c r="L134" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Financial service provider (FSP) type; Account type</t>
-        </is>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" t="inlineStr">
-        <is>
-          <t>Consumer protection</t>
-        </is>
-      </c>
-      <c r="B133" t="inlineStr">
-        <is>
-          <t>Fair treatment</t>
-        </is>
-      </c>
-      <c r="C133" t="inlineStr">
-        <is>
-          <t>Payments, Savings, Credit, Insurance, Pensions, Investments</t>
-        </is>
-      </c>
-      <c r="D133">
-        <v>226</v>
-      </c>
-      <c r="E133" t="inlineStr">
-        <is>
-          <t>Rejections of product applications</t>
-        </is>
-      </c>
-      <c r="F133" t="inlineStr">
-        <is>
-          <t>% of all applications that are rejected by product type</t>
-        </is>
-      </c>
-      <c r="G133" t="inlineStr">
-        <is>
-          <t>Measures the proportion of customer applications for financial products that are rejected by regulated financial institutions during the reporting period. The indicator is calculated as the percentage of total applications received—across products such as loans, credit cards, deposit accounts, or insurance policies—that were not approved or accepted. Captures the extent of unmet demand or access barriers in financial markets, as well as aspects of market conduct, underwriting practices, and risk appetite among providers. It provides insight into how easily consumers and businesses can obtain financial products. Monitoring rejection rates helps authorities: Identify potential access constraints or discriminatory lending or sales practices; Evaluate the tightness of credit or account-opening standards; Assess consumer protection outcomes and fair treatment; Detect sudden shifts in provider risk tolerance or macro-prudential conditions (e.g., post-crisis credit tightening). High rejection rates may indicate stringent eligibility criteria, weak applicant creditworthiness, or barriers to financial access. Declining rates may suggest improving inclusion or relaxation of underwriting standards. Cross-product comparisons reveal whether certain markets (e.g., credit vs. deposits) are more exclusionary. !- Definitions and concepts: Application: A formal request by a customer to obtain a financial product or service. Rejection: A decision by the provider not to approve, issue, or open the requested product, whether automated or manual. Product type: Category of financial service applied for (loan, deposit, insurance, card, etc.). !- Data requirements: Product application records from regulated financail institutions that can yield the total number of applications rejected and the total number of applications received during the reference period. Disaggregation variables for segmentation analysis: product type, applicant type (individual, MSME), gender etc.</t>
-        </is>
-      </c>
-      <c r="H133" t="inlineStr">
-        <is>
-          <t>How do rejection rates vary by gender? Are rejection rates higher for any gender in specific channels? How do rejection rates in physical channels compare to those in digital channels by gender? How do FSPs rank in terms of rejection rates by gender across available channels? For loans, when analyzed alongside the indicator "Customers by credit score," are there gender disparities in rejection rates by credit score?</t>
-        </is>
-      </c>
-      <c r="I133" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J133" t="inlineStr">
-        <is>
-          <t>Financial inclusion</t>
-        </is>
-      </c>
-      <c r="K133" t="inlineStr">
-        <is>
-          <t>Quality</t>
-        </is>
-      </c>
-      <c r="L133" t="inlineStr">
-        <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Product type</t>
-        </is>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" t="inlineStr">
-        <is>
-          <t>Consumer protection</t>
-        </is>
-      </c>
-      <c r="B134" t="inlineStr">
-        <is>
-          <t>Impact</t>
-        </is>
-      </c>
-      <c r="C134" t="inlineStr">
-        <is>
-          <t>Credit</t>
-        </is>
-      </c>
-      <c r="D134">
-        <v>175</v>
-      </c>
-      <c r="E134" t="inlineStr">
-        <is>
-          <t>Payroll loans</t>
-        </is>
-      </c>
-      <c r="F134" t="inlineStr">
-        <is>
-          <t>% of all retail borrowers (or loans) that have payroll loans (repayments deducted directly of wages deposited into the customer's account)</t>
-        </is>
-      </c>
-      <c r="G134" t="inlineStr">
-        <is>
-          <t>Measures the prevalence of payroll lending in the retail loan portfolio. !- Definitions and concepts: A payroll loan (also called a payroll-deducted loan, salary loan) is a personal consumer loan whose installments are automatically withheld from the borrower’s pay-check (or pension/social-security benefit) and remitted directly to the lender each pay period. Because repayment is taken “off the top” of the employee’s gross salary, the borrower’s future income effectively serves as collateral, giving lenders high repayment certainty and allowing them to charge lower rates than on unsecured personal loans. !- Data requirements:  Loan-level records with ability to identify payroll loans (e.g. product code or terms of loan that specify the repayment modality). Unique customer ID in order to extract unique number of borrowers with payroll loans.</t>
-        </is>
-      </c>
-      <c r="H134" t="inlineStr">
-        <is>
-          <t>Are there gender disparities in the share of retail borrowers accessing payroll loans, and how do these differences vary by age, income, and location? Do women or other gender groups have equal access to payroll loan products compared to men, or are there structural or employment-related barriers affecting uptake? How does the prevalence of payroll loans among borrowers relate to their employment types and sectors, and are certain gender groups more represented in these segments? Are financial service providers with greater gender diversity more likely to offer payroll loans equitably across genders? How do repayment behaviors and default rates on payroll loans differ by gender, and what implications does this have for financial inclusion and debt sustainability?</t>
-        </is>
-      </c>
-      <c r="J134" t="inlineStr">
-        <is>
-          <t>Financial inclusion</t>
-        </is>
-      </c>
-      <c r="K134" t="inlineStr">
-        <is>
-          <t>Uptake (account ownership)</t>
-        </is>
-      </c>
-      <c r="L134" t="inlineStr">
-        <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Loan type; Loan size; Loan term; Interest rate category</t>
         </is>
       </c>
     </row>
@@ -7618,36 +7504,35 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Impact</t>
+          <t>Fair treatment</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Credit</t>
+          <t>Payments, Savings, Credit, Insurance, Pensions, Investments</t>
         </is>
       </c>
       <c r="D135">
-        <v>172</v>
+        <v>226</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>First-time borrowers</t>
+          <t>Rejections of product applications</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>% of borrowers who are first-time borrowers with the FSP (or in the financial system)</t>
+          <t>% of all applications that are rejected by product type</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>This indicator shows the share of active borrowing retail customers who are new to the lender (new-to-bank/FSP) or new to formal credit altogether (new-to-credit, NTC). It is a direct barometer of financial inclusion and retail credit growth. A higher share can signal effective onboarding and market expansion, but it also shifts portfolio risk: NTC borrowers may lack repayment histories, making underwriting more model-driven and subject to greater uncertainty. Supervisors and lenders can monitor this metric to balance inclusion objectives with prudent risk management and to evaluate the effectiveness of credit-bureau coverage. !- Definitions and concepts: First-time borrower (FSP scope): a customer with no prior loan or credit line ever booked by the FSP before the reference period. First-time borrower (system scope / NTC): a customer with no prior loan or credit line reported to the national credit registry/bureau within a defined historical look-back (commonly “ever,” or a long horizon such as 5–10 years). This indicator is obtained by dividing the number of first-time borrowers by the total number of borrowers. Variants of this indicator include: value-weighted (by origination amount), new originations only (versus the entire active book), and cohort-based analysis (by origination month or quarter). !- Data requirements: Customer master records with unique, reliable identifiers (national ID/tax ID; deduplicated across branches). Loan-booking history from the FSP’s core systems. Credit-bureau/registry match results (for system-wide NTC status). Product taxonomy (include/exclude credit cards, overdrafts, BNPL) and reference dates. Limitaitons and considerations: Coverage gaps: thin or partial bureau coverage, informal lenders, or non-reporting segments can misclassify NTC status.
-Identifier quality: name changes, multiple IDs, or data-entry errors cause false “first-time” flags; robust deduplication is essential. Look-back window choice: shorter windows inflate “first-time” shares; disclose methodology. Product scope: excluding revolving credit or microloans biases results.</t>
+          <t>Measures the proportion of customer applications for financial products that are rejected by regulated financial institutions during the reporting period. The indicator is calculated as the percentage of total applications received—across products such as loans, credit cards, deposit accounts, or insurance policies—that were not approved or accepted. Captures the extent of unmet demand or access barriers in financial markets, as well as aspects of market conduct, underwriting practices, and risk appetite among providers. It provides insight into how easily consumers and businesses can obtain financial products. Monitoring rejection rates helps authorities: Identify potential access constraints or discriminatory lending or sales practices; Evaluate the tightness of credit or account-opening standards; Assess consumer protection outcomes and fair treatment; Detect sudden shifts in provider risk tolerance or macro-prudential conditions (e.g., post-crisis credit tightening). High rejection rates may indicate stringent eligibility criteria, weak applicant creditworthiness, or barriers to financial access. Declining rates may suggest improving inclusion or relaxation of underwriting standards. Cross-product comparisons reveal whether certain markets (e.g., credit vs. deposits) are more exclusionary. !- Definitions and concepts: Application: A formal request by a customer to obtain a financial product or service. Rejection: A decision by the provider not to approve, issue, or open the requested product, whether automated or manual. Product type: Category of financial service applied for (loan, deposit, insurance, card, etc.). !- Data requirements: Product application records from regulated financail institutions that can yield the total number of applications rejected and the total number of applications received during the reference period. Disaggregation variables for segmentation analysis: product type, applicant type (individual, MSME), gender etc.</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>Do first-time borrowers reflect a balanced gender representation, or are there gender disparities? How do FSPs rank in onboarding typically underserved borrowers, and does this ranking change when analyzed by gender?</t>
+          <t>How do rejection rates vary by gender? Are rejection rates higher for any gender in specific channels? How do rejection rates in physical channels compare to those in digital channels by gender? How do FSPs rank in terms of rejection rates by gender across available channels? For loans, when analyzed alongside the indicator "Customers by credit score," are there gender disparities in rejection rates by credit score?</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -7662,12 +7547,12 @@
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>Uptake (account ownership)</t>
+          <t>Quality</t>
         </is>
       </c>
       <c r="L135" t="inlineStr">
         <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Product type</t>
         </is>
       </c>
     </row>
@@ -7679,7 +7564,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Suitability, Impact</t>
+          <t>Suitability</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -9375,12 +9260,12 @@
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>Financial inclusion; Consumer protection; Stability, safety and soundness</t>
+          <t>Financial inclusion; Consumer protection</t>
         </is>
       </c>
       <c r="K164" t="inlineStr">
         <is>
-          <t>Outcomes, Suitability, Credit risk</t>
+          <t>Outcomes, Suitability</t>
         </is>
       </c>
       <c r="L164" t="inlineStr">
@@ -9435,12 +9320,12 @@
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>Financial inclusion; Consumer protection; Stability, safety and soundness</t>
+          <t>Financial inclusion; Consumer protection</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
         <is>
-          <t>Quality, Suitability,</t>
+          <t>Quality, Suitability</t>
         </is>
       </c>
       <c r="L165" t="inlineStr">
@@ -9495,12 +9380,12 @@
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>Financial inclusion; Consumer protection; Stability, safety and soundness</t>
+          <t>Financial inclusion; Consumer protection</t>
         </is>
       </c>
       <c r="K166" t="inlineStr">
         <is>
-          <t>Quality, Suitability,</t>
+          <t>Quality, Suitability</t>
         </is>
       </c>
       <c r="L166" t="inlineStr">
@@ -9550,12 +9435,12 @@
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>Financial inclusion; Consumer protection; Stability, safety and soundness</t>
+          <t>Consumer protection</t>
         </is>
       </c>
       <c r="K167" t="inlineStr">
         <is>
-          <t>Outcomes, Safety and security, Credit risk</t>
+          <t>Safety and security</t>
         </is>
       </c>
       <c r="L167" t="inlineStr">
@@ -9605,12 +9490,12 @@
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>Financial inclusion; Consumer protection; Stability, safety and soundness</t>
+          <t>Financial inclusion; Consumer protection</t>
         </is>
       </c>
       <c r="K168" t="inlineStr">
         <is>
-          <t>Outcomes, Suitability, Credit risk</t>
+          <t>Outcomes, Suitability</t>
         </is>
       </c>
       <c r="L168" t="inlineStr">
@@ -9665,12 +9550,12 @@
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>Financial inclusion; Consumer protection; Stability, safety and soundness</t>
+          <t>Financial inclusion; Consumer protection</t>
         </is>
       </c>
       <c r="K169" t="inlineStr">
         <is>
-          <t>Outcomes, Suitability, Credit risk, Soundness, Stability</t>
+          <t>Outcomes, Suitability</t>
         </is>
       </c>
       <c r="L169" t="inlineStr">
@@ -9806,16 +9691,6 @@
       <c r="H172" t="inlineStr">
         <is>
           <t>Is there a correlation between higher levels of gender diversity in FSPs and lower risk levels?</t>
-        </is>
-      </c>
-      <c r="J172" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="K172" t="inlineStr">
-        <is>
-          <t>Statistics and research</t>
         </is>
       </c>
       <c r="L172" t="inlineStr">
@@ -10092,7 +9967,7 @@
       </c>
       <c r="K177" t="inlineStr">
         <is>
-          <t>Quality,Suitability</t>
+          <t>Quality, Suitability</t>
         </is>
       </c>
       <c r="L177" t="inlineStr">
@@ -10531,16 +10406,6 @@
           <t>Do financial service providers (FSPs) with higher gender diversity in leadership or governance report different interest margin ratios compared to less gender‑diverse peers? Are there associations between the gender composition of the customer base (e.g. share of women borrowers/depositors) and margin outcomes? Could gendered pricing—such as differential rates offered to male vs. female clients—impact FSP interest margins? Over time, do changes in margin ratios correlate with shifts in gender inclusion (e.g. more women customers or staff)?</t>
         </is>
       </c>
-      <c r="J186" t="inlineStr">
-        <is>
-          <t>Consumer protection</t>
-        </is>
-      </c>
-      <c r="K186" t="inlineStr">
-        <is>
-          <t>Impact</t>
-        </is>
-      </c>
       <c r="L186" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
@@ -10588,12 +10453,12 @@
       </c>
       <c r="J187" t="inlineStr">
         <is>
-          <t>Financial inclusion; Other</t>
+          <t>Financial inclusion</t>
         </is>
       </c>
       <c r="K187" t="inlineStr">
         <is>
-          <t>Outcomes, Statistics and research</t>
+          <t>Outcomes</t>
         </is>
       </c>
       <c r="L187" t="inlineStr">
@@ -10745,7 +10610,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Soundness</t>
+          <t>Soundness, Credit risk</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
@@ -10774,16 +10639,6 @@
       <c r="H191" t="inlineStr">
         <is>
           <t>Is there a relationship between gender diversity in leadership or equity ownership and ROE performance across FSPs? Are FSPs that prioritize gender inclusion more likely to achieve higher equity returns, possibly through broader market reach or more balanced risk management? How does the gender mix of customers, especially depositors and borrowers, relate to ROE outcomes? Over time, do improvements in gender inclusion (in staffing or customer base) precede or follow changes in ROE?</t>
-        </is>
-      </c>
-      <c r="J191" t="inlineStr">
-        <is>
-          <t>Other; Consumer protection; Stability, safety and soundness</t>
-        </is>
-      </c>
-      <c r="K191" t="inlineStr">
-        <is>
-          <t>Statistics and research, Impact, Credit risk</t>
         </is>
       </c>
       <c r="L191" t="inlineStr">
@@ -11070,12 +10925,12 @@
       </c>
       <c r="J197" t="inlineStr">
         <is>
-          <t>Other; Stability, safety and soundness</t>
+          <t>Stability, safety and soundness</t>
         </is>
       </c>
       <c r="K197" t="inlineStr">
         <is>
-          <t>Statistics and research, Credit risk, Stability</t>
+          <t>Credit risk, Stability</t>
         </is>
       </c>
       <c r="L197" t="inlineStr">
@@ -11235,12 +11090,12 @@
       </c>
       <c r="J200" t="inlineStr">
         <is>
-          <t>Financial inclusion; Other; Stability, safety and soundness</t>
+          <t>Financial inclusion</t>
         </is>
       </c>
       <c r="K200" t="inlineStr">
         <is>
-          <t>Uptake, Statistics and research, Impact</t>
+          <t>Uptake (account ownership)</t>
         </is>
       </c>
       <c r="L200" t="inlineStr">
@@ -11295,12 +11150,12 @@
       </c>
       <c r="J201" t="inlineStr">
         <is>
-          <t>Financial inclusion; Consumer protection</t>
+          <t>Financial inclusion</t>
         </is>
       </c>
       <c r="K201" t="inlineStr">
         <is>
-          <t>Uptake, Impact</t>
+          <t>Uptake (account ownership)</t>
         </is>
       </c>
       <c r="L201" t="inlineStr">
@@ -11355,12 +11210,12 @@
       </c>
       <c r="J202" t="inlineStr">
         <is>
-          <t>Financial inclusion; Consumer protection</t>
+          <t>Financial inclusion</t>
         </is>
       </c>
       <c r="K202" t="inlineStr">
         <is>
-          <t>Usage, Impact</t>
+          <t>Usage</t>
         </is>
       </c>
       <c r="L202" t="inlineStr">
@@ -11410,12 +11265,12 @@
       </c>
       <c r="J203" t="inlineStr">
         <is>
-          <t>Financial inclusion; Other</t>
+          <t>Financial inclusion</t>
         </is>
       </c>
       <c r="K203" t="inlineStr">
         <is>
-          <t>Usage, Statistics and research</t>
+          <t>Usage</t>
         </is>
       </c>
       <c r="L203" t="inlineStr">
@@ -11463,16 +11318,6 @@
           <t>Are there gender disparities in the acquisition/holding of green/sustainable bonds? Are FSPs with higher levels of gender diversity more likely to distribute sustainable or green bonds to a more diverse investor base?  Comparing this with gender diversity at FSPs, are institutions with higher levels of gender diversity more likely to have larger green/sustainable portfolios?</t>
         </is>
       </c>
-      <c r="J204" t="inlineStr">
-        <is>
-          <t>Other; Market development</t>
-        </is>
-      </c>
-      <c r="K204" t="inlineStr">
-        <is>
-          <t>Statistics and research, Sustainability</t>
-        </is>
-      </c>
       <c r="L204" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
@@ -11520,12 +11365,12 @@
       </c>
       <c r="J205" t="inlineStr">
         <is>
-          <t>Financial inclusion; Other; Market development</t>
+          <t>Financial inclusion</t>
         </is>
       </c>
       <c r="K205" t="inlineStr">
         <is>
-          <t>Usage, Statistics and research, Sustainability</t>
+          <t>Usage</t>
         </is>
       </c>
       <c r="L205" t="inlineStr">
@@ -11628,11 +11473,6 @@
           <t>Are there gender disparities in workforce participation across different types of FSPs? At what responsibility levels? How does gender diversity in FSP management correlate with key financial indicators (e.g., Stability, Financial Inclusion, Customer Protection, Sustainability)? Comparing with climate-related financial data (e.g., green loan portfolios, green insurance), does gender diversity in FSPs correlate with the growth of these portfolios? If legal or regulatory gender equity requirements exist for FSPs, are they being met? Does gender diversity correlate with variations in supervisory risk scores? How does gender diversity correlate with staff turnover (if data is available)? How does gender diversity correlate with enforcement and other supervisory actions?</t>
         </is>
       </c>
-      <c r="J207" t="inlineStr">
-        <is>
-          <t>Financial inclusion; Consumer protection; Stability, safety and soundness; Market development</t>
-        </is>
-      </c>
       <c r="L207" t="inlineStr">
         <is>
           <t>Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
@@ -11678,11 +11518,6 @@
           <t>Are there significant gender disparities in the composition of customers across different types of financial service providers (FSPs)? How does the gender diversity of the FSP customer base vary by institution size, sector, and geographic region? What correlations exist between the gender diversity of the customer base and key financial inclusion metrics such as account ownership, loan uptake, and insurance coverage? How does greater gender diversity among customers relate to customer protection outcomes, including complaint resolution and fair treatment? Are FSPs with more gender-diverse customer bases also demonstrating stronger prudential performance and sustainability indicators? How do gender disparities in the customer base influencefinancila outcomes such as Financial Health? And broader social and economic outcomes, such as women's economic empowerment, MSME growth, climate change, jobs creation or poverty reduction?</t>
         </is>
       </c>
-      <c r="J208" t="inlineStr">
-        <is>
-          <t>Financial inclusion; Consumer protection; Stability, safety and soundness; Market development</t>
-        </is>
-      </c>
       <c r="L208" t="inlineStr">
         <is>
           <t>Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
@@ -11728,11 +11563,6 @@
           <t>Are there gender disparities in compensation for similar positions or responsibilities (Board, management, staff)? How does this compare with other macro indicators related to financial stability and portfolio performance across FSPs (credit, insurance, investment funds, pensions)? Are FSPs with greater gender diversity in the Board more likely to present lower gender pay gap?</t>
         </is>
       </c>
-      <c r="J209" t="inlineStr">
-        <is>
-          <t>Financial inclusion; Consumer protection; Stability, safety and soundness; Market development</t>
-        </is>
-      </c>
       <c r="L209" t="inlineStr">
         <is>
           <t>Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
@@ -11779,11 +11609,6 @@
           <t>How do financial service providers (FSPs) compare in their Human Resources Gender Index (HRGI) scores? Are FSPs with higher levels of gender diversity in their workforce more likely to perform better across the various HRGI dimensions, such as recruitment, retention, promotion, and leadership representation? When comparing HRGI scores with key performance indicators (e.g., capital and liquidity, profitability, efficiency, customer satisfaction, innovation), is there evidence of a positive correlation? How do HRGI scores vary by FSP type, size, or region, and what best practices can be identified from top performers? How does HRGI performance relate to gender-related outcomes, such as gender-balanced customer bases or inclusive product offerings?</t>
         </is>
       </c>
-      <c r="J210" t="inlineStr">
-        <is>
-          <t>Financial inclusion; Consumer protection; Stability, safety and soundness; Market development</t>
-        </is>
-      </c>
       <c r="L210" t="inlineStr">
         <is>
           <t>Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
@@ -11807,36 +11632,26 @@
         </is>
       </c>
       <c r="D211">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>New licenses granted to diverse FSPs</t>
+          <t>Success rate of license applications by diverse FSPs</t>
         </is>
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t>% of all new licenses that are issued to diverse FSPs</t>
+          <t>% of all license applications by diverse FSPs that are issued</t>
         </is>
       </c>
       <c r="G211" t="inlineStr">
         <is>
-          <t>This indicator is a measure of the gender composition of newly licensed financial institutions. It helps regulators and policy makers identify trends in the gender diversity in the financial sector by looking at the leadership of financial institutions. For fuller more complete analysis, this indicator can be complemented by an indicator of the success rate of licensing applications, considering the gender of the lead sponsor.</t>
+          <t>This indicator is a measure of potential gender biases in licensing decisions by the financial authority. It helps authorities analyze the success rate of license pplications by segmenting applications by their final oucome (rejection/approval), and the gender of the lead sponsor of the application (e.g., the majority individual shareholder). The definition of lead sponsor will vary across countries and the indicator should align with local practices.</t>
         </is>
       </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>What are the trends in the number of new licenses issued to diverse FSPs?</t>
-        </is>
-      </c>
-      <c r="J211" t="inlineStr">
-        <is>
-          <t>Other; Stability, safety and soundness</t>
-        </is>
-      </c>
-      <c r="K211" t="inlineStr">
-        <is>
-          <t>Statistics and research,  Stability</t>
+          <t>To what extent does the gender of individuals in leadership or control positions within the proposed FSPs influence the likelihood of obtaining a license from the regulatory authority?</t>
         </is>
       </c>
       <c r="L211" t="inlineStr">
@@ -11848,45 +11663,55 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>Sustainability</t>
+          <t>Market development</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Gender equality</t>
+          <t>Capital markets development</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>Payments, Savings, Credit, Insurance, Pensions, Investments</t>
+          <t>Investments</t>
         </is>
       </c>
       <c r="D212">
-        <v>13</v>
+        <v>45</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>Success rate of license applications by diverse FSPs</t>
+          <t>Crowdfunding - Differential rate of return (equity)</t>
         </is>
       </c>
       <c r="F212" t="inlineStr">
         <is>
-          <t>% of all license applications by diverse FSPs that are issued</t>
+          <t>Difference between the advertised/promised rate of return and the actual rate of return of equity in crowdfunding projects</t>
         </is>
       </c>
       <c r="G212" t="inlineStr">
         <is>
-          <t>This indicator is a measure of potential gender biases in licensing decisions by the financial authority. It helps authorities analyze the success rate of license pplications by segmenting applications by their final oucome (rejection/approval), and the gender of the lead sponsor of the application (e.g., the majority individual shareholder). The definition of lead sponsor will vary across countries and the indicator should align with local practices.</t>
+          <t>Measures the gap between the projected or advertised rate of return presented to investors before a project is funded and the actual rate of return realized after the project is completed. This is a critical conduct indicator that measures the accuracy of a project's promises versus its real-world performance. For investors, this metric is a tool for due diligence. For conduct supervisors, it can be used to detect mis-selling and fraud. A large and persistent negative differential (where actual returns are consistently far below promised returns) is a red flag. it could flag issues such as inadequate risk disclosure and fraud. When gender disaggregated by the gender of the main sponsor or lead executive, the indicator can provide additional information. If projects led by women consistently show a smaller negative "reality gap" (meaning their actual returns are closer to their promised returns), it could suggest they are more conservative or accurate in their financial projections. This would be a crucial data point in assessing risk and investor protection. Using this indicator together with the indicator on rejected crowddfunding projects could strenghten the identification of gender bias inside the securities authority. Return Differential (%) = Actual Rate of Return - Advertised/Promised Rate of Return.</t>
         </is>
       </c>
       <c r="H212" t="inlineStr">
         <is>
-          <t>To what extent does the gender of individuals in leadership or control positions within the proposed FSPs influence the likelihood of obtaining a license from the regulatory authority?</t>
+          <t>Are there differences in the rates of return for crowdfunding projects depending on the gender assigned to the MSME seeking funding?</t>
+        </is>
+      </c>
+      <c r="J212" t="inlineStr">
+        <is>
+          <t>Financial inclusion</t>
+        </is>
+      </c>
+      <c r="K212" t="inlineStr">
+        <is>
+          <t>Uptake (account ownership)</t>
         </is>
       </c>
       <c r="L212" t="inlineStr">
         <is>
-          <t>Financial service provider (FSP) gender diversity; Financial service provider (FSP) type</t>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type</t>
         </is>
       </c>
     </row>
@@ -11907,36 +11732,26 @@
         </is>
       </c>
       <c r="D213">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>Crowdfunding - Differential rate of return (equity)</t>
+          <t>Crowdfunding - Authorization rejection rate</t>
         </is>
       </c>
       <c r="F213" t="inlineStr">
         <is>
-          <t>Difference between the advertised/promised rate of return and the actual rate of return of equity in crowdfunding projects</t>
+          <t>% of all crowfunding applications that are rejected (not authorized by the securities authority)</t>
         </is>
       </c>
       <c r="G213" t="inlineStr">
         <is>
-          <t>Measures the gap between the projected or advertised rate of return presented to investors before a project is funded and the actual rate of return realized after the project is completed. This is a critical conduct indicator that measures the accuracy of a project's promises versus its real-world performance. For investors, this metric is a tool for due diligence. For conduct supervisors, it can be used to detect mis-selling and fraud. A large and persistent negative differential (where actual returns are consistently far below promised returns) is a red flag. it could flag issues such as inadequate risk disclosure and fraud. When gender disaggregated by the gender of the main sponsor or lead executive, the indicator can provide additional information. If projects led by women consistently show a smaller negative "reality gap" (meaning their actual returns are closer to their promised returns), it could suggest they are more conservative or accurate in their financial projections. This would be a crucial data point in assessing risk and investor protection. Using this indicator together with the indicator on rejected crowddfunding projects could strenghten the identification of gender bias inside the securities authority. Return Differential (%) = Actual Rate of Return - Advertised/Promised Rate of Return.</t>
+          <t>Measures the percentage of all crowdfunding applications submitted to a securities authority that are denied or not authorized to proceed with fundraising. This is a key regulatory indicator that reflects the quality of applications being submitted and the stringency of the regulator's vetting process, which is designed to protect investors from fraud and non-viable projects. When disaggregated by the gender of the main sponsor, the lead executive of the company, it could draw insights into potential gender biases working within the securities authority.</t>
         </is>
       </c>
       <c r="H213" t="inlineStr">
         <is>
-          <t>Are there differences in the rates of return for crowdfunding projects depending on the gender assigned to the MSME seeking funding?</t>
-        </is>
-      </c>
-      <c r="J213" t="inlineStr">
-        <is>
-          <t>Financial inclusion; Other</t>
-        </is>
-      </c>
-      <c r="K213" t="inlineStr">
-        <is>
-          <t>Uptake (account ownership), Statistics and research</t>
+          <t>Are there gender disparities in the rejection rates and the reasons for rejection of crowdfunding projects presented for authorization by the securities regulator?</t>
         </is>
       </c>
       <c r="L213" t="inlineStr">
@@ -11962,26 +11777,36 @@
         </is>
       </c>
       <c r="D214">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>Crowdfunding - Authorization rejection rate</t>
+          <t>Crowdfunding - Success rate</t>
         </is>
       </c>
       <c r="F214" t="inlineStr">
         <is>
-          <t>% of all crowfunding applications that are rejected (not authorized by the securities authority)</t>
+          <t>% of all crowfunding projects that are successful in raising the asked amount</t>
         </is>
       </c>
       <c r="G214" t="inlineStr">
         <is>
-          <t>Measures the percentage of all crowdfunding applications submitted to a securities authority that are denied or not authorized to proceed with fundraising. This is a key regulatory indicator that reflects the quality of applications being submitted and the stringency of the regulator's vetting process, which is designed to protect investors from fraud and non-viable projects. When disaggregated by the gender of the main sponsor, the lead executive of the company, it could draw insights into potential gender biases working within the securities authority.</t>
+          <t>The indicator is a metric that measures the proportion of projects on a crowdfunding platform (or the sum of all crowdfunding platforms) that successfully reach their predetermined funding goal within a specified timeframe. This indicator is a vital sign of a platform's effectiveness, credibility, and the overall health of its ecosystem. It helps gauge the ability of a platform to connect viable projects with interested backers. For MSMEs, crowdfunding can be a viable and less onerous funding source, so the indicator provids important information for monitoring development of MSME finance markets. From a market conduct perspective, while a high success rate is generally positive, an unusually high or artificially inflated rate could be a red flag for misconduct. Platforms could be setting trivially low funding goals to boost statistics,  failing to conduct proper due diligence on projects, or not being transparent about how the success rate is calculated. Successful projects is the number of projects that met or exceeded their funding target during a specific period (e.g., a month, quarter, or year).</t>
         </is>
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the rejection rates and the reasons for rejection of crowdfunding projects presented for authorization by the securities regulator?</t>
+          <t>Are there gender disparities in the success rates of crowdfunding projects? Are smaller or younger MSMEs headed by women more likely to face challenges in crowdfunding?</t>
+        </is>
+      </c>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t>Financial inclusion</t>
+        </is>
+      </c>
+      <c r="K214" t="inlineStr">
+        <is>
+          <t>Usage</t>
         </is>
       </c>
       <c r="L214" t="inlineStr">
@@ -12007,36 +11832,26 @@
         </is>
       </c>
       <c r="D215">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
-          <t>Crowdfunding - Success rate</t>
+          <t>Crowdfunding - Transactions</t>
         </is>
       </c>
       <c r="F215" t="inlineStr">
         <is>
-          <t>% of all crowfunding projects that are successful in raising the asked amount</t>
+          <t>Volume (number of offerings) and value (amount raised) of crowdfunding transactions</t>
         </is>
       </c>
       <c r="G215" t="inlineStr">
         <is>
-          <t>The indicator is a metric that measures the proportion of projects on a crowdfunding platform (or the sum of all crowdfunding platforms) that successfully reach their predetermined funding goal within a specified timeframe. This indicator is a vital sign of a platform's effectiveness, credibility, and the overall health of its ecosystem. It helps gauge the ability of a platform to connect viable projects with interested backers. For MSMEs, crowdfunding can be a viable and less onerous funding source, so the indicator provids important information for monitoring development of MSME finance markets. From a market conduct perspective, while a high success rate is generally positive, an unusually high or artificially inflated rate could be a red flag for misconduct. Platforms could be setting trivially low funding goals to boost statistics,  failing to conduct proper due diligence on projects, or not being transparent about how the success rate is calculated. Successful projects is the number of projects that met or exceeded their funding target during a specific period (e.g., a month, quarter, or year).</t>
+          <t>Metric that measures the total volume of individual investments or pledges made across all projects on a crowdfunding platform or in the entire market (across multiple platforms) over a specific period. This indicator is a direct measure of market activity and investor engagement with crowdfunding, which is increasingly important for MSME finance.</t>
         </is>
       </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the success rates of crowdfunding projects? Are smaller or younger MSMEs headed by women more likely to face challenges in crowdfunding?</t>
-        </is>
-      </c>
-      <c r="J215" t="inlineStr">
-        <is>
-          <t>Financial inclusion; Other</t>
-        </is>
-      </c>
-      <c r="K215" t="inlineStr">
-        <is>
-          <t>Usage, Statistics and research</t>
+          <t>Are there disparities in crowdfunding volumes and values raised, according to the gender of the MSMEs asking for funds? Are there disparities in terms of funding periods? Among women-owned MSMEs, which types and ages (years in operation) are driving growth in crowdfunding transactions? Are crowdfunding platforms operated by diverse management more likely to attract women-owned MSMEs, and young MSMEs headed by women?</t>
         </is>
       </c>
       <c r="L215" t="inlineStr">
@@ -12062,26 +11877,26 @@
         </is>
       </c>
       <c r="D216">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>Crowdfunding - Transactions</t>
+          <t>P2P - Investors</t>
         </is>
       </c>
       <c r="F216" t="inlineStr">
         <is>
-          <t>Volume (number of offerings) and value (amount raised) of crowdfunding transactions</t>
+          <t>Number of P2P investors</t>
         </is>
       </c>
       <c r="G216" t="inlineStr">
         <is>
-          <t>Metric that measures the total volume of individual investments or pledges made across all projects on a crowdfunding platform or in the entire market (across multiple platforms) over a specific period. This indicator is a direct measure of market activity and investor engagement with crowdfunding, which is increasingly important for MSME finance.</t>
+          <t>This indicator counts the number of investors registered in P2P lending platforms, as a measure of development of digital finance, and specifically P2P lending, which can potentially benefit MSMEs. It is a key metric to monitor market development in platform lending. It helps assess the effectiveness of marketing campaigns, measure market reach, and forecast potential loan demand or the ability of platforms to meet demand. A growing investor base indicates increased trust and interest, enabling the business to scale and optimize revenue generation. The indicator should be segmented by type of investor (e.g., retail investor, institutional investor), according to local regulatory definitions.</t>
         </is>
       </c>
       <c r="H216" t="inlineStr">
         <is>
-          <t>Are there disparities in crowdfunding volumes and values raised, according to the gender of the MSMEs asking for funds? Are there disparities in terms of funding periods? Among women-owned MSMEs, which types and ages (years in operation) are driving growth in crowdfunding transactions? Are crowdfunding platforms operated by diverse management more likely to attract women-owned MSMEs, and young MSMEs headed by women?</t>
+          <t>Are there gender disparities in the growth of reatil investors in P2P lending platforms? How do invested amounts and types vary by investor gender and other demographics? For example, do women prefer to invest in women-led MSMEs, smaller projects, or younger enterprises? Do P2P platforms operated by diverse management more likely to attract a more diverse investor base?</t>
         </is>
       </c>
       <c r="L216" t="inlineStr">
@@ -12107,26 +11922,36 @@
         </is>
       </c>
       <c r="D217">
-        <v>46</v>
+        <v>9</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
-          <t>P2P - Investors</t>
+          <t>Total investment fund shares</t>
         </is>
       </c>
       <c r="F217" t="inlineStr">
         <is>
-          <t>Number of P2P investors</t>
+          <t>Number of investment fund shares held by retail investors in the system</t>
         </is>
       </c>
       <c r="G217" t="inlineStr">
         <is>
-          <t>This indicator counts the number of investors registered in P2P lending platforms, as a measure of development of digital finance, and specifically P2P lending, which can potentially benefit MSMEs. It is a key metric to monitor market development in platform lending. It helps assess the effectiveness of marketing campaigns, measure market reach, and forecast potential loan demand or the ability of platforms to meet demand. A growing investor base indicates increased trust and interest, enabling the business to scale and optimize revenue generation. The indicator should be segmented by type of investor (e.g., retail investor, institutional investor), according to local regulatory definitions.</t>
+          <t>Market-wide metric that quantifies the volume of investment fund shares owned by individual, non-professional investors within a financial system. This market develoment indicator serves as a crucial gauge of retail investor participation in the capital markets, and their overall exposure to market risks. Companion indicators include the share of investment fund shares held by retail investors as percentage of total investment fund shares, and the average holding size by retail investors.</t>
         </is>
       </c>
       <c r="H217" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the growth of reatil investors in P2P lending platforms? How do invested amounts and types vary by investor gender and other demographics? For example, do women prefer to invest in women-led MSMEs, smaller projects, or younger enterprises? Do P2P platforms operated by diverse management more likely to attract a more diverse investor base?</t>
+          <t>How has participation in investment funds evolved by gender, both for individuals and MSMEs considering the gender of their owners? What types of investment funds show growing participation by women?</t>
+        </is>
+      </c>
+      <c r="J217" t="inlineStr">
+        <is>
+          <t>Financial inclusion</t>
+        </is>
+      </c>
+      <c r="K217" t="inlineStr">
+        <is>
+          <t>Uptake (account ownership)</t>
         </is>
       </c>
       <c r="L217" t="inlineStr">
@@ -12143,50 +11968,55 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>Capital markets development</t>
+          <t>Competition</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>Investments</t>
+          <t>Savings, Credit</t>
         </is>
       </c>
       <c r="D218">
-        <v>9</v>
+        <v>267</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t>Total investment fund shares</t>
+          <t>Interest rate spreads (loans)</t>
         </is>
       </c>
       <c r="F218" t="inlineStr">
         <is>
-          <t>Number of investment fund shares held by retail investors in the system</t>
+          <t>Difference between the average lending rate and a reference rate (e.g. deposit rate or external reference rate)</t>
         </is>
       </c>
       <c r="G218" t="inlineStr">
         <is>
-          <t>Market-wide metric that quantifies the volume of investment fund shares owned by individual, non-professional investors within a financial system. This market develoment indicator serves as a crucial gauge of retail investor participation in the capital markets, and their overall exposure to market risks. Companion indicators include the share of investment fund shares held by retail investors as percentage of total investment fund shares, and the average holding size by retail investors.</t>
+          <t>The interest-rate spread on loans captures the margin between the average contractual rate a lender charges borrowers and an external reference rate—typically the policy rate. It is a concise gauge of (i) lenders’ credit-risk pricing, (ii) competitive conditions in the lending market, and (iii) monetary-policy transmission. Wider spreads may reflect higher perceived borrower risk, limited competition, or funding-cost pressures; persistently narrow spreads can point to aggressive underwriting or excess liquidity that may undermine future asset quality. Tracked over time and across peer institutions, interest-rate spreads provide insights into credit-cycle turning points, profitability dynamics, and the effectiveness of monetary-policy signals reaching the real economy. !- Definitions and concepts:  Loan interest rate spread (simple): Average contractual loan rate minus Reference rate measured for new originations or for the stock of loans. Net lending spread: average loan rate minus average deposit rate, often used when policy benchmarks are volatile. Segmented spreads: calculated by product (e.g., mortgages, SMEs, credit cards). Non-interest charges: fees and cross-selling income are excluded; the true all-in lending margin may be higher.</t>
         </is>
       </c>
       <c r="H218" t="inlineStr">
         <is>
-          <t>How has participation in investment funds evolved by gender, both for individuals and MSMEs considering the gender of their owners? What types of investment funds show growing participation by women?</t>
+          <t>Are there gender disparities in interest rate spreads offered to borrowers, and how do these differences vary across regions, income levels, and types of financial service providers? Do women or other gender groups consistently face higher lending rates relative to reference rates compared to men, potentially indicating unequal credit costs? How do interest rate spreads differ by loan type or sector, and are there gender patterns in these variations? Are financial service providers with higher gender diversity more likely to offer more equitable interest rate spreads across gender groups? How do differences in interest rate spreads impact borrowing behavior and access to credit for different gender groups?</t>
+        </is>
+      </c>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
         </is>
       </c>
       <c r="J218" t="inlineStr">
         <is>
-          <t>Financial inclusion; Statistics &amp; research</t>
+          <t>Financial inclusion</t>
         </is>
       </c>
       <c r="K218" t="inlineStr">
         <is>
-          <t>Uptake (account ownership), Other</t>
+          <t>Quality</t>
         </is>
       </c>
       <c r="L218" t="inlineStr">
         <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type</t>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Loan type; Loan size; Loan term; Interest rate category</t>
         </is>
       </c>
     </row>
@@ -12203,30 +12033,30 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>Savings</t>
+          <t>Payments, Savings, Credit, Insurance, Pensions, Investments</t>
         </is>
       </c>
       <c r="D219">
-        <v>156</v>
+        <v>35</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t>Depositors who actively close deposit accounts</t>
+          <t>Open finance - % of customers that have given data sharing consent to FSPs</t>
         </is>
       </c>
       <c r="F219" t="inlineStr">
         <is>
-          <t>% of retail depositors who actively closed a deposit account</t>
+          <t>% of all customers that have given consent to participate in the open finance scheme</t>
         </is>
       </c>
       <c r="G219" t="inlineStr">
         <is>
-          <t>A measure of the incidence of account closing among depositors, if the measure is high, it could potentially signal issues with the quality of accounts or concerns about the safety of funds. !- Definitions and concepts: Deposit accounts include transaction and non-transaction deposit accounts, for example: Checking/demand, savings, time/term deposit accounts, pensions. 'Active' closure of an account refers to cases where the closure is initiated at the request of the customer, and not due to inactivity or dormancy. !- Data requirements: List of unique deposit account holders (i.e. an individual  must be counted as one depositor irrespective of the number of deposit accounts held) who actively close any of their accounts over a specified period of time (e.g. quarter or year); Total number of unique depositors at the beginning of the specified period.</t>
+          <t>The indicator shows how many customers have actively opted in to share their data via the open finance rails (e.g., with account information service providers or payment initiation service providers). A higher share signals trust, clear value propositions, and mature consent customer interfaces (mobile apps); a low or falling rate may reflect friction in UX or Strong Customer Authentication (SCA), poor messaging, or privacy concerns. It’s a headline adoption KPI for open finance schemes. !- Definitions and concepts: Explicit consent: a clear, affirmative action tied to a specific purpose with the ability to manage and withdraw. Active consent: valid as of the reference date (not expired/withdrawn). Open finance consenting customers (%) = [# unique customers with at least 1 open finance consent / # eligible customers] x 100%. Denominator options: all active retail/MSME customers (preferred) or customers with eligible accounts (state choice). Segment by purpose of consent, scope (accounts included), and channel (mobile/web). Duplication &amp; scope: a customer may hold multiple consents across TPPs; count unique customers, and compare with total count of consents. Lawful-basis nuance: exclude sharing done under contractual necessity or legal obligation (e.g., consultation to credit bureaus for a loan application)—this metric is about explicit consent only.</t>
         </is>
       </c>
       <c r="H219" t="inlineStr">
         <is>
-          <t>How do active closure rates compare by gender? Which types of accounts are most frequently closed by each gender? How do FSPs rank in active account closures, and does this ranking change when analyzed by gender?</t>
+          <t>Are there gender disparities in data-sharing consent within the open finance scheme, including for MSMEs based on the ownership gender and low-value accounts? What types of accounts are more commonly subject to data-sharing consents? Which types of FSPs have a higher percentage of customers who have given data-sharing consent, and do these percentages vary by gender? If the information is available, what are the most common types and terms for these consents?</t>
         </is>
       </c>
       <c r="I219" t="inlineStr">
@@ -12236,17 +12066,17 @@
       </c>
       <c r="J219" t="inlineStr">
         <is>
-          <t>Financial inclusion; Consumer protection; Stability, safety and soundness</t>
+          <t>Consumer protection; Stability, safety and soundness</t>
         </is>
       </c>
       <c r="K219" t="inlineStr">
         <is>
-          <t>Quality, Fair treatment, Soundness, Stability</t>
+          <t>Data privacy and protection, Reputational and legal risk</t>
         </is>
       </c>
       <c r="L219" t="inlineStr">
         <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type</t>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
         </is>
       </c>
     </row>
@@ -12263,30 +12093,30 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>Savings, Credit</t>
+          <t>Payments, Savings, Credit, Insurance, Pensions, Investments</t>
         </is>
       </c>
       <c r="D220">
-        <v>267</v>
+        <v>36</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
-          <t>Interest rate spreads (loans)</t>
+          <t>Open finance - API availability</t>
         </is>
       </c>
       <c r="F220" t="inlineStr">
         <is>
-          <t>Difference between the average lending rate and a reference rate (e.g. deposit rate or external reference rate)</t>
+          <t>Average % of time APIs are available</t>
         </is>
       </c>
       <c r="G220" t="inlineStr">
         <is>
-          <t>The interest-rate spread on loans captures the margin between the average contractual rate a lender charges borrowers and an external reference rate—typically the policy rate. It is a concise gauge of (i) lenders’ credit-risk pricing, (ii) competitive conditions in the lending market, and (iii) monetary-policy transmission. Wider spreads may reflect higher perceived borrower risk, limited competition, or funding-cost pressures; persistently narrow spreads can point to aggressive underwriting or excess liquidity that may undermine future asset quality. Tracked over time and across peer institutions, interest-rate spreads provide insights into credit-cycle turning points, profitability dynamics, and the effectiveness of monetary-policy signals reaching the real economy. !- Definitions and concepts:  Loan interest rate spread (simple): Average contractual loan rate minus Reference rate measured for new originations or for the stock of loans. Net lending spread: average loan rate minus average deposit rate, often used when policy benchmarks are volatile. Segmented spreads: calculated by product (e.g., mortgages, SMEs, credit cards). Non-interest charges: fees and cross-selling income are excluded; the true all-in lending margin may be higher.</t>
+          <t>Shows the proportion of clock time that open finance endpoints can successfully serve requests. High availability is critical for data users such as third-party providers (TPPs) to deliver reliable account information and payment initiation; poor uptime breaks customer journeys, breaches SLAs/SLOs, and can trigger regulatory scrutiny in open finance schemes. !- Definitions and concepts: Availability (uptime):  time-weighted share of intervals in which an endpoint meets both reachability and success criteria. Scope — include account information service, payment initiation service, consent/token endpoints, and webhooks if they’re required for completion. Planned vs. unplanned:  exclude planned maintenance time; report maintenance windows separately. SLO period: availability is usually measured monthly/quarterly (e.g., 99.9% per calendar month), but preferably in shorter periods (e.g., weekly, daily). Granularity: overall availability, by endpoint family, region/zone, and time of day. Example indicator: Availability = 1 - [Downtime / Total scheduled time] where Downtime aggregates intervals failing the success criterion (5xx gateway/network timeouts, auth outages, or latency breaches). !- Limitations and considerations: Including latency SLOs will lower availability vs. status-only measurements. Publish thresholds.</t>
         </is>
       </c>
       <c r="H220" t="inlineStr">
         <is>
-          <t>Are there gender disparities in interest rate spreads offered to borrowers, and how do these differences vary across regions, income levels, and types of financial service providers? Do women or other gender groups consistently face higher lending rates relative to reference rates compared to men, potentially indicating unequal credit costs? How do interest rate spreads differ by loan type or sector, and are there gender patterns in these variations? Are financial service providers with higher gender diversity more likely to offer more equitable interest rate spreads across gender groups? How do differences in interest rate spreads impact borrowing behavior and access to credit for different gender groups?</t>
+          <t>Open finance performance will vary across FSPs for a range of reasons such as their current data architecture and other firm-specific aspects. The objective of looking into this indicator from a gender perspective is to identify whether FSPs that concentrate underserved, low-income women and women-led MSMEs also present poor open finance performance. This indicator can be analyzed together with other open finance performance indicators (Unsuccessful API calls, API response time), and open finance adoption indicators (% customer that have given consent, payment initiation transactions)</t>
         </is>
       </c>
       <c r="I220" t="inlineStr">
@@ -12296,17 +12126,17 @@
       </c>
       <c r="J220" t="inlineStr">
         <is>
-          <t>Financial inclusion; Consumer protection; Stability, safety and soundness</t>
+          <t>Financial inclusion; Stability, safety and soundness</t>
         </is>
       </c>
       <c r="K220" t="inlineStr">
         <is>
-          <t>Data privacy and protection, Operational risk</t>
+          <t>Quality, Operational risk</t>
         </is>
       </c>
       <c r="L220" t="inlineStr">
         <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Loan type; Loan size; Loan term; Interest rate category</t>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
         </is>
       </c>
     </row>
@@ -12327,26 +12157,26 @@
         </is>
       </c>
       <c r="D221">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
-          <t>Open finance - % of customers that have given data sharing consent to FSPs</t>
+          <t>Open finance - API error rate</t>
         </is>
       </c>
       <c r="F221" t="inlineStr">
         <is>
-          <t>% of all customers that have given consent to participate in the open finance scheme</t>
+          <t>% of all API calls that are unsuccessful</t>
         </is>
       </c>
       <c r="G221" t="inlineStr">
         <is>
-          <t>The indicator shows how many customers have actively opted in to share their data via the open finance rails (e.g., with account information service providers or payment initiation service providers). A higher share signals trust, clear value propositions, and mature consent customer interfaces (mobile apps); a low or falling rate may reflect friction in UX or Strong Customer Authentication (SCA), poor messaging, or privacy concerns. It’s a headline adoption KPI for open finance schemes. !- Definitions and concepts: Explicit consent: a clear, affirmative action tied to a specific purpose with the ability to manage and withdraw. Active consent: valid as of the reference date (not expired/withdrawn). Open finance consenting customers (%) = [# unique customers with at least 1 open finance consent / # eligible customers] x 100%. Denominator options: all active retail/MSME customers (preferred) or customers with eligible accounts (state choice). Segment by purpose of consent, scope (accounts included), and channel (mobile/web). Duplication &amp; scope: a customer may hold multiple consents across TPPs; count unique customers, and compare with total count of consents. Lawful-basis nuance: exclude sharing done under contractual necessity or legal obligation (e.g., consultation to credit bureaus for a loan application)—this metric is about explicit consent only.</t>
+          <t>This indicator tracks the reliability of open-finance interfaces by showing what share of API requests do not complete successfully due to errors. It is a key API performance indicator monitored by financial authorities implementing open finance. High failure rates degrade customer journeys (consent, data retrieval, payment initiation), inflate support costs, and can breach SLA/SLO commitments. !- Definitions and concepts: API call (request): one HTTP request to a documented endpoint, for example: Account Information Services (AIS) data, Payment Initiatiion Services (PIS) payment, consent, token, webhook, etc. Unsuccessful call: define as per local regulation. This indicator can be collected segmented by types of errors, to be defined as per local regulation (e.g., gateway/network timeouts, invalid/expired token/consent, error in validation, authentication failures. It should also be segmented by type of endpoint, as per local categorization (e.g., account information request, payment initiation request, other). Example indicator: [# of errors  /  # total API calls] x 100%.</t>
         </is>
       </c>
       <c r="H221" t="inlineStr">
         <is>
-          <t>Are there gender disparities in data-sharing consent within the open finance scheme, including for MSMEs based on the ownership gender and low-value accounts? What types of accounts are more commonly subject to data-sharing consents? Which types of FSPs have a higher percentage of customers who have given data-sharing consent, and do these percentages vary by gender? If the information is available, what are the most common types and terms for these consents?</t>
+          <t>Open finance performance will vary across FSPs for a range of reasons such as their current data architecture and other firm-specific aspects. The objective of looking into this indicator from a gender perspective is to identify whether FSPs that concentrate underserved, low-income women and women-led MSMEs also present poor open finance performance. This indicator can be analyzed together with other open finance performance indicators (Unsuccessful API calls, API response time), and open finance adoption indicators (% customer that have given consent, payment initiation transactions)</t>
         </is>
       </c>
       <c r="I221" t="inlineStr">
@@ -12356,12 +12186,12 @@
       </c>
       <c r="J221" t="inlineStr">
         <is>
-          <t>Consumer protection; Stability, safety and soundness</t>
+          <t>Financial inclusion; Stability, safety and soundness</t>
         </is>
       </c>
       <c r="K221" t="inlineStr">
         <is>
-          <t>Data privacy and protection, Reputational and legal risk</t>
+          <t>Quality, Operational risk</t>
         </is>
       </c>
       <c r="L221" t="inlineStr">
@@ -12387,21 +12217,21 @@
         </is>
       </c>
       <c r="D222">
-        <v>36</v>
+        <v>69</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
-          <t>Open finance - API availability</t>
+          <t>Open finance - API response time</t>
         </is>
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t>Average % of time APIs are available</t>
+          <t>Average API response time</t>
         </is>
       </c>
       <c r="G222" t="inlineStr">
         <is>
-          <t>Shows the proportion of clock time that open finance endpoints can successfully serve requests. High availability is critical for data users such as third-party providers (TPPs) to deliver reliable account information and payment initiation; poor uptime breaks customer journeys, breaches SLAs/SLOs, and can trigger regulatory scrutiny in open finance schemes. !- Definitions and concepts: Availability (uptime):  time-weighted share of intervals in which an endpoint meets both reachability and success criteria. Scope — include account information service, payment initiation service, consent/token endpoints, and webhooks if they’re required for completion. Planned vs. unplanned:  exclude planned maintenance time; report maintenance windows separately. SLO period: availability is usually measured monthly/quarterly (e.g., 99.9% per calendar month), but preferably in shorter periods (e.g., weekly, daily). Granularity: overall availability, by endpoint family, region/zone, and time of day. Example indicator: Availability = 1 - [Downtime / Total scheduled time] where Downtime aggregates intervals failing the success criterion (5xx gateway/network timeouts, auth outages, or latency breaches). !- Limitations and considerations: Including latency SLOs will lower availability vs. status-only measurements. Publish thresholds.</t>
+          <t>Shows how quickly open-finance endpoints answer requests. Faster responses improve user experience during consent, account-information retrieval, and payment initiation, reducing frictions and drop-offs. Response time is a core performance KPI that complements availability and error rate. !- Definitions and concepts: Response time (latency): elapsed time between request start and final byte received (client-observed) or gateway in → gateway out (server-observed). Track both when possible. Averages vs. tails: report p50/median, p95, p99, and the mean; tails (p95/p99) best reflect user pain. Track both. Granularity: report by endpoint family (types of APIs), potentially segmented into priority levels (see https://www.cdr.gov.au/performance). Units &amp; window: milliseconds, by calendar month (preferably shorter SLO period, such as weekly or daily).</t>
         </is>
       </c>
       <c r="H222" t="inlineStr">
@@ -12421,7 +12251,7 @@
       </c>
       <c r="K222" t="inlineStr">
         <is>
-          <t>Quality, Suitability, Operational risk</t>
+          <t>Quality, Operational risk</t>
         </is>
       </c>
       <c r="L222" t="inlineStr">
@@ -12447,41 +12277,31 @@
         </is>
       </c>
       <c r="D223">
-        <v>37</v>
+        <v>68</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>Open finance - API error rate</t>
+          <t>Open finance - Payment initiation transactions</t>
         </is>
       </c>
       <c r="F223" t="inlineStr">
         <is>
-          <t>% of all API calls that are unsuccessful</t>
+          <t>Number of payment initiation transactions conducted in the open finance scheme</t>
         </is>
       </c>
       <c r="G223" t="inlineStr">
         <is>
-          <t>This indicator tracks the reliability of open-finance interfaces by showing what share of API requests do not complete successfully due to errors. It is a key API performance indicator monitored by financial authorities implementing open finance. High failure rates degrade customer journeys (consent, data retrieval, payment initiation), inflate support costs, and can breach SLA/SLO commitments. !- Definitions and concepts: API call (request): one HTTP request to a documented endpoint, for example: Account Information Services (AIS) data, Payment Initiatiion Services (PIS) payment, consent, token, webhook, etc. Unsuccessful call: define as per local regulation. This indicator can be collected segmented by types of errors, to be defined as per local regulation (e.g., gateway/network timeouts, invalid/expired token/consent, error in validation, authentication failures. It should also be segmented by type of endpoint, as per local categorization (e.g., account information request, payment initiation request, other). Example indicator: [# of errors  /  # total API calls] x 100%.</t>
+          <t>Counts how many account-to-account (A2A) payment orders were successfully initiated via open-finance rails in the period. It’s a core adoption and usage KPI for Payment Initiation Services (PIS): more transactions imply growing merchant and P2P acceptance of openb finance, customer trust, and TPP–bank interoperability. !- Definitions and concepts: Payment initiation transaction (PIT): a payment order created via an authorized PISP/TPP and accepted by the ASPSP (account holder) for processing. Companion counts: Failed payment initiation transactions. Refunds/returns/chargebacks tracked separately. Sub-types: single immediate payments, scheduled payments, recurring/VRP (variable recurring payments), instant vs. ACH/batch. !- Data requirements: Total number of successful payment initiation transactions. !- Limitations and considerations: Duplicates: avoid double counting by using operation IDs.</t>
         </is>
       </c>
       <c r="H223" t="inlineStr">
         <is>
-          <t>Open finance performance will vary across FSPs for a range of reasons such as their current data architecture and other firm-specific aspects. The objective of looking into this indicator from a gender perspective is to identify whether FSPs that concentrate underserved, low-income women and women-led MSMEs also present poor open finance performance. This indicator can be analyzed together with other open finance performance indicators (Unsuccessful API calls, API response time), and open finance adoption indicators (% customer that have given consent, payment initiation transactions)</t>
+          <t>Are there gender disparities in the adoption of payment initiation transactions within the open finance scheme, including for MSMEs by the owner's gender? Do FSPs with higher levels of gender diversity tend to have a larger share of diverse customers conducting payment initiation transactions?</t>
         </is>
       </c>
       <c r="I223" t="inlineStr">
         <is>
           <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J223" t="inlineStr">
-        <is>
-          <t>Financial inclusion; Stability, safety and soundness</t>
-        </is>
-      </c>
-      <c r="K223" t="inlineStr">
-        <is>
-          <t>Quality, Operational risk</t>
         </is>
       </c>
       <c r="L223" t="inlineStr">
@@ -12507,26 +12327,27 @@
         </is>
       </c>
       <c r="D224">
-        <v>69</v>
+        <v>150</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
-          <t>Open finance - API response time</t>
+          <t>Bundled product uptake rate</t>
         </is>
       </c>
       <c r="F224" t="inlineStr">
         <is>
-          <t>Average API response time</t>
+          <t>% of customers taking up additional products during onboarding</t>
         </is>
       </c>
       <c r="G224" t="inlineStr">
         <is>
-          <t>Shows how quickly open-finance endpoints answer requests. Faster responses improve user experience during consent, account-information retrieval, and payment initiation, reducing frictions and drop-offs. Response time is a core performance KPI that complements availability and error rate. !- Definitions and concepts: Response time (latency): elapsed time between request start and final byte received (client-observed) or gateway in → gateway out (server-observed). Track both when possible. Averages vs. tails: report p50/median, p95, p99, and the mean; tails (p95/p99) best reflect user pain. Track both. Granularity: report by endpoint family (types of APIs), potentially segmented into priority levels (see https://www.cdr.gov.au/performance). Units &amp; window: milliseconds, by calendar month (preferably shorter SLO period, such as weekly or daily).</t>
+          <t>Measures the percentage of customers who acquire one or more additional financial products or services at the time of onboarding (i.e., when opening their primary account or initiating a new relationship with a financial service provider). These additional products may include insurance, savings, credit, or investment add-ons linked to the initial product. Captures the prevalence of product bundling and cross-selling practices during customer onboarding. It provides insight into market behavior, product integration, and the extent to which customers are being offered or encouraged to take multiple products simultaneously. Monitoring product bundling helps regulators and providers:
+Assess consumer choice and informed consent during onboarding; Identify potential coercive or mis-selling practices; Evaluate financial literacy and customer understanding of product combinations; Analyze the integration of complementary services (e.g., savings plus micro-insurance); Support efforts to ensure responsible cross-selling and transparent disclosure. Bundling can enhance value and convenience when responsibly designed, but may also raise conduct or affordability risks if customers are not well-informed. High bundling rates may reflect integrated product offerings or effective cross-selling, but warrant review for consent and suitability. Low rates may indicate limited product integration or narrow customer engagement at onboarding. Trends can reveal shifts in market strategy, regulatory compliance, or consumer protection outcomes. !- Definitions and concepts: Bundled product: A package of two or more financial services offered together at onboarding (e.g., transaction account + insurance or credit line). Onboarding: The process of establishing a new customer relationship, including account opening and KYC verification. Cross-selling: Offering additional, often related, financial products to a new or existing customer. Informed consent: The customer’s clear understanding and voluntary acceptance of each product taken. !- Data requirements: Bundled product uptake rate (%)=Number of customers who acquired ≥1 additional product at onboarding​/Total number of new customers onboarded. Administrative or CRM data from financial institutions on new customer onboarding and product uptake. Disaggregation by institution type, customer segment (individual, SME), region, and product category. !- Derivable indicators: Average number of products per new customer; Distribution of additional products (e.g., % taking insurance, credit, savings add-ons)</t>
         </is>
       </c>
       <c r="H224" t="inlineStr">
         <is>
-          <t>Open finance performance will vary across FSPs for a range of reasons such as their current data architecture and other firm-specific aspects. The objective of looking into this indicator from a gender perspective is to identify whether FSPs that concentrate underserved, low-income women and women-led MSMEs also present poor open finance performance. This indicator can be analyzed together with other open finance performance indicators (Unsuccessful API calls, API response time), and open finance adoption indicators (% customer that have given consent, payment initiation transactions)</t>
+          <t>How many products does each gender take up on average during the onboarding stage, and how do these numbers compare? What are the gender disparities in the likelihood of adopting multiple products? Which FSPs stand out in multi-product onboarding, and does their ranking change when analyzed by gender? Note: Active usage of products should also be assessed for multiple products taken up during onboarding.</t>
         </is>
       </c>
       <c r="I224" t="inlineStr">
@@ -12536,17 +12357,17 @@
       </c>
       <c r="J224" t="inlineStr">
         <is>
-          <t>Financial inclusion; Stability, safety and soundness</t>
+          <t>Financial inclusion</t>
         </is>
       </c>
       <c r="K224" t="inlineStr">
         <is>
-          <t>Quality, Operational risk</t>
+          <t>Uptake (account ownership)</t>
         </is>
       </c>
       <c r="L224" t="inlineStr">
         <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type</t>
         </is>
       </c>
     </row>
@@ -12567,26 +12388,26 @@
         </is>
       </c>
       <c r="D225">
-        <v>68</v>
+        <v>32</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>Open finance - Payment initiation transactions</t>
+          <t>Product portability requests</t>
         </is>
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>Number of payment initiation transactions conducted in the open finance scheme</t>
+          <t>Number of product portability requests</t>
         </is>
       </c>
       <c r="G225" t="inlineStr">
         <is>
-          <t>Counts how many account-to-account (A2A) payment orders were successfully initiated via open-finance rails in the period. It’s a core adoption and usage KPI for Payment Initiation Services (PIS): more transactions imply growing merchant and P2P acceptance of openb finance, customer trust, and TPP–bank interoperability. !- Definitions and concepts: Payment initiation transaction (PIT): a payment order created via an authorized PISP/TPP and accepted by the ASPSP (account holder) for processing. Companion counts: Failed payment initiation transactions. Refunds/returns/chargebacks tracked separately. Sub-types: single immediate payments, scheduled payments, recurring/VRP (variable recurring payments), instant vs. ACH/batch. !- Data requirements: Total number of successful payment initiation transactions. !- Limitations and considerations: Duplicates: avoid double counting by using operation IDs.</t>
+          <t>Measures the volume of formal requests initiated by customers to transfer their financial product or relationship from one provider to another within a specific period. This includes activities like switching a mortgage, transferring a loan to a new lender, or moving a current account to a new bank. This indicator is a gauge of market competition, consumer empowerment, and potential frictions or risks within the financial system. Very low switching rates can indicate significant barriers to entry or anti-competitive behavior, suggesting that customers are "trapped" with their current providers due to high exit fees, complex processes, or a lack of clear alternatives. This indicator is even more important in countries where product switching platforms or open finance exist and whose effectiveness should be monitored. A companion indicator to the total number of product switch requests is the total number of switches effected in the period, in comparison to the total number of requests. Another companion indicator is the total number of requests (or successful requests) relative to the number of active customers. The central bank of Brazil has calculated the number of loan portability requests relative to the number of loans with an interest rate above the market average rates, using the number of loans with above-market interest rates as a proxy for the untapped potential of the portability system. https://www.bcb.gov.br/content/publicacoes/Documents/reb/boxesreb2020/boxe_2_evolucao_portabilidade_credito_brasil.pdf</t>
         </is>
       </c>
       <c r="H225" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the adoption of payment initiation transactions within the open finance scheme, including for MSMEs by the owner's gender? Do FSPs with higher levels of gender diversity tend to have a larger share of diverse customers conducting payment initiation transactions?</t>
+          <t>Are there customer gender, income and location disparities in account and loan portability or FSP switching requests? Are FSPs with higher levels of gender diversity more likely to receive portability or switching requests or be the destination FSP (rather than the origin) for such requests?</t>
         </is>
       </c>
       <c r="I225" t="inlineStr">
@@ -12594,9 +12415,19 @@
           <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
         </is>
       </c>
+      <c r="J225" t="inlineStr">
+        <is>
+          <t>Financial inclusion; Consumer protection</t>
+        </is>
+      </c>
+      <c r="K225" t="inlineStr">
+        <is>
+          <t>Usage, Suitability</t>
+        </is>
+      </c>
       <c r="L225" t="inlineStr">
         <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Product type</t>
         </is>
       </c>
     </row>
@@ -12617,27 +12448,26 @@
         </is>
       </c>
       <c r="D226">
-        <v>150</v>
+        <v>33</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>Bundled product uptake rate</t>
+          <t>Rejected product portability requests</t>
         </is>
       </c>
       <c r="F226" t="inlineStr">
         <is>
-          <t>% of customers taking up additional products during onboarding</t>
+          <t>% of all product portability requests that are rejected</t>
         </is>
       </c>
       <c r="G226" t="inlineStr">
         <is>
-          <t>Measures the percentage of customers who acquire one or more additional financial products or services at the time of onboarding (i.e., when opening their primary account or initiating a new relationship with a financial service provider). These additional products may include insurance, savings, credit, or investment add-ons linked to the initial product. Captures the prevalence of product bundling and cross-selling practices during customer onboarding. It provides insight into market behavior, product integration, and the extent to which customers are being offered or encouraged to take multiple products simultaneously. Monitoring product bundling helps regulators and providers:
-Assess consumer choice and informed consent during onboarding; Identify potential coercive or mis-selling practices; Evaluate financial literacy and customer understanding of product combinations; Analyze the integration of complementary services (e.g., savings plus micro-insurance); Support efforts to ensure responsible cross-selling and transparent disclosure. Bundling can enhance value and convenience when responsibly designed, but may also raise conduct or affordability risks if customers are not well-informed. High bundling rates may reflect integrated product offerings or effective cross-selling, but warrant review for consent and suitability. Low rates may indicate limited product integration or narrow customer engagement at onboarding. Trends can reveal shifts in market strategy, regulatory compliance, or consumer protection outcomes. !- Definitions and concepts: Bundled product: A package of two or more financial services offered together at onboarding (e.g., transaction account + insurance or credit line). Onboarding: The process of establishing a new customer relationship, including account opening and KYC verification. Cross-selling: Offering additional, often related, financial products to a new or existing customer. Informed consent: The customer’s clear understanding and voluntary acceptance of each product taken. !- Data requirements: Bundled product uptake rate (%)=Number of customers who acquired ≥1 additional product at onboarding​/Total number of new customers onboarded. Administrative or CRM data from financial institutions on new customer onboarding and product uptake. Disaggregation by institution type, customer segment (individual, SME), region, and product category. !- Derivable indicators: Average number of products per new customer; Distribution of additional products (e.g., % taking insurance, credit, savings add-ons)</t>
+          <t>Measures the volume of formal portability requests initiated by customers to transfer their financial product or relationship from one provider to another within a specific period, which are rejected by the financial service provider. Product portability includes activities like switching a mortgage, transferring a loan to a new lender, or moving a current account to a new bank. This indicator is a gauge of market competition, consumer empowerment, and potential frictions or risks within the financial system. Very low switching rates can indicate significant barriers to entry or anti-competitive behavior, suggesting that customers are "trapped" with their current providers due to high exit fees, complex processes, or a lack of clear alternatives. This indicator is even more important in countries where product switching platforms or open finance exist and whose effectiveness should be monitored. When providers reject too many portability requests, this could be a sign of anti-competitive practices. This indicator should be analyzed together with the indicator on the total number of portability requests.</t>
         </is>
       </c>
       <c r="H226" t="inlineStr">
         <is>
-          <t>How many products does each gender take up on average during the onboarding stage, and how do these numbers compare? What are the gender disparities in the likelihood of adopting multiple products? Which FSPs stand out in multi-product onboarding, and does their ranking change when analyzed by gender? Note: Active usage of products should also be assessed for multiple products taken up during onboarding.</t>
+          <t>Are there customer gender, income, and location disparities in the approval of portability requests? Are FSPs with higher levels of gender diversity more likely to approve portability requests?</t>
         </is>
       </c>
       <c r="I226" t="inlineStr">
@@ -12647,135 +12477,15 @@
       </c>
       <c r="J226" t="inlineStr">
         <is>
-          <t>Financial inclusion</t>
+          <t>Financial inclusion; Consumer protection</t>
         </is>
       </c>
       <c r="K226" t="inlineStr">
         <is>
-          <t>Uptake</t>
+          <t>Usage, Suitability</t>
         </is>
       </c>
       <c r="L226" t="inlineStr">
-        <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type</t>
-        </is>
-      </c>
-    </row>
-    <row r="227">
-      <c r="A227" t="inlineStr">
-        <is>
-          <t>Market development</t>
-        </is>
-      </c>
-      <c r="B227" t="inlineStr">
-        <is>
-          <t>Competition</t>
-        </is>
-      </c>
-      <c r="C227" t="inlineStr">
-        <is>
-          <t>Payments, Savings, Credit, Insurance, Pensions, Investments</t>
-        </is>
-      </c>
-      <c r="D227">
-        <v>32</v>
-      </c>
-      <c r="E227" t="inlineStr">
-        <is>
-          <t>Product portability requests</t>
-        </is>
-      </c>
-      <c r="F227" t="inlineStr">
-        <is>
-          <t>Number of product portability requests</t>
-        </is>
-      </c>
-      <c r="G227" t="inlineStr">
-        <is>
-          <t>Measures the volume of formal requests initiated by customers to transfer their financial product or relationship from one provider to another within a specific period. This includes activities like switching a mortgage, transferring a loan to a new lender, or moving a current account to a new bank. This indicator is a gauge of market competition, consumer empowerment, and potential frictions or risks within the financial system. Very low switching rates can indicate significant barriers to entry or anti-competitive behavior, suggesting that customers are "trapped" with their current providers due to high exit fees, complex processes, or a lack of clear alternatives. This indicator is even more important in countries where product switching platforms or open finance exist and whose effectiveness should be monitored. A companion indicator to the total number of product switch requests is the total number of switches effected in the period, in comparison to the total number of requests. Another companion indicator is the total number of requests (or successful requests) relative to the number of active customers. The central bank of Brazil has calculated the number of loan portability requests relative to the number of loans with an interest rate above the market average rates, using the number of loans with above-market interest rates as a proxy for the untapped potential of the portability system. https://www.bcb.gov.br/content/publicacoes/Documents/reb/boxesreb2020/boxe_2_evolucao_portabilidade_credito_brasil.pdf</t>
-        </is>
-      </c>
-      <c r="H227" t="inlineStr">
-        <is>
-          <t>Are there customer gender, income and location disparities in account and loan portability or FSP switching requests? Are FSPs with higher levels of gender diversity more likely to receive portability or switching requests or be the destination FSP (rather than the origin) for such requests?</t>
-        </is>
-      </c>
-      <c r="I227" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J227" t="inlineStr">
-        <is>
-          <t>Financial inclusion; Consumer protection</t>
-        </is>
-      </c>
-      <c r="K227" t="inlineStr">
-        <is>
-          <t>Usage, Suitability</t>
-        </is>
-      </c>
-      <c r="L227" t="inlineStr">
-        <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Product type</t>
-        </is>
-      </c>
-    </row>
-    <row r="228">
-      <c r="A228" t="inlineStr">
-        <is>
-          <t>Market development</t>
-        </is>
-      </c>
-      <c r="B228" t="inlineStr">
-        <is>
-          <t>Competition</t>
-        </is>
-      </c>
-      <c r="C228" t="inlineStr">
-        <is>
-          <t>Payments, Savings, Credit, Insurance, Pensions, Investments</t>
-        </is>
-      </c>
-      <c r="D228">
-        <v>33</v>
-      </c>
-      <c r="E228" t="inlineStr">
-        <is>
-          <t>Rejected product portability requests</t>
-        </is>
-      </c>
-      <c r="F228" t="inlineStr">
-        <is>
-          <t>% of all product portability requests that are rejected</t>
-        </is>
-      </c>
-      <c r="G228" t="inlineStr">
-        <is>
-          <t>Measures the volume of formal portability requests initiated by customers to transfer their financial product or relationship from one provider to another within a specific period, which are rejected by the financial service provider. Product portability includes activities like switching a mortgage, transferring a loan to a new lender, or moving a current account to a new bank. This indicator is a gauge of market competition, consumer empowerment, and potential frictions or risks within the financial system. Very low switching rates can indicate significant barriers to entry or anti-competitive behavior, suggesting that customers are "trapped" with their current providers due to high exit fees, complex processes, or a lack of clear alternatives. This indicator is even more important in countries where product switching platforms or open finance exist and whose effectiveness should be monitored. When providers reject too many portability requests, this could be a sign of anti-competitive practices. This indicator should be analyzed together with the indicator on the total number of portability requests.</t>
-        </is>
-      </c>
-      <c r="H228" t="inlineStr">
-        <is>
-          <t>Are there customer gender, income, and location disparities in the approval of portability requests? Are FSPs with higher levels of gender diversity more likely to approve portability requests?</t>
-        </is>
-      </c>
-      <c r="I228" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers (i.e., natural persons) and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J228" t="inlineStr">
-        <is>
-          <t>Financial inclusion; Consumer protection</t>
-        </is>
-      </c>
-      <c r="K228" t="inlineStr">
-        <is>
-          <t>Usage, Suitability</t>
-        </is>
-      </c>
-      <c r="L228" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Product type</t>
         </is>

</xml_diff>

<commit_message>
Refresh indicator data from Google Sheets (230 indicators)
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/www/LENS_INDICATORS_DB.xlsx
+++ b/www/LENS_INDICATORS_DB.xlsx
@@ -6683,7 +6683,7 @@
       </c>
       <c r="L121" t="inlineStr">
         <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Complaints filing channel; Complaints issue category; Complaints processing status; Complaints resolution outcome; Complaints resolution time</t>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Product type; Complaints filing channel; Complaints issue category; Complaints processing status; Complaints resolution outcome; Complaints resolution time</t>
         </is>
       </c>
     </row>
@@ -7957,7 +7957,7 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>Frauds resulting in costumer losses</t>
+          <t>Frauds resulting in customer losses</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
@@ -7987,7 +7987,7 @@
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>Quality</t>
+          <t>Quality, Outcomes</t>
         </is>
       </c>
       <c r="L143" t="inlineStr">

</xml_diff>

<commit_message>
Rename "Gender equality" objective to "Diversity and inclusion"
Rename the Sustainability sub-objective everywhere it surfaces in the
catalog: the MND_OBJ_2 hierarchy (drives the objective filter) in
globals.R and the data values themselves via a rename step in the
data connector, applied before derived mandate-objective labels are
built so it propagates to main/secondary_mandate_objective and stays
consistent with the filter. Regenerated indicators.RData and the public
xlsx from the live Google Sheet (230 indicators).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/www/LENS_INDICATORS_DB.xlsx
+++ b/www/LENS_INDICATORS_DB.xlsx
@@ -559,7 +559,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Access</t>
+          <t>Access, Quality</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Access point type; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Access point type</t>
         </is>
       </c>
     </row>
@@ -702,17 +702,17 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Stability, safety and soundness</t>
+          <t>Stability, safety and soundness; Consumer protection</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Operational risk</t>
+          <t>Operational risk, Fair treatment</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>MSME gender; Digital transaction type; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
+          <t>MSME gender; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Digital transaction type</t>
         </is>
       </c>
     </row>
@@ -757,17 +757,17 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Stability, safety and soundness</t>
+          <t>Stability, safety and soundness; Consumer protection</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Operational risk</t>
+          <t>Operational risk, Fair treatment</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>MSME gender; Digital transaction type; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
+          <t>MSME gender; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Digital transaction type</t>
         </is>
       </c>
     </row>
@@ -2965,12 +2965,12 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>Consumer protection</t>
+          <t>Market development</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>Suitability</t>
+          <t>Competition</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
@@ -3403,7 +3403,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Usage</t>
+          <t>Usage, Outcomes</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -3446,12 +3446,12 @@
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>Safety and security, Depositor protection</t>
+          <t>Safety and security</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>Customer gender; Product type; Loan size; Customer income category</t>
+          <t>Customer gender; Customer income category; Loan size; Product type</t>
         </is>
       </c>
     </row>
@@ -3463,7 +3463,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Usage</t>
+          <t>Usage, Quality</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -3601,12 +3601,12 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>Consumer protection; Financial inclusion</t>
+          <t>Consumer protection; Consumer protection</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>Suitability, Usage</t>
+          <t>Suitability, Suitability</t>
         </is>
       </c>
       <c r="L63" t="inlineStr">
@@ -3773,7 +3773,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Usage</t>
+          <t>Usage, Quality</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Usage</t>
+          <t>Usage, Quality</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -4664,7 +4664,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Usage</t>
+          <t>Usage, Quality</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -4872,12 +4872,12 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>Stability, safety and soundness</t>
+          <t>Stability, safety and soundness; Consumer protection</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t>AML/CFT, Operational risk</t>
+          <t>AML/CFT, Suitability</t>
         </is>
       </c>
       <c r="L88" t="inlineStr">
@@ -4927,17 +4927,17 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>Stability, safety and soundness</t>
+          <t>Stability, safety and soundness; Consumer protection</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>Operational risk</t>
+          <t>Operational risk, Fair treatment</t>
         </is>
       </c>
       <c r="L89" t="inlineStr">
         <is>
-          <t>MSME gender; Digital transaction type; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
+          <t>MSME gender; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Digital transaction type</t>
         </is>
       </c>
     </row>
@@ -4985,16 +4985,6 @@
           <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
         </is>
       </c>
-      <c r="J90" t="inlineStr">
-        <is>
-          <t>Consumer protection; Stability, safety and soundness</t>
-        </is>
-      </c>
-      <c r="K90" t="inlineStr">
-        <is>
-          <t>Suitability, Stability</t>
-        </is>
-      </c>
       <c r="L90" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
@@ -5392,17 +5382,17 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>Stability, safety and soundness</t>
+          <t>Stability, safety and soundness; Consumer protection</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
         <is>
-          <t>Soundness</t>
+          <t>Soundness, Suitability</t>
         </is>
       </c>
       <c r="L97" t="inlineStr">
         <is>
-          <t>Customer type; Product type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity;</t>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Product type</t>
         </is>
       </c>
     </row>
@@ -5453,6 +5443,16 @@
           <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
         </is>
       </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>Consumer protection</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>Fair treatment</t>
+        </is>
+      </c>
       <c r="L98" t="inlineStr">
         <is>
           <t>Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
@@ -5502,6 +5502,16 @@
       <c r="I99" t="inlineStr">
         <is>
           <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>Consumer protection</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>Fair treatment</t>
         </is>
       </c>
       <c r="L99" t="inlineStr">
@@ -5556,6 +5566,16 @@
           <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
         </is>
       </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>Consumer protection</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>Fair treatment</t>
+        </is>
+      </c>
       <c r="L100" t="inlineStr">
         <is>
           <t>Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
@@ -5606,6 +5626,16 @@
           <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
         </is>
       </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>Consumer protection</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>Fair treatment</t>
+        </is>
+      </c>
       <c r="L101" t="inlineStr">
         <is>
           <t>Customer type; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Account type</t>
@@ -5776,6 +5806,16 @@
           <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
         </is>
       </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>Consumer protection</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>Suitability</t>
+        </is>
+      </c>
       <c r="L104" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
@@ -5826,6 +5866,16 @@
           <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
         </is>
       </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>Consumer protection</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>Suitability</t>
+        </is>
+      </c>
       <c r="L105" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
@@ -5876,6 +5926,16 @@
           <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
         </is>
       </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>Consumer protection</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>Suitability</t>
+        </is>
+      </c>
       <c r="L106" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
@@ -5984,6 +6044,16 @@
       <c r="I108" t="inlineStr">
         <is>
           <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>Consumer protection</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>Suitability</t>
         </is>
       </c>
       <c r="L108" t="inlineStr">
@@ -6291,6 +6361,16 @@
           <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
         </is>
       </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>Consumer protection</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>Suitability</t>
+        </is>
+      </c>
       <c r="L114" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Account type; Channel type</t>
@@ -6455,7 +6535,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Usage</t>
+          <t>Usage, Quality</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -6510,40 +6590,40 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Consumer protection</t>
+          <t>Financial inclusion</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Complaints handling, Safety and security</t>
+          <t>Usage, Quality</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Payments, Savings, Credit, Insurance, Pensions, Investments</t>
+          <t>Insurance</t>
         </is>
       </c>
       <c r="D119">
-        <v>322</v>
+        <v>389</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Fraud prevalence in complaints</t>
+          <t>Insurance claims (number)</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>Portion and volume of complaints received by providers, regulators, and ombuds that are fraud-related.</t>
+          <t>Number of insurance claims</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>Tracks how much of the complaint landscape is driven by fraud—both the count (volume) and the share (portion) of total complaints. Rising prevalence of frauds signals elevated customer harm, control weaknesses (KYC/AML, authentication, data security), or new attack vectors (social engineering). It helps guide supervision, consumer protection responses, reimbursement policies, and investment in fraud controls. !- Definitions and concepts: Fraud-related complaint: a case alleging unauthorised or deceptive activity resulting in loss or attempted loss—e.g., account takeover, card-not-present, phishing/SMiShing, SIM-swap, mule accounts, synthetic identity, merchant fraud, insider abuse, and authorised push payment (APP) scams. Volume: number of fraud-related complaints received in the period. Share: [# of fraud complaints / # of all complaints] x 100%. Intensity companions: fraud complaints per 1,000 customers or per 1 million transactions, value lens using claimed or confirmed loss amounts. Outcome cuts: upheld rate, reimbursement rate, median loss, time-to-resolution. A standard taxonomy for fraud types is needed, including the differentiation between fraud and disputed transaction. !- Limitations and considerations:  Under-reporting: many victims never complain or only contact the bank—triangulate with dispute/chargeback data and incident logs.</t>
+          <t>The total count of insurance claims formally submitted by policyholders, beneficiaries, or authorized third parties to an insurer within a defined reporting period, regardless of whether the claims are accepted, rejected, paid, or still under review. Denominator for several key inclusion, consumer protection and prudential insurance ratios. !- Data requirements: Claim identifier, (unique ID per claim), Policyholder identifier, Date of claim submission.</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>Are there gender differences in the proportion of fraud-related complaints submitted to providers, regulators, or ombuds services?  Do individuals of different genders tend to report different types of fraud, such as identity theft, phishing, or agent misconduct, and are specific delivery channels more commonly associated with these complaints? Is the volume of fraud-related complaints disproportionately high among certain gender groups when compared to their levels of account ownership or usage? Do complaint resolution rates and timeframes differ by gender across various FSP or reporting channels?</t>
+          <t>How do claim numbers vary by gender? Are there any gender groups logging fewer claims compared to the market average? Are there FSPs with particularly low or high claim numbers for certain genders? How do claim statistics intersect with policy type and customer demographics?</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -6553,57 +6633,57 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>Financial inclusion; Stability, safety and soundness</t>
+          <t>Consumer protection; Stability, safety and soundness</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>Quality, AML/CFT</t>
+          <t>Suitability, Soundness</t>
         </is>
       </c>
       <c r="L119" t="inlineStr">
         <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Complaints resolution outcome; Complaints resolution time</t>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Insurance type</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Consumer protection</t>
+          <t>Financial inclusion</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Suitability</t>
+          <t>Usage, Quality</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Credit</t>
+          <t>Insurance</t>
         </is>
       </c>
       <c r="D120">
-        <v>103</v>
+        <v>390</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Borrowers whose collateral was seized</t>
+          <t>Insurance claims paid</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>% of borrowers whose collateral was seized</t>
+          <t>Value of insurance claims paid</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>A measure of loan portfolio/credit risk assessment quality or financial distress among borrowers. !- Data requirements: Granular data that can yield (1) A count of unique borrowers of secured loans (those with collateral requirements) who subsequently had collateral seized by lender due to default over a specific period of time (e.g. past quarter or past year), (2) Total unique borrowers of secured loans over a specific period of time.</t>
+          <t>"Claims paid" represents the total cash outflow or settled obligations by an insurer to policyholders or beneficiaries for claims events during a reporting period. It includes only claims for which payment has been disbursed, regardless of whether additional claims are still outstanding or whether reserves were previously established. Tracking claims paid helps supervisors monitor liquidity, operational efficiency, and consumer protection outcomes. It provides a concrete measure of the insurer’s fulfillment of contractual obligations and complements other claims indicators (e.g., claims incurred, claims outstanding, unpaid approved claims). !- Data requirements: Claim identifier, (unique ID per claim), Policyholder identifier, Date of claim submission, Date of payment, Amount paid (full or partial), Product / policy type; . !- Limitations and considerations: paid claims may lag claims incurred due to reporting delays or extended claims handling processes; some claims are paid in installments, methodology must specify whether to include full or partial amounts; severe events can cause sudden increases in paid claims, interpretation should consider context. Segmentation by product line or policy type is recommended for supervisory analysis.</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>How does the share of customers whose collateral was seized due to default vary by gender and other key sociodemographic of the customer or MSME owner? Are women/WMSME more or less likely than men to have their collateral seized following loan default? How does the share differ by gender across different loan sizes, loan products,  types of financial service providers (FSP), collateral type (e.g., movable, immovable, alternative)? And how do any of these differences relate to seizure rates? Are women more likely to be subject to stricter collateral requirements or less flexible repayment terms that increase the likelihood of asset seizure?</t>
+          <t>How do claim payments vary by gender? Are there any gender groups receiving fewer/lower payments compared to the market average? Are there FSPs with particularly low or high payment rate for certain genders? How do claim payment statistics intersect with policy type and customer demographics?</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -6613,17 +6693,17 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>Financial inclusion; Stability, safety and soundness</t>
+          <t>Consumer protection; Stability, safety and soundness</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>Outcomes, Credit risk</t>
+          <t>Fair treatment, Soundness</t>
         </is>
       </c>
       <c r="L120" t="inlineStr">
         <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Loan type; Collateral type; Loan size; Loan term; Interest rate category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Insurance type</t>
         </is>
       </c>
     </row>
@@ -6635,7 +6715,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Complaints handling</t>
+          <t>Complaints handling, Safety and security</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -6644,26 +6724,26 @@
         </is>
       </c>
       <c r="D121">
-        <v>239</v>
+        <v>322</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Customer complaints (number)</t>
+          <t>Fraud prevalence in complaints</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>Number of customer complaints (including processing status, channels, type)</t>
+          <t>Portion and volume of complaints received by providers, regulators, and ombuds that are fraud-related.</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>This indicator tallies the formal expressions of dissatisfaction that retail or MSME clients lodge with a financial-service provider (or an external ombudsman) about products, services, or staff conduct over a specified period and can be normalized by dividing by the customer basis to obtain an intensity metric (e.g. complaints per 1,000 active customers). A rising complaint count can signal service-quality gaps, mis-selling, opaque fees, or inadequate disclosure—issues that erode trust and may escalate into regulatory sanctions or litigation. Supervisors can track both the absolute number and complaint-to-account ratios to test consumer-protection frameworks, prioritise thematic reviews, and assess whether rapid product roll-outs (e.g., digital lending, mobile wallets) are being matched by robust after-sales support. Where granular data or more detailed reporting templates permit, customer complaints can be disaggregated by processing status (e.g. received, accepted/rejected, in process, resolved, escalated/disputed, withdrawn), product (e.g. consumer loan, deposit account, etc), channel (e.g. digital, phone, in-person), issue category (e.g. fraudulent or unauthorized transactions, unfair treatment, unexpected fees, errors on statements,  etc.), resolution status (open, resolved with monetary compensation, resolved without compensation, escalated to ombudsman/regulator, other). Combined with resolution-time, compensation and other metrics, the number of customer complaints provides a critical, early-warning lens on conduct risk and customer-experience health. !- Definitions and concepts:  Complaints are expressions of dissatisfaction by (or on behalf of) customers that are related to their experiences with FSPs and can include any written, digital or recorded verbal statement made through any available channel, such as a branch, call-centre, email, social media, chatbots and other portals. Complaints may relate to the quality of a product or service, treatment by an FSP (including its agents and other third parties), or suspected wrongdoing. Complaints are different from general inquiries (e.g., where can I find an ATM?) or legal disputes between parties that may require formal dispute resolution. For more information, see for example CGAP's toolkit on using complaints data for market conduct supervision: https://www.cgap.org/research/publication/market-monitoring-tool-analysis-complaints-data and the Alliance for Financial Inclusion's framework on 'Complaint handling in Central Banks': https://www.afi-global.org/sites/default/files/publications/2020-04/AFI_CEMC_framework_AW_digital%20v2.pdf. !- Data requirements:  Database or log of customer complaints, detailing date of complaint and additional information, such as channel through which complaint was lodged, associated product or account, details or brief description of the complaint, and resolution status. !- Limitations and considerations: Complaints processes differ across FSPs in terms of steps/levels for routing, hand-over, escalations to higher management levels and to external ombudsman. Customer details and demographics of complainants are not always capture/stored on FSPs' systems, or may be stored in fragmented data bases. Complaints logged at aggregator sites/portals may not request customer demographics. Limited to officially logged complaints and/or maintaining records of inbound customer communications. Dependent on having electronic complaints management system.  Reporting culture: firms with easy‐to‐use channels may record more complaints than peers, even if service quality is similar—benchmark using severity and uphold rates. Under-reporting bias: vulnerable customers may forgo formal complaints; mystery-shopping and survey data can complement administrative counts. Duplicate cases: the same issue voiced through multiple channels can inflate totals unless robust deduplication exists. Product mix effects: complaint propensity varies—e.g., complex investments draw more grievances than basic savings; segment analysis is essential. Regulatory divergence: definitions and mandatory reporting thresholds differ across jurisdictions, complicating cross-border comparisons.</t>
+          <t>Tracks how much of the complaint landscape is driven by fraud—both the count (volume) and the share (portion) of total complaints. Rising prevalence of frauds signals elevated customer harm, control weaknesses (KYC/AML, authentication, data security), or new attack vectors (social engineering). It helps guide supervision, consumer protection responses, reimbursement policies, and investment in fraud controls. !- Definitions and concepts: Fraud-related complaint: a case alleging unauthorised or deceptive activity resulting in loss or attempted loss—e.g., account takeover, card-not-present, phishing/SMiShing, SIM-swap, mule accounts, synthetic identity, merchant fraud, insider abuse, and authorised push payment (APP) scams. Volume: number of fraud-related complaints received in the period. Share: [# of fraud complaints / # of all complaints] x 100%. Intensity companions: fraud complaints per 1,000 customers or per 1 million transactions, value lens using claimed or confirmed loss amounts. Outcome cuts: upheld rate, reimbursement rate, median loss, time-to-resolution. A standard taxonomy for fraud types is needed, including the differentiation between fraud and disputed transaction. !- Limitations and considerations:  Under-reporting: many victims never complain or only contact the bank—triangulate with dispute/chargeback data and incident logs.</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>How does the number of complaints at each processing stage vary by gender? Are complaints disproportionately concentrated at certain processing stages for any gender? How do FSPs compare to market averages in the number of complaints at each processing stage?"</t>
+          <t>Are there gender differences in the proportion of fraud-related complaints submitted to providers, regulators, or ombuds services?  Do individuals of different genders tend to report different types of fraud, such as identity theft, phishing, or agent misconduct, and are specific delivery channels more commonly associated with these complaints? Is the volume of fraud-related complaints disproportionately high among certain gender groups when compared to their levels of account ownership or usage? Do complaint resolution rates and timeframes differ by gender across various FSP or reporting channels?</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -6673,17 +6753,17 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>Financial inclusion</t>
+          <t>Financial inclusion; Stability, safety and soundness</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>Quality</t>
+          <t>Quality, AML/CFT</t>
         </is>
       </c>
       <c r="L121" t="inlineStr">
         <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Product type; Complaints filing channel; Complaints issue category; Complaints processing status; Complaints resolution outcome; Complaints resolution time</t>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Complaints resolution outcome; Complaints resolution time</t>
         </is>
       </c>
     </row>
@@ -6695,35 +6775,35 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Complaints handling</t>
+          <t>Suitability</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Payments, Savings, Credit, Insurance, Pensions, Investments</t>
+          <t>Credit</t>
         </is>
       </c>
       <c r="D122">
-        <v>243</v>
+        <v>103</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Customer complaints resolved in the customer's favor</t>
+          <t>Borrowers whose collateral was seized</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>% of customer complaints that were solved in the customer's favor in the most recent period</t>
+          <t>% of borrowers whose collateral was seized</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>This indicator shows the share of complaints closed in the reference period that were resolved in the customer’s favor. It is a direct outcome metric for fair treatment and service quality. A higher “uphold rate” can indicate strong remediation and customer-centric policies; a very low rate may suggest poor triage, overly narrow eligibility rules, or weak guidance to customers on evidence requirements. Supervisors use it to benchmark conduct outcomes across firms and products; boards track it alongside complaint volumes and resolution times to target root-cause fixes. Tracked with complaint volume, resolution time, and compensation totals, this indicator provides a balanced view of consumer outcomes and conduct risk. !- Definitions and concepts: Resolved in the customer’s favor (upheld): final decision grants redress—monetary (refund/compensation/fee reversal) or non-monetary (policy correction, contract change, apology with tangible remedy). Many firms also count partially upheld cases; disclose whether partials are included. Denominator: all complaints closed in the period. Segment results by product, channel, and severtiy to avoid masking problem areas. !- Data requirements: Central complaint-management records with unique IDs, receipt date, closure date, product, channel, allegation type, decision outcome (upheld/partially/declined), and compensation amount. Deduplication logic across channels; linkages to ombudsman/regulator portals for escalations and reversals. Customer-base denominator (for intensity metrics) and service level agreement (SLA) timestamps for parallel monitoring* (see note below). !- Limitations and considerations: Classification discretion: definitions of “partial uphold” vary; publish inclusion rules. Case mix effects: a surge in low-merit mass claims can depress the percentage; report severity-adjusted or line-of-business cuts. Gaming risk: chasing high uphold rates may encourage paying weak claims; pair with fraud flags, root-cause fixes, and cost-per-case. Timing bias: complex cases close later and differ in uphold propensity; use rolling averages and track median resolution time. External outcomes: include overturned-on-appeal adjustments to reflect true customer outcome. *With granular time-stamped complaints data, timeliness of key milestones in the complaints resolution process can be tracked, for example time to acknowledge complaint, time to first response, time to resolution. With this data, supervisors can track not just outcomes, but also whether providers are meeting required timeframes per their own SLA.</t>
+          <t>A measure of loan portfolio/credit risk assessment quality or financial distress among borrowers. !- Data requirements: Granular data that can yield (1) A count of unique borrowers of secured loans (those with collateral requirements) who subsequently had collateral seized by lender due to default over a specific period of time (e.g. past quarter or past year), (2) Total unique borrowers of secured loans over a specific period of time.</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>How do the percentages of complaints resolved in favor of customers vary by gender? Are any genders more likely to receive favorable resolutions? How do FSPs rank in terms of favorable resolutions by gender?</t>
+          <t>How does the share of customers whose collateral was seized due to default vary by gender and other key sociodemographic of the customer or MSME owner? Are women/WMSME more or less likely than men to have their collateral seized following loan default? How does the share differ by gender across different loan sizes, loan products,  types of financial service providers (FSP), collateral type (e.g., movable, immovable, alternative)? And how do any of these differences relate to seizure rates? Are women more likely to be subject to stricter collateral requirements or less flexible repayment terms that increase the likelihood of asset seizure?</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -6733,17 +6813,17 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>Financial inclusion</t>
+          <t>Financial inclusion; Stability, safety and soundness</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>Quality</t>
+          <t>Outcomes, Credit risk</t>
         </is>
       </c>
       <c r="L122" t="inlineStr">
         <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Complaints filing channel; Complaints issue category; Complaints processing status; Complaints resolution outcome; Complaints resolution time</t>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Loan type; Collateral type; Loan size; Loan term; Interest rate category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
         </is>
       </c>
     </row>
@@ -6755,7 +6835,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Data privacy and protection</t>
+          <t>Complaints handling</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -6764,26 +6844,26 @@
         </is>
       </c>
       <c r="D123">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Consent rate for FSP contact</t>
+          <t>Customer complaints (number)</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>% of customers who provide consent to be contacted in the future by the FSP for sales, awareness and new offerings</t>
+          <t>Number of customer complaints (including processing status, channels, type)</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>Measures the percentage of customers who have provided explicit consent to be contacted in the future by their financial service provider (FSP) for purposes such as product marketing, customer awareness campaigns, or information on new offerings. This indicator reflects how institutions manage customer permissions for communication under applicable data privacy and marketing regulations. Captures the extent of customer consent and data-use transparency in the financial system, serving as a proxy for compliance with consent-based communication standards and the balance between customer engagement and data protection. Tracking customer contact consents helps regulators and providers: Monitor compliance with data protection and privacy laws (e.g., GDPR-like frameworks, data protection acts); Assess ethical marketing practices and responsible customer engagement; Evaluate trust and willingness of customers to maintain open communication with FSPs; Understand customer attitudes toward data sharing and digital outreach. For supervisors, it provides a measurable view of market conduct, customer empowerment, and institutional transparency. High consent rates suggest strong customer trust and engagement, but may require close monitoring to ensure non-coercive consent collection and ethical marketing practices. Low consent rates may reflect privacy concerns, limited digital literacy, or overly complex consent processes. Changes over time can signal shifts in consumer sentiment or compliance practices following new regulations. !- Definitions and concepts: Consent: A freely given, informed, and specific agreement by a customer allowing the FSP to contact them for defined purposes. Data privacy regulation: Legal framework governing the collection, storage, and use of personal data, including consent requirements for marketing communications. !- Data requirements: Administrative data from FSP customer relationship management (CRM) or consent-management systems to obtain the number of customers who provided consent to be contact and the total number of customers.</t>
+          <t>This indicator tallies the formal expressions of dissatisfaction that retail or MSME clients lodge with a financial-service provider (or an external ombudsman) about products, services, or staff conduct over a specified period and can be normalized by dividing by the customer basis to obtain an intensity metric (e.g. complaints per 1,000 active customers). A rising complaint count can signal service-quality gaps, mis-selling, opaque fees, or inadequate disclosure—issues that erode trust and may escalate into regulatory sanctions or litigation. Supervisors can track both the absolute number and complaint-to-account ratios to test consumer-protection frameworks, prioritise thematic reviews, and assess whether rapid product roll-outs (e.g., digital lending, mobile wallets) are being matched by robust after-sales support. Where granular data or more detailed reporting templates permit, customer complaints can be disaggregated by processing status (e.g. received, accepted/rejected, in process, resolved, escalated/disputed, withdrawn), product (e.g. consumer loan, deposit account, etc), channel (e.g. digital, phone, in-person), issue category (e.g. fraudulent or unauthorized transactions, unfair treatment, unexpected fees, errors on statements,  etc.), resolution status (open, resolved with monetary compensation, resolved without compensation, escalated to ombudsman/regulator, other). Combined with resolution-time, compensation and other metrics, the number of customer complaints provides a critical, early-warning lens on conduct risk and customer-experience health. !- Definitions and concepts:  Complaints are expressions of dissatisfaction by (or on behalf of) customers that are related to their experiences with FSPs and can include any written, digital or recorded verbal statement made through any available channel, such as a branch, call-centre, email, social media, chatbots and other portals. Complaints may relate to the quality of a product or service, treatment by an FSP (including its agents and other third parties), or suspected wrongdoing. Complaints are different from general inquiries (e.g., where can I find an ATM?) or legal disputes between parties that may require formal dispute resolution. For more information, see for example CGAP's toolkit on using complaints data for market conduct supervision: https://www.cgap.org/research/publication/market-monitoring-tool-analysis-complaints-data and the Alliance for Financial Inclusion's framework on 'Complaint handling in Central Banks': https://www.afi-global.org/sites/default/files/publications/2020-04/AFI_CEMC_framework_AW_digital%20v2.pdf. !- Data requirements:  Database or log of customer complaints, detailing date of complaint and additional information, such as channel through which complaint was lodged, associated product or account, details or brief description of the complaint, and resolution status. !- Limitations and considerations: Complaints processes differ across FSPs in terms of steps/levels for routing, hand-over, escalations to higher management levels and to external ombudsman. Customer details and demographics of complainants are not always capture/stored on FSPs' systems, or may be stored in fragmented data bases. Complaints logged at aggregator sites/portals may not request customer demographics. Limited to officially logged complaints and/or maintaining records of inbound customer communications. Dependent on having electronic complaints management system.  Reporting culture: firms with easy‐to‐use channels may record more complaints than peers, even if service quality is similar—benchmark using severity and uphold rates. Under-reporting bias: vulnerable customers may forgo formal complaints; mystery-shopping and survey data can complement administrative counts. Duplicate cases: the same issue voiced through multiple channels can inflate totals unless robust deduplication exists. Product mix effects: complaint propensity varies—e.g., complex investments draw more grievances than basic savings; segment analysis is essential. Regulatory divergence: definitions and mandatory reporting thresholds differ across jurisdictions, complicating cross-border comparisons.</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>How do consent rates for customer contact vary by gender? Are any genders more likely to provide consent to be contacted? How do FSPs rank in terms of consent rates by gender?</t>
+          <t>How does the number of complaints at each processing stage vary by gender? Are complaints disproportionately concentrated at certain processing stages for any gender? How do FSPs compare to market averages in the number of complaints at each processing stage?"</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -6803,7 +6883,7 @@
       </c>
       <c r="L123" t="inlineStr">
         <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Product type; Complaints filing channel; Complaints issue category; Complaints processing status; Complaints resolution outcome; Complaints resolution time</t>
         </is>
       </c>
     </row>
@@ -6815,28 +6895,148 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
+          <t>Complaints handling</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Payments, Savings, Credit, Insurance, Pensions, Investments</t>
+        </is>
+      </c>
+      <c r="D124">
+        <v>243</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Customer complaints resolved in the customer's favor</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>% of customer complaints that were solved in the customer's favor in the most recent period</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>This indicator shows the share of complaints closed in the reference period that were resolved in the customer’s favor. It is a direct outcome metric for fair treatment and service quality. A higher “uphold rate” can indicate strong remediation and customer-centric policies; a very low rate may suggest poor triage, overly narrow eligibility rules, or weak guidance to customers on evidence requirements. Supervisors use it to benchmark conduct outcomes across firms and products; boards track it alongside complaint volumes and resolution times to target root-cause fixes. Tracked with complaint volume, resolution time, and compensation totals, this indicator provides a balanced view of consumer outcomes and conduct risk. !- Definitions and concepts: Resolved in the customer’s favor (upheld): final decision grants redress—monetary (refund/compensation/fee reversal) or non-monetary (policy correction, contract change, apology with tangible remedy). Many firms also count partially upheld cases; disclose whether partials are included. Denominator: all complaints closed in the period. Segment results by product, channel, and severtiy to avoid masking problem areas. !- Data requirements: Central complaint-management records with unique IDs, receipt date, closure date, product, channel, allegation type, decision outcome (upheld/partially/declined), and compensation amount. Deduplication logic across channels; linkages to ombudsman/regulator portals for escalations and reversals. Customer-base denominator (for intensity metrics) and service level agreement (SLA) timestamps for parallel monitoring* (see note below). !- Limitations and considerations: Classification discretion: definitions of “partial uphold” vary; publish inclusion rules. Case mix effects: a surge in low-merit mass claims can depress the percentage; report severity-adjusted or line-of-business cuts. Gaming risk: chasing high uphold rates may encourage paying weak claims; pair with fraud flags, root-cause fixes, and cost-per-case. Timing bias: complex cases close later and differ in uphold propensity; use rolling averages and track median resolution time. External outcomes: include overturned-on-appeal adjustments to reflect true customer outcome. *With granular time-stamped complaints data, timeliness of key milestones in the complaints resolution process can be tracked, for example time to acknowledge complaint, time to first response, time to resolution. With this data, supervisors can track not just outcomes, but also whether providers are meeting required timeframes per their own SLA.</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>How do the percentages of complaints resolved in favor of customers vary by gender? Are any genders more likely to receive favorable resolutions? How do FSPs rank in terms of favorable resolutions by gender?</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>Financial inclusion</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Complaints filing channel; Complaints issue category; Complaints processing status; Complaints resolution outcome; Complaints resolution time</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Consumer protection</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Data privacy and protection</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Payments, Savings, Credit, Insurance, Pensions, Investments</t>
+        </is>
+      </c>
+      <c r="D125">
+        <v>234</v>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Consent rate for FSP contact</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>% of customers who provide consent to be contacted in the future by the FSP for sales, awareness and new offerings</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>Measures the percentage of customers who have provided explicit consent to be contacted in the future by their financial service provider (FSP) for purposes such as product marketing, customer awareness campaigns, or information on new offerings. This indicator reflects how institutions manage customer permissions for communication under applicable data privacy and marketing regulations. Captures the extent of customer consent and data-use transparency in the financial system, serving as a proxy for compliance with consent-based communication standards and the balance between customer engagement and data protection. Tracking customer contact consents helps regulators and providers: Monitor compliance with data protection and privacy laws (e.g., GDPR-like frameworks, data protection acts); Assess ethical marketing practices and responsible customer engagement; Evaluate trust and willingness of customers to maintain open communication with FSPs; Understand customer attitudes toward data sharing and digital outreach. For supervisors, it provides a measurable view of market conduct, customer empowerment, and institutional transparency. High consent rates suggest strong customer trust and engagement, but may require close monitoring to ensure non-coercive consent collection and ethical marketing practices. Low consent rates may reflect privacy concerns, limited digital literacy, or overly complex consent processes. Changes over time can signal shifts in consumer sentiment or compliance practices following new regulations. !- Definitions and concepts: Consent: A freely given, informed, and specific agreement by a customer allowing the FSP to contact them for defined purposes. Data privacy regulation: Legal framework governing the collection, storage, and use of personal data, including consent requirements for marketing communications. !- Data requirements: Administrative data from FSP customer relationship management (CRM) or consent-management systems to obtain the number of customers who provided consent to be contact and the total number of customers.</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>How do consent rates for customer contact vary by gender? Are any genders more likely to provide consent to be contacted? How do FSPs rank in terms of consent rates by gender?</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>Financial inclusion</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Consumer protection</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
           <t>Fair treatment</t>
         </is>
       </c>
-      <c r="C124" t="inlineStr">
+      <c r="C126" t="inlineStr">
         <is>
           <t>Credit</t>
         </is>
       </c>
-      <c r="D124">
+      <c r="D126">
         <v>284</v>
       </c>
-      <c r="E124" t="inlineStr">
+      <c r="E126" t="inlineStr">
         <is>
           <t>Annual percentage rate (APR) for retail credit</t>
         </is>
       </c>
-      <c r="F124" t="inlineStr">
+      <c r="F126" t="inlineStr">
         <is>
           <t>Average cost of borrowing money, including fees to get the loan, as a% of the loan principal (except for credit cards)</t>
         </is>
       </c>
-      <c r="G124" t="inlineStr">
+      <c r="G126" t="inlineStr">
         <is>
           <t>APR is the standardized annualized cost of borrowing that incorporates the contractual interest rate plus certain up-front or periodic fees required to obtain and maintain the credit. It lets consumers compare offers across lenders and products on a like-for-like basis, and helps supervisors monitor pricing fairness and market competitiveness. Unlike a simple “nominal” rate, APR reflects timing of cash flows and required charges, so it better approximates the true price of credit. !- Definitions and concepts: Installment credit APR (actuarial method): the internal rate of return (IRR) that equates the amount advanced to the borrower with the present value of all required payments (principal, interest, and included fees), expressed on an annual basis.
 Revolving credit APR (cards/overdrafts): the periodic rate applied to the average daily balance, annualized (e.g., daily rate × 365 or monthly rate × 12), plus disclosure of any mandatory fees as prescribed. Scope of fees: typically includes origination/processing fees and compulsory charges; excludes penalty fees and optional add-ons (unless mandated). APR vs. EIR: APR is a consumer disclosure metric (jurisdiction-specific rules); EIR is an accounting yield used to recognize interest income.!- Data requirements: Contract terms: principal advanced, repayment schedule (dates/amounts), nominal rate, compounding frequency, and variable-rate index/margins. Included fees: origination/processing, mandatory maintenance or platform fees, financed vs. paid-in-cash. For revolving products: periodic rate(s), balance computation method (average daily balance), mandatory annual fees, grace-period rules, promotional/teaser rates.
@@ -6844,144 +7044,24 @@
 Promotions &amp; step-ups: teaser or deferred-interest offers can make snapshot APRs unrepresentative—show lifetime-effective examples when possible. Variable rates: APR at origination may understate future cost if reference rates rise. Loan term effects: fixed fees loom larger on short tenors; present both APR and the fee share of cost for transparency.</t>
         </is>
       </c>
-      <c r="H124" t="inlineStr">
+      <c r="H126" t="inlineStr">
         <is>
           <t>Are there gender disparities in the APR applied to loans disbursed to women and men, including MSMEs by gender of ownership? Do women borrowers systematically face higher average APRs than men within the same loan type, amount range, or provider category? Are higher APRs for women associated with smaller loan sizes, shorter maturities, or higher perceived credit risk? Do FSPs with greater gender diversity or stronger inclusion policies show smaller gender gaps in average APRs? How do APR differences relate to borrower profiles and do they suggest the presence of gender-based pricing bias or structural credit segmentation?</t>
         </is>
       </c>
-      <c r="I124" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J124" t="inlineStr">
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
         <is>
           <t>Financial inclusion; Market development</t>
         </is>
       </c>
-      <c r="K124" t="inlineStr">
+      <c r="K126" t="inlineStr">
         <is>
           <t>Quality, Competition</t>
-        </is>
-      </c>
-      <c r="L124" t="inlineStr">
-        <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Loan type</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" t="inlineStr">
-        <is>
-          <t>Consumer protection</t>
-        </is>
-      </c>
-      <c r="B125" t="inlineStr">
-        <is>
-          <t>Data privacy and protection</t>
-        </is>
-      </c>
-      <c r="C125" t="inlineStr">
-        <is>
-          <t>Payments, Savings, Credit, Insurance, Pensions, Investments</t>
-        </is>
-      </c>
-      <c r="D125">
-        <v>235</v>
-      </c>
-      <c r="E125" t="inlineStr">
-        <is>
-          <t>Consents for sharing data with third-parties</t>
-        </is>
-      </c>
-      <c r="F125" t="inlineStr">
-        <is>
-          <t>% of customers who have given explicit consent for their data to be shared by FSPs with third parties, for various purposes</t>
-        </is>
-      </c>
-      <c r="G125" t="inlineStr">
-        <is>
-          <t>This indicator shows how many customers have actively opted in to let a financial service provider (FSP) share their data with external parties—for open-banking/aggregation, credit scoring, fraud prevention, marketing, analytics, etc. A higher share can reflect strong digital adoption and trust; low or falling rates may signal poor consent UX, unclear value propositions, or privacy concerns. It helps compliance teams evidence lawfulness, product teams gauge partner-integration reach, and supervisors assess the maturity of consent-based data-sharing ecosystems. !- Definitions and concepts: Explicit consent: a clear, affirmative action (e.g., checked box, strong-customer-authenticated authorization) tied to a specific purpose, with intelligible notice and the ability to withdraw at any time. Active consent: consent that is valid as of the reference date (not expired, not withdrawn, not superseded). Purpose taxonomy: e.g., account information services (AIS), payment initiation services (PIS), credit decisioning/bureau pulls, fraud/AML tools, personalised marketing, data portability. Metric: % of customer with active consent for purpose p = [# of unique customers with at least 1 active consent for p / # of active customers] x 100%. Indicator companions: Any-purpose consent, consents per consenting customer and revocation rate. !- Data requirements: Consent ledger that includes: customer ID, purpose(s) granted, third-party identity, channel, timestamp, expiry/refresh cycle, version of the privacy notice, proof of consent (hash, audit trail, SCA event). Status events: withdrawals, expiries, scope changes, third-party disconnects. Reference universe: deduplicated active-customer list (define “active”: e.g., ≥1 product in force or ≥1 login/transaction in last 12 months). !- Limitations and considerations: Granularity &amp; fragmentation: a customer may consent per app, per account, and per purpose; avoid double counting by using unique customers and report purpose-level cuts. Expiry &amp; refresh: open-banking tokens often have short authorizations; snapshot dates vs. rolling windows will yield different figures—disclose method. Consumer protection risk: high opt-ins driven by coercive UX can backfire (complaints, revocations); pair with revocation rate, time-to-revocation, and complaints about data sharing. Coverage gaps: legacy channels without digital capture may under-record historical consents; backfill or disclose limitations.</t>
-        </is>
-      </c>
-      <c r="H125" t="inlineStr">
-        <is>
-          <t>How do consent rates for data sharing with third parties vary by gender? Are any genders more likely to provide consent for data sharing? How do FSPs rank in terms of consent rates for data sharing by gender?</t>
-        </is>
-      </c>
-      <c r="I125" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J125" t="inlineStr">
-        <is>
-          <t>Market development</t>
-        </is>
-      </c>
-      <c r="K125" t="inlineStr">
-        <is>
-          <t>Competition</t>
-        </is>
-      </c>
-      <c r="L125" t="inlineStr">
-        <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="inlineStr">
-        <is>
-          <t>Consumer protection</t>
-        </is>
-      </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>Fair treatment</t>
-        </is>
-      </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t>Credit</t>
-        </is>
-      </c>
-      <c r="D126">
-        <v>260</v>
-      </c>
-      <c r="E126" t="inlineStr">
-        <is>
-          <t>Late penalty charges/fees on retail credit</t>
-        </is>
-      </c>
-      <c r="F126" t="inlineStr">
-        <is>
-          <t>Income from penalty fees as % of total net interest income</t>
-        </is>
-      </c>
-      <c r="G126" t="inlineStr">
-        <is>
-          <t>This indicator shows how much of a lender is relying on penalty fees for income. Revenue from penalty fees and other charges applied when a loan payment is late is compared with the total gross interest income. A high share could signal borrower stress and potential conduct risk (reliance on punitive pricing). Boards and supervisors use the metric to assess earnings quality, pricing fairness. !- Definitions and concepts: Penalty/default fees and charges: the fees and costs charged once a loan  is past due. Numerator (preferred “incremental” view): Penalty actually recognized as income on retail loans during the period. Denominator: Gross interest income. !- Data requirements: General-ledger mapping that identifies penalty income at product level. Period interest income totals for the denominator.  !- Limitations and considerations: Mix effects: card-heavy books show higher shares of penalty income; segment by product. Conduct lens: pair with % customers incurring penalty charges, related complaints.</t>
-        </is>
-      </c>
-      <c r="H126" t="inlineStr">
-        <is>
-          <t>What percentages of net interest income are attributable to penalties and other punitive charges earned from borrowers of unsecured loans/lines of credit, and how do these vary by gender across age bands and location types, at a total market level and by relevant FSP/type? How do these percentages compare across relevant FSPs/types and against market norms across age bands and location types? How do gender disparities manifest in these percentages at a total market level and by relevant FSP/type?</t>
-        </is>
-      </c>
-      <c r="I126" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J126" t="inlineStr">
-        <is>
-          <t>Financial inclusion</t>
-        </is>
-      </c>
-      <c r="K126" t="inlineStr">
-        <is>
-          <t>Quality</t>
         </is>
       </c>
       <c r="L126" t="inlineStr">
@@ -6998,177 +7078,177 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
+          <t>Data privacy and protection</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Payments, Savings, Credit, Insurance, Pensions, Investments</t>
+        </is>
+      </c>
+      <c r="D127">
+        <v>235</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Consents for sharing data with third-parties</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>% of customers who have given explicit consent for their data to be shared by FSPs with third parties, for various purposes</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>This indicator shows how many customers have actively opted in to let a financial service provider (FSP) share their data with external parties—for open-banking/aggregation, credit scoring, fraud prevention, marketing, analytics, etc. A higher share can reflect strong digital adoption and trust; low or falling rates may signal poor consent UX, unclear value propositions, or privacy concerns. It helps compliance teams evidence lawfulness, product teams gauge partner-integration reach, and supervisors assess the maturity of consent-based data-sharing ecosystems. !- Definitions and concepts: Explicit consent: a clear, affirmative action (e.g., checked box, strong-customer-authenticated authorization) tied to a specific purpose, with intelligible notice and the ability to withdraw at any time. Active consent: consent that is valid as of the reference date (not expired, not withdrawn, not superseded). Purpose taxonomy: e.g., account information services (AIS), payment initiation services (PIS), credit decisioning/bureau pulls, fraud/AML tools, personalised marketing, data portability. Metric: % of customer with active consent for purpose p = [# of unique customers with at least 1 active consent for p / # of active customers] x 100%. Indicator companions: Any-purpose consent, consents per consenting customer and revocation rate. !- Data requirements: Consent ledger that includes: customer ID, purpose(s) granted, third-party identity, channel, timestamp, expiry/refresh cycle, version of the privacy notice, proof of consent (hash, audit trail, SCA event). Status events: withdrawals, expiries, scope changes, third-party disconnects. Reference universe: deduplicated active-customer list (define “active”: e.g., ≥1 product in force or ≥1 login/transaction in last 12 months). !- Limitations and considerations: Granularity &amp; fragmentation: a customer may consent per app, per account, and per purpose; avoid double counting by using unique customers and report purpose-level cuts. Expiry &amp; refresh: open-banking tokens often have short authorizations; snapshot dates vs. rolling windows will yield different figures—disclose method. Consumer protection risk: high opt-ins driven by coercive UX can backfire (complaints, revocations); pair with revocation rate, time-to-revocation, and complaints about data sharing. Coverage gaps: legacy channels without digital capture may under-record historical consents; backfill or disclose limitations.</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>How do consent rates for data sharing with third parties vary by gender? Are any genders more likely to provide consent for data sharing? How do FSPs rank in terms of consent rates for data sharing by gender?</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>Market development; Financial inclusion</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>Competition, Quality</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Consumer protection</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
           <t>Fair treatment</t>
         </is>
       </c>
-      <c r="C127" t="inlineStr">
+      <c r="C128" t="inlineStr">
         <is>
           <t>Credit</t>
         </is>
       </c>
-      <c r="D127">
+      <c r="D128">
+        <v>260</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Late penalty charges/fees on retail credit</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>Income from penalty fees as % of total net interest income</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>This indicator shows how much of a lender is relying on penalty fees for income. Revenue from penalty fees and other charges applied when a loan payment is late is compared with the total gross interest income. A high share could signal borrower stress and potential conduct risk (reliance on punitive pricing). Boards and supervisors use the metric to assess earnings quality, pricing fairness. !- Definitions and concepts: Penalty/default fees and charges: the fees and costs charged once a loan  is past due. Numerator (preferred “incremental” view): Penalty actually recognized as income on retail loans during the period. Denominator: Gross interest income. !- Data requirements: General-ledger mapping that identifies penalty income at product level. Period interest income totals for the denominator.  !- Limitations and considerations: Mix effects: card-heavy books show higher shares of penalty income; segment by product. Conduct lens: pair with % customers incurring penalty charges, related complaints.</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>What percentages of net interest income are attributable to penalties and other punitive charges earned from borrowers of unsecured loans/lines of credit, and how do these vary by gender across age bands and location types, at a total market level and by relevant FSP/type? How do these percentages compare across relevant FSPs/types and against market norms across age bands and location types? How do gender disparities manifest in these percentages at a total market level and by relevant FSP/type?</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>Financial inclusion</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Loan type</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Consumer protection</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Fair treatment</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="D129">
         <v>185</v>
       </c>
-      <c r="E127" t="inlineStr">
+      <c r="E129" t="inlineStr">
         <is>
           <t>Processing and application fees or PAF (as % of loan principal)</t>
         </is>
       </c>
-      <c r="F127" t="inlineStr">
+      <c r="F129" t="inlineStr">
         <is>
           <t>PAF as % of loan principal in unsecured credit operations</t>
         </is>
       </c>
-      <c r="G127" t="inlineStr">
+      <c r="G129" t="inlineStr">
         <is>
           <t>This indicator expresses the total up-front charges borrowers pay to originate an unsecured loan—processing fees, application fees, documentation charges—as a percentage of the loan’s principal amount. Because unsecured credit often targets price-sensitive segments and carries higher risk-based interest rates, excessive PAFs can materially raise the all-in cost of borrowing, undermine affordability tests, and trigger consumer-protection scrutiny. Tracking the ratio helps regulators detect predatory pricing, compare lenders’ transparency practices, and gauge competition in loan-origination services. For lenders, it is a barometer of non-interest revenue reliance and a lever for recouping acquisition costs. Processing &amp; Application Fees (PAF): any non-refundable charge levied at or before disbursement for administrative tasks (credit checks, KYC, documentation, platform usage). Late-payment or insurance fees are excluded.
 PAF ratio (simple): [Total PAF charged/Gross loan principal]×100%
 Where multiple partial disbursements occur, use the aggregate principal amount. Annualised impact: when PAFs are capitalised into the Effective Annual Percentage Rate (APR), their weight declines as term length rises—monitor both absolute and APR-embedded views. !- Data requirements: Loan-level records capturing principal, disbursement date, PAF amount, and any rebates for cancellations. Product codes distinguishing personal instalment loans, credit-card cash advances, payday/BNPL equivalents. Borrower demographics and channel identifiers (branch, mobile app, marketplace) for segmentation. Accounting entries showing whether fees are recognised up-front (IFRS 15 “contract costs”) or amortised via the effective-interest-rate (EIR) method. !- Limitations and considerations: Amortisation differences: Lenders using EIR spread PAFs over the loan’s life; comparing ratios on a cash basis versus amortised income can mislead. Bundled products: Cross-selling (e.g., credit-life insurance) may shift income from PAF to commissions, understating the ratio. Regulatory caps &amp; disclosures: Jurisdictions with fee ceilings or mandatory APR disclosures compress PAF ratios; cross-country benchmarking must control for such rules. Loan term effects: Short-tenor payday or BNPL loans show high PAF percentages even when absolute fees are small; interpret in context of maturity profile and APR. Waivers &amp; promotions: Temporary fee holidays for marketing campaigns can distort time-series trends—flag promotional periods separately. Should FSPs not be allowed/willing to share sensitive revenue data, ratios/percentages can be performed in-house and then shared with regulator.</t>
         </is>
       </c>
-      <c r="H127" t="inlineStr">
+      <c r="H129" t="inlineStr">
         <is>
           <t>What are the origination fee percentages as a share of loan principal by gender? Are there gender disparities in the origination fee percentages incurred? How do FSPs rank in terms of origination fee percentages by gender?</t>
         </is>
       </c>
-      <c r="I127" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J127" t="inlineStr">
-        <is>
-          <t>Financial inclusion</t>
-        </is>
-      </c>
-      <c r="K127" t="inlineStr">
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>Financial inclusion</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
         <is>
           <t>Quality</t>
         </is>
       </c>
-      <c r="L127" t="inlineStr">
+      <c r="L129" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Product type</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" t="inlineStr">
-        <is>
-          <t>Consumer protection</t>
-        </is>
-      </c>
-      <c r="B128" t="inlineStr">
-        <is>
-          <t>Data privacy and protection</t>
-        </is>
-      </c>
-      <c r="C128" t="inlineStr">
-        <is>
-          <t>Payments, Savings, Credit, Insurance, Pensions, Investments</t>
-        </is>
-      </c>
-      <c r="D128">
-        <v>232</v>
-      </c>
-      <c r="E128" t="inlineStr">
-        <is>
-          <t>Data breaches</t>
-        </is>
-      </c>
-      <c r="F128" t="inlineStr">
-        <is>
-          <t>% of customers affected by data breaches</t>
-        </is>
-      </c>
-      <c r="G128" t="inlineStr">
-        <is>
-          <t>A measure of the depth of cyberattacks or other data security breach that result in unauthorized access to customer data. Definitions and concept: A data breach is any security incident in which unauthorized parties access sensitive or confidential information, including personal data (tax numbers, ID information, bank account numbers, healthcare data) and corporate data (customer records, intellectual property, financial information). Data requirement: Number of customers whose data was accessed without authorization during a specified period of time (e.g. quarter or year); Total number of customers at the beginning of the specified period (e.g. quarter or year).</t>
-        </is>
-      </c>
-      <c r="H128" t="inlineStr">
-        <is>
-          <t>How does the percentage of customers affected by data breaches vary by gender? Are any genders disproportionately affected by data breaches? Are data breaches more frequent in certain types of FSPs? Are data breaches more common in specific channels or interfaces?"</t>
-        </is>
-      </c>
-      <c r="I128" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J128" t="inlineStr">
-        <is>
-          <t>Financial inclusion; Stability, safety and soundness</t>
-        </is>
-      </c>
-      <c r="K128" t="inlineStr">
-        <is>
-          <t>Quality, Operational risk</t>
-        </is>
-      </c>
-      <c r="L128" t="inlineStr">
-        <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" t="inlineStr">
-        <is>
-          <t>Consumer protection</t>
-        </is>
-      </c>
-      <c r="B129" t="inlineStr">
-        <is>
-          <t>Depositor protection</t>
-        </is>
-      </c>
-      <c r="C129" t="inlineStr">
-        <is>
-          <t>Savings</t>
-        </is>
-      </c>
-      <c r="D129">
-        <v>15</v>
-      </c>
-      <c r="E129" t="inlineStr">
-        <is>
-          <t>Deposit accounts covered by direct deposit insurance</t>
-        </is>
-      </c>
-      <c r="F129" t="inlineStr">
-        <is>
-          <t>Volume and value (balances) of deposit accounts covered by direct deposit insurance</t>
-        </is>
-      </c>
-      <c r="G129" t="inlineStr">
-        <is>
-          <t>This indicator counts (or expresses as a percentage) the deposit accounts that fall within the scope of an explicit, statutory deposit insurance scheme (DIS) or deposit guarantee fund. It helps supervisors gauge how much of the retail/MSME funding base is protected against bank failure. This is key for financial stability monitoring, payout readiness, and for calibrating the deposit insurance/guarantee fund. High coverage supports confidence and can dampen run dynamics. Source: https://www.iadi.org/uploads/cprevised2014nov.pdf. !- Definitions and concepts: Covered (eligible) account: a deposit type included by law. Fully insured vs. partially insured: “Fully insured” balances are ≤ the coverage limit per depositor, per bank, per ownership category; “covered/eligible” may include accounts whose balances exceed the cap (partially insured). Ownership categories: individual, joint, trust/fiduciary, retirement—rules vary by jurisdiction and affect aggregation across accounts. Indicator variants: % Eligible accounts = eligible deposit accounts ÷ total deposit accounts. Insured balance share = insured amounts in eligible accounts ÷ total deposit balances in eligible accounts. Dormancy: dormant accounts may be treated differently in coverage statistics.</t>
-        </is>
-      </c>
-      <c r="H129" t="inlineStr">
-        <is>
-          <t>Are there gender disparities in the number of deposit accounts covered by direct deposit insurance? How do these disparities vary by age, income level, and geographic location? Are certain gender groups, especially within vulnerable or low-income populations, less likely to hold insured deposit accounts? How do the average insured deposit account balances differ across genders, and what might this indicate about savings behavior, access to financial protection, or economic security? Do financial service providers with higher levels of gender diversity in leadership or staff tend to offer more equitable access to insured deposit accounts and balanced coverage across genders? Additionally, how do gender differences in insured deposit accounts relate to broader financial inclusion and resilience against financial shocks?</t>
-        </is>
-      </c>
-      <c r="I129" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J129" t="inlineStr">
-        <is>
-          <t>Financial inclusion; Consumer protection</t>
-        </is>
-      </c>
-      <c r="K129" t="inlineStr">
-        <is>
-          <t>Quality, Suitability</t>
-        </is>
-      </c>
-      <c r="L129" t="inlineStr">
-        <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Deposit account type</t>
         </is>
       </c>
     </row>
@@ -7180,28 +7260,148 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
+          <t>Data privacy and protection</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Payments, Savings, Credit, Insurance, Pensions, Investments</t>
+        </is>
+      </c>
+      <c r="D130">
+        <v>232</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>Data breaches</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>% of customers affected by data breaches</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>A measure of the depth of cyberattacks or other data security breach that result in unauthorized access to customer data. Definitions and concept: A data breach is any security incident in which unauthorized parties access sensitive or confidential information, including personal data (tax numbers, ID information, bank account numbers, healthcare data) and corporate data (customer records, intellectual property, financial information). Data requirement: Number of customers whose data was accessed without authorization during a specified period of time (e.g. quarter or year); Total number of customers at the beginning of the specified period (e.g. quarter or year).</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>How does the percentage of customers affected by data breaches vary by gender? Are any genders disproportionately affected by data breaches? Are data breaches more frequent in certain types of FSPs? Are data breaches more common in specific channels or interfaces?"</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>Financial inclusion; Stability, safety and soundness</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>Quality, Operational risk</t>
+        </is>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Consumer protection</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
           <t>Depositor protection</t>
         </is>
       </c>
-      <c r="C130" t="inlineStr">
+      <c r="C131" t="inlineStr">
         <is>
           <t>Savings</t>
         </is>
       </c>
-      <c r="D130">
+      <c r="D131">
+        <v>15</v>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Deposit accounts covered by direct deposit insurance</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>Volume and value (balances) of deposit accounts covered by direct deposit insurance</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>This indicator counts (or expresses as a percentage) the deposit accounts that fall within the scope of an explicit, statutory deposit insurance scheme (DIS) or deposit guarantee fund. It helps supervisors gauge how much of the retail/MSME funding base is protected against bank failure. This is key for financial stability monitoring, payout readiness, and for calibrating the deposit insurance/guarantee fund. High coverage supports confidence and can dampen run dynamics. Source: https://www.iadi.org/uploads/cprevised2014nov.pdf. !- Definitions and concepts: Covered (eligible) account: a deposit type included by law. Fully insured vs. partially insured: “Fully insured” balances are ≤ the coverage limit per depositor, per bank, per ownership category; “covered/eligible” may include accounts whose balances exceed the cap (partially insured). Ownership categories: individual, joint, trust/fiduciary, retirement—rules vary by jurisdiction and affect aggregation across accounts. Indicator variants: % Eligible accounts = eligible deposit accounts ÷ total deposit accounts. Insured balance share = insured amounts in eligible accounts ÷ total deposit balances in eligible accounts. Dormancy: dormant accounts may be treated differently in coverage statistics.</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>Are there gender disparities in the number of deposit accounts covered by direct deposit insurance? How do these disparities vary by age, income level, and geographic location? Are certain gender groups, especially within vulnerable or low-income populations, less likely to hold insured deposit accounts? How do the average insured deposit account balances differ across genders, and what might this indicate about savings behavior, access to financial protection, or economic security? Do financial service providers with higher levels of gender diversity in leadership or staff tend to offer more equitable access to insured deposit accounts and balanced coverage across genders? Additionally, how do gender differences in insured deposit accounts relate to broader financial inclusion and resilience against financial shocks?</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>Financial inclusion; Consumer protection</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>Quality, Suitability</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Deposit account type</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Consumer protection</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Depositor protection</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Savings</t>
+        </is>
+      </c>
+      <c r="D132">
         <v>16</v>
       </c>
-      <c r="E130" t="inlineStr">
+      <c r="E132" t="inlineStr">
         <is>
           <t>G2P accounts covered by deposit insurance</t>
         </is>
       </c>
-      <c r="F130" t="inlineStr">
+      <c r="F132" t="inlineStr">
         <is>
           <t>% of all accounts receiving G2P payments that are covered by deposit protection</t>
         </is>
       </c>
-      <c r="G130" t="inlineStr">
+      <c r="G132" t="inlineStr">
         <is>
           <t>This indicator helps analyze the extent to which low-value accounts are covered by deposit insurance or other protection. It focuses on account holders who are recipients of G2P programs. It quantifies how many of the government-to-person (G2P) payments recipients are protected by an explicit deposit insurance scheme or guarantee fund. It can be shown as (a) the share of G2P accounts that are eligible/fully insured and/or (b) the insured share of G2P balances. This indicator informs strategies for insurance/coverage payouts and the calibration of the deposit insurance fund. Definitions  and concepts: G2P account: an account that receives social transfers, government pensions, subsidies, or cash-benefit programs.
 Covered (eligible) vs. fully insured: “Eligible” products fall within the deposit insurance scope; “fully insured” means the balance per beneficiary per insured bank does not exceed the coverage cap. 
@@ -7210,669 +7410,559 @@
 Core-banking (and, where applicable, e-money) extracts: product code, ownership category, end-of-day balance, currency. Rules engine encoding national deposit-insurance scope, limits, and aggregation logic (per depositor—per bank). Sub-ledger data for pooled/FBO accounts to support pass-through eligibility. Timing sensitivity: balances spike on disbursement days; define the snapshot (e.g., month-end vs. T+2 after payout).</t>
         </is>
       </c>
-      <c r="H130" t="inlineStr">
+      <c r="H132" t="inlineStr">
         <is>
           <t>Are there gender disparities in the number of G2P accounts covered by deposit insurance? How do these disparities vary across different age groups, income levels, and geographic locations? Are women and other gender groups within vulnerable populations less likely to have G2P accounts that are insured, potentially affecting their financial security? How do the average balances of insured G2P accounts compare across genders, and what does this imply about economic empowerment and financial resilience? Do government programs and financial service providers with greater gender diversity in design or delivery show more equitable insurance coverage of G2P accounts? Additionally, how do gender differences in insured G2P accounts influence overall inclusion and access to social safety nets?</t>
         </is>
       </c>
-      <c r="I130" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J130" t="inlineStr">
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
         <is>
           <t>Financial inclusion; Consumer protection; Stability, safety and soundness</t>
         </is>
       </c>
-      <c r="K130" t="inlineStr">
+      <c r="K132" t="inlineStr">
         <is>
           <t>Quality, Suitability, Stability</t>
         </is>
       </c>
-      <c r="L130" t="inlineStr">
+      <c r="L132" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
         </is>
       </c>
     </row>
-    <row r="131">
-      <c r="A131" t="inlineStr">
+    <row r="133">
+      <c r="A133" t="inlineStr">
         <is>
           <t>Consumer protection</t>
         </is>
       </c>
-      <c r="B131" t="inlineStr">
+      <c r="B133" t="inlineStr">
         <is>
           <t>Fair treatment</t>
         </is>
       </c>
-      <c r="C131" t="inlineStr">
+      <c r="C133" t="inlineStr">
         <is>
           <t>Credit</t>
         </is>
       </c>
-      <c r="D131">
+      <c r="D133">
         <v>183</v>
       </c>
-      <c r="E131" t="inlineStr">
+      <c r="E133" t="inlineStr">
         <is>
           <t>Average cost-to-borrower for unsecured lending</t>
         </is>
       </c>
-      <c r="F131" t="inlineStr">
+      <c r="F133" t="inlineStr">
         <is>
           <t>Average topline revenue earned from unsecured retail credit operations (as percentage of the average outstanding unsecured credit)</t>
         </is>
       </c>
-      <c r="G131" t="inlineStr">
+      <c r="G133" t="inlineStr">
         <is>
           <t>This indicator is a portfolio-level proxy for the all-in price actually paid by customers on unsecured retail credit during the period. It answers: How many currency units of revenue did the lender earn for each 100 units of average unpaid balance? Rising values may reflect higher base rates, heavier fee reliance (e.g., late/over-limit charges), or a shift toward shorter-tenor/high-yield products; falling values can indicate competitive pressure, promotional pricing, or relief programs. Boards, supervisors, and consumer-protection teams use it to benchmark pricing fairness, earnings quality, and sensitivity to interest-rate cycles. !- Definitions and concepts: Recommended numerator (topline revenue, P&amp;L-recognized): Interest income (EIR basis) + contractual fees (origination, servicing) + penalty/default interest actually recognized + punitive fees (late, over-limit, returned-payment) − waivers/reversals. Denominator: Average outstanding unsecured retail balances (use Average Daily Balance - ADB). Formula: Cost-to-customer yield = Topline revenue from unsecured retail credit divded by Average outstanding unsecured retail balances. This indicator can be reported separately for interest, contractual fees and penalities if the data is available and when the period is less than 12 months, report an annualized figure. !- Data requirements: General ledger and product-level revenue broken into interest, contractual fees, penalty interest, punitive fees; flags for waivers/reversals and non-accrual. Loan/card-level balances to compute ADB, segmented by product (cards, instalment, overdraft, BNPL), channel, and risk bucket. Accounting policies: EIR vs. cash, Stage-3/non-accrual treatment, capitalization rules.
 FX mapping for multi-currency portfolios. !- Limitations and considerations: Comparability: EIR vs. cash accounting and non-accrual practices differ; disclose methodology. Mix effects: more revolving/short-tenor loans inflate yields; always segment. Penalty bias: high ratios may be driven by a small cohort repeatedly paying fees—track % customers incurring penalties. Promotions/teasers: intro 0% and fee holidays distort short periods—show trailing-12-month and cohort views. Scope creep: exclude bundled insurance premiums or merchant discounts (BNPL) unless consistently included and disclosed.</t>
         </is>
       </c>
-      <c r="H131" t="inlineStr">
+      <c r="H133" t="inlineStr">
         <is>
           <t>Are there gender disparities in the percentage of topline revenue relative to outstanding loan balances? Is there any gender paying comparatively more than market percentages for the same account types? How do FSPs rank in terms of these percentages by gender?</t>
         </is>
       </c>
-      <c r="J131" t="inlineStr">
-        <is>
-          <t>Financial inclusion</t>
-        </is>
-      </c>
-      <c r="K131" t="inlineStr">
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>Financial inclusion</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
         <is>
           <t>Quality</t>
         </is>
       </c>
-      <c r="L131" t="inlineStr">
+      <c r="L133" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Loan type</t>
         </is>
       </c>
     </row>
-    <row r="132">
-      <c r="A132" t="inlineStr">
+    <row r="134">
+      <c r="A134" t="inlineStr">
         <is>
           <t>Consumer protection</t>
         </is>
       </c>
-      <c r="B132" t="inlineStr">
+      <c r="B134" t="inlineStr">
         <is>
           <t>Fair treatment</t>
         </is>
       </c>
-      <c r="C132" t="inlineStr">
+      <c r="C134" t="inlineStr">
         <is>
           <t>Credit</t>
         </is>
       </c>
-      <c r="D132">
+      <c r="D134">
         <v>181</v>
       </c>
-      <c r="E132" t="inlineStr">
+      <c r="E134" t="inlineStr">
         <is>
           <t>Revenue generated by unsecured credit</t>
         </is>
       </c>
-      <c r="F132" t="inlineStr">
+      <c r="F134" t="inlineStr">
         <is>
           <t>% of total topline revenue attributable to unsecured credit operations and interest and non-interest revenue proportions</t>
         </is>
       </c>
-      <c r="G132" t="inlineStr">
+      <c r="G134" t="inlineStr">
         <is>
           <t>This indicator captures the total income that a lending institution earns from unsecured credit products—credit cards, personal instalment loans, overdrafts, payday and buy-now-pay-later (BNPL) facilities—over a reporting period. Because unsecured lending is typically high-yield and high-risk, tracking its revenue helps supervisors and management understand how much of the institution’s top line depends on products that are more sensitive to economic downturns, job-market shocks and aggressive competition. A rising share can boost short-term profitability, but it may also presage higher future credit losses and conduct-risk concerns if underwriting standards slip. !- Definitions and concepts: Unsecured credit – loans that are not backed by collateral; repayment relies on the borrower’s cash flow and creditworthiness.
 Revenue components – Interest income (accrued and collected) from outstanding balances. Fee income: annual fees, origination fees, late-payment charges, interchange on card transactions, BNPL merchant discount rates. Net insurance or payment-protection premiums (if bundled) may be included subject to local accounting rules.
 Revenue share metric: Unsecured-credit revenue ÷ Total lending revenue expresses concentration risk. Risk-adjusted yield – revenue net of credit-loss provisions gives a clearer view of economic profitability. !- Data requirements: Product-level general-ledger extracts segregating interest, fees and other income. Loan-level flags identifying collateral status (secured vs. unsecured). Average daily or month-end balances to compute effective yields. Associated credit-loss provisions and write-offs for risk-adjusted analysis. !- Limitations and considerations: Mixed products: Some personal loans are partially secured (e.g., salary-linked) or carry optional collateral; clear taxonomy is essential. Fee recognition rules: Capitalised origination fees amortised under effective-interest-rate (EIR) accounting may blur timing comparisons across banks or jurisdictions. Regulatory caps: Interest-rate or fee ceilings (e.g., usury limits) affect revenue potential and comparability. Promotional pricing: Introductory 0 % card offers or BNPL “pay-in-4” models generate deferred revenue; headline figures may understate future income. Economic cyclicality: Unsecured-credit revenue can fall sharply in recessions as balances contract and charge-offs rise; pairing with delinquency and provision metrics is crucial for a full risk-return picture.</t>
         </is>
       </c>
-      <c r="H132" t="inlineStr">
+      <c r="H134" t="inlineStr">
         <is>
           <t>What proportion of total topline revenue comes from unsecured credit operations, and are there gender disparities in this distribution? How do FSPs rank in their reliance on unsecured credit revenue by gender?</t>
         </is>
       </c>
-      <c r="I132" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="L132" t="inlineStr">
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>Financial inclusion</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
+      <c r="L134" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Loan type</t>
         </is>
       </c>
     </row>
-    <row r="133">
-      <c r="A133" t="inlineStr">
+    <row r="135">
+      <c r="A135" t="inlineStr">
         <is>
           <t>Consumer protection</t>
         </is>
       </c>
-      <c r="B133" t="inlineStr">
+      <c r="B135" t="inlineStr">
         <is>
           <t>Fair treatment</t>
         </is>
       </c>
-      <c r="C133" t="inlineStr">
+      <c r="C135" t="inlineStr">
         <is>
           <t>Insurance</t>
         </is>
       </c>
-      <c r="D133">
+      <c r="D135">
         <v>198</v>
       </c>
-      <c r="E133" t="inlineStr">
+      <c r="E135" t="inlineStr">
         <is>
           <t>Insurance approved claims not paid</t>
         </is>
       </c>
-      <c r="F133" t="inlineStr">
+      <c r="F135" t="inlineStr">
         <is>
           <t>% of approved/accepted claims that remain unpaid to customers</t>
         </is>
       </c>
-      <c r="G133" t="inlineStr">
+      <c r="G135" t="inlineStr">
         <is>
           <t>This indicator shows the share of claims that have been approved (final liability accepted) but not yet disbursed to the claimant. A high rate flags operational bottlenecks or weak payout controls, directly impacting customer outcomes. Track alongside claims turnaround time, claims rejection rates, and complaints, to get a full picture of payout effectiveness and customer fairness. !- Definitions and concepts: Approved / accepted claim: a claim with a final decision to pay (post-analysis), a recorded payable, and no outstanding dispute. Unpaid status: no successful settlement to the beneficiary by period end. Formula: Amount weighted (unpaid approved amount ÷ approved amount) reveal economic impact. Count basis (# approved claims not paid by cut-off ÷ # claims approved in teh period). SLA variant: % not paid within X days of approval (e.g., 5/10/30 days) to neutralize end-period timing bias. Treatment of partial payments: disclose whether partially paid claims are counted as unpaid or excluded. The indicator may also track the reasons for non-payment, if these are standardized for reporting. !- Limitations and considerations: Cut-off effects: approvals late in the period will naturally be unpaid—use the SLA variant and report both snapshot and flow views. Reopened claims / appeals: specify whether reversals after approval are removed from both numerator and denominator. Segmentation: monitor by line of business, payment method, channel, and claim size to target fixes.</t>
         </is>
       </c>
-      <c r="H133" t="inlineStr">
+      <c r="H135" t="inlineStr">
         <is>
           <t>How do the average values of outstanding insurance claims compare by gender? Is there a gender group with consistently higher average unpaid claims? How do different FSPs rank in terms of outstanding claims by gender? Are vulnerable gender groups disproportionately affected by delayed or unpaid claims?</t>
         </is>
       </c>
-      <c r="I133" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J133" t="inlineStr">
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
         <is>
           <t>Financial inclusion; Stability, safety and soundness</t>
         </is>
       </c>
-      <c r="K133" t="inlineStr">
+      <c r="K135" t="inlineStr">
         <is>
           <t>Quality, Reputational and legal risk</t>
         </is>
       </c>
-      <c r="L133" t="inlineStr">
+      <c r="L135" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Insurance type</t>
         </is>
       </c>
     </row>
-    <row r="134">
-      <c r="A134" t="inlineStr">
+    <row r="136">
+      <c r="A136" t="inlineStr">
         <is>
           <t>Consumer protection</t>
         </is>
       </c>
-      <c r="B134" t="inlineStr">
+      <c r="B136" t="inlineStr">
         <is>
           <t>Fair treatment</t>
         </is>
       </c>
-      <c r="C134" t="inlineStr">
+      <c r="C136" t="inlineStr">
         <is>
           <t>Insurance</t>
         </is>
       </c>
-      <c r="D134">
+      <c r="D136">
         <v>256</v>
       </c>
-      <c r="E134" t="inlineStr">
+      <c r="E136" t="inlineStr">
         <is>
           <t>Insurance claims declined</t>
         </is>
       </c>
-      <c r="F134" t="inlineStr">
+      <c r="F136" t="inlineStr">
         <is>
           <t>% of claims logged by policyholders that are declined prior to substantive analysis</t>
         </is>
       </c>
-      <c r="G134" t="inlineStr">
+      <c r="G136" t="inlineStr">
         <is>
           <t>This indicator captures the share of claim notifications the insurer does not accept for assessment at the front door—typically during first notice of loss (FNOL)/triage—because they are ineligible or incomplete. A high intake-decline rate can point to unclear policy wording, poor customer guidance, data-capture frictions, or overly strict gatekeeping. It is a key conduct-risk and customer-experience signal and, operationally, helps size avoidable workload versus genuinely assessable claims. Claim logged / FNOL: the moment a policyholder submits a claim or loss notice. Declined at intake (non-acceptance): the insurer refuses to open an assessable claim before investigation (e.g., policy not in force, peril not covered, waiting period, duplicate claim, claim below deductible/threshold, incomplete mandatory data not cured within a set window). Indicator formula (count basis): # claims declined at intake in period divided by # claim notifications received in period . Variants: exclude cured cases later resubmitted; report by product/channel. !- Data requirements: Claims-intake system fields: FNOL timestamp, policy ID/status at loss date, coverage/peril checks, deductible, mandatory-document checklist, triage outcome. Standardised reason codes (e.g., not covered, lapsed, duplicate, below excess, incomplete info). Deduplication logic (policyholder ID + incident date + peril). Linkage to resubmissions/appeals and to complaint records for outcome tracking. !- Limitations and considerations: Definition variance: what counts as “prior to analysis” differs; some firms place incomplete cases in “pending info” instead of “declined,” affecting comparability.
 Gaming risk: shifting cases to “withdrawn” or “pending” to improve this metric; require audit trails and age-off rules. Mix effects: products with low deductibles or mandatory documents (e.g., health) have different baseline rates—segment results. Customer fairness: high early declines may reflect confusing onboarding or exclusion wording; monitor alongside claims rejection rate (post-assessment), turnaround time, and complaints upheld. Resubmission policy: disclose whether cured resubmissions are excluded from the numerator to avoid double counting.</t>
         </is>
       </c>
-      <c r="H134" t="inlineStr">
+      <c r="H136" t="inlineStr">
         <is>
           <t>What percentage of claims logged by policyholders are declined, disaggregated by gender? How do these decline rates vary across FSPs, policy types, age groups, and locations? Are there notable gender disparities in claim declines at the market level or within specific providers? Are women or other gender groups more likely to face claim denial?</t>
         </is>
       </c>
-      <c r="I134" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J134" t="inlineStr">
-        <is>
-          <t>Financial inclusion</t>
-        </is>
-      </c>
-      <c r="K134" t="inlineStr">
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>Financial inclusion</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
         <is>
           <t>Quality</t>
         </is>
       </c>
-      <c r="L134" t="inlineStr">
+      <c r="L136" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Insurance type</t>
         </is>
       </c>
     </row>
-    <row r="135">
-      <c r="A135" t="inlineStr">
+    <row r="137">
+      <c r="A137" t="inlineStr">
         <is>
           <t>Consumer protection</t>
         </is>
       </c>
-      <c r="B135" t="inlineStr">
+      <c r="B137" t="inlineStr">
         <is>
           <t>Fair treatment</t>
         </is>
       </c>
-      <c r="C135" t="inlineStr">
+      <c r="C137" t="inlineStr">
         <is>
           <t>Insurance</t>
         </is>
       </c>
-      <c r="D135">
+      <c r="D137">
         <v>60</v>
       </c>
-      <c r="E135" t="inlineStr">
+      <c r="E137" t="inlineStr">
         <is>
           <t>Insurance claims rejection rate</t>
         </is>
       </c>
-      <c r="F135" t="inlineStr">
+      <c r="F137" t="inlineStr">
         <is>
           <t>% of all insurance claims that are rejected by insurers (post-analysis)</t>
         </is>
       </c>
-      <c r="G135" t="inlineStr">
+      <c r="G137" t="inlineStr">
         <is>
           <t>The claims rejection rate shows the share of claims that an insurer declines to pay—fully or partially—relative to the total number (or value) of claims submitted in a period. Because denial directly affects customer trust, supervisors use the metric to monitor fair treatment outcomes, detect aggressive underwriting or opaque policy wording, and flag operational shortcomings. A sudden rise may presage reputational damage, regulatory sanctions, or litigation costs, while an unusually low rate can hint at lax fraud controls or inadequate claims processing. !- Definitions and concepts: Claims rejected (denied): claims for which the insurer issues a final communication refusing payment on contractual grounds (e.g., policy exclusions, lapsed cover, misrepresentation) or on fraud findings. !- Limitations and considerations: Definition divergence: Some regimes class “claims closed without payment” (due to missing documents) as rejections; others record them as pending, complicating cross-market comparison. Fraud vs. technical denial: Combining fraud rejections with contractual exclusions can blur very different issues. Separate reporting is best practice. Volume vs. value: A single large, legitimately denied loss can distort amount-based ratios; analysts should monitor both count and value metrics.
 Appeals and reversals: Denials overturned on review lower true rejection rates; timely data updates are essential.
 Incentive effects: Over-emphasis on low rejection rates may weaken fraud vigilance, whereas strict targets can push staff toward technical denials—pair the indicator with complaint ratios, turnaround times, and fraud-detection statistics for balanced oversight.</t>
         </is>
       </c>
-      <c r="H135" t="inlineStr">
+      <c r="H137" t="inlineStr">
         <is>
           <t>Are there gender disparities in the rejection rates of insurance claims, including for MSMEs by owner gender? Which types of policies or claims see higher rejection rates, and do these differ by gender? How does claim rejection relate to coverage levels and turnaround times? Do FSPs with higher gender diversity have lower rejection rates for vulnerable gender groups?</t>
         </is>
       </c>
-      <c r="I135" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J135" t="inlineStr">
-        <is>
-          <t>Financial inclusion</t>
-        </is>
-      </c>
-      <c r="K135" t="inlineStr">
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>Financial inclusion</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
         <is>
           <t>Quality</t>
         </is>
       </c>
-      <c r="L135" t="inlineStr">
+      <c r="L137" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Insurance type</t>
         </is>
       </c>
     </row>
-    <row r="136">
-      <c r="A136" t="inlineStr">
+    <row r="138">
+      <c r="A138" t="inlineStr">
         <is>
           <t>Consumer protection</t>
         </is>
       </c>
-      <c r="B136" t="inlineStr">
+      <c r="B138" t="inlineStr">
         <is>
           <t>Fair treatment</t>
         </is>
       </c>
-      <c r="C136" t="inlineStr">
+      <c r="C138" t="inlineStr">
         <is>
           <t>Insurance</t>
         </is>
       </c>
-      <c r="D136">
+      <c r="D138">
         <v>201</v>
       </c>
-      <c r="E136" t="inlineStr">
+      <c r="E138" t="inlineStr">
         <is>
           <t>Insurance claims settlement ratio</t>
         </is>
       </c>
-      <c r="F136" t="inlineStr">
+      <c r="F138" t="inlineStr">
         <is>
           <t>% of insurance claims logged by policyholders that have been paid by insurers</t>
         </is>
       </c>
-      <c r="G136" t="inlineStr">
+      <c r="G138" t="inlineStr">
         <is>
           <t>Measures the percentage of insurance claims settled by an insurer out of the total claims it receives. It is a direct measure of an insurer's reliability and its commitment to fulfilling its primary promise to policyholders. This indicator is a cornerstone of conduct supervision, as it provides a quantitative view of how an insurer treats its customers at their most critical moment of need. For prudential supervisors, it could help analysis of operational and reputational risk. This indicator should be used together with other indicators on the performance of the claims process in the insurance sector.</t>
         </is>
       </c>
-      <c r="H136" t="inlineStr">
+      <c r="H138" t="inlineStr">
         <is>
           <t>How do claim settlement ratios vary by gender? Are any gender groups receiving lower settlement ratios compared to the market average? Are there FSPs with particularly low or high settlement ratios for certain genders? How do these ratios intersect with policy type and customer demographics?</t>
         </is>
       </c>
-      <c r="I136" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J136" t="inlineStr">
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
         <is>
           <t>Financial inclusion; Stability, safety and soundness</t>
         </is>
       </c>
-      <c r="K136" t="inlineStr">
+      <c r="K138" t="inlineStr">
         <is>
           <t>Outcomes, Reputational and legal risk</t>
         </is>
       </c>
-      <c r="L136" t="inlineStr">
+      <c r="L138" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Insurance type</t>
         </is>
       </c>
     </row>
-    <row r="137">
-      <c r="A137" t="inlineStr">
+    <row r="139">
+      <c r="A139" t="inlineStr">
         <is>
           <t>Consumer protection</t>
         </is>
       </c>
-      <c r="B137" t="inlineStr">
+      <c r="B139" t="inlineStr">
         <is>
           <t>Fair treatment</t>
         </is>
       </c>
-      <c r="C137" t="inlineStr">
+      <c r="C139" t="inlineStr">
         <is>
           <t>Insurance</t>
         </is>
       </c>
-      <c r="D137">
+      <c r="D139">
         <v>59</v>
       </c>
-      <c r="E137" t="inlineStr">
+      <c r="E139" t="inlineStr">
         <is>
           <t>Insurance claims turnaround time</t>
         </is>
       </c>
-      <c r="F137" t="inlineStr">
+      <c r="F139" t="inlineStr">
         <is>
           <t>Average number of days to process insurance claims</t>
         </is>
       </c>
-      <c r="G137" t="inlineStr">
+      <c r="G139" t="inlineStr">
         <is>
           <t>This indicator captures the average calendar days an insurer takes to settle a claim—from the claim filing date to the final payment or formal denial. It is a direct yard-stick of operational efficiency and customer experience. Shorter turnaround times (TATs) enhance policy-holder trust, limit reputational risk, and can lower claims handling expenses. Supervisors use the metric to enforce fair-treatment rules, while actuaries and underwriters link it to reserving accuracy—prolonged settlement can signal documentation bottlenecks, fraud investigations, policy transparency issues, or catastrophic complexity that may keep outstanding reserves elevated. !- Definitions and concepts:  Start point – the timestamp when the insurer first receives the claim request. End point – the date the insurer issues full payment, partial final payment, or a written denial. Average turnaround time (TAT) – arithmetic mean; many firms also monitor median and 90th-percentile to limit outlier masking.
 Segmented TATs – tracked by line of business, claim severity band, and distribution channel to isolate problem areas.
 !- Limitations and considerations: Partial settlements: Recording the date of first partial payment can understate full-and-final completion time. Dispute and litigation pauses: Regulatory or court‐mandated suspensions inflate TAT yet lie outside managerial control.</t>
         </is>
       </c>
-      <c r="H137" t="inlineStr">
+      <c r="H139" t="inlineStr">
         <is>
           <t>Are there gender disparities in the average time taken to process and settle insurance claims? How does processing time vary by policy type, premium, claim amount, and customer demographics? Are insurers with lower gender diversity more likely to have longer turnaround times? Are vulnerable gender groups disproportionately affected by delays?</t>
         </is>
       </c>
-      <c r="J137" t="inlineStr">
-        <is>
-          <t>Financial inclusion</t>
-        </is>
-      </c>
-      <c r="K137" t="inlineStr">
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>Financial inclusion</t>
+        </is>
+      </c>
+      <c r="K139" t="inlineStr">
         <is>
           <t>Quality</t>
         </is>
       </c>
-      <c r="L137" t="inlineStr">
+      <c r="L139" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Insurance type</t>
         </is>
       </c>
     </row>
-    <row r="138">
-      <c r="A138" t="inlineStr">
+    <row r="140">
+      <c r="A140" t="inlineStr">
         <is>
           <t>Consumer protection</t>
         </is>
       </c>
-      <c r="B138" t="inlineStr">
+      <c r="B140" t="inlineStr">
         <is>
           <t>Fair treatment</t>
         </is>
       </c>
-      <c r="C138" t="inlineStr">
+      <c r="C140" t="inlineStr">
         <is>
           <t>Investments</t>
         </is>
       </c>
-      <c r="D138">
+      <c r="D140">
         <v>207</v>
       </c>
-      <c r="E138" t="inlineStr">
+      <c r="E140" t="inlineStr">
         <is>
           <t>Net rate of return on investments</t>
         </is>
       </c>
-      <c r="F138" t="inlineStr">
+      <c r="F140" t="inlineStr">
         <is>
           <t>% point differential between the average rates of returns on investments and the average performance/administration fees charged</t>
         </is>
       </c>
-      <c r="G138" t="inlineStr">
+      <c r="G140" t="inlineStr">
         <is>
           <t>Measures the profitability of a financial institution's own investment portfolio after accounting for all associated costs. It reveals the actual, bottom-line gain or loss generated by the institution's securities, real estate, or other investments. This is a fundamental indicator of an institution's ability to effectively manage its own capital and generate profit from non-lending activities, of particular importance to prudential supervisors, including supervisors of insurance and pension administrators. Net Rate of Return (%)= 
 [(Market Value final-Market Value initial+Income−Expenses)/Market Value initial]×100</t>
         </is>
       </c>
-      <c r="H138" t="inlineStr">
+      <c r="H140" t="inlineStr">
         <is>
           <t>How do net returns (% returns minus % performance fees and charges) on longer-term investments compare by gender? Do net returns for any gender differ from the overall market average for similar investment products? How do FSPs compare in terms of net returns earned by gender?</t>
         </is>
       </c>
-      <c r="J138" t="inlineStr">
-        <is>
-          <t>Market development</t>
-        </is>
-      </c>
-      <c r="K138" t="inlineStr">
-        <is>
-          <t>Capital markets development</t>
-        </is>
-      </c>
-      <c r="L138" t="inlineStr">
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>Market development; Financial inclusion</t>
+        </is>
+      </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>Capital markets development, Quality</t>
+        </is>
+      </c>
+      <c r="L140" t="inlineStr">
         <is>
           <t>Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
         </is>
       </c>
     </row>
-    <row r="139">
-      <c r="A139" t="inlineStr">
+    <row r="141">
+      <c r="A141" t="inlineStr">
         <is>
           <t>Consumer protection</t>
         </is>
       </c>
-      <c r="B139" t="inlineStr">
+      <c r="B141" t="inlineStr">
         <is>
           <t>Fair treatment</t>
         </is>
       </c>
-      <c r="C139" t="inlineStr">
+      <c r="C141" t="inlineStr">
         <is>
           <t>Savings</t>
         </is>
       </c>
-      <c r="D139">
+      <c r="D141">
         <v>159</v>
       </c>
-      <c r="E139" t="inlineStr">
+      <c r="E141" t="inlineStr">
         <is>
           <t>Average cost-to-customer for transaction accounts</t>
         </is>
       </c>
-      <c r="F139" t="inlineStr">
+      <c r="F141" t="inlineStr">
         <is>
           <t>Average topline revenue earned per account holder as % of average account balances</t>
         </is>
       </c>
-      <c r="G139" t="inlineStr">
+      <c r="G141" t="inlineStr">
         <is>
           <t>This indicator estimates the effective price of holding and using a transaction account, expressed as a yield on the customer’s average balance. By computing it for each account type (e.g., basic/no-frills, standard retail, premium, MSMEs, e-money wallet), it reveals where pricing and usage frictions are highest. It helps supervisors assess fairness, inclusion quality, and reliance on fee income. !- Definitions and concepts: Non-interest fees: maintenance/inactivity, ATM/network, FX/transfer, statement/card fees, overdraft &amp; returned-payment fees tied to the account. 
 Per account-holder basis: aggregate all accounts of the same type per customer, then average (also show balance-weighted results). !- Data requirements: Core-banking data: customer ID, account type tags, average daily balance by customer for each account type, interest credited, revenue by fee code linked to accounts; flags for waivers/refunds/chargebacks. Channel/product hierarchies (basic vs. premium, retail vs. MSMEs, wallet vs. bank account) and currency/FX mapping. Optional: usage indicators (transactions per month) to explain differences across types.</t>
         </is>
       </c>
-      <c r="H139" t="inlineStr">
+      <c r="H141" t="inlineStr">
         <is>
           <t>Are there gender disparities in the costs (fees, charges) borne by account holders of transaction accounts? Do women tend to hold transaction accounts with higher fee burdens (relative to income or transaction frequency) than men, particularly in certain regions or among lower‐income groups? How do costs compare across FSPs with different levels of gender diversity? Is fee structure or cost‐to‐customer a barrier to transaction usage for some gender/age/income cohorts?</t>
         </is>
       </c>
-      <c r="J139" t="inlineStr">
-        <is>
-          <t>Financial inclusion</t>
-        </is>
-      </c>
-      <c r="K139" t="inlineStr">
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>Financial inclusion</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
         <is>
           <t>Quality</t>
         </is>
       </c>
-      <c r="L139" t="inlineStr">
+      <c r="L141" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Financial service provider (FSP) type; Account type</t>
-        </is>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" t="inlineStr">
-        <is>
-          <t>Consumer protection</t>
-        </is>
-      </c>
-      <c r="B140" t="inlineStr">
-        <is>
-          <t>Fair treatment</t>
-        </is>
-      </c>
-      <c r="C140" t="inlineStr">
-        <is>
-          <t>Payments, Savings, Credit, Insurance, Pensions, Investments</t>
-        </is>
-      </c>
-      <c r="D140">
-        <v>226</v>
-      </c>
-      <c r="E140" t="inlineStr">
-        <is>
-          <t>Rejections of product applications</t>
-        </is>
-      </c>
-      <c r="F140" t="inlineStr">
-        <is>
-          <t>% of all applications that are rejected by product type</t>
-        </is>
-      </c>
-      <c r="G140" t="inlineStr">
-        <is>
-          <t>Measures the proportion of customer applications for financial products that are rejected by regulated financial institutions during the reporting period. The indicator is calculated as the percentage of total applications received—across products such as loans, credit cards, deposit accounts, or insurance policies—that were not approved or accepted. Captures the extent of unmet demand or access barriers in financial markets, as well as aspects of market conduct, underwriting practices, and risk appetite among providers. It provides insight into how easily consumers and businesses can obtain financial products. Monitoring rejection rates helps authorities: Identify potential access constraints or discriminatory lending or sales practices; Evaluate the tightness of credit or account-opening standards; Assess consumer protection outcomes and fair treatment; Detect sudden shifts in provider risk tolerance or macro-prudential conditions (e.g., post-crisis credit tightening). High rejection rates may indicate stringent eligibility criteria, weak applicant creditworthiness, or barriers to financial access. Declining rates may suggest improving inclusion or relaxation of underwriting standards. Cross-product comparisons reveal whether certain markets (e.g., credit vs. deposits) are more exclusionary. !- Definitions and concepts: Application: A formal request by a customer to obtain a financial product or service. Rejection: A decision by the provider not to approve, issue, or open the requested product, whether automated or manual. Product type: Category of financial service applied for (loan, deposit, insurance, card, etc.). !- Data requirements: Product application records from regulated financail institutions that can yield the total number of applications rejected and the total number of applications received during the reference period. Disaggregation variables for segmentation analysis: product type, applicant type (individual, MSME), gender etc.</t>
-        </is>
-      </c>
-      <c r="H140" t="inlineStr">
-        <is>
-          <t>How do rejection rates vary by gender for individuasl and MSME? Are rejection rates higher for any gender in specific channels? How do rejection rates in physical channels compare to those in digital channels by gender? How do FSPs rank in terms of rejection rates by gender across available channels, by type of customer (individuals, MSME)?</t>
-        </is>
-      </c>
-      <c r="I140" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J140" t="inlineStr">
-        <is>
-          <t>Financial inclusion</t>
-        </is>
-      </c>
-      <c r="K140" t="inlineStr">
-        <is>
-          <t>Quality</t>
-        </is>
-      </c>
-      <c r="L140" t="inlineStr">
-        <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Product type</t>
-        </is>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" t="inlineStr">
-        <is>
-          <t>Consumer protection</t>
-        </is>
-      </c>
-      <c r="B141" t="inlineStr">
-        <is>
-          <t>Suitability</t>
-        </is>
-      </c>
-      <c r="C141" t="inlineStr">
-        <is>
-          <t>Credit</t>
-        </is>
-      </c>
-      <c r="D141">
-        <v>171</v>
-      </c>
-      <c r="E141" t="inlineStr">
-        <is>
-          <t>Unsecured credit facilities per borrower</t>
-        </is>
-      </c>
-      <c r="F141" t="inlineStr">
-        <is>
-          <t>Average volume and value (outstanding amount) of unsecured credit operations per borrower</t>
-        </is>
-      </c>
-      <c r="G141" t="inlineStr">
-        <is>
-          <t>This indicator shows, for each unsecured credit type (e.g., credit cards, personal instalment loans, overdrafts/lines, BNPL/pay-in-4, microcredit), how many active facilities the typical borrower holds (volume) and how much they owe on average (value). It reveals product stacking, utilisation intensity, and pockets of affordability risk. Rising volumes with flat values can indicate product fragmentation (e.g., multiple small BNPL plans), while high values per borrower point to concentration risk and potential loss severity. !- Definitions and concepts: Borrower universe per type (t): unique customers with ≥1 active unsecured facility of type (t) during the period. Average volume (holders-only) = [Total number of active contracts of type t for borrow b] / [Total number of unique borrowers with facility of type t]. Average value (holders only) = [Average daily outstanding balance across all of borrower b's facility of type t] / [Total number of unique borrowers with facility of type t]. Outstanding amount: Gross carrying amount before prvisions, exclude undrawn limits. Attribution rules: Define treatment of joint borrowers (full vs. proportional), refinances/restructures and charged-off accounts (exclude once written off, unless still on-book). !- Data requirements: Loan/line-level records with borrower ID, product/credit-type tag, status, origination date, limit (revolving), currency, and daily balances. Deduped customer master across subsidiaries/channels; joint-borrower flags. FX rates for multi-currency portfolios; calendar to compute ADB over the period. !- Limitations and considerations: Seasonality: cards/overdrafts spike around holidays—use ADB and rolling windows. Mix effects: comparing cards (revolving) with instalments needs a utilisation companion metric. Policy choices: inclusion of dormant but open lines, re-aged accounts, or post-charge-off recoveries changes results—document choices. Distribution matters: report median and percentiles per type alongside means to avoid high-balance skew.</t>
-        </is>
-      </c>
-      <c r="H141" t="inlineStr">
-        <is>
-          <t>How does the average number of outstanding loans per borrower vary by gender? Are outstanding balances more concentrated in long- or short-term loans, and does this differ by gender? Have gender disparities in loan terms evolved over time?</t>
-        </is>
-      </c>
-      <c r="I141" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J141" t="inlineStr">
-        <is>
-          <t>Financial inclusion; Stability, safety and soundness</t>
-        </is>
-      </c>
-      <c r="K141" t="inlineStr">
-        <is>
-          <t>Outcomes, Credit risk</t>
-        </is>
-      </c>
-      <c r="L141" t="inlineStr">
-        <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Loan type</t>
         </is>
       </c>
     </row>
@@ -7884,7 +7974,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Safety and security</t>
+          <t>Fair treatment</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -7893,26 +7983,26 @@
         </is>
       </c>
       <c r="D142">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>Frauds faced by customers</t>
+          <t>Rejections of product applications</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>% of customers affected by fraud</t>
+          <t>% of all applications that are rejected by product type</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>Fraud directly erodes consumer confidence, trust in financial institutions and can trigger liquidity or solvency stress for institutions, tracking its incidence lets supervisors spot emerging threats before they undermine financial stability. Consistent monitoring also reveals control weaknesses, helping authorities direct enforcement, bolster preventive regulation, and keep the payments and deposit system trusted and resilient. This indicator measures the share of customers of financial services that have been victims of fraud over a specific period. !- Definitions and concepts: Several definitions of fraud exist and vary depending on the jurisdiction, local definitions of fraud for statistical reporting purposes should be used. For example, the European Banking Authority splits fraudelent payment transactions into two categories: (1) Unauthorised payment transactions: transfers made “as a result of the loss, theft or misappropriation of sensitive payment data or a payment instrument … executed in the absence of consent by the payer.” and (2) Manipulation of the payer: transactions “made as a result of the payer being manipulated … to issue a payment order … in good faith, to a payment account it believes belongs to a legitimate payee.” This definition anchors EU-wide fraud statistics and stresses both technical compromise (e.g., stolen credentials) and social-engineering scams (e.g., authorised push-payment fraud). !- Data requirements: Transactions initiated and executed during a specified period that are flagged as fraudulent linked to a unique customer ID; Total number of customer at the beginning of the specified period.</t>
+          <t>Measures the proportion of customer applications for financial products that are rejected by regulated financial institutions during the reporting period. The indicator is calculated as the percentage of total applications received—across products such as loans, credit cards, deposit accounts, or insurance policies—that were not approved or accepted. Captures the extent of unmet demand or access barriers in financial markets, as well as aspects of market conduct, underwriting practices, and risk appetite among providers. It provides insight into how easily consumers and businesses can obtain financial products. Monitoring rejection rates helps authorities: Identify potential access constraints or discriminatory lending or sales practices; Evaluate the tightness of credit or account-opening standards; Assess consumer protection outcomes and fair treatment; Detect sudden shifts in provider risk tolerance or macro-prudential conditions (e.g., post-crisis credit tightening). High rejection rates may indicate stringent eligibility criteria, weak applicant creditworthiness, or barriers to financial access. Declining rates may suggest improving inclusion or relaxation of underwriting standards. Cross-product comparisons reveal whether certain markets (e.g., credit vs. deposits) are more exclusionary. !- Definitions and concepts: Application: A formal request by a customer to obtain a financial product or service. Rejection: A decision by the provider not to approve, issue, or open the requested product, whether automated or manual. Product type: Category of financial service applied for (loan, deposit, insurance, card, etc.). !- Data requirements: Product application records from regulated financail institutions that can yield the total number of applications rejected and the total number of applications received during the reference period. Disaggregation variables for segmentation analysis: product type, applicant type (individual, MSME), gender etc.</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>How does the number of fraud cases vary by gender? Are any genders disproportionately affected by fraud? Are fraud cases more frequent in certain types of FSPs?</t>
+          <t>How do rejection rates vary by gender for individuasl and MSME? Are rejection rates higher for any gender in specific channels? How do rejection rates in physical channels compare to those in digital channels by gender? How do FSPs rank in terms of rejection rates by gender across available channels, by type of customer (individuals, MSME)?</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -7922,17 +8012,17 @@
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>Financial inclusion; Stability, safety and soundness</t>
+          <t>Financial inclusion</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>Quality, AML/CFT</t>
+          <t>Quality</t>
         </is>
       </c>
       <c r="L142" t="inlineStr">
         <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Product type</t>
         </is>
       </c>
     </row>
@@ -7944,35 +8034,35 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Safety and security</t>
+          <t>Suitability</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Payments, Savings, Credit, Insurance, Pensions, Investments</t>
+          <t>Credit</t>
         </is>
       </c>
       <c r="D143">
-        <v>233</v>
+        <v>171</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>Frauds resulting in customer losses</t>
+          <t>Unsecured credit facilities per borrower</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>Average volume and value (losses incurred) of frauds experienced by customers</t>
+          <t>Average volume and value (outstanding amount) of unsecured credit operations per borrower</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>Fraud directly erodes consumer confidence, trust in financial institutions and can trigger liquidity or solvency stress for institutions, tracking its incidence lets supervisors spot emerging threats before they undermine financial stability. Consistent monitoring also reveals control weaknesses, helping authorities direct enforcement, bolster preventive regulation, and keep the payments and deposit system trusted and resilient. This indicator measures the number of transactions that have been flagged as fraudulent and their corresponding value in currency.  !- Definitions and concepts: Several definitions of fraud exist and vary depending on the jurisdiction, local definitions of fraud for statistical reporting purposes should be used. For example, the European Banking Authority splits fraudelent payment transactions into two categories: (1) Unauthorised payment transactions: transfers made “as a result of the loss, theft or misappropriation of sensitive payment data or a payment instrument … executed in the absence of consent by the payer.” and (2) Manipulation of the payer: transactions “made as a result of the payer being manipulated … to issue a payment order … in good faith, to a payment account it believes belongs to a legitimate payee.” This definition anchors EU-wide fraud statistics and stresses both technical compromise (e.g., stolen credentials) and social-engineering scams (e.g., authorised push-payment fraud). !- Data requirements: Total number of transactions initiated and executed during a specified period that are flagged as fraudulent;  Total value of transactions initiated and executed during a specified period that are flagged as fraudulent.</t>
+          <t>This indicator shows, for each unsecured credit type (e.g., credit cards, personal instalment loans, overdrafts/lines, BNPL/pay-in-4, microcredit), how many active facilities the typical borrower holds (volume) and how much they owe on average (value). It reveals product stacking, utilisation intensity, and pockets of affordability risk. Rising volumes with flat values can indicate product fragmentation (e.g., multiple small BNPL plans), while high values per borrower point to concentration risk and potential loss severity. !- Definitions and concepts: Borrower universe per type (t): unique customers with ≥1 active unsecured facility of type (t) during the period. Average volume (holders-only) = [Total number of active contracts of type t for borrow b] / [Total number of unique borrowers with facility of type t]. Average value (holders only) = [Average daily outstanding balance across all of borrower b's facility of type t] / [Total number of unique borrowers with facility of type t]. Outstanding amount: Gross carrying amount before prvisions, exclude undrawn limits. Attribution rules: Define treatment of joint borrowers (full vs. proportional), refinances/restructures and charged-off accounts (exclude once written off, unless still on-book). !- Data requirements: Loan/line-level records with borrower ID, product/credit-type tag, status, origination date, limit (revolving), currency, and daily balances. Deduped customer master across subsidiaries/channels; joint-borrower flags. FX rates for multi-currency portfolios; calendar to compute ADB over the period. !- Limitations and considerations: Seasonality: cards/overdrafts spike around holidays—use ADB and rolling windows. Mix effects: comparing cards (revolving) with instalments needs a utilisation companion metric. Policy choices: inclusion of dormant but open lines, re-aged accounts, or post-charge-off recoveries changes results—document choices. Distribution matters: report median and percentiles per type alongside means to avoid high-balance skew.</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>How do financial loss-related fraud cases impact genders differently? Are any genders disproportionately affected by frauds that result in financial losses? Are fraud cases involving financial losses more common in certain types of FSPs?</t>
+          <t>How does the average number of outstanding loans per borrower vary by gender? Are outstanding balances more concentrated in long- or short-term loans, and does this differ by gender? Have gender disparities in loan terms evolved over time?</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -7987,12 +8077,12 @@
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>Outcomes, AML/CFT</t>
+          <t>Quality, Credit risk</t>
         </is>
       </c>
       <c r="L143" t="inlineStr">
         <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Loan type</t>
         </is>
       </c>
     </row>
@@ -8013,162 +8103,162 @@
         </is>
       </c>
       <c r="D144">
+        <v>231</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Frauds faced by customers</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>% of customers affected by fraud</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>Fraud directly erodes consumer confidence, trust in financial institutions and can trigger liquidity or solvency stress for institutions, tracking its incidence lets supervisors spot emerging threats before they undermine financial stability. Consistent monitoring also reveals control weaknesses, helping authorities direct enforcement, bolster preventive regulation, and keep the payments and deposit system trusted and resilient. This indicator measures the share of customers of financial services that have been victims of fraud over a specific period. !- Definitions and concepts: Several definitions of fraud exist and vary depending on the jurisdiction, local definitions of fraud for statistical reporting purposes should be used. For example, the European Banking Authority splits fraudelent payment transactions into two categories: (1) Unauthorised payment transactions: transfers made “as a result of the loss, theft or misappropriation of sensitive payment data or a payment instrument … executed in the absence of consent by the payer.” and (2) Manipulation of the payer: transactions “made as a result of the payer being manipulated … to issue a payment order … in good faith, to a payment account it believes belongs to a legitimate payee.” This definition anchors EU-wide fraud statistics and stresses both technical compromise (e.g., stolen credentials) and social-engineering scams (e.g., authorised push-payment fraud). !- Data requirements: Transactions initiated and executed during a specified period that are flagged as fraudulent linked to a unique customer ID; Total number of customer at the beginning of the specified period.</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>How does the number of fraud cases vary by gender? Are any genders disproportionately affected by fraud? Are fraud cases more frequent in certain types of FSPs?</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>Financial inclusion; Stability, safety and soundness</t>
+        </is>
+      </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>Quality, AML/CFT</t>
+        </is>
+      </c>
+      <c r="L144" t="inlineStr">
+        <is>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Consumer protection</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Safety and security</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Payments, Savings, Credit, Insurance, Pensions, Investments</t>
+        </is>
+      </c>
+      <c r="D145">
+        <v>233</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Frauds resulting in customer losses</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>Average volume and value (losses incurred) of frauds experienced by customers</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>Fraud directly erodes consumer confidence, trust in financial institutions and can trigger liquidity or solvency stress for institutions, tracking its incidence lets supervisors spot emerging threats before they undermine financial stability. Consistent monitoring also reveals control weaknesses, helping authorities direct enforcement, bolster preventive regulation, and keep the payments and deposit system trusted and resilient. This indicator measures the number of transactions that have been flagged as fraudulent and their corresponding value in currency.  !- Definitions and concepts: Several definitions of fraud exist and vary depending on the jurisdiction, local definitions of fraud for statistical reporting purposes should be used. For example, the European Banking Authority splits fraudelent payment transactions into two categories: (1) Unauthorised payment transactions: transfers made “as a result of the loss, theft or misappropriation of sensitive payment data or a payment instrument … executed in the absence of consent by the payer.” and (2) Manipulation of the payer: transactions “made as a result of the payer being manipulated … to issue a payment order … in good faith, to a payment account it believes belongs to a legitimate payee.” This definition anchors EU-wide fraud statistics and stresses both technical compromise (e.g., stolen credentials) and social-engineering scams (e.g., authorised push-payment fraud). !- Data requirements: Total number of transactions initiated and executed during a specified period that are flagged as fraudulent;  Total value of transactions initiated and executed during a specified period that are flagged as fraudulent.</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>How do financial loss-related fraud cases impact genders differently? Are any genders disproportionately affected by frauds that result in financial losses? Are fraud cases involving financial losses more common in certain types of FSPs?</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>Financial inclusion; Stability, safety and soundness</t>
+        </is>
+      </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>Outcomes, AML/CFT</t>
+        </is>
+      </c>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Consumer protection</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Safety and security</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Payments, Savings, Credit, Insurance, Pensions, Investments</t>
+        </is>
+      </c>
+      <c r="D146">
         <v>230</v>
       </c>
-      <c r="E144" t="inlineStr">
+      <c r="E146" t="inlineStr">
         <is>
           <t>Physical safety</t>
         </is>
       </c>
-      <c r="F144" t="inlineStr">
+      <c r="F146" t="inlineStr">
         <is>
           <t>Number of physical security incidents and number of customers affected</t>
         </is>
       </c>
-      <c r="G144" t="inlineStr">
+      <c r="G146" t="inlineStr">
         <is>
           <t>This indicator captures the total number of reported physical security incidents that occur in connection with the operations of financial service providers (FSPs) — including banks, microfinance institutions, payment service providers, and other regulated entities — as well as the number of customers directly affected by such incidents. Physical security incidents include events such as armed robberies, thefts, assaults, vandalism, or damage to property occurring at branches, ATMs, cash-in-transit vehicles, or other service delivery points. The “number of customers affected” reflects individuals who have experienced harm, loss, or disruption of service as a result of these events.This indicator measures the operational risk exposure of the financial sector to physical threats and criminal activity, and the extent to which such incidents impact customers and public trust. It forms part of the broader construct of operational resilience and consumer protection, providing insights into the safety of physical access points within the financial system. Supervisory reporting could record:
 Number of incidents = Total count of reported physical security incidents during the reference period (e.g., quarterly or annually). Number of customers affected = Total number of customers who suffered loss, injury, or service disruption due to those incidents. !- Derivable indicators: Incident rate = (Number of incidents / Total number of service points) × 1,000; Customer impact rate = (Number of customers affected / Total number of customers) × 100</t>
         </is>
       </c>
-      <c r="H144" t="inlineStr">
+      <c r="H146" t="inlineStr">
         <is>
           <t>How does the number of physical security incidents vary by gender? Are any genders disproportionately affected? Are physical security incidents more common in certain types of FSPs?</t>
         </is>
       </c>
-      <c r="J144" t="inlineStr">
+      <c r="J146" t="inlineStr">
         <is>
           <t>Financial inclusion; Stability, safety and soundness</t>
         </is>
       </c>
-      <c r="K144" t="inlineStr">
+      <c r="K146" t="inlineStr">
         <is>
           <t>Outcomes, Reputational and legal risk</t>
         </is>
       </c>
-      <c r="L144" t="inlineStr">
+      <c r="L146" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
-        </is>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" t="inlineStr">
-        <is>
-          <t>Consumer protection</t>
-        </is>
-      </c>
-      <c r="B145" t="inlineStr">
-        <is>
-          <t>Suitability</t>
-        </is>
-      </c>
-      <c r="C145" t="inlineStr">
-        <is>
-          <t>Credit</t>
-        </is>
-      </c>
-      <c r="D145">
-        <v>152</v>
-      </c>
-      <c r="E145" t="inlineStr">
-        <is>
-          <t>Deposit account holders qualifying for credit</t>
-        </is>
-      </c>
-      <c r="F145" t="inlineStr">
-        <is>
-          <t>% of all deposit account holders that meet the minimum qualifying criteria for a loan or line of credit</t>
-        </is>
-      </c>
-      <c r="G145" t="inlineStr">
-        <is>
-          <t>A measure of the assessed creditworthiness of depositors. Digital financial tools such as mobile money and e-wallets have opened up access to financal services to millions around the world. This indicator tries to measure the degree to which users of accounts can unlock access to addiitonal services, in the case credit. !- Definitions and concepts: Deposit accounts include transaction and non-transaction deposit accounts, for example: Checking/demand, savings, time/term deposit accounts, pensions. !- Data requirements: Total number of unique deposit account holders that also either have (1) an open loan account, (2) do not have an open loan account but would be approved for a loan or line of credit given their current credit history, credit score or other basic requirements (such as minimum balance or savings history); Total number of unique deposit account holders (i.e. an individual must be counted as one depositor irrespective of the number of deposit accounts held) at the end of a specified period (e.g. quarter or year).  !- Limitations and considerations: If individuals or MSMEs own deposit accounts across multiple different financial institutions, sector or system wide aggregates which add up accounts across institutions will, as a result, overstate the degree of financial inclusion unless granular data and unique national IDs can be used to identify individuals with multiple accounts across financial institutions.</t>
-        </is>
-      </c>
-      <c r="H145" t="inlineStr">
-        <is>
-          <t>What are the credit-qualifying rates for transaction account holders by gender? How do these rates compare? Which FSPs rank highest and lowest in credit-qualifying rates for typically underserved groups, and does this ranking change when analyzed by gender?</t>
-        </is>
-      </c>
-      <c r="I145" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J145" t="inlineStr">
-        <is>
-          <t>Financial inclusion; Stability, safety and soundness</t>
-        </is>
-      </c>
-      <c r="K145" t="inlineStr">
-        <is>
-          <t>Outcomes, Credit risk</t>
-        </is>
-      </c>
-      <c r="L145" t="inlineStr">
-        <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Loan type</t>
-        </is>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" t="inlineStr">
-        <is>
-          <t>Consumer protection</t>
-        </is>
-      </c>
-      <c r="B146" t="inlineStr">
-        <is>
-          <t>Suitability</t>
-        </is>
-      </c>
-      <c r="C146" t="inlineStr">
-        <is>
-          <t>Credit</t>
-        </is>
-      </c>
-      <c r="D146">
-        <v>176</v>
-      </c>
-      <c r="E146" t="inlineStr">
-        <is>
-          <t>Early loan payoff</t>
-        </is>
-      </c>
-      <c r="F146" t="inlineStr">
-        <is>
-          <t>% of borrowers who paid loans in full before due date</t>
-        </is>
-      </c>
-      <c r="G146" t="inlineStr">
-        <is>
-          <t>The early-loan-payoff (or prepayment) indicator tracks the share of outstanding loans that borrowers settle—partly or fully—before the contractually scheduled maturity. High prepayment activity can squeeze interest income, change expected cash-flow profiles that underpin asset-liability management, and distort credit-loss models. For lenders, rising early payoffs may flag aggressive refinancing campaigns by competitors, interest rate declines that make refinancing attractive, or borrowers’ improved liquidity. Supervisors and investors monitor the metric to evaluate revenue volatility, among others. !- Definitions and concepts: Early payoff / prepayment: any unscheduled principal reduction exceeding the contractual amortisation, including full settlement (loan closed) and partial prepayments (lump-sum curtailments).</t>
-        </is>
-      </c>
-      <c r="H146" t="inlineStr">
-        <is>
-          <t>Are there gender disparities in the likelihood of making early payments before due dates? Which credit products are most frequently paid early by each gender?</t>
-        </is>
-      </c>
-      <c r="I146" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J146" t="inlineStr">
-        <is>
-          <t>Financial inclusion; Stability, safety and soundness</t>
-        </is>
-      </c>
-      <c r="K146" t="inlineStr">
-        <is>
-          <t>Outcomes, Credit risk</t>
-        </is>
-      </c>
-      <c r="L146" t="inlineStr">
-        <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Loan type</t>
         </is>
       </c>
     </row>
@@ -8189,26 +8279,26 @@
         </is>
       </c>
       <c r="D147">
-        <v>189</v>
+        <v>152</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>Grace period/payment leeway</t>
+          <t>Deposit account holders qualifying for credit</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>% of borrowers using payment holidays, grace periods and other relief measures</t>
+          <t>% of all deposit account holders that meet the minimum qualifying criteria for a loan or line of credit</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>Shows how many borrowers are under temporary repayment relief, signalling household stress, policy effectiveness, and potential payment cliffs when relief ends. Rising usage can reduce near-term delinquencies but may defer (not eliminate) credit risk and revenue. !- Definitions and concepts: Relief measures (forbearance): payment holiday/deferral, interest-only period, reduced instalment, term extension, fee/penalty waiver, capitalization of arrears, hardship programs.Borrower-based indicator: % of borrowers on relief = [Total unique borrowers with at least 1 active relief measure in period]/[Total unique active borrowing customers] x 100%. Account-based variant uses loan count instead of borrowers. Status: Active (relief in effect), Approved but not started, Expired. Intensity companions: % of balances under relief, avg. relief days used, new entrants to relief ÷ active borrowers. !- Data requirements: Loan-level flags: relief type, start/end dates, approval date, terms (interest accrual, capitalization), reason code (income loss, disaster, medical), product type. Borrower ID (deduplicated across products/entities). !- Limitations and considerations: Definition variance: some programs auto-enrol; others require hardship evidence—harmful to cross-bank comparisons. Double counting: a borrower may receive multiple reliefs across loans—use borrower-level dedupe and report per-loan as a companion. Masking effect: relief suppresses DPD/NPL temporarily; pair with balances under relief and post-exit performance. Cohort effects &amp; timing: shocks (e.g., disasters) create spikes; use cohort tracking (by approval month) and rolling windows. Conduct risk: prolonged or opaque relief terms can mislead customers; monitor complaints and repeat relief rates. Segment by product (mortgage, card, personal, MSMEs), risk grade, tenure, and demographics to pinpoint vulnerability and program effectiveness.</t>
+          <t>A measure of the assessed creditworthiness of depositors. Digital financial tools such as mobile money and e-wallets have opened up access to financal services to millions around the world. This indicator tries to measure the degree to which users of accounts can unlock access to addiitonal services, in the case credit. !- Definitions and concepts: Deposit accounts include transaction and non-transaction deposit accounts, for example: Checking/demand, savings, time/term deposit accounts, pensions. !- Data requirements: Total number of unique deposit account holders that also either have (1) an open loan account, (2) do not have an open loan account but would be approved for a loan or line of credit given their current credit history, credit score or other basic requirements (such as minimum balance or savings history); Total number of unique deposit account holders (i.e. an individual must be counted as one depositor irrespective of the number of deposit accounts held) at the end of a specified period (e.g. quarter or year).  !- Limitations and considerations: If individuals or MSMEs own deposit accounts across multiple different financial institutions, sector or system wide aggregates which add up accounts across institutions will, as a result, overstate the degree of financial inclusion unless granular data and unique national IDs can be used to identify individuals with multiple accounts across financial institutions.</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>How do the percentages of borrowers using grace periods or payment leeways compare by gender? Is there any gender more likely to use them? How does the use of grace periods or payment leeways vary by credit product and gender?</t>
+          <t>What are the credit-qualifying rates for transaction account holders by gender? How do these rates compare? Which FSPs rank highest and lowest in credit-qualifying rates for typically underserved groups, and does this ranking change when analyzed by gender?</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -8249,162 +8339,162 @@
         </is>
       </c>
       <c r="D148">
+        <v>176</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>Early loan payoff</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>% of borrowers who paid loans in full before due date</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>The early-loan-payoff (or prepayment) indicator tracks the share of outstanding loans that borrowers settle—partly or fully—before the contractually scheduled maturity. High prepayment activity can squeeze interest income, change expected cash-flow profiles that underpin asset-liability management, and distort credit-loss models. For lenders, rising early payoffs may flag aggressive refinancing campaigns by competitors, interest rate declines that make refinancing attractive, or borrowers’ improved liquidity. Supervisors and investors monitor the metric to evaluate revenue volatility, among others. !- Definitions and concepts: Early payoff / prepayment: any unscheduled principal reduction exceeding the contractual amortisation, including full settlement (loan closed) and partial prepayments (lump-sum curtailments).</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>Are there gender disparities in the likelihood of making early payments before due dates? Which credit products are most frequently paid early by each gender?</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>Financial inclusion; Stability, safety and soundness</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>Outcomes, Credit risk</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Loan type</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Consumer protection</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Suitability</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="D149">
+        <v>189</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Grace period/payment leeway</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>% of borrowers using payment holidays, grace periods and other relief measures</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>Shows how many borrowers are under temporary repayment relief, signalling household stress, policy effectiveness, and potential payment cliffs when relief ends. Rising usage can reduce near-term delinquencies but may defer (not eliminate) credit risk and revenue. !- Definitions and concepts: Relief measures (forbearance): payment holiday/deferral, interest-only period, reduced instalment, term extension, fee/penalty waiver, capitalization of arrears, hardship programs.Borrower-based indicator: % of borrowers on relief = [Total unique borrowers with at least 1 active relief measure in period]/[Total unique active borrowing customers] x 100%. Account-based variant uses loan count instead of borrowers. Status: Active (relief in effect), Approved but not started, Expired. Intensity companions: % of balances under relief, avg. relief days used, new entrants to relief ÷ active borrowers. !- Data requirements: Loan-level flags: relief type, start/end dates, approval date, terms (interest accrual, capitalization), reason code (income loss, disaster, medical), product type. Borrower ID (deduplicated across products/entities). !- Limitations and considerations: Definition variance: some programs auto-enrol; others require hardship evidence—harmful to cross-bank comparisons. Double counting: a borrower may receive multiple reliefs across loans—use borrower-level dedupe and report per-loan as a companion. Masking effect: relief suppresses DPD/NPL temporarily; pair with balances under relief and post-exit performance. Cohort effects &amp; timing: shocks (e.g., disasters) create spikes; use cohort tracking (by approval month) and rolling windows. Conduct risk: prolonged or opaque relief terms can mislead customers; monitor complaints and repeat relief rates. Segment by product (mortgage, card, personal, MSMEs), risk grade, tenure, and demographics to pinpoint vulnerability and program effectiveness.</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>How do the percentages of borrowers using grace periods or payment leeways compare by gender? Is there any gender more likely to use them? How does the use of grace periods or payment leeways vary by credit product and gender?</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>Financial inclusion; Stability, safety and soundness</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>Outcomes, Credit risk</t>
+        </is>
+      </c>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Loan type</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Consumer protection</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Suitability</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="D150">
         <v>190</v>
       </c>
-      <c r="E148" t="inlineStr">
+      <c r="E150" t="inlineStr">
         <is>
           <t>Borrowers in debt counselling and rehabilitation</t>
         </is>
       </c>
-      <c r="F148" t="inlineStr">
+      <c r="F150" t="inlineStr">
         <is>
           <t>% of borrowers participating in debt counselling and/or debt rehabilitation progams</t>
         </is>
       </c>
-      <c r="G148" t="inlineStr">
+      <c r="G150" t="inlineStr">
         <is>
           <t>This indicator tracks the prevalence of individuals formally enrolled in debt-counselling or rehabilitation programmes: legal or contractual processes that restructure debt, impose spending plans, or provide financial-literacy support. A rising level signals household over-indebtedness pressures, tighter monetary or labour-market conditions, or aggressive credit expansion in the recent past. Regulators, consumer-protection agencies, and lenders track the metric to gauge systemic consumer-credit risk, calibrate responsible-lending rules and supervision, and anticipate write-off or provisioning needs. !- Definitions and concepts: Borrowers refers to individuals that have obtained any type of credit from financial institutions. Individuals are counted as one borrower, irrespective of the number of loan accounts held. Debt-counselling / debt-review: A court-sanctioned or regulator-approved process (e.g., South Africa’s National Credit Act, UK Debt Management Plans) where a certified counsellor assesses affordability, negotiates new payment schedules with all creditors, and disburses consolidated instalments. Debt rehabilitation / discharge: The stage at which the borrower has completed the plan, obtained a clearance certificate, or been legally discharged from remaining obligations (analogous to Chapter 13 completion in the US). Indicator forms:
 Stock measure: number of active borrowers under counselling ÷ total number of retail borrowers. Flow measure: new counselling entrants during the period ÷ new defaults. !- Data requirements: Registry or court filings identifying unique borrowers, start and end dates, original and restructured debt balances, and counsellor accreditation. Credit-bureau data to link counselling status with credit scores, delinquency buckets, and new credit enquiries. !- Limitations and considerations: Coverage gaps: Informal or NGO-led advice services may not report centrally, understating prevalence. Regime differences: Some jurisdictions treat insolvency, debt management, and bankruptcy as separate processes; harmonising counts is non-trivial. Multiple enrolments: Borrowers can exit and re-enter counselling; deduplicating unique individuals is essential for accurate stock figures. Moral-hazard concerns: Easy access to rehabilitation might weaken repayment discipline; analysts pair this indicator with post-rehabilitation re-default rates.Privacy restrictions: Personally identifiable data are often masked, limiting segmentation by income, gender, or geography unless aggregated extracts are provided. Used alongside delinquency trends, restructuring volumes, and loan-loss provisions, the “borrowers in debt counselling and rehabilitation” metric offers a forward-looking lens on household financial stress and the effectiveness of consumer-protection frameworks.</t>
         </is>
       </c>
-      <c r="H148" t="inlineStr">
+      <c r="H150" t="inlineStr">
         <is>
           <t>How do the percentages of borrowers in debt counseling or rehabilitation compare by gender? Is there any gender more likely to enroll in debt counseling or rehabilitation? How do FSPs compare in terms of debt counseling or rehabilitation enrollment by gender?</t>
         </is>
       </c>
-      <c r="I148" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J148" t="inlineStr">
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
         <is>
           <t>Financial inclusion; Stability, safety and soundness</t>
         </is>
       </c>
-      <c r="K148" t="inlineStr">
+      <c r="K150" t="inlineStr">
         <is>
           <t>Outcomes, Credit risk</t>
-        </is>
-      </c>
-      <c r="L148" t="inlineStr">
-        <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" t="inlineStr">
-        <is>
-          <t>Consumer protection</t>
-        </is>
-      </c>
-      <c r="B149" t="inlineStr">
-        <is>
-          <t>Suitability</t>
-        </is>
-      </c>
-      <c r="C149" t="inlineStr">
-        <is>
-          <t>Credit</t>
-        </is>
-      </c>
-      <c r="D149">
-        <v>27</v>
-      </c>
-      <c r="E149" t="inlineStr">
-        <is>
-          <t>Borrowers in risky indebtedness (risk of over-indebtedness)</t>
-        </is>
-      </c>
-      <c r="F149" t="inlineStr">
-        <is>
-          <t>Number of borrowers classified as at risk of over-indebtedness, as per risk-indebtedness calculation</t>
-        </is>
-      </c>
-      <c r="G149" t="inlineStr">
-        <is>
-          <t>Tracking over-indebtedness gives authorities a measure of systemic distress: when large segments of retail borrowers can’t meet their obligations, it highlights consumer-protection gaps. Persistent debt burdens signal predatory lending or inadequate affordability assessments. The indicator helps calibrate market-conduct supervision and regulation. This particular indicator that identifies borrowers at risk of overindebtedness was developed by the Central Bank of Brazil: https://www.bcb.gov.br/content/cidadaniafinanceira/documentos_cidadania/serie_cidadania/serie_cidadania_financeira_8_endividamento_risco_2ed.pdf ad https://www.researchgate.net/publication/376634051_Risky_Indebtedness_Behavior_Impacts_on_Financial_Preparation_for_Retirement_and_Perceived_Financial_Well-Being. It is a composite of four components. A borrower is flagged as being in "risky indebtedness" when any two of the following four criteria are met: (1) Has defaulted on credit installments, that is, has had payment delays of more than 90 days in meeting credit obligations, (2) Monthly income devoted to debt-service payments exceeds 50 percent, (3) Has simultaneous exposure to the following forms of credit: overdraft, unsecured personal loan, and revolving credit card debt, (4) Monthly disposable income (after debt-service payments) that falls below the poverty line. Generating this indicator at the system level requires a unique national ID in order to match granular loan data to unique borrowers. The indicator also requires access to income data. !- Derivable indicators: Percent of borrowers in risky indebtendess; Percent of adults in risky indebtedness.</t>
-        </is>
-      </c>
-      <c r="H149" t="inlineStr">
-        <is>
-          <t>Are there gender disparities in the classification of risky indebtedness? Are low-income borrowers more at risk of risky indebtedness and how does it compare across genders? Comparing this indicator with gender diversity, do FSPs with higher levels of gender diversity present lower levels of risky indebtedness?</t>
-        </is>
-      </c>
-      <c r="I149" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J149" t="inlineStr">
-        <is>
-          <t>Stability, safety and soundness</t>
-        </is>
-      </c>
-      <c r="K149" t="inlineStr">
-        <is>
-          <t>Credit risk</t>
-        </is>
-      </c>
-      <c r="L149" t="inlineStr">
-        <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
-        </is>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" t="inlineStr">
-        <is>
-          <t>Consumer protection</t>
-        </is>
-      </c>
-      <c r="B150" t="inlineStr">
-        <is>
-          <t>Suitability</t>
-        </is>
-      </c>
-      <c r="C150" t="inlineStr">
-        <is>
-          <t>Credit</t>
-        </is>
-      </c>
-      <c r="D150">
-        <v>285</v>
-      </c>
-      <c r="E150" t="inlineStr">
-        <is>
-          <t>Debt service-to-income ratio</t>
-        </is>
-      </c>
-      <c r="F150" t="inlineStr">
-        <is>
-          <t>% of income allocated to retail credit debt repayment</t>
-        </is>
-      </c>
-      <c r="G150" t="inlineStr">
-        <is>
-          <t>The debt service-to-Income ratio,  sometimes referred to more concisely as the debt service ratio (DSR) expresses a borrower’s (or household’s) total debt-service burden relative to recurring income, answering a simple question: How much of each income unit is already pledged to repay existing debt? At the micro level, lenders use DSR to assess repayment capacity, price credit, and comply with responsible-lending rules. At the macro level, supervisors track average or distributional DSR to gauge household vulnerability to interest-rate shocks and to calibrate macro-prudential tools such as loan-to-income caps. !- Definitions and concepts: Debt payments include principal, interest, mandatory insurance on retail credit facilities;  Income can be defined in gross terms (pre-tax income (salary) plus verifiable recurring earning) or net terms (income after taxes and social-security contributions). !- Data requirements: Current loan statements or credit-bureau/registry reports detailing payment amounts, remaiming term, and interest rate for all obligations; Recent payslips, audited financial statements (self-fmployed), tax returns, and verified rental or pension income. !- Limitations and considerations: Income volatility: informal or gig-economy or commission-based earnings make future cash flows uncertain; Undisclosed liabilities: informal or unreported debts escape bureau coverage, understating true DSR. Household composition: shared living expenses and co-borrower support can distort individual ratios; some frameworks use household disposable income instead. Interest-rate path: fixed-rate loans keep payments stable, while floating-rate debt can raise DSR sharply when policy rates rise. Cross-country comparability: tax structures, social-welfare benefits, and healthcare costs influence disposable income, so identical DSR thresholds may imply different real affordability across jurisdictions.</t>
-        </is>
-      </c>
-      <c r="H150" t="inlineStr">
-        <is>
-          <t>How do debt service-to-income ratios vary by gender and across different loan sizes and terms? Do loans with higher rates and shorter terms show gender disparities in ratios? Comparing this indicator with gender diversity, do FSPs with higher levels of gender diversity present lower debt-service to income ratios?</t>
-        </is>
-      </c>
-      <c r="I150" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J150" t="inlineStr">
-        <is>
-          <t>Financial inclusion; Stability, safety and soundness</t>
-        </is>
-      </c>
-      <c r="K150" t="inlineStr">
-        <is>
-          <t>Quality, Credit risk</t>
         </is>
       </c>
       <c r="L150" t="inlineStr">
@@ -8426,30 +8516,30 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Insurance</t>
+          <t>Credit</t>
         </is>
       </c>
       <c r="D151">
-        <v>194</v>
+        <v>27</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>Insurance lapse rates</t>
+          <t>Borrowers in risky indebtedness (risk of over-indebtedness)</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>% of all insurance policies (or policyholders) that have lapsed</t>
+          <t>Number of borrowers classified as at risk of over-indebtedness, as per risk-indebtedness calculation</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>This indicator measures the number of policies discontinued due to non-payment of premiums by the policyholder relative to the total number of policies at the beginning of the period. It is a key indicator to assess quality of advice, quality of service, product appropriateness, and mis-selling risk in the insurance sector. https://www.iais.org/uploads/2022/06/Report-on-Supervisors-Use-of-Key-Indicators-to-Assess-Insurer-Conduct.pdf</t>
+          <t>Tracking over-indebtedness gives authorities a measure of systemic distress: when large segments of retail borrowers can’t meet their obligations, it highlights consumer-protection gaps. Persistent debt burdens signal predatory lending or inadequate affordability assessments. The indicator helps calibrate market-conduct supervision and regulation. This particular indicator that identifies borrowers at risk of overindebtedness was developed by the Central Bank of Brazil: https://www.bcb.gov.br/content/cidadaniafinanceira/documentos_cidadania/serie_cidadania/serie_cidadania_financeira_8_endividamento_risco_2ed.pdf ad https://www.researchgate.net/publication/376634051_Risky_Indebtedness_Behavior_Impacts_on_Financial_Preparation_for_Retirement_and_Perceived_Financial_Well-Being. It is a composite of four components. A borrower is flagged as being in "risky indebtedness" when any two of the following four criteria are met: (1) Has defaulted on credit installments, that is, has had payment delays of more than 90 days in meeting credit obligations, (2) Monthly income devoted to debt-service payments exceeds 50 percent, (3) Has simultaneous exposure to the following forms of credit: overdraft, unsecured personal loan, and revolving credit card debt, (4) Monthly disposable income (after debt-service payments) that falls below the poverty line. Generating this indicator at the system level requires a unique national ID in order to match granular loan data to unique borrowers. The indicator also requires access to income data. !- Derivable indicators: Percent of borrowers in risky indebtendess; Percent of adults in risky indebtedness.</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>How do insurance lapse rates differ by gender? Are certain types of insurance policies associated with higher lapse rates among specific genders, suggesting potential issues with product suitability? How do different financial service providers (FSPs) compare in terms of lapse rates across genders? Are there notable differences when considering age, location, or income alongside gender?</t>
+          <t>Are there gender disparities in the classification of risky indebtedness? Are low-income borrowers more at risk of risky indebtedness and how does it compare across genders? Comparing this indicator with gender diversity, do FSPs with higher levels of gender diversity present lower levels of risky indebtedness?</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
@@ -8459,17 +8549,17 @@
       </c>
       <c r="J151" t="inlineStr">
         <is>
-          <t>Financial inclusion; Stability, safety and soundness</t>
+          <t>Stability, safety and soundness; Financial inclusion</t>
         </is>
       </c>
       <c r="K151" t="inlineStr">
         <is>
-          <t>Outcomes, Credit risk</t>
+          <t>Credit risk, Quality</t>
         </is>
       </c>
       <c r="L151" t="inlineStr">
         <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Insurance type</t>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
         </is>
       </c>
     </row>
@@ -8486,30 +8576,30 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Insurance</t>
+          <t>Credit</t>
         </is>
       </c>
       <c r="D152">
-        <v>197</v>
+        <v>285</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>Reinstatement of lapsed insurance policies</t>
+          <t>Debt service-to-income ratio</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>% of lapsed insurance policies that have been re-instated after customer made back-payments</t>
+          <t>% of income allocated to retail credit debt repayment</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>This indicator shows the share of policies that lapsed for non-payment and were later reinstated after the customer cleared arrears (and, where required, satisfied evidence-of-insurability). A higher reinstatement rate can indicate effective retention outreach and product value to customers; very low rates may signal affordability stress, weak follow-up, or poor customer experience. From a risk perspective, reinstatements affect cash flows, reserve dynamics, and anti-selection (customers may reinstate when risk has increased). Pair this indicator with persistency, tenure of cancellations, and complaint metrics to diagnose retention quality and customer outcomes. !- Definitions and concepts: Lapse (non-payment): policy terminated after the grace period due to unpaid premium (distinct from surrender, maturity, or death). Reinstatement: restoration of coverage after lapse once back-premiums (and any interest/fees) are paid and underwriting/administrative conditions are met. Coverage may be backdated or resume prospectively per policy terms. Measurement window: define a fixed look-back (e.g., reinstated within 90/180 days of lapse). Formula (cohort basis): # policies that lapsed in period and were reinstated within {days} divided by the # policies that lapsed in period. Variants: policyholder-level (deduplicated), premium-weighted share, and calendar-period “reinstatements ÷ lapses” with a stated window. !- Data requirements: Policy-level: product/LOB, activation date, lapse date, grace-period end, arrears amount, reinstatement date, back-payment amount, underwriting outcome (medical/financial), and whether coverage backdated. Channel, geography, tenure at lapse, and prior claims/loan status. Cohort tags (issue or lapse month) for like-for-like tracking. !- Limitations and considerations: Window sensitivity: longer window raises the rate; disclose and keep constant. Classification noise: grace-period statuses mis-tagged as lapses depress apparent reinstatement. Anti-selection: reinstated policies may have higher subsequent claims—monitor post-reinstatement loss experience. Operational variance: some firms “rewrite” new policies rather than reinstate, understating the metric. Coverage basis: backdated vs. prospective reinstatement changes exposure and reserve treatment—report the split if material.</t>
+          <t>The debt service-to-Income ratio,  sometimes referred to more concisely as the debt service ratio (DSR) expresses a borrower’s (or household’s) total debt-service burden relative to recurring income, answering a simple question: How much of each income unit is already pledged to repay existing debt? At the micro level, lenders use DSR to assess repayment capacity, price credit, and comply with responsible-lending rules. At the macro level, supervisors track average or distributional DSR to gauge household vulnerability to interest-rate shocks and to calibrate macro-prudential tools such as loan-to-income caps. !- Definitions and concepts: Debt payments include principal, interest, mandatory insurance on retail credit facilities;  Income can be defined in gross terms (pre-tax income (salary) plus verifiable recurring earning) or net terms (income after taxes and social-security contributions). !- Data requirements: Current loan statements or credit-bureau/registry reports detailing payment amounts, remaiming term, and interest rate for all obligations; Recent payslips, audited financial statements (self-fmployed), tax returns, and verified rental or pension income. !- Limitations and considerations: Income volatility: informal or gig-economy or commission-based earnings make future cash flows uncertain; Undisclosed liabilities: informal or unreported debts escape bureau coverage, understating true DSR. Household composition: shared living expenses and co-borrower support can distort individual ratios; some frameworks use household disposable income instead. Interest-rate path: fixed-rate loans keep payments stable, while floating-rate debt can raise DSR sharply when policy rates rise. Cross-country comparability: tax structures, social-welfare benefits, and healthcare costs influence disposable income, so identical DSR thresholds may imply different real affordability across jurisdictions.</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>How do rates of reinstating lapsed insurance policies vary by gender? Is any gender more likely to make back payments and reinstate their policies? How do these reinstatement patterns differ across FSPs, policy types, and demographic groups such as age or income? What might these patterns indicate about barriers to maintaining continuous coverage?</t>
+          <t>How do debt service-to-income ratios vary by gender and across different loan sizes and terms? Do loans with higher rates and shorter terms show gender disparities in ratios? Comparing this indicator with gender diversity, do FSPs with higher levels of gender diversity present lower debt-service to income ratios?</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -8519,17 +8609,17 @@
       </c>
       <c r="J152" t="inlineStr">
         <is>
-          <t>Financial inclusion</t>
+          <t>Financial inclusion; Stability, safety and soundness</t>
         </is>
       </c>
       <c r="K152" t="inlineStr">
         <is>
-          <t>Quality</t>
+          <t>Quality, Credit risk</t>
         </is>
       </c>
       <c r="L152" t="inlineStr">
         <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Insurance type</t>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity</t>
         </is>
       </c>
     </row>
@@ -8550,26 +8640,26 @@
         </is>
       </c>
       <c r="D153">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>Risk of insurance coverage lapse</t>
+          <t>Insurance lapse rates</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>% of all insurance policies (or policyholders) that missed one or more premium payments (depending on product rules and polcies) but are still within the grace period</t>
+          <t>% of all insurance policies (or policyholders) that have lapsed</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>Measures the percentage of active insurance policies (or policyholders) that have missed one or more scheduled premium payments but remain within the contractual grace period before formal lapse or cancellation takes effect. It reflects the proportion of insurance coverage that is at risk of lapsing due to non-payment but still eligible for reinstatement under product rules. Captures policyholder payment continuity risk and the vulnerability of insurance coverage within a given portfolio. It serves as an early-warning measure of potential lapse rates, affordability pressures, and retention dynamics in insurance markets. Monitoring the risk of coverage lapse helps regulators, supervisors, and insurers to: Identify emerging risks to policy continuity and financial protection coverage; Assess household liquidity stress and premium affordability; Evaluate insurer risk management practices regarding collections and grace-period handling; Strengthen consumer protection and financial health monitoring, especially in low-income or microinsurance segments. It provides an early signal of future lapse or surrender trends, which can affect both household resilience and insurer liquidity. Higher values indicate rising vulnerability to policy lapse, which may reflect household financial strain, ineffective premium collection, or weak payment reminders.Persistent high rates suggest potential issues in affordability or product suitability. Declining values reflect improved payment discipline, automatic premium collection mechanisms, or targeted retention strategies. !- Definitions and concepts: Grace period: A contractually defined period after a missed premium during which coverage remains active and can be reinstated upon payment. Lapse: Termination of an insurance policy due to non-payment of premiums after the grace period expires. !- Data requirements: Administrative data from licensed insurance companies or supervisory reporting systems. Disaggregation by product type (life, health, motor, microinsurance, etc.), customer segment (individual, group), and insurer type. Definition of grace period based on product category (e.g., 30 days for life insurance, 7–15 days for general insurance).</t>
+          <t>This indicator measures the number of policies discontinued due to non-payment of premiums by the policyholder relative to the total number of policies at the beginning of the period. It is a key indicator to assess quality of advice, quality of service, product appropriateness, and mis-selling risk in the insurance sector. https://www.iais.org/uploads/2022/06/Report-on-Supervisors-Use-of-Key-Indicators-to-Assess-Insurer-Conduct.pdf</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>How well does the non-life insurance policy market reflect gender-based differences in policyholding and insured benefits? How do the types of non-life insurance policies held compare by gender? How are gender disparities evolving in the distribution of non-life insurance policies across different FSPs?</t>
+          <t>How do insurance lapse rates differ by gender? Are certain types of insurance policies associated with higher lapse rates among specific genders, suggesting potential issues with product suitability? How do different financial service providers (FSPs) compare in terms of lapse rates across genders? Are there notable differences when considering age, location, or income alongside gender?</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -8579,12 +8669,12 @@
       </c>
       <c r="J153" t="inlineStr">
         <is>
-          <t>Financial inclusion</t>
+          <t>Financial inclusion; Stability, safety and soundness</t>
         </is>
       </c>
       <c r="K153" t="inlineStr">
         <is>
-          <t>Outcomes</t>
+          <t>Quality, Stability</t>
         </is>
       </c>
       <c r="L153" t="inlineStr">
@@ -8610,19 +8700,139 @@
         </is>
       </c>
       <c r="D154">
+        <v>197</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Reinstatement of lapsed insurance policies</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>% of lapsed insurance policies that have been re-instated after customer made back-payments</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>This indicator shows the share of policies that lapsed for non-payment and were later reinstated after the customer cleared arrears (and, where required, satisfied evidence-of-insurability). A higher reinstatement rate can indicate effective retention outreach and product value to customers; very low rates may signal affordability stress, weak follow-up, or poor customer experience. From a risk perspective, reinstatements affect cash flows, reserve dynamics, and anti-selection (customers may reinstate when risk has increased). Pair this indicator with persistency, tenure of cancellations, and complaint metrics to diagnose retention quality and customer outcomes. !- Definitions and concepts: Lapse (non-payment): policy terminated after the grace period due to unpaid premium (distinct from surrender, maturity, or death). Reinstatement: restoration of coverage after lapse once back-premiums (and any interest/fees) are paid and underwriting/administrative conditions are met. Coverage may be backdated or resume prospectively per policy terms. Measurement window: define a fixed look-back (e.g., reinstated within 90/180 days of lapse). Formula (cohort basis): # policies that lapsed in period and were reinstated within {days} divided by the # policies that lapsed in period. Variants: policyholder-level (deduplicated), premium-weighted share, and calendar-period “reinstatements ÷ lapses” with a stated window. !- Data requirements: Policy-level: product/LOB, activation date, lapse date, grace-period end, arrears amount, reinstatement date, back-payment amount, underwriting outcome (medical/financial), and whether coverage backdated. Channel, geography, tenure at lapse, and prior claims/loan status. Cohort tags (issue or lapse month) for like-for-like tracking. !- Limitations and considerations: Window sensitivity: longer window raises the rate; disclose and keep constant. Classification noise: grace-period statuses mis-tagged as lapses depress apparent reinstatement. Anti-selection: reinstated policies may have higher subsequent claims—monitor post-reinstatement loss experience. Operational variance: some firms “rewrite” new policies rather than reinstate, understating the metric. Coverage basis: backdated vs. prospective reinstatement changes exposure and reserve treatment—report the split if material.</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>How do rates of reinstating lapsed insurance policies vary by gender? Is any gender more likely to make back payments and reinstate their policies? How do these reinstatement patterns differ across FSPs, policy types, and demographic groups such as age or income? What might these patterns indicate about barriers to maintaining continuous coverage?</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>Financial inclusion</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Insurance type</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Consumer protection</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Suitability</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Insurance</t>
+        </is>
+      </c>
+      <c r="D155">
+        <v>193</v>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Risk of insurance coverage lapse</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>% of all insurance policies (or policyholders) that missed one or more premium payments (depending on product rules and polcies) but are still within the grace period</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>Measures the percentage of active insurance policies (or policyholders) that have missed one or more scheduled premium payments but remain within the contractual grace period before formal lapse or cancellation takes effect. It reflects the proportion of insurance coverage that is at risk of lapsing due to non-payment but still eligible for reinstatement under product rules. Captures policyholder payment continuity risk and the vulnerability of insurance coverage within a given portfolio. It serves as an early-warning measure of potential lapse rates, affordability pressures, and retention dynamics in insurance markets. Monitoring the risk of coverage lapse helps regulators, supervisors, and insurers to: Identify emerging risks to policy continuity and financial protection coverage; Assess household liquidity stress and premium affordability; Evaluate insurer risk management practices regarding collections and grace-period handling; Strengthen consumer protection and financial health monitoring, especially in low-income or microinsurance segments. It provides an early signal of future lapse or surrender trends, which can affect both household resilience and insurer liquidity. Higher values indicate rising vulnerability to policy lapse, which may reflect household financial strain, ineffective premium collection, or weak payment reminders.Persistent high rates suggest potential issues in affordability or product suitability. Declining values reflect improved payment discipline, automatic premium collection mechanisms, or targeted retention strategies. !- Definitions and concepts: Grace period: A contractually defined period after a missed premium during which coverage remains active and can be reinstated upon payment. Lapse: Termination of an insurance policy due to non-payment of premiums after the grace period expires. !- Data requirements: Administrative data from licensed insurance companies or supervisory reporting systems. Disaggregation by product type (life, health, motor, microinsurance, etc.), customer segment (individual, group), and insurer type. Definition of grace period based on product category (e.g., 30 days for life insurance, 7–15 days for general insurance).</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>How well does the non-life insurance policy market reflect gender-based differences in policyholding and insured benefits? How do the types of non-life insurance policies held compare by gender? How are gender disparities evolving in the distribution of non-life insurance policies across different FSPs?</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>Financial inclusion</t>
+        </is>
+      </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Insurance type</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Consumer protection</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Suitability</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Insurance</t>
+        </is>
+      </c>
+      <c r="D156">
         <v>196</v>
       </c>
-      <c r="E154" t="inlineStr">
+      <c r="E156" t="inlineStr">
         <is>
           <t>Surrendered insurance policies</t>
         </is>
       </c>
-      <c r="F154" t="inlineStr">
+      <c r="F156" t="inlineStr">
         <is>
           <t>% of eligible insurance policies (or policyholders) de-activated/lapsed that paid-out surrender values</t>
         </is>
       </c>
-      <c r="G154" t="inlineStr">
+      <c r="G156" t="inlineStr">
         <is>
           <t>This indicator shows the share of terminated policies that generated a cash surrender payout. It helps distinguish benign expiries or non-cash lapses from value-bearing exits that can strain liquidity, depress embedded value, and signal product-fit or conduct issues (e.g., early surrenders after aggressive sales). Supervisors and boards use it to gauge customer outcomes, the health of savings-type books, and potential mis-selling or affordability problems. !- Definitions and concepts: Eligible policy: contracts with a cash value (e.g., whole life, endowment, unit-linked). Pure risk covers (term, many GI lines) are ineligible. Surrender vs. lapse: a surrender pays cash value on termination; a lapse ends cover without payout. De-activatd here excludes natural maturaties and deaths. Full vs. partial surrender: count full surrenders tied to termination; report partial withdrawals separately unless they trigger de-activation.
 Indicator (count basis): Policies terminated in period with a surrender payout divided by the number of eligible policies terminated (non-maturity) in period. Variants: policyholder-based (unique customers), and amount-based (surrender amounts ÷ cash values of terminated policies). Segment by tenure (&lt;1y, 1–3y, &gt;3y), product, and channel. Data requirements
@@ -8630,206 +8840,91 @@
 Data granularity: partial withdrawals that don’t terminate cover should be excluded or separately disclosed. Conduct lens: high early-tenure surrender shares point to mis-selling or affordability issues—pair with complaints, persistency, and tenure-of-cancellation indicators.</t>
         </is>
       </c>
-      <c r="H154" t="inlineStr">
+      <c r="H156" t="inlineStr">
         <is>
           <t>Are surrender values and payouts equitably distributed by gender among eligible policyholders? Is there any gender that is less likely to receive surrender payouts, and does this vary by policy type or FSP? How do surrender rates differ by gender when combined with other demographics like income or location?</t>
         </is>
       </c>
-      <c r="I154" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J154" t="inlineStr">
-        <is>
-          <t>Financial inclusion</t>
-        </is>
-      </c>
-      <c r="K154" t="inlineStr">
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>Financial inclusion</t>
+        </is>
+      </c>
+      <c r="K156" t="inlineStr">
         <is>
           <t>Quality</t>
         </is>
       </c>
-      <c r="L154" t="inlineStr">
+      <c r="L156" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Insurance type</t>
         </is>
       </c>
     </row>
-    <row r="155">
-      <c r="A155" t="inlineStr">
+    <row r="157">
+      <c r="A157" t="inlineStr">
         <is>
           <t>Consumer protection</t>
         </is>
       </c>
-      <c r="B155" t="inlineStr">
+      <c r="B157" t="inlineStr">
         <is>
           <t>Suitability</t>
         </is>
       </c>
-      <c r="C155" t="inlineStr">
+      <c r="C157" t="inlineStr">
         <is>
           <t>Insurance</t>
         </is>
       </c>
-      <c r="D155">
+      <c r="D157">
         <v>195</v>
       </c>
-      <c r="E155" t="inlineStr">
+      <c r="E157" t="inlineStr">
         <is>
           <t>Tenure of  insurance policies</t>
         </is>
       </c>
-      <c r="F155" t="inlineStr">
+      <c r="F157" t="inlineStr">
         <is>
           <t>Average time elapsed since policy activation, by chosen time periods (e.g., &lt;3 months, 3-6 months, 6-12 months, etc)</t>
         </is>
       </c>
-      <c r="G155" t="inlineStr">
+      <c r="G157" t="inlineStr">
         <is>
           <t>This indicator measures how long policies have stayed in force -including policies that were cancelled or lapsed mid-term. It captures the stability, maturity, and longevity of customer relationships with insurers, distinguishing recently opened accounts from those that have remained active and in use over time, and identifying which policies were cancelled after a short period of activity. A concentration of early-tenure cancellations is a red flag for mis-selling, poor onboarding, pricing/friction issues, or product-fit problems. It also matters for economics: early lapses strand acquisition costs, depress embedded value, and erode persistency. Tracking tenure helps regulators and financial institutions to: Assess policyholder retention and churn rates; Identify short-lived policies that may inflate access statistics; Evaluate the depth and continuity of customer engagement; Analyze cancellations by product and channel to target remediation measures (e.g., agent training, cooling-off disclosures, claim-time communications). From a supervisory perspective, it provides insights into stability, consumer loyalty, and the effectiveness of insurance acquisition campaigns. A longer average tenure indicates stable customer relationships, active usage, and mature market penetration. A high share of new policies may suggest recent inclusion initiatives, but also potential fragility if those policies are cancelled quickly. Monitoring shifts over time can reveal trends in account retention and digital adoption maturity !- Definitions and concepts: Activation (policy start): the in-force date (not the issue date, if different). Cancellation: termination of cover before the natural renewal/expiry date—may be customer-initiated (voluntary), insurer-initiated (non-payment, underwriting, fraud), or regulatory. Tenure of active policies (days/months) = date at the end of the reference period – activation date. Tenure of cancelled policies (days/months) = cancelation date – activation date.
 Buckets: choose stable, business-meaningful bands (e.g., &lt;3m, 3–6m, 6–12m, 12–24m, &gt;24m). Report count-weighted and premium-weighted shares. Scope: life and non-life.  Clarify whether non-renewals at anniversary are counted (usually not) and how cooling-off/free-look rescissions are treated (often reported separately). Data requirements: Policy-level fields: policy ID, product/LOB, distribution channel, activation date, cancellation date, cancellation reason code, written premium/sum assured, payment mode, and claim history. Status logic to exclude simple expiries and to de-duplicate reinstated policies (see below). Calendar and cohort views (by issue month/quarter) to remove seasonality. !- Limitations and considerations: Selection bias: averaging only cancelled policies ignores still-active ones. For a fuller view of lifetime behaviour, complement with survival analysis (e.g., Kaplan–Meier) and standard persistency ratios (13/25/61-month). Reinstatements: define whether a reinstated policy’s earlier cancellation is (a) ignored, (b) treated as a separate episode, or (c) measured to the first cancellation only.
 For cancelled policies, consider including reason codes and analyze results by product type (voluntary, non-payment, underwriting, fraud). Early non-payment suggests billing/channel issues; early voluntary points to product fit. Channel &amp; product mix: bancassurance, digital, and agency books have distinct early-tenure profiles—always segment. Cooling-off: report &lt;30-day rescissions separately to avoid overstating issues that are procedural rather than structural.</t>
         </is>
       </c>
-      <c r="H155" t="inlineStr">
+      <c r="H157" t="inlineStr">
         <is>
           <t>Do genders differ in how long they hold their policies? Are there disproportionate gender differences in longer, medium, or shorter tenures? Does any gender show higher loyalty across different insurers/types? At what tenure points do insurance policies tend to be canceled, and do these patterns vary by gender? Is there a gender more likely to cancel policies earlier? How do cancellation patterns differ across policy types, age groups, locations, or income levels? What might early cancellations suggest about policy suitability or customer experience for different genders?</t>
         </is>
       </c>
-      <c r="I155" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J155" t="inlineStr">
-        <is>
-          <t>Financial inclusion</t>
-        </is>
-      </c>
-      <c r="K155" t="inlineStr">
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>Financial inclusion</t>
+        </is>
+      </c>
+      <c r="K157" t="inlineStr">
         <is>
           <t>Quality</t>
         </is>
       </c>
-      <c r="L155" t="inlineStr">
+      <c r="L157" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Insurance type</t>
-        </is>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" t="inlineStr">
-        <is>
-          <t>Consumer protection</t>
-        </is>
-      </c>
-      <c r="B156" t="inlineStr">
-        <is>
-          <t>Suitability, Fair treatment</t>
-        </is>
-      </c>
-      <c r="C156" t="inlineStr">
-        <is>
-          <t>Insurance</t>
-        </is>
-      </c>
-      <c r="D156">
-        <v>61</v>
-      </c>
-      <c r="E156" t="inlineStr">
-        <is>
-          <t>Insurance policy downgrade rate</t>
-        </is>
-      </c>
-      <c r="F156" t="inlineStr">
-        <is>
-          <t>% of policies downgraded at the customer's request (e.g.,  lower coverage, higher deductiblees, removal of riders, switch to a lower tier plan)</t>
-        </is>
-      </c>
-      <c r="G156" t="inlineStr">
-        <is>
-          <t>This indicator tracks the share of in-force policies that customers voluntarily reduce in coverage during the period. Elevated downgrade activity can signal affordability stress, product misfit, or competitive pressure (customers trading down to cheaper plans). It affects revenue (lower premiums), risk mix (higher deductibles shift loss ratios), and persistency (downgrades may precede lapses or surrenders). Supervisors and boards use the metric to monitor customer outcomes and pricing adequacy, and to gauge the effectiveness of retention strategies that preserve cover while easing budgets. !- Definitions and concepts: Downgrade (customer-initiated): a mid-term endorsement or renewal change that reduces coverage level—e.g., lower sum assured/benefit limits, higher deductibles/co-pays, downgrade of plan tier. Formula (count basis): # policies with customer-requested downgrades in period divided by # active (or renewing) policies in period. !- Limitations and considerations: Multiple events: the same policy may downgrade more than once—decide event vs. policy-unique counting. Product mapping: ensure consistent tier/benefit taxonomy across products. Group policies: member-level downgrades may not map cleanly to master policy counts—state scope.</t>
-        </is>
-      </c>
-      <c r="H156" t="inlineStr">
-        <is>
-          <t>Are there gender disparities in policy downgrade rates, including for MSMEs based on owner gender? Which types of policies experience higher downgrade rates, and could this reflect issues like unsuitable product features or unfavorable premium-to-coverage ratios? How might these downgrade rates relate to claims rejection rates and coverage ratios? Could poor claims experiences or misunderstandings about coverage terms contribute to downgrades? Do FSPs with greater gender diversity exhibit lower downgrade rates?</t>
-        </is>
-      </c>
-      <c r="I156" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J156" t="inlineStr">
-        <is>
-          <t>Financial inclusion</t>
-        </is>
-      </c>
-      <c r="K156" t="inlineStr">
-        <is>
-          <t>Quality</t>
-        </is>
-      </c>
-      <c r="L156" t="inlineStr">
-        <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Insurance type</t>
-        </is>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" t="inlineStr">
-        <is>
-          <t>Consumer protection</t>
-        </is>
-      </c>
-      <c r="B157" t="inlineStr">
-        <is>
-          <t>Suitability</t>
-        </is>
-      </c>
-      <c r="C157" t="inlineStr">
-        <is>
-          <t>Investments</t>
-        </is>
-      </c>
-      <c r="D157">
-        <v>206</v>
-      </c>
-      <c r="E157" t="inlineStr">
-        <is>
-          <t>Unpaid matured long-term investments</t>
-        </is>
-      </c>
-      <c r="F157" t="inlineStr">
-        <is>
-          <t>% of long-term investments that have matured but have not yet been paid to investors</t>
-        </is>
-      </c>
-      <c r="H157" t="inlineStr">
-        <is>
-          <t>What percentage of unpaid matured longer-term investments is attributable to each gender? Are unpaid amounts disproportionately concentrated in any gender? How do FSPs rank in terms of unpaid proportions of matured longer-term investments by gender?</t>
-        </is>
-      </c>
-      <c r="I157" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J157" t="inlineStr">
-        <is>
-          <t>Market development</t>
-        </is>
-      </c>
-      <c r="K157" t="inlineStr">
-        <is>
-          <t>Capital markets development</t>
-        </is>
-      </c>
-      <c r="L157" t="inlineStr">
-        <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type</t>
         </is>
       </c>
     </row>
@@ -8846,30 +8941,30 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Pensions</t>
+          <t>Insurance</t>
         </is>
       </c>
       <c r="D158">
-        <v>34</v>
+        <v>61</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>Pension fund switching rate</t>
+          <t>Insurance policy downgrade rate</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>% of all pension accounts that have switched to another pension fund administrator</t>
+          <t>% of policies downgraded at the customer's request (e.g.,  lower coverage, higher deductiblees, removal of riders, switch to a lower tier plan)</t>
         </is>
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>An indicator of switching rates among pension recipients is a metric used to measure the frequency or volume of pension fund members who transfer their accumulated savings from one pension fund administrator (PFA) to another within a specific timeframe. This indicator can be used in countries where there is a private pension fund adminsitration industry, but not in countries where the entirety of the pension system is publicly-funded. This indicator serves as a key barometer of competition, customer satisfaction, and market dynamics within the pension industry. It can signal trends to administrators, regulators, and members themselves.  Switching Rate (%) = Total average number of members in the system / number of members who switched pension fund administrators  ×100</t>
+          <t>This indicator tracks the share of in-force policies that customers voluntarily reduce in coverage during the period. Elevated downgrade activity can signal affordability stress, product misfit, or competitive pressure (customers trading down to cheaper plans). It affects revenue (lower premiums), risk mix (higher deductibles shift loss ratios), and persistency (downgrades may precede lapses or surrenders). Supervisors and boards use the metric to monitor customer outcomes and pricing adequacy, and to gauge the effectiveness of retention strategies that preserve cover while easing budgets. !- Definitions and concepts: Downgrade (customer-initiated): a mid-term endorsement or renewal change that reduces coverage level—e.g., lower sum assured/benefit limits, higher deductibles/co-pays, downgrade of plan tier. Formula (count basis): # policies with customer-requested downgrades in period divided by # active (or renewing) policies in period. !- Limitations and considerations: Multiple events: the same policy may downgrade more than once—decide event vs. policy-unique counting. Product mapping: ensure consistent tier/benefit taxonomy across products. Group policies: member-level downgrades may not map cleanly to master policy counts—state scope.</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>How do transfers of pension fund balances to a different pension fund administrator vary by gender? Does this vary according to the level of FSP gender diversity? What percentage of contributors transferred funds compared to all customers, and are there gender disparities in this proportion? Are certain customer segments, such as women, women-owned MSMEs owners, and low-value accounts, more likely to make high-to-low transfers (switching to a fund administrator that has been paying lower returns)? Are FSPs with higher levels of gender diversity less likely to receive savers coming from an administrator that previously paid higher returns?</t>
+          <t>Are there gender disparities in policy downgrade rates, including for MSMEs based on owner gender? Which types of policies experience higher downgrade rates, and could this reflect issues like unsuitable product features or unfavorable premium-to-coverage ratios? How might these downgrade rates relate to claims rejection rates and coverage ratios? Could poor claims experiences or misunderstandings about coverage terms contribute to downgrades? Do FSPs with greater gender diversity exhibit lower downgrade rates?</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -8889,7 +8984,7 @@
       </c>
       <c r="L158" t="inlineStr">
         <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Pension type</t>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Insurance type</t>
         </is>
       </c>
     </row>
@@ -8906,30 +9001,25 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Savings</t>
+          <t>Investments</t>
         </is>
       </c>
       <c r="D159">
-        <v>151</v>
+        <v>206</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>Tenure of deposit and payment accounts</t>
+          <t>Unpaid matured long-term investments</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>Average time elapsed since account opening</t>
-        </is>
-      </c>
-      <c r="G159" t="inlineStr">
-        <is>
-          <t>Measures the length of time that deposit and payment accounts have been open, can be expressed as an average or as the share of accounts in tenure categories such as &lt;3 months, 3–6 months, 6–12 months, 1–3 years, &gt;3 years, etc. It reflects the age profile of active accounts held by customers at regulated financial institutions and payment service providers. Captures the stability, maturity, and longevity of customer relationships with financial institutions. It is a key behavioral measure of financial inclusion sustainability, distinguishing recently opened accounts from those that have remained active and in use over time. Tracking account tenure helps regulators and financial institutions to: Assess account retention and churn rates in deposit and payment systems; Monitor sustained usage versus one-off account openings, especially under inclusion programs; Identify short-lived or dormant accounts that may inflate access statistics; Evaluate the depth and continuity of customer engagement with the financial system. From a supervisory perspective, it provides insights into financial system stability, consumer loyalty, and the effectiveness of account-opening campaigns. A longer average tenure indicates stable customer relationships, active usage, and mature market penetration. A high share of newly opened accounts may suggest recent inclusion initiatives, but also potential fragility if those accounts become inactive. Monitoring shifts over time can reveal trends in account retention and digital adoption maturity. !- Definitions and concepts: Deposit accounts: Savings, current, or term accounts offered by regulated deposit-taking institutions. Payment accounts: Accounts used to execute payment transactions or access funds on demand, including e-money and digital wallets. !- Data requirements: Account-level data from administrative records containing the account opening date; Total number of accounts. The tenure is calculated as the difference between the data of the end of the reference period and the account opening data (expressed in years or months).</t>
+          <t>% of long-term investments that have matured but have not yet been paid to investors</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>Do genders differ in how long they hold their transaction accounts? Are some genders disproportionately represented in longer, medium, or shorter account tenures? Which genders show higher account loyalty across different FSPs/types, and which tend to close accounts sooner?</t>
+          <t>What percentage of unpaid matured longer-term investments is attributable to each gender? Are unpaid amounts disproportionately concentrated in any gender? How do FSPs rank in terms of unpaid proportions of matured longer-term investments by gender?</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -8939,12 +9029,12 @@
       </c>
       <c r="J159" t="inlineStr">
         <is>
-          <t>Stability, safety and soundness</t>
+          <t>Market development; Financial inclusion</t>
         </is>
       </c>
       <c r="K159" t="inlineStr">
         <is>
-          <t>Liquidity risk</t>
+          <t>Capital markets development, Quality</t>
         </is>
       </c>
       <c r="L159" t="inlineStr">
@@ -8961,176 +9051,176 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
+          <t>Suitability, Fair treatment</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Pensions</t>
+        </is>
+      </c>
+      <c r="D160">
+        <v>34</v>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>Pension fund switching rate</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>% of all pension accounts that have switched to another pension fund administrator</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>An indicator of switching rates among pension recipients is a metric used to measure the frequency or volume of pension fund members who transfer their accumulated savings from one pension fund administrator (PFA) to another within a specific timeframe. This indicator can be used in countries where there is a private pension fund adminsitration industry, but not in countries where the entirety of the pension system is publicly-funded. This indicator serves as a key barometer of competition, customer satisfaction, and market dynamics within the pension industry. It can signal trends to administrators, regulators, and members themselves.  Switching Rate (%) = Total average number of members in the system / number of members who switched pension fund administrators  ×100</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>How do transfers of pension fund balances to a different pension fund administrator vary by gender? Does this vary according to the level of FSP gender diversity? What percentage of contributors transferred funds compared to all customers, and are there gender disparities in this proportion? Are certain customer segments, such as women, women-owned MSMEs owners, and low-value accounts, more likely to make high-to-low transfers (switching to a fund administrator that has been paying lower returns)? Are FSPs with higher levels of gender diversity less likely to receive savers coming from an administrator that previously paid higher returns?</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>Financial inclusion</t>
+        </is>
+      </c>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
+      <c r="L160" t="inlineStr">
+        <is>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Pension type</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Consumer protection</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
           <t>Suitability</t>
         </is>
       </c>
-      <c r="C160" t="inlineStr">
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Savings</t>
+        </is>
+      </c>
+      <c r="D161">
+        <v>151</v>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>Tenure of deposit and payment accounts</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>Average time elapsed since account opening</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>Measures the length of time that deposit and payment accounts have been open, can be expressed as an average or as the share of accounts in tenure categories such as &lt;3 months, 3–6 months, 6–12 months, 1–3 years, &gt;3 years, etc. It reflects the age profile of active accounts held by customers at regulated financial institutions and payment service providers. Captures the stability, maturity, and longevity of customer relationships with financial institutions. It is a key behavioral measure of financial inclusion sustainability, distinguishing recently opened accounts from those that have remained active and in use over time. Tracking account tenure helps regulators and financial institutions to: Assess account retention and churn rates in deposit and payment systems; Monitor sustained usage versus one-off account openings, especially under inclusion programs; Identify short-lived or dormant accounts that may inflate access statistics; Evaluate the depth and continuity of customer engagement with the financial system. From a supervisory perspective, it provides insights into financial system stability, consumer loyalty, and the effectiveness of account-opening campaigns. A longer average tenure indicates stable customer relationships, active usage, and mature market penetration. A high share of newly opened accounts may suggest recent inclusion initiatives, but also potential fragility if those accounts become inactive. Monitoring shifts over time can reveal trends in account retention and digital adoption maturity. !- Definitions and concepts: Deposit accounts: Savings, current, or term accounts offered by regulated deposit-taking institutions. Payment accounts: Accounts used to execute payment transactions or access funds on demand, including e-money and digital wallets. !- Data requirements: Account-level data from administrative records containing the account opening date; Total number of accounts. The tenure is calculated as the difference between the data of the end of the reference period and the account opening data (expressed in years or months).</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>Do genders differ in how long they hold their transaction accounts? Are some genders disproportionately represented in longer, medium, or shorter account tenures? Which genders show higher account loyalty across different FSPs/types, and which tend to close accounts sooner?</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>Stability, safety and soundness; Financial inclusion</t>
+        </is>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>Liquidity risk, Quality</t>
+        </is>
+      </c>
+      <c r="L161" t="inlineStr">
+        <is>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Consumer protection</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Suitability</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
         <is>
           <t>Payments, Savings, Pensions, Investments</t>
         </is>
       </c>
-      <c r="D160">
+      <c r="D162">
         <v>158</v>
       </c>
-      <c r="E160" t="inlineStr">
+      <c r="E162" t="inlineStr">
         <is>
           <t>Inactive and dormant accounts (balance)</t>
         </is>
       </c>
-      <c r="F160" t="inlineStr">
+      <c r="F162" t="inlineStr">
         <is>
           <t>% of total account balances that are held in inactive and dormant accounts</t>
         </is>
       </c>
-      <c r="G160" t="inlineStr">
+      <c r="G162" t="inlineStr">
         <is>
           <t>This indicator shows the share of funds sitting in deposit and payment accounts (excluding term deposits) that are not actively used by customers. High concentrations of idle balances can signal weak customer engagement, poor product fit, or frictions in account usage—important for financial-inclusion quality, liquidity management, and conduct risk. From a prudential angle, large dormant balances may look “stable” but can reverse if reactivation drives or policy changes prompt withdrawals. For consumer protection, persistent dormancy raises risks around unclaimed funds, fees, and fraud. Recommended to analyze of this indicator by product type (e.g. current/checking, mobile money, etc). !- Definitions and concepts: Accounts: demand/current accounts and other payment-capable deposit accounts. Inactive account: no customer-initiated debit/credit (card use, cash withdrawal/deposit, transfer) for a defined window (e.g., ≥90 or 180 days). System entries (interest, fees, bank corrections) don’t count. Dormant account: extended inactivity beyond a longer threshold (commonly ≥12 months) that may trigger special handling (restricted access, outreach, escheatment). Indicator formula: Balances in inactive + dormant transaction accounts divided by total transaction-account balances. Reporting the split (inactive vs. dormant) can provide further detail. !- Data requirements: Core-banking ledger with end-of-day balances, product codes, and last customer-initiated activity timestamp per account. Classification rules reflecting local definitions (inactive/dormant thresholds; treatment of standing orders/auto-debits). Ownership segment (retail/MSMEs), currency, and insured/uninsured flags. Optional: outreach attempts, reactivation outcomes, and fee assessments to monitor conduct risk. Limitations &amp; considerations: Definition divergence: thresholds and what counts as “activity” vary by jurisdiction and even by institution—state methodology clearly. Data quality: some channels (agents, fintech front-ends) may not update the core “last activity” field, overstating dormancy.
 Seasonality &amp; cycles: balances can spike around payroll/tax periods; use consistent month-end or averages. Policy effects: dormancy fees, auto-closures, and unclaimed-funds rules materially affect trends. Coverage scope: exclude escrow, trust, and suspense ledgers to avoid inflating inactive balances.</t>
         </is>
       </c>
-      <c r="H160" t="inlineStr">
+      <c r="H162" t="inlineStr">
         <is>
           <t>What proportion of balances held in inactive/dormant/suspense accounts is attributable to each gender? Are these balances disproportionately skewed by gender? Which FSPs have notable skews (higher than market averages) in balances held in inactive/dormant/suspense accounts by gender?</t>
         </is>
       </c>
-      <c r="I160" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J160" t="inlineStr">
-        <is>
-          <t>Financial inclusion</t>
-        </is>
-      </c>
-      <c r="K160" t="inlineStr">
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
+        </is>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>Financial inclusion</t>
+        </is>
+      </c>
+      <c r="K162" t="inlineStr">
         <is>
           <t>Quality</t>
         </is>
       </c>
-      <c r="L160" t="inlineStr">
+      <c r="L162" t="inlineStr">
         <is>
           <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Account type</t>
-        </is>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" t="inlineStr">
-        <is>
-          <t>Consumer protection</t>
-        </is>
-      </c>
-      <c r="B161" t="inlineStr">
-        <is>
-          <t>Suitability</t>
-        </is>
-      </c>
-      <c r="C161" t="inlineStr">
-        <is>
-          <t>Payments, Savings, Pensions, Investments</t>
-        </is>
-      </c>
-      <c r="D161">
-        <v>161</v>
-      </c>
-      <c r="E161" t="inlineStr">
-        <is>
-          <t>Revenue from inactive and dormant accounts</t>
-        </is>
-      </c>
-      <c r="F161" t="inlineStr">
-        <is>
-          <t>Average non-interest revenue earned on inactive and dormant accounts per account holder</t>
-        </is>
-      </c>
-      <c r="G161" t="inlineStr">
-        <is>
-          <t>This indicator estimates how much fee income a provider earns, on average, from customers whose transaction accounts are inactive or dormant. It highlights potential conduct-risk hotspots (“junk fees”), tests whether inclusion policies translate into active use, and helps gauge earnings reliance on non-usage charges. Regulators often scrutinize such revenue because it may disproportionately affect vulnerable or low-balance customers and can conflict with fair-treatment principles or local dormancy rules. Used alongside % balances in inactive/dormant accounts, reactivation rates, and complaints upheld about fees, this metric provides a balanced view of inclusion quality and earnings fairness. !- Definitions and concepts: Inactive account: no customer-initiated transaction over a defined window (e.g., ≥90/180 days). Dormant account: extended inactivity (e.g., ≥12 months) triggering special handling (restricted access, outreach, or escheatment). Non-interest revenue: maintenance/inactivity fees, SMS/statement charges, card fees, ATM/network fees, account closure fees—exclude interest, FX spreads, and lending-related fees. Metric (per holder): Avg. fee per inactive/dormant holder = [Non interest fees charged to inactive+dormant accounts in period (net of waivers/refunds)] divided by unique customers with ≥1 inactive or dormant account in period. Report per-account as a companion view, and show inactive vs dormant separately. !- Data requirements: Core-banking extracts: account status, last customer-initiated activity timestamp, balances, product code. General-ledger fee income by fee code with identifiers to tie fees to specific accounts/customers; flags for waivers/refunds/chargebacks. Customer master data to deduplicate holders with multiple accounts. Policy tables: inactivity/dormancy thresholds, fee schedules, and escheatment rules; time-at-risk (days classified as inactive/dormant). !- Limitations and considerations: Definition variance: thresholds and what counts as “activity” differ—state methodology. Partial-period bias: accounts turning dormant late in the period face fewer fee days; consider normalizing by days inactive/dormant. Outliers &amp; distribution: averages can be skewed; also report median, 90th percentile, and % of affected customers. Conduct/regulatory constraints: some jurisdictions cap or ban dormancy fees or require fee cessation before escheatment—track compliance and annotate series breaks after rule changes. Mix effects: product/channel mixes (e.g., basic accounts, youth or social-transfer accounts) drive fee propensity—segment results by product and customer segment.</t>
-        </is>
-      </c>
-      <c r="H161" t="inlineStr">
-        <is>
-          <t>How does the average revenue earned from inactive and dormant accounts compare by gender? Are there gender disparities in the charges applied to these accounts compared to the overall market average? How do relevant FSPs rank in terms of the average revenue earned from these accounts, and does this ranking change when analyzed by gender?</t>
-        </is>
-      </c>
-      <c r="I161" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J161" t="inlineStr">
-        <is>
-          <t>Financial inclusion</t>
-        </is>
-      </c>
-      <c r="K161" t="inlineStr">
-        <is>
-          <t>Quality</t>
-        </is>
-      </c>
-      <c r="L161" t="inlineStr">
-        <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Account type</t>
-        </is>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" t="inlineStr">
-        <is>
-          <t>Consumer protection</t>
-        </is>
-      </c>
-      <c r="B162" t="inlineStr">
-        <is>
-          <t>Suitability</t>
-        </is>
-      </c>
-      <c r="C162" t="inlineStr">
-        <is>
-          <t>Payments, Savings, Credit, Insurance, Pensions, Investments</t>
-        </is>
-      </c>
-      <c r="D162">
-        <v>229</v>
-      </c>
-      <c r="E162" t="inlineStr">
-        <is>
-          <t>Product take-up ratio</t>
-        </is>
-      </c>
-      <c r="F162" t="inlineStr">
-        <is>
-          <t>% of approved applicants who take-up the approved products by product type</t>
-        </is>
-      </c>
-      <c r="G162" t="inlineStr">
-        <is>
-          <t>Share of applicants that are approved for a specific product type that take-up the product. This indicator can be viewed together with the product application indicator to allow for a more comprehensive analysis of the demand for financial products. Product categoreis to consider for analysis include: deposits, investments, insurance, credit.</t>
-        </is>
-      </c>
-      <c r="H162" t="inlineStr">
-        <is>
-          <t>How do take-up rates vary by gender? Do any genders have higher take-up rates than the overall market average? How do FSPs compare in terms of take-up rates by gender?</t>
-        </is>
-      </c>
-      <c r="I162" t="inlineStr">
-        <is>
-          <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
-        </is>
-      </c>
-      <c r="J162" t="inlineStr">
-        <is>
-          <t>Financial inclusion</t>
-        </is>
-      </c>
-      <c r="K162" t="inlineStr">
-        <is>
-          <t>Uptake (account ownership)</t>
-        </is>
-      </c>
-      <c r="L162" t="inlineStr">
-        <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Product type</t>
         </is>
       </c>
     </row>
@@ -9142,35 +9232,35 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Fair treatment</t>
+          <t>Suitability</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Savings</t>
+          <t>Payments, Savings, Pensions, Investments</t>
         </is>
       </c>
       <c r="D163">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>Account closure costs paid by customers</t>
+          <t>Revenue from inactive and dormant accounts</t>
         </is>
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>Average customer-paid account closure charges</t>
+          <t>Average non-interest revenue earned on inactive and dormant accounts per account holder</t>
         </is>
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>This indicator captures the out-of-pocket costs borne by customers when they close their transaction account(s). It focuses on fees directly tied to the closure process (not ongoing usage fees). High averages or wide dispersion can signal unfair fee structures, poor process design (e.g., costly payout rails), or weak disclosures—issues that draw conduct-risk scrutiny and harm inclusion goals. Tracking this metric alongside complaints upheld about closure, time to close, and payout failure/return rates gives a rounded view of off-boarding fairness and efficiency. !- Definitions and concepts: Transaction accounts are broadly defined as an account held with a bank or other authorised and/or regulated service provider (including a non-bank) which can be used to make and receive payments. Transaction accounts can be further differentiated into deposit transaction accounts and e-money accounts. Customer-paid closure charges: amounts debited to the customer because of closure, including: explicit closure fees, final statement/document fees, card/cheque deactivation fees, balance-refund/payout charges (e.g., wire/RTGS, cheque issuance, e-money cash-out), account package early-termination fees, statutory taxes/levies linked to these items, and FX/transfer margins if required to remit funds. Exclusions: regular monthly maintenance already charged prior to the closure request, penalty interest on unrelated lending, and third-party fees not passed through. !- Data requirements: Event log with closure request date and closure completion date; customer ID (deduplicated), number of accounts closed, channel, reason code. Transaction-level fee taxonomy to flag closure-related charges; payout transactions (method, amount, fees, FX). Reversal/waiver flags and timestamps to net back rescinded charges. Recommended charge window: from request date through T+30 days after completion to catch settlement/payout fees. Number of customers who closed at least 1 account in period. !- Limitations and considerations: Attribution: define the fee list upfront to avoid counting routine usage fees; publish the measurement window.</t>
+          <t>This indicator estimates how much fee income a provider earns, on average, from customers whose transaction accounts are inactive or dormant. It highlights potential conduct-risk hotspots (“junk fees”), tests whether inclusion policies translate into active use, and helps gauge earnings reliance on non-usage charges. Regulators often scrutinize such revenue because it may disproportionately affect vulnerable or low-balance customers and can conflict with fair-treatment principles or local dormancy rules. Used alongside % balances in inactive/dormant accounts, reactivation rates, and complaints upheld about fees, this metric provides a balanced view of inclusion quality and earnings fairness. !- Definitions and concepts: Inactive account: no customer-initiated transaction over a defined window (e.g., ≥90/180 days). Dormant account: extended inactivity (e.g., ≥12 months) triggering special handling (restricted access, outreach, or escheatment). Non-interest revenue: maintenance/inactivity fees, SMS/statement charges, card fees, ATM/network fees, account closure fees—exclude interest, FX spreads, and lending-related fees. Metric (per holder): Avg. fee per inactive/dormant holder = [Non interest fees charged to inactive+dormant accounts in period (net of waivers/refunds)] divided by unique customers with ≥1 inactive or dormant account in period. Report per-account as a companion view, and show inactive vs dormant separately. !- Data requirements: Core-banking extracts: account status, last customer-initiated activity timestamp, balances, product code. General-ledger fee income by fee code with identifiers to tie fees to specific accounts/customers; flags for waivers/refunds/chargebacks. Customer master data to deduplicate holders with multiple accounts. Policy tables: inactivity/dormancy thresholds, fee schedules, and escheatment rules; time-at-risk (days classified as inactive/dormant). !- Limitations and considerations: Definition variance: thresholds and what counts as “activity” differ—state methodology. Partial-period bias: accounts turning dormant late in the period face fewer fee days; consider normalizing by days inactive/dormant. Outliers &amp; distribution: averages can be skewed; also report median, 90th percentile, and % of affected customers. Conduct/regulatory constraints: some jurisdictions cap or ban dormancy fees or require fee cessation before escheatment—track compliance and annotate series breaks after rule changes. Mix effects: product/channel mixes (e.g., basic accounts, youth or social-transfer accounts) drive fee propensity—segment results by product and customer segment.</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>How do relevant FSPs rank in terms of closing costs (from highest to lowest), and does this ranking change when the average is computed by gender? Are women and men equally likely to incur account closure fees, or are there gendered patterns in the types of financial service providers (FSPs) they use that influence the likelihood or amount of such fees? How might account closure costs act as a barrier to financial flexibility or mobility? Are women more likely to avoid formal financial services due to concerns over the cost of exiting the system? Additionally, are FSPs that charge lower or no closure fees more accessible to certain gender groups, and does this vary by geography or provider type?</t>
+          <t>How does the average revenue earned from inactive and dormant accounts compare by gender? Are there gender disparities in the charges applied to these accounts compared to the overall market average? How do relevant FSPs rank in terms of the average revenue earned from these accounts, and does this ranking change when analyzed by gender?</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -9180,17 +9270,17 @@
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>Financial inclusion; Market development</t>
+          <t>Financial inclusion</t>
         </is>
       </c>
       <c r="K163" t="inlineStr">
         <is>
-          <t>Outcomes, Capital markets development</t>
+          <t>Quality</t>
         </is>
       </c>
       <c r="L163" t="inlineStr">
         <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type</t>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Account type</t>
         </is>
       </c>
     </row>
@@ -9207,30 +9297,30 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>Insurance</t>
+          <t>Payments, Savings, Credit, Insurance, Pensions, Investments</t>
         </is>
       </c>
       <c r="D164">
-        <v>389</v>
+        <v>229</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>Insurance claims (number)</t>
+          <t>Product take-up ratio</t>
         </is>
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>Number of insurance claims</t>
+          <t>% of approved applicants who take-up the approved products by product type</t>
         </is>
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>The total count of insurance claims formally submitted by policyholders, beneficiaries, or authorized third parties to an insurer within a defined reporting period, regardless of whether the claims are accepted, rejected, paid, or still under review. Denominator for several key inclusion, consumer protection and prudential insurance ratios. !- Data requirements: Claim identifier, (unique ID per claim), Policyholder identifier, Date of claim submission.</t>
+          <t>Share of applicants that are approved for a specific product type that take-up the product. This indicator can be viewed together with the product application indicator to allow for a more comprehensive analysis of the demand for financial products. Product categoreis to consider for analysis include: deposits, investments, insurance, credit.</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>How do claim numbers vary by gender? Are there any gender groups logging fewer claims compared to the market average? Are there FSPs with particularly low or high claim numbers for certain genders? How do claim statistics intersect with policy type and customer demographics?</t>
+          <t>How do take-up rates vary by gender? Do any genders have higher take-up rates than the overall market average? How do FSPs compare in terms of take-up rates by gender?</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -9240,17 +9330,17 @@
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>Financial inclusion; Stability, safety and soundness</t>
+          <t>Financial inclusion</t>
         </is>
       </c>
       <c r="K164" t="inlineStr">
         <is>
-          <t>Usage, Soundness</t>
+          <t>Uptake (account ownership)</t>
         </is>
       </c>
       <c r="L164" t="inlineStr">
         <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Insurance type</t>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Product type</t>
         </is>
       </c>
     </row>
@@ -9267,30 +9357,30 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Insurance</t>
+          <t>Savings</t>
         </is>
       </c>
       <c r="D165">
-        <v>390</v>
+        <v>162</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>Insurance claims paid</t>
+          <t>Account closure costs paid by customers</t>
         </is>
       </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t>Value of insurance claims paid</t>
+          <t>Average customer-paid account closure charges</t>
         </is>
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>"Claims paid" represents the total cash outflow or settled obligations by an insurer to policyholders or beneficiaries for claims events during a reporting period. It includes only claims for which payment has been disbursed, regardless of whether additional claims are still outstanding or whether reserves were previously established. Tracking claims paid helps supervisors monitor liquidity, operational efficiency, and consumer protection outcomes. It provides a concrete measure of the insurer’s fulfillment of contractual obligations and complements other claims indicators (e.g., claims incurred, claims outstanding, unpaid approved claims). !- Data requirements: Claim identifier, (unique ID per claim), Policyholder identifier, Date of claim submission, Date of payment, Amount paid (full or partial), Product / policy type; . !- Limitations and considerations: paid claims may lag claims incurred due to reporting delays or extended claims handling processes; some claims are paid in installments, methodology must specify whether to include full or partial amounts; severe events can cause sudden increases in paid claims, interpretation should consider context. Segmentation by product line or policy type is recommended for supervisory analysis.</t>
+          <t>This indicator captures the out-of-pocket costs borne by customers when they close their transaction account(s). It focuses on fees directly tied to the closure process (not ongoing usage fees). High averages or wide dispersion can signal unfair fee structures, poor process design (e.g., costly payout rails), or weak disclosures—issues that draw conduct-risk scrutiny and harm inclusion goals. Tracking this metric alongside complaints upheld about closure, time to close, and payout failure/return rates gives a rounded view of off-boarding fairness and efficiency. !- Definitions and concepts: Transaction accounts are broadly defined as an account held with a bank or other authorised and/or regulated service provider (including a non-bank) which can be used to make and receive payments. Transaction accounts can be further differentiated into deposit transaction accounts and e-money accounts. Customer-paid closure charges: amounts debited to the customer because of closure, including: explicit closure fees, final statement/document fees, card/cheque deactivation fees, balance-refund/payout charges (e.g., wire/RTGS, cheque issuance, e-money cash-out), account package early-termination fees, statutory taxes/levies linked to these items, and FX/transfer margins if required to remit funds. Exclusions: regular monthly maintenance already charged prior to the closure request, penalty interest on unrelated lending, and third-party fees not passed through. !- Data requirements: Event log with closure request date and closure completion date; customer ID (deduplicated), number of accounts closed, channel, reason code. Transaction-level fee taxonomy to flag closure-related charges; payout transactions (method, amount, fees, FX). Reversal/waiver flags and timestamps to net back rescinded charges. Recommended charge window: from request date through T+30 days after completion to catch settlement/payout fees. Number of customers who closed at least 1 account in period. !- Limitations and considerations: Attribution: define the fee list upfront to avoid counting routine usage fees; publish the measurement window.</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>How do claim payments vary by gender? Are there any gender groups receiving fewer/lower payments compared to the market average? Are there FSPs with particularly low or high payment rate for certain genders? How do claim payment statistics intersect with policy type and customer demographics?</t>
+          <t>How do relevant FSPs rank in terms of closing costs (from highest to lowest), and does this ranking change when the average is computed by gender? Are women and men equally likely to incur account closure fees, or are there gendered patterns in the types of financial service providers (FSPs) they use that influence the likelihood or amount of such fees? How might account closure costs act as a barrier to financial flexibility or mobility? Are women more likely to avoid formal financial services due to concerns over the cost of exiting the system? Additionally, are FSPs that charge lower or no closure fees more accessible to certain gender groups, and does this vary by geography or provider type?</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
@@ -9300,17 +9390,17 @@
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>Financial inclusion; Stability, safety and soundness</t>
+          <t>Financial inclusion; Market development</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
         <is>
-          <t>Usage, Soundness</t>
+          <t>Quality, Competition</t>
         </is>
       </c>
       <c r="L165" t="inlineStr">
         <is>
-          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type; Financial service provider (FSP) main activity; Insurance type</t>
+          <t>Customer type; Customer gender; Customer age; Customer location; Customer income category; Financial service provider (FSP) type</t>
         </is>
       </c>
     </row>
@@ -9460,17 +9550,17 @@
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>Consumer protection</t>
+          <t>Consumer protection; Financial inclusion</t>
         </is>
       </c>
       <c r="K168" t="inlineStr">
         <is>
-          <t>Fair treatment</t>
+          <t>Fair treatment, Quality</t>
         </is>
       </c>
       <c r="L168" t="inlineStr">
         <is>
-          <t>Customer gender; Financial service provider (FSP) gender diversity; Customer type; Financial service provider (FSP) type; Product type</t>
+          <t>Customer type; Customer gender; Financial service provider (FSP) type; Financial service provider (FSP) gender diversity; Product type</t>
         </is>
       </c>
     </row>
@@ -9525,7 +9615,7 @@
       </c>
       <c r="K169" t="inlineStr">
         <is>
-          <t>Outcomes, Suitability</t>
+          <t>Quality, Outcomes, Suitability</t>
         </is>
       </c>
       <c r="L169" t="inlineStr">
@@ -9695,12 +9785,12 @@
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>Consumer protection</t>
+          <t>Market development</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
         <is>
-          <t>Safety and security</t>
+          <t>Competition</t>
         </is>
       </c>
       <c r="L172" t="inlineStr">
@@ -9755,7 +9845,7 @@
       </c>
       <c r="K173" t="inlineStr">
         <is>
-          <t>Outcomes, Suitability</t>
+          <t>Quality, Outcomes, Suitability</t>
         </is>
       </c>
       <c r="L173" t="inlineStr">
@@ -9815,12 +9905,12 @@
       </c>
       <c r="K174" t="inlineStr">
         <is>
-          <t>Outcomes, Suitability</t>
+          <t>Quality, Suitability</t>
         </is>
       </c>
       <c r="L174" t="inlineStr">
         <is>
-          <t>Customer gender; Financial service provider (FSP) gender diversity; Customer type; Financial service provider (FSP) type; Product type; Loan size</t>
+          <t>Customer type; Customer gender; Financial service provider (FSP) type; Financial service provider (FSP) gender diversity; Loan size; Product type</t>
         </is>
       </c>
     </row>
@@ -10005,7 +10095,7 @@
       </c>
       <c r="K178" t="inlineStr">
         <is>
-          <t>Usage, Suitability</t>
+          <t>Quality, Suitability</t>
         </is>
       </c>
       <c r="L178" t="inlineStr">
@@ -10060,7 +10150,7 @@
       </c>
       <c r="K179" t="inlineStr">
         <is>
-          <t>Usage, Suitability</t>
+          <t>Quality, Suitability</t>
         </is>
       </c>
       <c r="L179" t="inlineStr">
@@ -10282,7 +10372,7 @@
       </c>
       <c r="K183" t="inlineStr">
         <is>
-          <t>Usage, Suitability</t>
+          <t>Usage, Quality, Suitability</t>
         </is>
       </c>
       <c r="L183" t="inlineStr">
@@ -10337,7 +10427,7 @@
       </c>
       <c r="K184" t="inlineStr">
         <is>
-          <t>Quality, Suitability</t>
+          <t>Usage, Quality, Suitability</t>
         </is>
       </c>
       <c r="L184" t="inlineStr">
@@ -10718,7 +10808,7 @@
       </c>
       <c r="K192" t="inlineStr">
         <is>
-          <t>Outcomes</t>
+          <t>Usage, Outcomes</t>
         </is>
       </c>
       <c r="L192" t="inlineStr">
@@ -11702,7 +11792,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Gender equality</t>
+          <t>Diversity and inclusion</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
@@ -11747,7 +11837,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>Gender equality</t>
+          <t>Diversity and inclusion</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
@@ -11792,7 +11882,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>Gender equality</t>
+          <t>Diversity and inclusion</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
@@ -11837,7 +11927,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>Gender equality</t>
+          <t>Diversity and inclusion</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
@@ -11883,7 +11973,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>Gender equality</t>
+          <t>Diversity and inclusion</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
@@ -12326,12 +12416,12 @@
       </c>
       <c r="J224" t="inlineStr">
         <is>
-          <t>Consumer protection; Stability, safety and soundness</t>
+          <t>Consumer protection; Stability, safety and soundness; Financial inclusion</t>
         </is>
       </c>
       <c r="K224" t="inlineStr">
         <is>
-          <t>Data privacy and protection, Reputational and legal risk</t>
+          <t>Data privacy and protection, Reputational and legal risk, Quality</t>
         </is>
       </c>
       <c r="L224" t="inlineStr">
@@ -12386,12 +12476,12 @@
       </c>
       <c r="J225" t="inlineStr">
         <is>
-          <t>Financial inclusion; Stability, safety and soundness</t>
+          <t>Financial inclusion; Stability, safety and soundness; Consumer protection</t>
         </is>
       </c>
       <c r="K225" t="inlineStr">
         <is>
-          <t>Quality, Operational risk</t>
+          <t>Quality, Operational risk, Fair treatment</t>
         </is>
       </c>
       <c r="L225" t="inlineStr">
@@ -12506,12 +12596,12 @@
       </c>
       <c r="J227" t="inlineStr">
         <is>
-          <t>Financial inclusion; Stability, safety and soundness</t>
+          <t>Financial inclusion; Stability, safety and soundness; Consumer protection</t>
         </is>
       </c>
       <c r="K227" t="inlineStr">
         <is>
-          <t>Quality, Operational risk</t>
+          <t>Quality, Operational risk, Fair treatment</t>
         </is>
       </c>
       <c r="L227" t="inlineStr">
@@ -12682,7 +12772,7 @@
       </c>
       <c r="K230" t="inlineStr">
         <is>
-          <t>Usage, Suitability</t>
+          <t>Quality, Suitability</t>
         </is>
       </c>
       <c r="L230" t="inlineStr">
@@ -12742,7 +12832,7 @@
       </c>
       <c r="K231" t="inlineStr">
         <is>
-          <t>Usage, Suitability</t>
+          <t>Quality, Suitability</t>
         </is>
       </c>
       <c r="L231" t="inlineStr">

</xml_diff>

<commit_message>
Remove "Stability" and "Reputational and legal risk" objectives
Drop both objectives from the Stability mandate in MND_OBJ_2 (cascades to the
objectives filter UI and the connector's objective->mandate lookup). Refresh
data/indicators.RData and the public xlsx from the updated Google Sheet
(230 indicators) where these objectives were removed/reclassified — verified
0 remaining references in any objective column.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/www/LENS_INDICATORS_DB.xlsx
+++ b/www/LENS_INDICATORS_DB.xlsx
@@ -6209,12 +6209,12 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>Consumer protection; Stability, safety and soundness</t>
+          <t>Consumer protection</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>Fair treatment, Stability</t>
+          <t>Fair treatment</t>
         </is>
       </c>
       <c r="L111" t="inlineStr">
@@ -7422,12 +7422,12 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>Financial inclusion; Consumer protection; Stability, safety and soundness</t>
+          <t>Financial inclusion; Consumer protection</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>Quality, Suitability, Stability</t>
+          <t>Quality, Suitability</t>
         </is>
       </c>
       <c r="L132" t="inlineStr">
@@ -7605,7 +7605,7 @@
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>Quality, Reputational and legal risk</t>
+          <t>Quality, Operational risk</t>
         </is>
       </c>
       <c r="L135" t="inlineStr">
@@ -7788,7 +7788,7 @@
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>Outcomes, Reputational and legal risk</t>
+          <t>Outcomes, Operational risk</t>
         </is>
       </c>
       <c r="L138" t="inlineStr">
@@ -8253,7 +8253,7 @@
       </c>
       <c r="K146" t="inlineStr">
         <is>
-          <t>Outcomes, Reputational and legal risk</t>
+          <t>Outcomes, Operational risk</t>
         </is>
       </c>
       <c r="L146" t="inlineStr">
@@ -8669,7 +8669,7 @@
       </c>
       <c r="J153" t="inlineStr">
         <is>
-          <t>Financial inclusion; Stability, safety and soundness</t>
+          <t>Financial inclusion</t>
         </is>
       </c>
       <c r="K153" t="inlineStr">
@@ -11280,7 +11280,7 @@
       </c>
       <c r="K202" t="inlineStr">
         <is>
-          <t>Credit risk, Stability</t>
+          <t>Credit risk</t>
         </is>
       </c>
       <c r="L202" t="inlineStr">
@@ -11335,7 +11335,7 @@
       </c>
       <c r="K203" t="inlineStr">
         <is>
-          <t>Credit risk, Stability</t>
+          <t>Credit risk</t>
         </is>
       </c>
       <c r="L203" t="inlineStr">
@@ -11390,7 +11390,7 @@
       </c>
       <c r="K204" t="inlineStr">
         <is>
-          <t>Credit risk, Stability</t>
+          <t>Credit risk</t>
         </is>
       </c>
       <c r="L204" t="inlineStr">
@@ -12421,7 +12421,7 @@
       </c>
       <c r="K224" t="inlineStr">
         <is>
-          <t>Data privacy and protection, Reputational and legal risk, Quality</t>
+          <t>Data privacy and protection, Operational risk, Quality</t>
         </is>
       </c>
       <c r="L224" t="inlineStr">

</xml_diff>

<commit_message>
Rename "Sustainability" mandate to "Sustainability (ESG)"
Add a rename step in data_prep.R: rename the mandate across the mandate
columns and rebuild the mandate-objective labels from the renamed values
(factor levels updated too). Update the app's hardcoded references in
globals.R — MND_OBJ_2 key (objectives filter), MANDATE_TG_ID key
(technical-guide icon), and the tech-guide memo title. Regenerated
indicators.RData + public xlsx (16 indicators; 0 bare "Sustainability"
remaining).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/www/LENS_INDICATORS_DB.xlsx
+++ b/www/LENS_INDICATORS_DB.xlsx
@@ -11177,7 +11177,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>Sustainability</t>
+          <t>Sustainability (ESG)</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -11237,7 +11237,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>Sustainability</t>
+          <t>Sustainability (ESG)</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -11292,7 +11292,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>Sustainability</t>
+          <t>Sustainability (ESG)</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -11347,7 +11347,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>Sustainability</t>
+          <t>Sustainability (ESG)</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -11402,7 +11402,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>Sustainability</t>
+          <t>Sustainability (ESG)</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -11457,7 +11457,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>Sustainability</t>
+          <t>Sustainability (ESG)</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -11517,7 +11517,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>Sustainability</t>
+          <t>Sustainability (ESG)</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -11577,7 +11577,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>Sustainability</t>
+          <t>Sustainability (ESG)</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -11632,7 +11632,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>Sustainability</t>
+          <t>Sustainability (ESG)</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -11677,7 +11677,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>Sustainability</t>
+          <t>Sustainability (ESG)</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -11732,7 +11732,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>Sustainability</t>
+          <t>Sustainability (ESG)</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
@@ -11787,7 +11787,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>Sustainability</t>
+          <t>Sustainability (ESG)</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -11832,7 +11832,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>Sustainability</t>
+          <t>Sustainability (ESG)</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -11877,7 +11877,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>Sustainability</t>
+          <t>Sustainability (ESG)</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -11922,7 +11922,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>Sustainability</t>
+          <t>Sustainability (ESG)</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -11968,7 +11968,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>Sustainability</t>
+          <t>Sustainability (ESG)</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">

</xml_diff>

<commit_message>
Refresh indicator data from master database
Re-ran data_prep.R against the upstream Google Sheet. 230 indicators
(232 loaded, 2 dropped per the catalog exclusion list).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/www/LENS_INDICATORS_DB.xlsx
+++ b/www/LENS_INDICATORS_DB.xlsx
@@ -452,7 +452,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Are the infrastructures for access well dimensioned and designed to meet the customers needs, including by gender and other sociodemographics? This indicator could be analyzed together with indicators for transactions and against indicators for gender diversity</t>
+          <t>Are physical access points distributed in a way that adequately serves the needs of all sociodemographic groups, including in underserved or low-income areas (e.g., higher proportions of female-headed households receiving G2P payments)? Variations in this indicator may be explored across type of access point, FSP type, and location. Answering this question requires matching access point location with socio-demographic and economics information about each location. This indicator can be analyzed alongside indicators for transaction volumes. Also, do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -497,7 +497,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Do administrative units without any financial access points have substantially different population characteristics (gender, age, location, income) compared to those with at least one access point (e.g., higher proportions of women, female-headed households, or other vulnerable subgroups)? Are there differences in the types of financial access points/physical channels (e.g., ATM, branch, agent/merchants) present in administrative units with higher versus lower shares of female population? Are FSPs with higher levels of gender diversity more likely to deploy access points in underserved administrative units?. NOTE: these questions are meant to analyze the territorial distribution of physical access points and how it aligns with gender-related characteristics of administrative units. To understand the effective population coverage by gender, see the related indicator on “Population living in administrative units with at least one access point.</t>
+          <t>Do administrative units without financial access points have substantially different gender compositions (higher proportions of women or female-headed households)? Answering this question requires matching access point location with socio-demographic and economics information about each location. This indicator can be analyzed alongside population coverage by access point indicator, and the indicator on physical access points. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? Variations in this indicator may be explored across type of access point and location.</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -542,7 +542,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Are women, including female-headed households, disproportionately concentrated in administrative units without financial access points, resulting in lower effective coverage? Does the share of women living in covered areas differ significantly from that of men, and how does this vary across regions or demographic groups? Are FSPs with higher levels of gender diversity more likely to extend access coverage to administrative units with higher shares of women or underserved female populations?</t>
+          <t>This question requires matching access point location with population size for each location. Are women, particularly those in female-headed households, disproportionately concentrated in areas without financial access points? Variations in this indicator may be explored across access point type.</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -587,7 +587,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the likelihood of being located in areas with low levels of access to transaction points, including for elderly customers, low-income customers, low-value accounts, and MSMEs based on the ownership gender?  Are FSPs with higher levels of gender diversity more or less likely to have more clients in areas with a low density of access points?</t>
+          <t>is there gender disparity of customer location in areas with high or low financial access point density? if there is such information by location, does low access point density intersect with areas of high informality, or with low income? Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside administrative units with at least one physical access point to explore whether areas without any access point have substantially higher shares of vulnerable customer groups. Variations in this indicator may be explored across customer type, gender, age, income, location, and FSP type.</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -647,7 +647,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Are there gender disparities in registration on digital banking platforms and access to digital banking channels? Are banks with higher levels of gender diversity more or less likely to have more clients registered on their digital channels? Are there differences for other sociodemographic traits, in isolate or in combination (eg; young rural women)</t>
+          <t>Are there gender disparities in the volume or value of premiums written? Variations in this indicator may be explored across customer type, gender, age, income, location, FSP type, type of insurance, and average premium. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -697,7 +697,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Are there differences based on the owner's gender and/or manager of the MSME in the acceptance of digital or cashless transactions? Are FSPs with higher levels of gender diversity more likely to have more women-owned MSMEs accepting digital payments in their networks?</t>
+          <t>Are there gender disparities in the share of MSMEs using digital payment tools? Variations in this indicator may be explored across MSME gender of owner, business sector, location, income, age, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Are there differences based on the owner's gender and/or manager of the MSME in: participation in merchant and agent networks, payment instruments accepted, and geographical distribution? Are FSPs with higher levels of gender diversity more likely to have greater participation of women-owned MSMEs in their networks?</t>
+          <t>Are there gender disparities in the share of MSMEs using digital payment tools? Variations in this indicator may be explored across MSME gender of owner, business sector, age, location, income, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? This indicator can be analyzed alongside MSMEs accepting digital transactions and MSMEs using digital payments to explore whether participation in payment networks translates into active digital transaction acceptance and payment usage.</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -807,7 +807,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the number of accounts registered in or connected to the instant payment system (IPS)? Are FSPs with higher levels of gender diversity more likely to sign up a more diverse customer base? How do sign-up rates compare with the indicator on IPS usage? Are lower levels of sign-ups concentrated in specific FSP types, FSP gender diversity rate, geographic regions, or account balance segments?</t>
+          <t>Are there gender disparities in the number of accounts registered in the instant payment system? Variations in this indicator may be explored across customer gender, age, income, location, customer type, and FSP type. This indicator can be analyzed alongside instant/fast payment transactions per account. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -852,7 +852,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the number of unique current account holders, and how do these vary across age groups, income levels, and urban or rural locations? Do individuals from specific gender and age groups—particularly those in low-income or remote areas—disproportionately lack access to current accounts? Are financial service providers with higher levels of gender diversity in their customer base or workforce more likely to serve a more balanced gender distribution of depositors? Does greater gender diversity among FSP leadership or staff correlate with more equitable account access across gender, age, and income groups? Among MSMEs, are current accounts equally held across enterprises led by individuals of different genders and age groups, and does this vary by region or business type?</t>
+          <t>Are there gender disparities in the number of unique current account holders? Variations in this indicator may be explored across customer type, gender, age, income, location, FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -903,7 +903,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Are there differences in the average number of current accounts held by individuals of different genders, ages, and income levels, including the incidence of multiple account ownership? How do patterns of account ownership vary across financial institutions or regions, and do certain age or gender groups tend to concentrate their accounts in particular provider types? Do FSPs with more gender-diverse teams offer more flexible or inclusive account structures that promote usage among underrepresented gender and age groups?</t>
+          <t>Are there gender disparities in the average number of accounts held per person? Variations in this indicator may be explored across customer type, gender, age, income, location, FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -953,8 +953,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the number of unique deposit account holders, and how do these vary across age groups, income levels, and urban or rural locations? Do individuals from certain gender and age groups, particularly those in low-income or remote areas, disproportionately lack access to deposit accounts? Are deposit accounts equally held across MSMEs led by individuals of different genders and ages?
-Does greater gender diversity in the staff or leadership of financial service providers correlate with more inclusive patterns of deposit account ownership?</t>
+          <t>Are there gender disparities in the number of unique deposit account holders? Variations in this indicator may be explored across customer gender, age, income, location, customer type, product type and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1004,8 +1003,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Are there differences in the number of deposit accounts held by individuals across gender, age, and income groups, including the incidence of multiple accounts per person? Do certain gender groups tend to hold more deposit accounts in specific types of financial institutions or regions? Among MSMEs, do ownership patterns of multiple deposit accounts differ based on the gender of the business owner?
-Do FSPs with more gender-diverse teams or customer bases offer products that encourage account use and retention among underserved gender and age segments?</t>
+          <t>Are there gender disparities in the average number of accounts held per person? Variations in this indicator may be explored across customer type, gender, age, income, location, FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside active deposit accounts (number) to explore whether socio-demographic gaps in total deposit account ownership are larger or smaller than gaps in active usage.</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1056,8 +1054,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the number of unique e-money account holders, and how do these vary by age group, income level, and urban vs. rural location? Do certain gender and age groups, particularly in low-income or remote communities, face greater barriers to registering or maintaining e-money accounts? Among MSMEs, are e-money accounts equally adopted by businesses led by individuals of different genders and age groups?
-Does gender diversity within mobile money operators or e-money providers influence the inclusiveness of account ownership across gender, age, and income segments?</t>
+          <t>Are there gender disparities in the number of e-money accounts? Variations in this indicator may be explored across customer gender, age, income, location, customer type, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1107,8 +1104,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Are there differences across gender, age, and income groups in the number of e-money accounts held, including the prevalence of multiple accounts per person? Do certain types of providers or platforms attract more account ownership from specific gender or age groups? Among MSMEs, does the number of e-money accounts vary depending on the gender and age of the business owner, and are there differences in account use by region or sector?
-Are FSPs or non-bank e-money providers with more gender-diverse staff or leadership more likely to support broader account ownership among underrepresented groups?</t>
+          <t>Are there gender disparities in the number of e-money accounts? Variations in this indicator may be explored across customer gender, age, income, location, customer type, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1158,8 +1154,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the number of unique mobile money account holders, and how do these vary across age groups, income levels, and rural versus urban areas? Do individuals of certain genders and ages, particularly in low-income or remote communities, face greater challenges in accessing or registering mobile money accounts? Among MSMEs, are mobile money accounts equally held by enterprises led by individuals of different genders and age groups, and do these patterns differ by region or sector?
-Does greater gender diversity within mobile money providers’ leadership or agent networks correlate with more equitable access to accounts across gender, age, and income groups?</t>
+          <t>Are there gender disparities in the unique holders of mobile money accounts? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, account average balance. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside active mobile money accounts (number) to explore whether socio-demographic gaps in mobile money account ownership translate into similar gaps in active usage.</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1209,8 +1204,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Are there gender differences in the number of mobile money accounts held per person, and how do these patterns vary by age, income level, or provider type? Do specific groups, such as women or youth, tend to rely on single-account setups while others hold multiple accounts, and does this affect usage behavior? Among MSMEs, does the number of mobile money accounts differ by gender or age of the business owner, and is this linked to business type or transaction volume?
-Do mobile money providers with more gender-inclusive teams or outreach strategies facilitate wider account ownership among underrepresented gender and age groups?</t>
+          <t>Are there gender disparities in the accounts per person of mobile money accounts? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, average account balance. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside mobile money account holders to explore whether sociio-demographic disparities in accounts per person reflect patterns of multiple account use.</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1258,6 +1252,11 @@
           <t>Measures the number of individuals or entities that hold at least one payment account with a regulated payment service provider or financial institution. Each holder is counted once, regardless of the number of accounts they maintain. Captures the extent of access to formal payment infrastructure, indicating the proportion of the population or firms that can send, receive, and store funds electronically through regulated accounts. Payment account ownership is a core measure of financial inclusion and digital financial participation. It helps assess: the reach of cashless transaction systems, the effectiveness instant payment schemes, and the integration of individuals and MSMEs into formal payment networks. Higher values indicate wider participation in the digital payment ecosystem; low values suggest barriers to access, especially in underserved regions or demographics. !- Definitions and concepts: Payment account: An account that allows customers to execute payment transactions (deposits, withdrawals, transfers) and access funds on demand. Includes current accounts, e-money accounts, mobile money accounts, and other regulated transaction accounts. !- Data requirements: Administrative or supervisory data from banks, mobile money operators, e-money issuers, and payment service providers. Disaggregation variables for segmentation analysis, for example, customer type, product type, gender. !- Derivable indicators: Payment account ownership rate = (Number of payment account holders / Adult population) × 100</t>
         </is>
       </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Are there gender disparities in the number of unique payment account holders? Variations in this indicator may be explored across customer type, gender, age, income, location and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
+        </is>
+      </c>
       <c r="I18" t="inlineStr">
         <is>
           <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
@@ -1306,7 +1305,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Are there differences in the number of  payment accounts held across gender, age, and income groups, including the prevalence of multiple account ownership? Do individuals of certain gender or age groups tend to hold multiple payment accounts with different providers, and what might explain these patterns? Among MSMEs, does the number of such accounts vary based on the gender and age of the owner, and is this linked to digital payment adoption or business type? Are providers with greater gender inclusion in product development or distribution channels more successful in supporting wider account ownership among underserved gender and age groups?</t>
+          <t>Are there gender disparities in the average number of accounts held per person,? Variations in this indicator may be explored across customer type, gender, age, income, location, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1356,7 +1355,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the number of unique savings account holders, and how do these vary by age group, income level, and rural vs. urban location? Do certain gender and age groups, particularly low-income individuals or those in remote areas, face greater barriers to opening or maintaining savings accounts? Does greater gender diversity within financial service providers correlate with more equitable savings account ownership across demographic groups?</t>
+          <t>Are there gender disparities in the number of unique savings account holders? Variations in this indicator may be explored across customer type, gender, age, income, location, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1407,7 +1406,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Are there differences across gender, age, and income groups in the number of savings accounts held, including multiple accounts per individual? Do specific demographic groups tend to maintain more savings accounts, and how does this relate to financial goals or access to different types of savings products? Are financial institutions with gender-diverse teams or inclusive policies more likely to support broader savings account ownership among underserved groups?</t>
+          <t>Are there gender disparities in the average number of accounts held per person? Variations in this indicator may be explored across customer type, gender, age, income, location, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1458,7 +1457,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the number of unique term deposit account holders, and how do these vary by age group, income level, and urban versus rural location? Do women or other gender groups face particular barriers in accessing term deposit products, such as minimum balance requirements or lack of tailored products? Do financial institutions with higher gender diversity in management or customer-facing roles show more balanced term deposit ownership across demographic groups?</t>
+          <t>Are there gender disparities in the number of unique term deposit account holders? Variations in this indicator may be explored across customer type, gender, age, income, location, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1508,7 +1507,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Are there differences by gender, age, and income in the number of term deposit accounts held, including multiple accounts per individual or business? Do certain gender or age groups tend to maintain more term deposits, possibly reflecting differing savings strategies or access to credit alternatives? Are providers with greater gender diversity more effective in expanding term deposit ownership among underrepresented gender and demographic groups?</t>
+          <t>Are there gender disparities in the average number of term deposit accounts held per person? Variations in this indicator may be explored across customer type, gender, age, income, location, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1558,7 +1557,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the number of unique pension account holders, and how do these vary by age group, income level, and urban versus rural location? Are women or other gender groups underrepresented in pension coverage, particularly among informal sector workers or MSMEs owners? Do pension providers or administrators with higher gender diversity in governance or management correlate with more inclusive pension account ownership across gender, age, and income groups?</t>
+          <t>Are there gender disparities in the number of pension account holders? Variations in this indicator may be explored across customer type, gender, age, income, location, FSP type, and pension type. Do FSPs with higher gender diversity show higher pension account ownership rates among women? This indicator can be analyzed alongside pension contributors to explore whether socio-demographic gaps in account holding are larger or smaller than gaps in active contribution.</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1608,7 +1607,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Are there differences by gender, age, and income in the number of pension accounts held, including cases where individuals hold multiple pension schemes? Do women tend to hold fewer or more pension accounts than men, and how does this relate to employment patterns or access to formal pension systems? Are pension providers with gender-diverse leadership more effective in expanding pension coverage among underrepresented gender and demographic groups?</t>
+          <t>Are there gender disparities in the number of pension account holders? Variations in this indicator may be explored across customer type, gender, age, income, location, FSP type, and pension type. Do FSPs with higher gender diversity show higher pension account ownership rates among women?</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1658,7 +1657,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the growth of investor participation in capital markets, including among MSMEs based on the gender of ownership? Which gender is underrepresented in the pool of retail investors, and how does this vary by age, income level, and location? Are certain market niches or investment products particularly skewed toward one gender? Do financial service providers (brokers, investment platforms, etc.) with higher levels of gender diversity tend to attract a more diverse investor base, including greater participation from women and women-owned MSMEs?</t>
+          <t>Are there gender disparities in the number or value of investment accounts held? Variations in this indicator may be explored across customer type, gender, age, income, location, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1719,7 +1718,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Are there differences by gender, age, and income in the number of investment accounts held by retail investors, including those linked to multiple providers or products? Are certain demographic groups or MSMEs more likely to hold multiple accounts, and does this vary with the gender of the investor or business owner? Are investment firms with greater gender diversity in leadership or advisory roles more successful in broadening account ownership among underrepresented groups?</t>
+          <t>Are there gender disparities in the number or value of investment accounts held? Variations in this indicator may be explored across customer type, gender, age, income, location, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside investment account holders (retail investors) to explore whether socio-demographic gaps in the number of investment accounts reflect differences in account ownership or in the tendency to hold multiple accounts.</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1779,7 +1778,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the number of unique debit card holders, and how do these differences vary across regions, income levels, or types of FSP? Do individuals of different genders have equal access to credit card products, or are there structural or eligibility barriers affecting uptake? How does the distribution of credit card ownership reflect broader patterns in formal credit access and usage across gender groups? Among MSMEs, are credit cards equally accessible regardless of the gender of the business owner, and do uptake patterns differ by sector or region? Are FSPs with higher levels of gender diversity more likely to issue credit cards to a more gender-diverse customer base?</t>
+          <t>Are there gender disparities in the number of unique debit card holders? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, product type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1829,7 +1828,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the average number of debit cards held per person, particularly across regions or FSP types? Is the total value transacted through debit cards lower for women, and how might this relate to income levels or account balances? Are women more</t>
+          <t>Are there gender disparities in the number of debit cards in circulation? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, product type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1880,7 +1879,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the number of unique credit card holders, and how do these differences vary across regions, income levels, or types of FSP? Do individuals of different genders have equal access to credit card products, or are there structural or eligibility barriers affecting uptake? How does the distribution of credit card ownership reflect broader patterns in formal credit access and usage across gender groups? Among MSMEs, are credit cards equally accessible regardless of the gender of the business owner, and do uptake patterns differ by sector or region? Are FSPs with higher levels of gender diversity more likely to issue credit cards to a more gender-diverse customer base?</t>
+          <t>Are there gender disparities in the number of unique credit card holders? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, average balance. Are FSPs with higher gender diversity more likely to issue credit cards to a more gender-diverse customer base? This indicator can be analyzed alongside credit cards (credit limit) to explore whether socio-demographic gaps in credit card access are compounded by lower credit limits assigned to differnt customer segments, suggesting a dual disadvantage in both access and credit depth.</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -1930,7 +1929,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the volume of credit cards issued, especially when analyzed by FSP type or region? Do providers serving a higher proportion of women issue fewer credit cards per capita? Is the volume of credit cards higher among FSPs with stronger gender diversity practices?</t>
+          <t>Are there gender disparities in the number of credit cards in circulation? Variations in this indicator may be explored across customer type, gender, age, income, location, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside credit cards (credit limit) and credit cards (outstanding balance) to explore whether customer groups with fewer credit cards in circulation are also those with lower limits and lower balances.</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -1980,9 +1979,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the number of unique loan borrowers, disaggregated by age, income level, location (urban/rural), and borrower type (individuals vs. MSMEs)? How do FSPs and different types of financial institutions differ in the gender composition of their borrower base? Are certain gender groups underrepresented among loan borrowers across loan types, sectors, or regions? To what extent do structural or eligibility barriers affect loan access for different gender and demographic groups? 
-How do multiple loan holdings by borrowers vary by gender and demographic characteristics?  Are FSPs with higher levels of gender diversity in leadership, credit teams, or customer-facing roles more likely to serve a balanced gender distribution among borrowers?
-How does gender diversity within FSPs correlate with borrower participation rates and broader financial inclusion outcomes?</t>
+          <t>Are there gender disparities in the number of unique loan borrowers? Variations in this indicator may be explored across customer type, gender, age, income, location, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside loans (number) to explore whether socio-demographic gaps in unique borrowers are similar to gaps in the total number of loans.</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2042,8 +2039,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>How do financial service providers (FSPs), including different types of FSPs, differ in the gender composition of their loan portfolios? Are there gender disparities in loan portfolio participation across various loan types and sectors?  When disaggregated by gender, age, income, and location, how do loan uptake patterns vary for individuals and MSMEs? Are women, WMSME or other customer groups underrepresented as borrowers in specific loan categories or regions? Are there differences in multiple loan holdings by gender or other sociodemographic group? 
-Comparing this indicator with FSP gender diversity, are lower gender disparities in loan portfolio participation correlated with higher levels of gender diversity within FSPs? How do gender disparities in loan portfolios relate to market-average interest rates or return rates on loan balances? For instance, do FSPs with predominantly female or male loan portfolios offer different rates compared to the market average? Are lower gender disparities in loan portfolio participation correlated with lower non-performing loan (NPL) ratios, and does this correlation vary when women’s representation in the loan portfolio is above or below market averages?</t>
+          <t>Are there gender disparities in the number of loans? Variations in this indicator may be explored across customer gender, customer type, FSP type, product type, loan size, and loan term. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside loans (principal disbursed) to explore whether socio-demographic gaps in the number of loans are proportional to gaps in the value disbursed.</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2103,8 +2099,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the number of unique loan borrowers of secured loans, disaggregated by age, income level, location (urban/rural), and borrower type (individuals vs. MSMEs)? How do FSPs and different types of financial institutions differ in the gender composition of their borrower base of this type of loans? Are certain gender groups underrepresented among these borrowers across secured loan types, sectors, or regions? To what extent do structural or eligibility barriers affect secured loan access for different gender and demographic groups? How do multiple secured loan holdings by borrowers vary by gender and demographic characteristics?  Are FSPs with higher levels of gender diversity in leadership, credit teams, or customer-facing roles more likely to serve a balanced gender distribution among secured loan borrowers?
-How does gender diversity within FSPs correlate with borrower participation rates and broader financial inclusion outcomes?</t>
+          <t>Are there gender disparities in the number of unique secured loan borrowers? Variations in this indicator may be explored across customer type, gender, age, income, location, FSP type, loan type, term and size. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside collateral pledges on credit (borrowers) to explore whether socio-demographic gaps in secured loan access are associated with differences in the type or value of collateral pledged by each customer group.</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2164,7 +2159,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>How do financial service providers (FSPs), including different types of FSPs, differ in the gender composition of their secured loan portfolios? Are there gender disparities in loan portfolio participation across various loan types and sectors? When disaggregated by gender, age, income, and location, how do secured loan uptake patterns vary? Are women or other gender groups underrepresented as borrowers in specific secured loan categories or regions? Are there differences in multiple loan holdings by gender or demographic group? Comparing this indicator with FSP gender diversity, are lower gender disparities in the secured loan portfolio participation correlated with higher levels of gender diversity within FSPs? How do gender disparities in this portfolio relate to market-average interest rates or return rates on loan balances? For instance, do FSPs with predominantly female or male loan portfolios offer different rates compared to the market average? Are lower gender disparities in loan portfolio participation correlated with lower non-performing loan (NPL) ratios, and does this correlation vary when women’s representation in the loan portfolio is above or below market averages? Are there gender differences in the types of collateral pledged for secured loans, such as movable versus immovable assets? To what extent do collateral requirements create gender-specific barriers to accessing secured credit, especially for women who may have limited ownership of traditionally accepted assets?</t>
+          <t>Are there gender disparities in the number of secured loans? Variations in this indicator may be explored across customer type, gender, age, income, FSP type, loan type, size, term. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2224,8 +2219,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the number of unique borrowers of secured loans, disaggregated by age, income level, location (urban/rural), and borrower type (individuals vs. MSMEs)? How do FSPs and different types of financial institutions differ in the gender composition of their secured loan borrower base? Are women or other gender groups underrepresented among secured loan borrowers across loan types, sectors, or regions? To what extent do collateral requirements create gender-specific barriers to accessing secured credit, especially for borrowers who may have limited ownership or control over accepted types of collateral? Are there gender differences in the types of collateral pledged by borrowers, such as movable versus immovable assets?
-How do multiple secured loan holdings by borrowers vary by gender and other demographic characteristics? Are FSPs with higher levels of gender diversity in leadership, credit teams, or customer-facing roles more likely to serve a balanced gender distribution among secured loan borrowers? How does gender diversity within FSPs correlate with borrower participation rates and secured credit access outcomes?</t>
+          <t>Are there gender disparities in the number of unique unsecured loan borrowers? Variations in this indicator may be explored across customer type, gender, age, income, location, FSP type, loan type, term and size. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside loans, secured (borrowers) to explore whether customer groups underrepresented among secured borrowers compensate through higher unsecured credit uptake.</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2285,7 +2279,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the number of unique borrowers of unsecured loans, disaggregated by age, income level, location (urban/rural), and borrower type (individuals vs. MSMEs)? How do FSPs and different types of financial institutions differ in the gender composition of their unsecured loan borrower base? Are women or other gender groups underrepresented among unsecured loan borrowers across loan types, sectors, or regions? To what extent do the absence of collateral requirements improve or hinder loan access for different gender groups? Are there specific barriers related to creditworthiness or other factors that disproportionately affect certain genders? How do multiple unsecured loan holdings by borrowers vary by gender and other demographic characteristics?  Are FSPs with higher levels of gender diversity in leadership, credit teams, or customer-facing roles more likely to serve a balanced gender distribution among unsecured loan borrowers? How does gender diversity within FSPs correlate with borrower participation rates and unsecured credit access outcomes?</t>
+          <t>Are there gender disparities in the number of unsecured loans? Variations in this indicator may be explored across customer type, gender, age, income, location, FSP type, loan type, size, and term. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2345,7 +2339,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>What is the share of new borrowers by gender?</t>
+          <t>Are new borrowers representative of a gender-balanced population? Variations in this indicator may be explored across customer type, gender, age, income, location, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside first-time borrowers to explore whether socio-demographic disparities in new borrower acquisition are driven primarily by first-time credit access.</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -2400,7 +2394,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>How does the gender composition of the new loans disbursed vary by FSP type and FSP loan?  When further disaggregated by age, income, and location, do patterns vary? Are women/WMSE or other customer groups underrepresented as new borrowers in specific loan categories or regions? Comparing this indicator with FSP gender diversity, are lower gender disparities in new loans correlated with higher levels of gender diversity within FSPs?</t>
+          <t>Are there gender disparities in the volume of new loan originations? Variations in this indicator may be explored across customer type, gender, customer type, age, income, location, FSP type, loan type, size and term. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2460,7 +2454,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the overall number of unique insurance policy holders when considering all insurance types? How do these disparities vary by age, income, location, and other demographic factors? Are vulnerable populations particularly affected by gender gaps in insurance coverage? Do providers with higher gender diversity in workforce and leadership tend to have a more balanced gender distribution among all insurance policy holders? How do gender disparities differ between life and non-life insurance within the same provider or market?</t>
+          <t>Are there gender disparities in the number of unique all insurance policies? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, type of insurance, and average premium. Do insurers with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -2510,7 +2504,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the share of retail borrowers holding multiple outstanding credit operations? Do certain gender groups, such as women/WMSME , experience higher rates of potential over-indebtedness compared to others? How does the prevalence of multiple loans vary across age groups, income levels, and geographic locations by gender? Are women or other gender groups more likely to have overlapping loans from different types of financial service providers or loan products, indicating possible gaps in credit assessment? How do financial service providers with higher gender diversity in their workforce or leadership influence the incidence of multiple borrowing among different gender groups? Are there patterns in repayment behavior or default rates among borrowers with multiple loans that differ by gender?</t>
+          <t>Are there gender disparities in the share of retail borrowers holding multiple outstanding credit operations, as a potential indicator of over-indebtedness or some level of debt stress? Variations in this indicator may be explored across customer gender, age, income, location, FSP type, product type, loan size, and loan term. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside borrowers in risky indebtedness to explore whether customer segments with higher rates of multiple loans are also more frequently classified as at risk of over-indebtedness.</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -2565,7 +2559,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Are there gender differences in the total number of insurance policies held overall, including across product types and providers? How do multiple policy ownership and coverage amounts vary by gender, age, income, and location? To what extent do providers with higher gender diversity attract more gender-balanced insurance policy portfolios? Are gender disparities consistent or do they vary across life and non-life insurance policies within the overall market?</t>
+          <t>Are there gender disparities in the number of unique all insurance holders? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, type of insurance, and average premium. Do insurers with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do insurers with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -2615,7 +2609,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the number of unique life insurance policy holders? How do these disparities vary by age, income level, and geographic location? Are certain gender groups underrepresented among life insurance holders, particularly within vulnerable populations? How do differences in life insurance policy ownership relate to the types of policies held and the insured benefits across genders? Are financial service providers with greater gender diversity in leadership or workforce more likely to achieve balanced gender representation among life insurance policy holders?</t>
+          <t>Are there gender disparities in the number of unique life insurance holders? Variations in this indicator may be explored across customer type, gender, age, income, location, FSP type, type of insurance, and average premium. Do insurers with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -2665,7 +2659,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Are there gender differences in the total number of life insurance policies held, including tendencies for multiple policy ownership? How does the distribution of life insurance policies across different product types vary by gender, age, income, and location? Are coverage amounts and renewal rates equitable across gender groups? To what extent do providers with higher gender diversity attract a more diverse and balanced pool of life insurance policyholders?</t>
+          <t>Are there gender disparities in the number of unique life insurance policies? Variations in this indicator may be explored across customer gender, age, income, location, customer type, insurer type, type of insurance, and average premium. Do insurers with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do insurers with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2715,7 +2709,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>How do gender groups differ in the total number of non-life insurance policies held, including multiple policy ownership? Are there disparities in the mix of non-life insurance products held by gender, across age groups, income levels, and locations? How do coverage amounts and claim experiences vary by gender? Are providers with higher gender diversity more successful in attracting a balanced gender distribution of non-life insurance policy holders and policies?</t>
+          <t>Are there gender disparities in the number of unique non-life insurance policies? Variations in this indicator may be explored across customer type, gender, age, income, location, FSP type, type of insurance, and average premium. Do insurers with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -2765,7 +2759,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the number of unique non-life insurance policy holders, and do these disparities differ by demographic factors such as age, income, and location? How are vulnerable groups affected by access to non-life insurance coverage, and are gender gaps more pronounced in these populations? How do gender differences manifest in the types of non-life insurance policies held? Do financial service providers with greater gender diversity in their workforce or management show more balanced gender representation in non-life insurance policy holders?</t>
+          <t>Are there gender disparities in the number of unique non-life insurance holders? Variations in this indicator may be explored across customer gender, age, income, location, customer type, insurer type, type of insurance, and average premium. Do insurers with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do insurers with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -2815,7 +2809,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the number of adults receiving pension benefits, and do these reflect differences in past participation, contribution histories, or retirement age? Are women more likely to access smaller or non-contributory pensions compared to men, and how does this vary across regions or types of pension plans? Do pension systems with more inclusive design features (e.g., minimum benefit floors, crediting for unpaid care work) show smaller gender gaps in beneficiary coverage? How does the share of women among pension beneficiaries compare to their share among retirement-age adults?</t>
+          <t>Are there gender disparities in the number of adults receiving pension benefits? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, pension type average balance. Do FSPs or employers with higher gender diversity show more equitable coverage of pension beneficiaries across genders? This indicator can be analyzed alongside retirement income per pension beneficiary to explore whether socio-demographic gaps in the number of beneficiaries are accompanied by gaps in the average income received, compounding the overall pension inequality.</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -2865,7 +2859,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the proportion of adults contributing to a pension account, and how do these relate to differences in labor force participation, formality, or income levels? Do women contribute through fewer or less diversified pension plans than men (e.g., occupational vs. individual plans)? Are FSPs or employers with higher levels of gender diversity or inclusive practices more likely to enroll female workers in pension systems? How does the share of women among contributors compare to their share in the labor force, and what does this suggest about structural gaps in retirement planning?</t>
+          <t>Are there gender disparities in the proportion of adults contributing to a pension account? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, pension type, average balance. Do FSPs with higher gender diversity show higher gender balance in pension enrollment or contribution rates? This indicator can be analyzed alongside pension account holders to explore whether socio-demographic disparities in the number of pension accounts are driven primarily by gaps in active contributions.</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -2915,7 +2909,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the use of digital payments among MSMEs based on the gender of the owner?</t>
+          <t>Are there gender disparities in the share of MSMEs using digital payments? Variations in this indicator may be explored across MSME type, gender of owner, business sector, location, income, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
@@ -2960,7 +2954,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the volume of cashless transactions, and how do these relate to account ownership and usage patterns across gender, age, income, and location? When analyzed alongside the number of accounts per capita disaggregated by gender and other demographics, does this indicator reveal correlations between gender representation in account ownership and the adoption of cashless payment methods? Are certain demographic groups, such as younger individuals or those in urban areas, particularly active in driving increases in cashless transactions? How do these patterns vary across types of financial service providers (FSPs)? Do FSPs with greater gender diversity tend to serve more balanced or higher volumes of cashless transactions across gender groups?</t>
+          <t>Are there gender disparities in the frequency of cash transactions? Variations in this indicator may be explored across customer type, gender, age, income, location, FSP type, and transaction type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -3015,7 +3009,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the likelihood of engaging in e-commerce transactions, including for MSMEs based on the gender of the owner? Do transaction patterns—such as frequency and average ticket size—differ by gender, and how do these vary across income groups, age brackets, and locations? Are e-commerce transactions concentrated within specific financial service providers (FSPs) or market segments, and does this concentration reflect gender imbalances? Could differences in transaction volumes by gender indicate limited access to e-commerce payment channels or the unsuitability of available solutions for certain groups? Are FSPs with higher levels of gender diversity more likely to support inclusive e-commerce participation across genders?</t>
+          <t>Are there gender disparities in engagement with e-commerce transactions, frequency and average ticket size? Variations in this indicator may be explored across customer gender, age, income, location, customer type, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside MSMEs accepting digital transactions to explore whether gender gaps in e-commerce usage among individual consumers are mirrored by gaps in digital payment acceptance among women-led MSMEs.</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
@@ -3060,7 +3054,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>How do the number of e‑money transactions per user differ by gender, and how are these differences affected by age, income, or geographic location? Do women use e‑money more for small frequent transactions or different types (P2P, bill pay, merchant pay) compared to men? Are there FSPs with higher gender diversity which show more similar usage (in number)  of e‑money between genders? Over time, have gender gaps in e‑money transaction usage narrowed, especially among lower income or rural populations?</t>
+          <t>Are there gender disparities in the number of e-money transactions? Variations in this indicator may be explored across customer type, gender, age, income, location, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -3111,7 +3105,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>How do the value of e‑money transactions per user differ by gender, and how are these differences affected by age, income, or geographic location? Do women use e‑money more for small frequent transactions or different types (P2P, bill pay, merchant pay) compared to men? Are there FSPs with higher gender diversity which show more similar usage (in value)  of e‑money between genders? Over time, have gender gaps in e‑money transaction values narrowed, especially among lower income or rural populations?</t>
+          <t>Are there gender disparities in the value of e-money transactions? Variations in this indicator may be explored across customer type, gender, age, income, location, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -3161,7 +3155,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the value of mobile money transactions per user, and do these differences vary by income level, age group, or rural/urban location? Do women more often conduct many small transactions while men conduct fewer larger ones, or vice versa? Are MSMEs led by different gender owners showing differences in mobile money usage patterns? Do providers with more gender‐diversity show less skew in usage between genders?</t>
+          <t>Are there gender disparities in the value of mobile money transactions per person? Variations in this indicator may be explored across customer type, gender, age, income, location, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
@@ -3206,7 +3200,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the number of mobile and internet banking transactions per person? Do women use digital banking channels at similar rates and intensities as men, and how does this vary across regions or FSP types? Are FSPs with higher levels of gender diversity more likely to promote and support greater digital banking usage among women?</t>
+          <t>Are there gender disparities in the volume of mobile money transactions? Variations in this indicator may be explored across customer gender, age, income, location, customer type, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside mobile money transactions (value) to explore whether customer groups conducting more frequent mobile money transactions also transact at lower average values.</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
@@ -3251,7 +3245,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>What are the gender dynamics in remittance transactions? Is there a gender that is the predominant recipient of international remittances? What are the gender differences in the size and frequency of remittances? Are remittances concentrated in certain geographical areas, FSP types, and account types? Which channels are mostly used to receive remittances? Are these areas considered low-income locations or locations with low cash access point density? Comparing with indicators on transaction channel locations, how do they compare with remittance reception? Are remittance recipients particularly underserved by access points? Is there any correlation between the gender of recipients and FSP gender diversity? Which countries originate the most remittances to low-income locations and populations? Do these coincide with countries with higher remittance costs?</t>
+          <t>Are there gender disparities in the value of international remittances, and is there a gender that is the predominant recipient? Variations in this indicator may be explored across customer gender, age, income, location, FSP type, channel type, and transaction type. Are remittances concentrated in specific geographic areas, FSP types, or channels associated with low-income or low-access communities? Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside cost of remittances and speed of remittances to explore whether disparities in remittance value are compounded by higher costs or longer processing times.</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
@@ -3296,7 +3290,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>What are the gender dynamics in remittance transactions? Is there a gender that is the predominant recipient of international remittances? What are the gender differences in the size and frequency of remittances? Are remittances concentrated in certain geographical areas, FSP types, and account types? Which channels are mostly used to receive remittances? Are these areas considered low-income locations or locations with low cash access point density? Comparing with indicators on transaction channel locations, how do they compare with remittance reception? Are remittance recipients particularly underserved by access points? Is there any correlation between the gender of recipients and FSP gender diversity? Which countries originate the most remittances to low-income locations and populations? Do these coincide with countries with higher remittance costs?</t>
+          <t>Are there gender disparities in the volume of international remittances, and is there a gender that is the predominant recipient? Variations in this indicator may be explored across customer gender, age, income, location, FSP type, channel type, and transaction type. Are remittances concentrated in specific geographic areas, FSP types, or channels associated with low-income or low-access communities?Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside remittances, total (value) to explore whether disparities in the number and value of remittances point in the same direction, or whether different customer groups send or receive more frequent but smaller transfers.</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
@@ -3341,7 +3335,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>How do genders differ in how much and how often they transact through different channels (cash, ATM, digital, agents, mobile, etc.), by transaction value and frequency? Are there gender differences in the choice of channels associated with high‐value vs low‐value transactions? How have channel usage patterns for different genders evolved over time, especially for younger, lower‐income, or rural women? Do providers who are more gender‐inclusive tend to offer or promote more equitable access and usage across channels?</t>
+          <t>Are there gender disparities in the value of transactions conducted through different channels (cash, ATM, digital, agents, mobile)? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, and transaction type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside financial transactions by channel (volume) to explore whether disparities in transaction value and frequency point in the same direction.</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
@@ -3386,7 +3380,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>How do genders differ in how much and how often they transact through different channels (cash, ATM, digital, agents, mobile, etc.)? How have channel usage patterns for different genders evolved over time, especially for younger, lower‐income, or rural women? Do providers who are more gender‐inclusive tend to offer or promote more equitable access and usage across channels?</t>
+          <t>Are there gender disparities in the volume of transactions conducted through different channels (cash, ATM, digital, agents, mobile)? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, transaction type and average size. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
@@ -3431,7 +3425,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>How do the genders differ in terms of average number and values of transfers to deposit accounts or savings pockets?  Are there differences in averages between transfers made to deposits accounts (held at deposit-taking FSPs) compared with transfers to built-in savings pockets on mobile banking/eWallets/prepaid cards) by gender? How do the averages for the genders compare when taking age group and location into account?</t>
+          <t>Are there gender disparities in the average number and value of transfers from mobile money or e-money accounts to savings accounts? Variations in this indicator may be explored across customer gender, age, income, location, and product type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside net savings account flows to explore whether customer groups that more frequently transfer from mobile wallets to savings accounts also show more positive net savings flows, indicating disciplined savings behavior.</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -3489,6 +3483,11 @@
           <t>Measures the proportion of G2P (government-to-person) payment recipients who withdraw the full amount of their transfer within a short period after disbursement — typically within a few days. It reflects how beneficiaries use digital G2P transfers once funds are received. Captures the degree of digital payment usage versus cash-out behavior among G2P recipients. It serves as a proxy for the “stickiness” of digital transfers — indicating whether beneficiaries are retaining value in their accounts for savings, payments, or transfers, or instead immediately converting digital funds into cash. Monitoring early cash-out rates helps regulators, policymakers, and program administrators to: Assess the effectiveness of G2P digitization efforts in promoting financial inclusion; Identify whether accounts are being used only as pass-through channels; Understand beneficiary trust, access, and usability constraints (e.g., merchant acceptance, withdrawal costs, distance to agents); Evaluate program design and payment infrastructure adequacy for promoting digital ecosystem usage. High early cash-out rates may indicate that beneficiaries do not retain or use funds digitally, often due to acceptance, trust, or liquidity constraints. Declining rates over time suggest growing comfort with digital usage and ecosystem maturity. Comparison across programs or regions helps identify where policy interventions are needed to enhance digital value retention. !- Definitions and concepts: G2P payment: A government-to-person transfer made via digital or electronic means (e.g., social benefits, pensions, cash transfers). !- Data requirements: Transaction-level data from G2P program administrators, payment service providers, or e-money issuers; Disaggregation by program type (social transfer, pension, subsidy), channel (bank, mobile money, prepaid card), gender, and region. Early cash-out rate (%)= Number of G2P recipients who withdraw the full payment within defined period​/ Total number of G2P payment recipients. "Short period" can be defined based on local context, could be less than 24 hours after disbursement, 7 days,  or 1 month.</t>
         </is>
       </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Are there gender disparities in the rate of early cash-out of G2P payments? Variations in this indicator may be explored across customer gender, age, income, location, and FSP type. This indicator can be analyzed alongside G2P payments received (value) and G2P accounts covered by deposit insurance. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
+        </is>
+      </c>
       <c r="J61" t="inlineStr">
         <is>
           <t>Consumer protection</t>
@@ -3539,6 +3538,11 @@
           <t>Measures the total monetary value of government-to-person (G2P) payments received by beneficiaries during the reporting period. G2P payments include cash transfers, social benefits, pensions, wages, and subsidies disbursed by government entities to individuals through bank accounts, mobile money, prepaid cards, or other regulated payment channels. Captures the financial scale and flow of public transfers to individuals, providing insight into the extent and monetary magnitude of G2P programs and their integration into the formal financial system. It serves as an indicator of both government expenditure channeled through digital or formal platforms and the liquidity entering beneficiary accounts. racking the value of G2P payments helps regulators, policymakers, and social program administrators to: Assess the total volume of public transfers supporting households and vulnerable groups; Monitor the digitization of government payments and progress toward cashless public disbursement systems; Evaluate program efficiency, transparency, and inclusion outcomes; Analyze the role of G2P payments in household liquidity, consumption smoothing, and resilience. At the macro level, it informs estimates of fiscal transfers, financial inclusion impacts, and digital ecosystem flows. Higher total values indicate expanded fiscal transfer programs, increased inclusion, or economic support measures (e.g., during crises). Growing digital share suggests progress in government payment digitization and ecosystem integration. Declines may signal program consolidation, budget cuts, or transition to alternative delivery methods. !- Definitions and concepts: G2P payment: A government-initiated transfer made to individuals, typically for social protection, salary, pension, or subsidy purposes. !- Data requirements: Administrative data from government ministries, social protection agencies, payment service providers, and financial institutions. Disaggregation by program type (social transfer, wage, pension, subsidy), delivery channel (bank, e-money, prepaid card), and region. !- Derivable indicators: Average G2P payment per recipient = (Total value of G2P payments received) ÷ (Number of G2P recipients). Share of digital G2P payments (%) = (Value of G2P payments received digitally / Total G2P payments) × 100</t>
         </is>
       </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Are there gender disparities in the value of G2P payments received? Variations in this indicator may be explored across customer gender, age, income, location, and FSP type. This indicator can be analyzed alongside G2P accounts covered by deposit insurance and G2P payment early cash-out rate. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
+        </is>
+      </c>
       <c r="J62" t="inlineStr">
         <is>
           <t>Consumer protection</t>
@@ -3591,7 +3595,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Are there disparities in average net savings account flows, across different types of transaction accounts by gender, and/or age, location or income? How do average net savings behaviours on different types of transaction accounts vary by gender (i.e., are net savings or spending more prevalent for certain account-types more)? How have the net savings patterns and gender-disparities changed over time, taking age group and location into account?</t>
+          <t>Are there gender disparities in average net savings account flows? Variations in this indicator may be explored across customer gender, age, income, location, customer type, product type, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside deposit stability/volatility to explore whether accounts showing higher net savings flows also tend to be more stable, and whether customer groups with positive net savings show lower balance volatility.</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -3651,7 +3655,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>Are there gender disparities in participation in the growth of projects funded via P2P lending platforms? Are there gender disparities in the amounts raised and interest rates paid, including for MSMEs based on the owner's gender? Do platforms with higher levels of gender diversity attract a more diverse pool of borrowers, including more women and women-owned MSMEs?</t>
+          <t>Are there gender disparities in the representation of P2P credit operations (borrowers)? Variations in this indicator may be explored across customer type, gender, age, income, location, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -3701,7 +3705,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>Are there gender disparities in average outstanding credit card balances? Do individuals of different genders tend to carry lower or higher balances, and how might this relate to credit limits, income levels, or repayment behavior? Are credit card portfolios with higher participation from different gender groups associated with distinct risk, delinquency, or usage patterns across financial service providers? How do these patterns vary by region or provider type?</t>
+          <t>Are there gender disparities in average outstanding balances on credit cards? Variations in this indicator may be explored across customer type, gender, age, income, location, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside credit cards (credit limit) to explore whether socio-demographic disparities in outstanding balances reflect differences in the limits assigned or in utilization rates.</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -3751,7 +3755,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>Are there gender disparities in average credit limits on credit cards, and how do these vary across financial service providers, income levels, or business sectors? Do credit limits assigned to different gender groups reflect differences in credit scoring, income, or collateral requirements? Among MSMEs, are there consistent gaps in credit limit allocations based on the gender of the owner, and how might this affect business growth or credit utilization?</t>
+          <t>Are there gender disparities in credit card limits? Variations in this indicator may be explored across customer type, gender, age, income, location, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -3801,7 +3805,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the total outstanding loan balances held by individuals orMSMEs, disaggregated by borrower gender or business owner gender? Do women tend to have lower outstanding balances due to smaller initial loan amounts, shorter loan terms, or faster repayment schedules? How do outstanding loan balances vary across age, income levels, and location for different gender groups? Are portfolios with higher female participation associated with different risk profiles, credit exposure patterns, or lower NPL rates? How does the share of total outstanding balances held by women compare to that held by men, and what does this imply about scale of credit access and usage? Are FSPs with greater gender diversity more likely to have balanced outstanding loan amounts across genders?</t>
+          <t>Are there gender disparities in the outstanding loan balance? Variations in this indicator may be explored across customer gender, customer type, FSP type, product type, loan size, and loan term. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside loans (number) to explore whether socio-demographic disparities in outstanding balances are explained by the number of loans held or by differences in the size and term of loans accessed by each customer segment.</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -3861,7 +3865,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the total principal amount of loans disbursed to individuals and MSMEs, disaggregated by borrower or business owner gender? Do women systematically receive smaller loan disbursements than men when controlling for loan type, income level, and sector? Are these disparities more pronounced in certain types of FSPs, geographic regions, or demographic groups? How does the share of total credit disbursed to women compare with their share of total loan applicants or potential borrowers? What does this reveal about credit allocation and approval processes? Are FSPs with higher gender diversity more likely to disburse a larger proportion of credit to women or women-owned MSMEs? How do disbursement patterns by gender relate to broader financial inclusion goals and barriers?</t>
+          <t>Are there gender disparities in the principal disbursed? Variations in this indicator may be explored across customer gender, customer type, FSP type, product type, loan size, and loan term. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside new loans (number) to explore whether socio-demographic disparities in the value disbursed are driven by fewer loans or by systematically smaller loan sizes.</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -3921,7 +3925,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>For the outstanding balance of secured credit, are there gender disparities in the total amount of outstanding loan balances held by individuals and MSMEs when disaggregated by gender? Do women tend to hold lower outstanding balances due to smaller initial loan amounts, shorter loan terms, or faster repayment rates? Are secured loan portfolios with higher female representation associated with different patterns of credit exposure or risk, such as lower non-performing loan (NPL) ratios? How do outstanding balances vary across age, income levels, and geographic locations by gender? Are there gender differences in the types and values of collateral pledged, and how might these differences affect the size and terms of outstanding secured loans? Are FSPs with greater gender diversity more likely to exhibit a balanced distribution of outstanding secured loan amounts across genders?</t>
+          <t>Are there gender disparities in the outstanding balance of secured loans? Variations in this indicator may be explored across customer type, age, gender, income, location, FSP type, product type, loan size, and loan term. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="L69" t="inlineStr">
@@ -3966,7 +3970,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the total amount of loans disbursed to individuals and MSMEs, disaggregated by the borrower’s gender? Do women receive systematically smaller disbursements than men within comparable secured loan types, sectors, or regions, and what does this imply about differences in access to productive credit? Are these disparities more pronounced in certain types of financial service providers or geographic areas? To what extent do collateral requirements influence the size of disbursements across gender groups? Are there differences in the acceptance or valuation of collateral provided by women versus men, and how does this impact loan approval and amounts disbursed? Do FSPs with higher levels of gender diversity tend to disburse a greater share of secured loan value to women or women-owned MSMEs? How does the share of total secured credit disbursed to women compare to their share of total loan applicants or potential borrowers, and what insights does this provide about credit allocation and approval processes?</t>
+          <t>Are there gender disparities in the principal disbursed of secured loans? Variations in this indicator may be explored across customer type, gender, age, income, location, FSP type, product type, loan size, and loan term. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="L70" t="inlineStr">
@@ -4011,7 +4015,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the total amount of outstanding loan balances held by individuals and MSMEs when disaggregated by gender? Do women tend to hold lower outstanding balances due to smaller initial loan amounts, shorter loan terms, or faster repayment rates? Are unsecured loan portfolios with higher female representation associated with different patterns of credit exposure or risk, such as lower non-performing loan (NPL) ratios? How do outstanding balances vary across age, income levels, and geographic locations by gender? Are FSPs with greater gender diversity more likely to exhibit a balanced distribution of outstanding unsecured loan amounts across genders?</t>
+          <t>Are there gender disparities in the outstanding balance of unsecured loans? Variations in this indicator may be explored across customer type, gender, age, income, location, FSP type, loan type, size, and term. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="L71" t="inlineStr">
@@ -4056,7 +4060,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the total amount of loans disbursed to individuals and MSMEs, disaggregated by borrower gender? Do women receive systematically smaller disbursements than men within comparable unsecured loan types, sectors, or regions, and what does this imply about differences in access to productive credit? Are these disparities more pronounced in certain types of financial service providers or geographic areas? How do credit approval criteria or lending terms for unsecured loans impact different gender groups? Do FSPs with higher levels of gender diversity tend to disburse a greater share of unsecured loan value to women or women-owned MSMEs? How does the share of total unsecured credit disbursed to women compare to their share of total loan applicants or potential borrowers, and what insights does this provide about credit allocation and approval processes?</t>
+          <t>Are there gender disparities in the principal disbursed of unsecured loans? Variations in this indicator may be explored across customer type, gender, age, income, location, FSP type, loan type, size, and term. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="L72" t="inlineStr">
@@ -4101,7 +4105,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>Are there differences in the number of active deposit accounts held by individuals across gender, age, and income groups, including the incidence of multiple accounts per person? Do certain gender groups tend to hold more active deposit accounts in specific types of financial institutions or regions? Do FSPs with more gender-diverse teams or customer bases show higher account use rates among underserved gender and age segments?</t>
+          <t>Are there gender disparities in the balances held in active deposit accounts? Variations in this indicator may be explored across customer gender, age, income, location, customer type, pruduct type and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside active deposit accounts (number) to explore whether disparities in balances are proportional to gaps in account ownership.</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -4152,7 +4156,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>Are there differences in the number of active deposit accounts held by individuals across gender, age, and income groups, including the incidence of multiple accounts per person? Do certain gender groups tend to hold more active deposit accounts in specific types of financial institutions or regions? Do FSPs with more gender-diverse teams or customer bases show higher account use rates among underserved gender and age segments?</t>
+          <t>Are there gender disparities in the number of active deposit accounts? Variations in this indicator may be explored across customer type, gender, age, income, location, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside deposit accounts (number) to explore whether socio-demographic gaps in total deposit account ownership translate into similar gaps in active usage.</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -4203,7 +4207,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>Are there differences across gender, age, and income groups in the number of active e-money accounts held, including the prevalence of multiple accounts per person? Do certain types of providers or platforms have higher rates of active accounts of this type from specific gender or age groups? Among MSMEs, does the number of active e-money accounts vary depending on the gender and age of the business owner, and are there differences in account use by region or sector? Are FSPs or non-bank e-money providers with more gender-diverse staff or leadership more likely to have higher activity rates among underrepresented groups?</t>
+          <t>Are there gender disparities in the number of active e-money accounts? Variations in this indicator may be explored across customer type, gender, age, income, location, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="L75" t="inlineStr">
@@ -4248,7 +4252,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>Are there differences across gender, age, and income groups in the number of active mobile-money accounts held, including the prevalence of multiple accounts per person? Do certain types of providers or platforms have higher rates of active accounts of this type from specific gender or age groups? Among MSMEs, does the number of active mobile-money accounts vary depending on the gender and age of the business owner, and are there differences in account use by region or sector? Are FSPs or non-bank e-money providers with more gender-diverse staff or leadership more likely to have higher activity rates among underrepresented groups?</t>
+          <t>Are there gender disparities in the number of active mobile money accounts? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, account type and average balance. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside mobile money accounts (number) to explore whether socio-demographic disparities in total mobile money account ownership are wider or narrower than gaps in active usage.</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -4298,7 +4302,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>Are there differences across gender, age, and income groups in the number of active payment accounts held, including the prevalence of multiple accounts per person? Do certain types of providers or platforms have higher rates of active accounts of this type from specific gender or age groups? Among MSMEs, does the number of active payment accounts vary depending on the gender and age of the business owner, and are there differences in account use by region or sector? Are FSPs or non-bank e-money providers with more gender-diverse staff or leadership more likely to have higher activity rates among underrepresented groups?</t>
+          <t>Are there gender disparities in the number of active payment accounts? Variations in this indicator may be explored across customer type, gender, age, income, location, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="L77" t="inlineStr">
@@ -4343,7 +4347,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>Are there gender disparities in average balances held in current accounts, and how do these differ by age group, income level, region, or provider type? Do individuals of different genders and age groups—particularly those who are younger, older, or low-income—tend to maintain lower balances, and how might this relate to income patterns, employment status, or usage behavior? Among MSMEs, do average current account balances differ by both the gender and age of the business owner, and what might this indicate about financial resilience, cash flow, or access to complementary financial services? Is there any relationship between the gender diversity of FSP staff or leadership and the balance levels maintained by different gender and age groups?</t>
+          <t>Are there gender disparities in average balances held in current accounts, and how do these vary by age, income, location, and FSP type? Variations in this indicator may be explored across customer gender, age, income, location, customer type, and FSP type. . Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -4393,7 +4397,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>Are there gender-based disparities in the average balances held in deposit accounts by individuals or MSMEs, and how do these vary by age group, income level, location, or provider type? Do certain groups—such as low-income women, youth, or older adults—tend to maintain lower balances, and what factors (e.g., income, financial behavior, limited access to credit) might explain this? Among MSMEs, are deposit account balances different based on the gender and age of the business owner, possibly reflecting liquidity constraints or unequal access to finance? Is there a relationship between the gender composition of FSP leadership or frontline staff and the balance levels maintained by different gender and age groups?</t>
+          <t>Are there gender disparities in average balances held in deposit accounts? Variations in this indicator may be explored across customer type, gender, age, income, location, FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -4443,8 +4447,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>Are there gender-based differences in the average balances maintained in e-money accounts, and how do these differences vary by age, income level, location, and provider type? Do women, youth, or lower-income individuals tend to hold lower balances, and how might this relate to differences in income flow, trust, or usage patterns? Among MSMEs, do average e-money account balances differ by the gender and age of the owner, and what does this suggest about digital financial inclusion for small businesses?
-Is there a link between gender diversity within e-money providers and the ability of different groups to maintain meaningful balances in their accounts?</t>
+          <t>Are there gender disparities in average balances held in e-money accounts? Variations in this indicator may be explored across customer type, gender, age, income, location, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="L80" t="inlineStr">
@@ -4489,8 +4492,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the average balances maintained in mobile money accounts, and how do these vary across age groups, income levels, geographic locations, and provider types? Do individuals of different genders and ages—particularly those who are low-income or live in rural areas—tend to maintain lower balances, and how might this relate to income patterns, transaction habits, or access to cash-out points? Among MSMEs, are mobile money account balances different depending on the gender and age of the business owner, possibly reflecting differences in business liquidity or customer bases?
-Is there a correlation between gender diversity in provider operations or agent networks and higher balance levels among underrepresented user groups?</t>
+          <t>Are there gender disparities in average balances held in e-money or mobile money accounts? Variations in this indicator may be explored across customer type, gender, age, income, location, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="L81" t="inlineStr">
@@ -4535,7 +4537,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>Are there gender disparities in average balances maintained in  payment accounts, and how do these differ across income levels, age groups, provider types, and geographic areas? Do lower-income individuals, younger adults, or women and other underrepresented gender groups tend to keep smaller balances in these accounts, and how might this relate to transaction frequency, income stability, or trust in digital services? Among MSMEs, do balances differ by the gender and age of the owner, possibly indicating variations in usage for business versus personal purposes? Does gender diversity within provider institutions correlate with more balanced usage and value retention in these account types across different demographic groups?</t>
+          <t>Are there gender disparities in average balances held in payment accounts? Variations in this indicator may be explored across customer type, gender, age, income, location, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="L82" t="inlineStr">
@@ -4581,8 +4583,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>Are there gender-based disparities in the average balances held in savings accounts, and how do these vary by age, income, location, and provider type? Do lower-income women, youth, or rural populations tend to maintain smaller balances, and what factors (such as income volatility, trust, or financial literacy) might explain these differences? Among MSMEs, do average savings account balances differ depending on the gender and age of the business owner, potentially reflecting varying access to capital or savings priorities?
-Is there a relationship between gender diversity in FSP leadership or frontline staff and the balance levels maintained by different gender and demographic groups?</t>
+          <t>Are there gender disparities in average balances held in savings accounts? Variations in this indicator may be explored across customer type, gender, age, income, location, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -4632,7 +4633,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>Are there gender disparities in average balances held in term deposit accounts, and how do these vary by age, income, location, and provider type? Do women and youth tend to hold smaller term deposit balances, and what might this indicate about savings behavior, risk preferences, or access to formal savings instruments? Among MSMEs, do term deposit balances differ depending on the gender and age of the owner? Is there a correlation between gender diversity in financial institutions and more equitable term deposit balances across demographic groups?</t>
+          <t>Are there gender disparities in average term deposit balances? Variations in this indicator may be explored across customer gender, age, income, location, customer type, product type and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -4692,7 +4693,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the likelihood of holding dormant accounts, including for MSMEs based on the gender of the owner? How does this indicator compare with other indicators of account inactivity and activity levels? Are FSPs with higher levels of gender diversity less likely to have high numbers of dormant accounts? How does dormancy correlate with mobile financial application adoption and access to payment infrastructure? Are customers who hold dormant accounts more likely to be low-income or G2P recipients? Are they at particular risk of being charged fees for dormant accounts? Are dormant accounts concentrated in specific FSP types or geographic regions?  Are there gender disparities in the likelihood of abandoning specific types of transaction accounts and cards (debit and credit)? Which FSPs rank highest and lowest in inactivity ratios, and does this ranking change when analyzed by gender?</t>
+          <t>Are there gender disparities in the likelihood of holding dormant or inactive accounts? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, and account type. This indicator can be analyzed alongside inactive and dormant accounts (balance) and revenue from inactive/dormant accounts. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -4752,7 +4753,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>Are there gender disparities in average investment account balances, and how do these vary across age, income, geographic location, and provider type? Do women and youth tend to hold smaller investment portfolios, and what factors might explain this difference? Among MSMEs, do investment balances differ based on the gender of ownership, reflecting differing investment goals or access? Is there a correlation between gender diversity within investment firms and more equitable investment balances across demographic groups?</t>
+          <t>Are there gender disparities in the number or value of investment accounts held? Variations in this indicator may be explored across customer type, gender, age, income, location, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -4812,7 +4813,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the use of transaction accounts for making or receiving digital payments?</t>
+          <t>Are there gender disparities in the adoption or registration of digital payment or banking channels? Variations in this indicator may be explored across customer type, gender, age, income, location, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
@@ -4867,7 +4868,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the active usage of the instant payment system (IPS), including for MSMEs based on the gender of the owner? Are FSPs with higher levels of gender diversity more likely to have a greater proportion of clients actively using the IPS? How does IPS usage correlate with the indicator on mobile financial application adoption? Are lower levels of IPS usage concentrated in specific FSP types, geographic regions, or account balance segments?</t>
+          <t>Are there gender disparities in the active usage intensity of the instant payment system (IPS)? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, and account type. This indicator can be analyzed alongside access to the instant/fast payment system. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -4922,7 +4923,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>Are there gender disparities in MSMEs' access to POS, depending on the owner's gender?</t>
+          <t>Are there gender disparities in the adoption of POS for in-store or online purchases? Variations in this indicator may be explored across MSME types, size, age, income, location, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -4977,7 +4978,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>Are there gender disparities in voluntary deposits into pension accounts? Are voluntary deposits geographically concentrated, and do these patterns vary by gender? Which types of pension administrators attract higher volumes of voluntary deposits, and do these trends differ by gender? Do FSPs with higher levels of gender diversity attract more voluntary deposits, and within these, are there gender disparities in the distribution of depositors?</t>
+          <t>Are there gender disparities in voluntary pension contributions? Variations in this indicator may be explored across customer gender, age, income, location, FSP type, and pension type. Do FSPs with higher gender diversity show higher voluntary contribution rates among women?</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -5027,7 +5028,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>Are there gender-related differences in the likelihood of pledging collateral when accessing credit? And by age and/or location nd/or income? Do borrowers of different genders tend to pledge different types of collateral (e.g., movable vs. immovable)? Are certain FSP types or loan products more likely to require collateral and are there differences acros gender groups? THis variable cna be analized along with indicators for credit access to see if the requirement or use of collateral influences credit access across genders.</t>
+          <t>Are there gender disparities in the requirement to pledge collateral? Variations in this indicator may be explored across customer type, gender, age, income, location, FSP type, product type, and collateral type. This indicator can be analyzed alongside the indicator on borrowers whose collateral was seized. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -5087,7 +5088,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the use of cooling-off periods for loans across gender and age? Are FSPs with higher levels of gender diversity more likely to apply or communicate the cooling-off period consistently across all clients? Does the presence of a cooling-off period reduce over-indebtedness more significantly among women?</t>
+          <t>Are there gender disparities in the use of cooling-off periods for loans. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Variations in this indicator may be explored across customer gender, age, income, location, FSP type, credit type, loan size, and loan term. Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside grace period/payment leeway to explore whether FSPs offering cooling-off periods on loans are also more likely to offer grace periods on repayment, and whether these two consumer-protective features are correlated with FSP gender diversity.</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -5147,7 +5148,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>What are the gender patterns in remittance costs for sending and receiving transactions? Comparing with the location of most recipients, are costs higher in lower-income areas? Do average costs vary based on the channels mostly available to low-income customers and locations? Is there any correlation between average remittance costs for a given provider and its gender diversity?</t>
+          <t>Are there gender disparities in the cost of sending or receiving remittances across provider types and corridors? Variations in this indicator may be explored across customer gender, age, income, location, FSP type, channel type, and transaction type. Are costs higher in areas or channels predominantly used by low-income customers or women? Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside speed of remittances to explore whether costlier remittance channels are also slower, and whether the channels most used by certain customer groups are doubly disadvantaged.</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -5207,7 +5208,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the likelihood of being affected by remittances that take longer to process? Do smaller remittances take longer? What types of FSPs and remittance channels have longer processing times? Are low-income communities particularly affected? Are slower remittances also the most expensive? Is there any correlation between this indicator and FSP gender diversity?</t>
+          <t>Are there gender disparities in the likelihood of experiencing slow remittance processing, and do slower remittances tend to be more expensive? Variations in this indicator may be explored across customer gender, age, income, location, FSP type, channel type, and transaction type. Are low-income communities and women particularly affected by longer processing times? Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -5267,7 +5268,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>Are there gender disparities in net pension replacement rates among retirees, and how do these differences vary across income levels or pension types (micro, mandatory, publice, etc )? Is there a correlation between gender diversity in pension system participation and overall replacement rate outcomes? Do individuals of different genders tend to have different contribution histories or retirement ages that affect their net replacement rates? How do life expectancy differences by gender interact with replacement rates to influence income security in old age</t>
+          <t>Are there gender disparities in the net pension replacement rate? Variations in this indicator may be explored across customer gender, age, income, location, FSP type, and pension type. Do FSPs or employers with higher gender diversity show higher or more equitable replacement rates among women? This indicator can be analyzed alongside pension contributors to explore whether customer groups with lower or shorter contribution histories also show lower replacement rates.</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -5327,7 +5328,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>How has participation in pension entitlements in pension funds evolved over time by gender, both for individuals and MSMEs considering the gender of the owner? Are there gender disparities in pension accumulation levels?</t>
+          <t>Are there gender disparities in pension entitlements? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, and product type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside pension contributors and pension beneficiaries to explore whether disparities in entitlements reflect differences in contribution history, participation rates, or benefit design.</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -5377,7 +5378,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>Are there gender disparities in average pension income?</t>
+          <t>Are there gender disparities in retirement income per pension beneficiary? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, and pension type. Do FSPs with higher gender diversity show more equitable retirement income outcomes across genders? This indicator can be analyzed alongside net pension replacement rate to explore whether socio-demographic gaps in absolute retirement income are proportional to gaps in the replacement rate.</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
@@ -5435,7 +5436,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>Are the portions of female account holders different for these accounts than for other account types offered by this provider?</t>
+          <t>Are there gender disparities in access to low-cost accounts or products? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, product type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside average cost-to-customer for transaction accounts to explore whether customer groups with lower access to FSPs offering low-cost products face higher effective transaction account costs.</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -5496,7 +5497,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>Are the portions of female account holders different for these accounts than for other account types offered by this provider?</t>
+          <t>Are there gender disparities in ownership of zero minimum balance accounts? Variations in this indicator may be explored across customer gender, age, income, location, customer type, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside deposit accounts (balance) to explore whether customer groups with lower access to zero minimum balance products also show lower average deposit balances, suggesting that minimum balance requirements may be an active barrier.</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -5558,7 +5559,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>How does the gender composition of the customer base of the FSPs correlate with the level of access to free accounts?, Are FSPs with higher levels of gender diversity more likely to offer free accounts?”</t>
+          <t>Are there gender disparities in onwership of free accounts? Variations in this indicator may be explored across customer type, gender, age, income, location, FSP type, account average balance. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside account opening costs to explore whether customer groups with lower access to FSPs offering free accounts face higher average account opening costs.</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -5618,7 +5619,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the total cost of opening retail accounts, considering all fees and charges? Do individuals of different genders tend to access providers or account types with higher upfront costs, and how does this affect account uptake? Are there geographic or income-based patterns that intersect with gender, leading to unequal cost burdens when entering the formal financial system? How does the structure of account opening fees influence financial access for different gender groups, particularly in low-income or rural segments?</t>
+          <t>Are there gender disparities in total account opening costs? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, and account type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -5678,7 +5679,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>How does the gender composition of the customer base of the FSPs correlate with the level of access to complaints channels?</t>
+          <t>Are there gender disparities in the availability of complaints channels? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, and complaints filing channel. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside access to free complaints channels to explore whether socio-economic disparities in complaints channel availability are compounded by disparities in the cost of those channels.</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -5738,7 +5739,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>Are free complaints channels equally available to women, particularly those from low-income or rural populations? Do women disproportionately rely on complaints channels that incur costs (e.g., phone calls requiring airtime)? Are FSPs with higher levels of gender diversity more likely to provide free complaints channels across all modalities?</t>
+          <t>Are free complaints channels equally available across customer genders? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, and complaints filing channel. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -5798,7 +5799,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>Are there gender disparities in savings discipline, particularly in whether term deposits are retained until maturity or withdrawn early? Is there evidence that term deposit savings serve as coping mechanisms differently by gender? How do term deposit savings behaviors differ among more vulnerable or underserved individuals by gender?</t>
+          <t>Are there gender disparities in the likelihood of extracting term deposit savings before maturity? Variations in this indicator may be explored across customer gender, age, income, location, customer type, product type and FSP type. This indicator can be analyzed alongside the resumption of savings after early extraction from term deposits. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -5858,7 +5859,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the likelihood of resuming term deposit savings after withdrawing them before maturity? What are the characteristics of individuals who resume term deposit savings by gender? Which FSPs rank highest and lowest in the resumption of term deposit savings, and does this ranking change when analyzed by gender?</t>
+          <t>Are there gender disparities in the likelihood of resuming term deposit savings after an early withdrawal? Variations in this indicator may be explored across customer gender, age, income, location, customer type, product type and FSP type. This indicator can be analyzed alongside the early extraction of term deposits indicator. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -5918,7 +5919,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>How common is it for individuals holding transaction accounts to also maintain interest-bearing term deposit accounts? Are there gender disparities in the multiple ownership and distribution of these different account types across age groups and location types, both at the total market level and by relevant FSP/type? How prevalent is the cross-sell of term deposit accounts among vulnerable customer segments, and are there gender disparities within these segments? How do average balances differ between transaction and term deposit accounts across gender, age groups, and location types, both at the total market level and by relevant FSP/type? Are there gender disparities in average balances across these account types? How do average balances vary among vulnerable customer segments, and are there gender disparities within these segments? What are the gender disparities in cross-selling and average balances of transaction accounts and term deposit accounts across age groups and location types, both at the total market level and by relevant FSP/type?</t>
+          <t>Are there gender disparities in the proportion of account holders who also maintain term deposits (cross-selling)? Variations in this indicator may be explored across customer gender, age, income, location, customer type, product type, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside tenure of deposit and payment accounts to explore whether customers with longer account tenure are more likely to also hold term deposits, and whether disparities in tenure explain disparities in term deposit cross-selling.</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -5978,7 +5979,7 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>Are there sociodemographic (gender, age, location, income) disparities in borrowers' cross-sell ratios of deposit accounts and in the likelihood of being a stand-alone borrower? Have gender disparities in cross-sell ratios changed over time, particularly for underserved borrowers?</t>
+          <t>Are there gender disparities in the likelihood of unsecured borrowers also holding a deposit account? Variations in this indicator may be explored across customer gender, age, income, location, customer type, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside savings to borrowings ratio to explore whether customer groups more likely to be stand-alone borrowers without deposit accounts are also those with lower savings-to-borrowings coverage ratios.</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -6038,7 +6039,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>Are there disparities in borrowers' cross-sell ratios of deposit accounts by gender, and/or age, location or income?? And in the likelihood of being a stand-alone borrower? Have gender disparities in cross-sell ratios changed over time, particularly for underserved borrowers?</t>
+          <t>Are there gender disparities in the ratio of savings to borrowings (likelihood of being a stand-alone borrower without savings coverage)? Variations in this indicator may be explored across customer type, gender, age, income, location, and FSP type. This indicator can be analyzed alongside the depositors-borrowers ratio. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -6099,7 +6100,7 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>Do first-time borrowers reflect a balanced gender representation, or are there gender disparities? How do FSPs rank in onboarding typically underserved borrowers, and does this ranking change when analyzed by gender?</t>
+          <t>Do first-time borrowers reflect a balanced gender representation? Variations in this indicator may be explored across customer gender, age, income, location, customer type, product type, and FSP type. How do FSPs rank in onboarding first-time borrowers from typically underserved groups? Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside new borrowers to explore whether socio-economic disparities in first-time borrowers differ from disparities in all new borrowers.</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -6149,7 +6150,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>What are the gender disparities in the average frequency of different types of cash transactions, such as withdrawals and deposits, performed across various cash-enabled channels (e.g., branches, ATMs, agents, retail stores)? Do different gender groups, when disaggregated by account type, age, income, and location, show distinct preferences in their use of cash channels? Are certain customer segments more reliant on cash due to limited access to digital alternatives? How have gender-related patterns in the use of cash evolved over time, and are these shifts consistent across regions or types of financial service providers?</t>
+          <t>Are there gender disparities in the frequency of cash transactions across different channels and account types? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, transaction type and average size. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside cashless transactions (volume) to explore whether customer groups with higher cash transaction volumes show lower cashless adoption, and how this trade-off evolves over time and across regions.</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -6199,7 +6200,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>How do active closure rates compare by gender? Which types of accounts are most frequently closed by each gender? How do FSPs rank in active account closures, and does this ranking change when analyzed by gender?</t>
+          <t>Are there gender disparities in active account closure rates? Variations in this indicator may be explored across customer gender, age, income, location, customer type, product type and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside account closure costs paid by customers to explore whether higher closure fees are associated with lower active closure rates for certain customer groups, potentially trapping customers in unsuitable accounts.</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -6623,7 +6624,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>How do claim numbers vary by gender? Are there any gender groups logging fewer claims compared to the market average? Are there FSPs with particularly low or high claim numbers for certain genders? How do claim statistics intersect with policy type and customer demographics?</t>
+          <t>Are there gender disparities in the number of claims? Variations in this indicator may be explored across customer type, gender, age, income, location, FSP type, type of insurance, and average premium. Do insurers with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do insurers with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside insurance claims paid to explore whether customer groups filing more claims also receive payment on a proportionally similar share.</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -6683,7 +6684,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>How do claim payments vary by gender? Are there any gender groups receiving fewer/lower payments compared to the market average? Are there FSPs with particularly low or high payment rate for certain genders? How do claim payment statistics intersect with policy type and customer demographics?</t>
+          <t>Are there gender disparities in the value of claims paid? Variations in this indicator may be explored across customer type, gender, age, income, location, FSP type, type of insurance, and average premium. Do insurers with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -6743,7 +6744,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>Are there gender differences in the proportion of fraud-related complaints submitted to providers, regulators, or ombuds services?  Do individuals of different genders tend to report different types of fraud, such as identity theft, phishing, or agent misconduct, and are specific delivery channels more commonly associated with these complaints? Is the volume of fraud-related complaints disproportionately high among certain gender groups when compared to their levels of account ownership or usage? Do complaint resolution rates and timeframes differ by gender across various FSP or reporting channels?</t>
+          <t>Are there gender disparities in the proportion of fraud-related complaints? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, complaints resolution outcome and complaints resolution time (turnaround time). Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside frauds faced by customers to explore whether customer groups submitting more fraud-related complaints are also those with higher rates of actual fraud exposure.</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -6803,7 +6804,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>How does the share of customers whose collateral was seized due to default vary by gender and other key sociodemographic of the customer or MSME owner? Are women/WMSME more or less likely than men to have their collateral seized following loan default? How does the share differ by gender across different loan sizes, loan products,  types of financial service providers (FSP), collateral type (e.g., movable, immovable, alternative)? And how do any of these differences relate to seizure rates? Are women more likely to be subject to stricter collateral requirements or less flexible repayment terms that increase the likelihood of asset seizure?</t>
+          <t>Are there gender disparities in collateral seizure rates? Variations in this indicator may be explored across customer gender, customer type, FSP type, credit type, loan size, loan term, and collateral type. This indicator can be analyzed alongside information about collateral requirements and repayment terms across customer segments, to explore whether higher likelihood of asset seizure is correlated with product terms and conditions. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -6863,7 +6864,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>How does the number of complaints at each processing stage vary by gender? Are complaints disproportionately concentrated at certain processing stages for any gender? How do FSPs compare to market averages in the number of complaints at each processing stage?"</t>
+          <t>Are there gender disparities in the number of complaints? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, complaints issue category, complaints filing channel, and complaints resolution status. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside customer complaints resolved in the customer's favor to explore whether FSPs receiving more complaints per customer also resolve a higher or lower share in the customer's favor, and whether any customer group both complains more and achieves less favorable outcomes.</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -6923,7 +6924,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>How do the percentages of complaints resolved in favor of customers vary by gender? Are any genders more likely to receive favorable resolutions? How do FSPs rank in terms of favorable resolutions by gender?</t>
+          <t>Are there gender disparities in the rate of complaints resolved in favor of customers? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, product type, complaints issue category. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -6983,7 +6984,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>How do consent rates for customer contact vary by gender? Are any genders more likely to provide consent to be contacted? How do FSPs rank in terms of consent rates by gender?</t>
+          <t>Are there gender disparities in consent rates for FSP contact for marketing or awareness purposes? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside consents for sharing data with third parties to explore whether customer groups more willing to be contacted by FSPs are also more willing to share data with third parties, or whether these represent distinct privacy preferences.</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
@@ -7046,7 +7047,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the APR applied to loans disbursed to women and men, including MSMEs by gender of ownership? Do women borrowers systematically face higher average APRs than men within the same loan type, amount range, or provider category? Are higher APRs for women associated with smaller loan sizes, shorter maturities, or higher perceived credit risk? Do FSPs with greater gender diversity or stronger inclusion policies show smaller gender gaps in average APRs? How do APR differences relate to borrower profiles and do they suggest the presence of gender-based pricing bias or structural credit segmentation?</t>
+          <t>Are there gender disparities in the APR applied to loans disbursed? Variations in this indicator may be explored across customer gender, customer type, age, income, location, FSP type, credit type, and loan size and term. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside processing and application fees (PAF) to explore whether customer groups facing higher APRs also pay higher upfront fees, pointing to a compounding cost disadvantage across the full borrowing lifecycle.</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -7106,7 +7107,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>How do consent rates for data sharing with third parties vary by gender? Are any genders more likely to provide consent for data sharing? How do FSPs rank in terms of consent rates for data sharing by gender?</t>
+          <t>Are there gender disparities in rates of consent for sharing data with third parties? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, and purpose of data sharing (e. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?g., credit scoring, marketing, open banking).</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -7166,7 +7167,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>What percentages of net interest income are attributable to penalties and other punitive charges earned from borrowers of unsecured loans/lines of credit, and how do these vary by gender across age bands and location types, at a total market level and by relevant FSP/type? How do these percentages compare across relevant FSPs/types and against market norms across age bands and location types? How do gender disparities manifest in these percentages at a total market level and by relevant FSP/type?</t>
+          <t>Are there gender disparities in the share of net interest income attributable to penalty charges? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, credit type, loan size and term. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside grace period/payment leeway to explore whether customer groups that make more use of grace periods subsequently incur fewer penalty charges, or whether grace periods simply delay rather than prevent fees.</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -7228,7 +7229,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>What are the origination fee percentages as a share of loan principal by gender? Are there gender disparities in the origination fee percentages incurred? How do FSPs rank in terms of origination fee percentages by gender?</t>
+          <t>Are there gender disparities in the origination fee percentages incurred as a share of loan principal? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, product type, and loan size and term. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside annual percentage rate (APR) for retail credit to explore whether customer groups facing higher upfront fees also pay higher overall borrowing costs.</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -7288,7 +7289,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>How does the percentage of customers affected by data breaches vary by gender? Are any genders disproportionately affected by data breaches? Are data breaches more frequent in certain types of FSPs? Are data breaches more common in specific channels or interfaces?"</t>
+          <t>Are there gender disparities in the share of customers affected by data breaches? Variations in this indicator may be explored across customer gender, age, income, location, customer type, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside consents for sharing data with third parties to explore whether FSPs where more customers have shared data with third parties also show higher rates of data breaches, and whether any customer group is disproportionately exposed.</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -7348,7 +7349,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the number of deposit accounts covered by direct deposit insurance? How do these disparities vary by age, income level, and geographic location? Are certain gender groups, especially within vulnerable or low-income populations, less likely to hold insured deposit accounts? How do the average insured deposit account balances differ across genders, and what might this indicate about savings behavior, access to financial protection, or economic security? Do financial service providers with higher levels of gender diversity in leadership or staff tend to offer more equitable access to insured deposit accounts and balanced coverage across genders? Additionally, how do gender differences in insured deposit accounts relate to broader financial inclusion and resilience against financial shocks?</t>
+          <t>Are there gender disparities in the share of deposit accounts covered by direct deposit insurance? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, and product type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside G2P accounts covered by deposit insurance to explore whether disparities in deposit insurance coverage are especially pronounced among G2P recipients, who are often predominantly women.</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -7412,7 +7413,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the number of G2P accounts covered by deposit insurance? How do these disparities vary across different age groups, income levels, and geographic locations? Are women and other gender groups within vulnerable populations less likely to have G2P accounts that are insured, potentially affecting their financial security? How do the average balances of insured G2P accounts compare across genders, and what does this imply about economic empowerment and financial resilience? Do government programs and financial service providers with greater gender diversity in design or delivery show more equitable insurance coverage of G2P accounts? Additionally, how do gender differences in insured G2P accounts influence overall inclusion and access to social safety nets?</t>
+          <t>Are there gender disparities in the share of G2P recipient accounts covered by deposit insurance, given that women are often the primary recipients of G2P transfers? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, product type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -7473,7 +7474,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the percentage of topline revenue relative to outstanding loan balances? Is there any gender paying comparatively more than market percentages for the same account types? How do FSPs rank in terms of these percentages by gender?</t>
+          <t>Are there gender disparities in the effective cost of unsecured lending? Variations in this indicator may be explored across customer gender, age, income, location, FSP type, and credit type, size and term. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside interest rate spreads (loans) to explore whether disparities in effective borrowing costs reflect broader pricing differences at the FSP level or differences in the specific products accessed by each customer group.</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
@@ -7530,7 +7531,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>What proportion of total topline revenue comes from unsecured credit operations, and are there gender disparities in this distribution? How do FSPs rank in their reliance on unsecured credit revenue by gender?</t>
+          <t>Are there gender disparities in the distribution of revenue from unsecured credit operations? Variations in this indicator may be explored across customer gender, customer type, age, income, location, FSP type, and loan type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside average cost-to-borrower for unsecured retail lending to explore whether FSPs generating a higher share of revenue from unsecured credit also charge higher effective costs to borrowers.</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -7590,7 +7591,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>How do the average values of outstanding insurance claims compare by gender? Is there a gender group with consistently higher average unpaid claims? How do different FSPs rank in terms of outstanding claims by gender? Are vulnerable gender groups disproportionately affected by delayed or unpaid claims?</t>
+          <t>Are there gender disparities in the average value of outstanding approved but unpaid insurance claims? Variations in this indicator may be explored across customer gender, age, income, location, customer type, insurer type, type of insurance, and average premium. Do insurers with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside insurance claims settlement ratio to explore whether customer groups with higher outstanding approved-but-unpaid claims also show lower overall settlement ratios, indicating systemic delays rather than isolated cases.</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -7651,7 +7652,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>What percentage of claims logged by policyholders are declined, disaggregated by gender? How do these decline rates vary across FSPs, policy types, age groups, and locations? Are there notable gender disparities in claim declines at the market level or within specific providers? Are women or other gender groups more likely to face claim denial?</t>
+          <t>Are there gender disparities in the share of insurance claims declined at intake? Variations in this indicator may be explored across customer gender, age, income, location, customer type, insurer type, type of insurance, and average premium. Do insurers with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do insurers with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -7713,7 +7714,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the rejection rates of insurance claims, including for MSMEs by owner gender? Which types of policies or claims see higher rejection rates, and do these differ by gender? How does claim rejection relate to coverage levels and turnaround times? Do FSPs with higher gender diversity have lower rejection rates for vulnerable gender groups?</t>
+          <t>Are there gender disparities in insurance claims rejection rates? Variations in this indicator may be explored across customer type, gender, age, income, location, FSP type, type of insurance, average premium. Do insurers with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside insurance claims declined to explore whether socio-demographic disparities in front-door declines are compounded by higher rejection rates after substantive review.</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -7773,7 +7774,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>How do claim settlement ratios vary by gender? Are any gender groups receiving lower settlement ratios compared to the market average? Are there FSPs with particularly low or high settlement ratios for certain genders? How do these ratios intersect with policy type and customer demographics?</t>
+          <t>Are there gender disparities in insurance claims settlement ratios, with any gender receiving systematically lower settlement rates? Variations in this indicator may be explored across customer gender, age, income, location, customer type, insurer type, type of insurance, and average premium. Do insurers with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do insurers with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -7835,7 +7836,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the average time taken to process and settle insurance claims? How does processing time vary by policy type, premium, claim amount, and customer demographics? Are insurers with lower gender diversity more likely to have longer turnaround times? Are vulnerable gender groups disproportionately affected by delays?</t>
+          <t>Are there gender disparities in insurance claims turnaround times? Variations in this indicator may be explored across customer type, gender, age, income, location, FSP type, type of insurance, and average premium. Do insurers with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside insurance approved claims not paid to explore whether insurers with longer turnaround times also accumulate higher stocks of approved-but-unpaid claims.</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
@@ -7891,7 +7892,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>How do net returns (% returns minus % performance fees and charges) on longer-term investments compare by gender? Do net returns for any gender differ from the overall market average for similar investment products? How do FSPs compare in terms of net returns earned by gender?</t>
+          <t>Are there gender disparities in net returns (percentage returns minus fees and charges) on longer-term investments for different customer groups? Variations in this indicator may be explored across FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? This indicator can be analyzed alongside unpaid matured long-term investments to explore whether socio-demographic disparities in net returns are compounded by disparities in the timely payment of matured investments.</t>
         </is>
       </c>
       <c r="J140" t="inlineStr">
@@ -7947,7 +7948,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the costs (fees, charges) borne by account holders of transaction accounts? Do women tend to hold transaction accounts with higher fee burdens (relative to income or transaction frequency) than men, particularly in certain regions or among lower‐income groups? How do costs compare across FSPs with different levels of gender diversity? Is fee structure or cost‐to‐customer a barrier to transaction usage for some gender/age/income cohorts?</t>
+          <t>Are there gender disparities in the cost of holding and using transaction accounts? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, and product type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside average cost-to-borrower for unsecured retail lending to explore whether customer groups that face higher transaction account costs also face higher credit costs, suggesting a compounding pricing disadvantage.</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
@@ -8002,7 +8003,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>How do rejection rates vary by gender for individuasl and MSME? Are rejection rates higher for any gender in specific channels? How do rejection rates in physical channels compare to those in digital channels by gender? How do FSPs rank in terms of rejection rates by gender across available channels, by type of customer (individuals, MSME)?</t>
+          <t>Are there gender disparities in rejection rates for financial product applications? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, and product type. When analyzed alongside the customers by credit score indicator, is there a correlation between product rejection and credit score? Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside deposit account holders qualifying for credit to explore whether socio-demographic gaps in formal creditworthiness qualification explain a significant share of gaps in loan application rejection rates.</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -8062,7 +8063,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>How does the average number of outstanding loans per borrower vary by gender? Are outstanding balances more concentrated in long- or short-term loans, and does this differ by gender? Have gender disparities in loan terms evolved over time?</t>
+          <t>Are there gender disparities in the average number and value of outstanding unsecured credit facilities per borrower? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, product type, loan term and average size. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside borrowers with multiple outstanding loans to explore whether customer groups with higher average credit facilities per borrower are also more likely to hold loans across multiple FSPs.</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -8122,7 +8123,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>How does the number of fraud cases vary by gender? Are any genders disproportionately affected by fraud? Are fraud cases more frequent in certain types of FSPs?</t>
+          <t>Are there gender disparities in the prevalence or financial impact of fraud? Variations in this indicator may be explored across customer gender, age, income, location, customer type, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside frauds resulting in customer losses to explore whether customer groups exposed to more fraud incidents also suffer higher financial losses per incident.</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -8182,7 +8183,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>How do financial loss-related fraud cases impact genders differently? Are any genders disproportionately affected by frauds that result in financial losses? Are fraud cases involving financial losses more common in certain types of FSPs?</t>
+          <t>Are there gender disparities in the prevalence or financial impact of fraud? Variations in this indicator may be explored across customer gender, age, income, location, customer type, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -8243,7 +8244,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>How does the number of physical security incidents vary by gender? Are any genders disproportionately affected? Are physical security incidents more common in certain types of FSPs?</t>
+          <t>Are there gender disparities in the number of physical security incidents affecting customers? Variations in this indicator may be explored across customer gender, age, income, location, customer type, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside physical access points to explore whether socio-demographic disparities in physical safety incidents are concentrated in areas or access point types with lower infrastructure quality or fewer alternative channels.</t>
         </is>
       </c>
       <c r="J146" t="inlineStr">
@@ -8298,7 +8299,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>What are the credit-qualifying rates for transaction account holders by gender? How do these rates compare? Which FSPs rank highest and lowest in credit-qualifying rates for typically underserved groups, and does this ranking change when analyzed by gender?</t>
+          <t>Are there gender disparities in credit qualification rates among deposit account holders? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, and credit type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside loan applications and rejections of product applications to explore whether disparities in credit qualification translate directly into gaps in application rates and approval outcomes.</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -8358,7 +8359,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the likelihood of making early payments before due dates? Which credit products are most frequently paid early by each gender?</t>
+          <t>Are there gender disparities in the likelihood of making early loan repayments? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, credit type, loan size and term. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside annual percentage rate (APR) for retail credit to explore whether customer groups facing higher APRs are more motivated to repay early, or whether higher costs instead reduce their capacity to do so.</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -8418,7 +8419,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>How do the percentages of borrowers using grace periods or payment leeways compare by gender? Is there any gender more likely to use them? How does the use of grace periods or payment leeways vary by credit product and gender?</t>
+          <t>Are there gender disparities in the use of payment grace periods or leeways? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, and credit type, size and term. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside borrowers in debt counselling and rehabilitation to explore whether access to grace periods reduces the likelihood of entering debt counseling, and whether oscio-demographic differences in grace period use correspond to differences in debt distress rates.</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -8479,7 +8480,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>How do the percentages of borrowers in debt counseling or rehabilitation compare by gender? Is there any gender more likely to enroll in debt counseling or rehabilitation? How do FSPs compare in terms of debt counseling or rehabilitation enrollment by gender?</t>
+          <t>Are there gender disparities in enrollment in debt counseling or rehabilitation programs? Variations in this indicator may be explored across customer gender, age, income, location, FSP type, product type, and loan size and term. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside borrowers in risky indebtedness to explore whether customer groups classified as at risk of over-indebtedness are subsequently more likely to enroll in debt counseling or rehabilitation programs.</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
@@ -8539,7 +8540,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the classification of risky indebtedness? Are low-income borrowers more at risk of risky indebtedness and how does it compare across genders? Comparing this indicator with gender diversity, do FSPs with higher levels of gender diversity present lower levels of risky indebtedness?</t>
+          <t>Are there gender disparities in the classification of borrowers as being in risky indebtedness? Variations in this indicator may be explored across customer gender, age, income, location, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside borrowers with multiple outstanding loans to explore whether holding loans across multiple FSPs is the primary driver of risky indebtedness classification, and whether this concentration risk falls disproportionately on a particular cusomter group.</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
@@ -8599,7 +8600,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>How do debt service-to-income ratios vary by gender and across different loan sizes and terms? Do loans with higher rates and shorter terms show gender disparities in ratios? Comparing this indicator with gender diversity, do FSPs with higher levels of gender diversity present lower debt-service to income ratios?</t>
+          <t>Are there gender disparities in debt service-to-income ratios? Variations in this indicator may be explored across customer gender, age, income, location, FSP type, credit type, and loan size and term. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside borrowers in risky indebtedness to explore whether customer groups with higher debt service-to-income ratios are also more frequently classified as being in risky indebtedness, validating the ratio as a predictor of financial distress by group.</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -8659,7 +8660,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>How do insurance lapse rates differ by gender? Are certain types of insurance policies associated with higher lapse rates among specific genders, suggesting potential issues with product suitability? How do different financial service providers (FSPs) compare in terms of lapse rates across genders? Are there notable differences when considering age, location, or income alongside gender?</t>
+          <t>Are there gender disparities in insurance lapse rates? Variations in this indicator may be explored across customer gender, age, income, location, customer type, insurer type, type of insurance, and average premium. Do insurers with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside insurance policy renewal (persistency) ratio to explore whether socio-demographic patterns in lapse rates are the mirror image of patterns in renewal rates, and whether any FSP-level gender diversity effect is consistent across both measures.</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -8719,7 +8720,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>How do rates of reinstating lapsed insurance policies vary by gender? Is any gender more likely to make back payments and reinstate their policies? How do these reinstatement patterns differ across FSPs, policy types, and demographic groups such as age or income? What might these patterns indicate about barriers to maintaining continuous coverage?</t>
+          <t>Are there gender disparities in the rate of reinstating lapsed insurance policies after back-payments? Variations in this indicator may be explored across customer gender, age, income, location, customer type, insurer type, type of insurance, and average premium. Do insurers with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do insurers with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside insurance lapse rates and risk of insurance coverage lapse to explore whether FSPs with higher lapse rates also show higher reinstatement rates, and whether socio-demographic differences in financial resilience predict reinstatement behavior.</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -8779,7 +8780,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>How well does the non-life insurance policy market reflect gender-based differences in policyholding and insured benefits? How do the types of non-life insurance policies held compare by gender? How are gender disparities evolving in the distribution of non-life insurance policies across different FSPs?</t>
+          <t>Are there gender disparities in the share of policies at risk of lapse? Variations in this indicator may be explored across customer gender, age, income, location, customer type, insurer type, type of insurance, and average premium. Do insurers with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do insurers with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside insurance lapse rates to explore whether customer groups with higher shares of policies at risk of lapse also have higher realized lapse rates, or whether interventions during the grace period prevent them from lapsing.</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
@@ -8842,7 +8843,7 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>Are surrender values and payouts equitably distributed by gender among eligible policyholders? Is there any gender that is less likely to receive surrender payouts, and does this vary by policy type or FSP? How do surrender rates differ by gender when combined with other demographics like income or location?</t>
+          <t>Are surrender values and payouts equitably distributed by gender among eligible policyholders? Variations in this indicator may be explored across customer gender, age, income, location, customer type, insurer type, type of insurance, and average premium. Do insurers with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside insurance lapse rates to explore whether customer groups with higher lapse rates are more or less likely to receive surrender values, which has direct implications for the financial losses they incur upon exit.</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -8904,7 +8905,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>Do genders differ in how long they hold their policies? Are there disproportionate gender differences in longer, medium, or shorter tenures? Does any gender show higher loyalty across different insurers/types? At what tenure points do insurance policies tend to be canceled, and do these patterns vary by gender? Is there a gender more likely to cancel policies earlier? How do cancellation patterns differ across policy types, age groups, locations, or income levels? What might early cancellations suggest about policy suitability or customer experience for different genders?</t>
+          <t>At what tenure points do insurance policies tend to be cancelled? Do insurers with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do insurer with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside insurance lapse rates to explore whether policies cancelled at shorter tenures drive the overall lapse rate, and whether early cancellation is disproportionately concentrated among certain customer groups or policy types. Variations in this indicator may be explored across customer gender, age, income, location, customer type, insurer type, and type of insurance.</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -8964,7 +8965,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>Are there gender disparities in policy downgrade rates, including for MSMEs based on owner gender? Which types of policies experience higher downgrade rates, and could this reflect issues like unsuitable product features or unfavorable premium-to-coverage ratios? How might these downgrade rates relate to claims rejection rates and coverage ratios? Could poor claims experiences or misunderstandings about coverage terms contribute to downgrades? Do FSPs with greater gender diversity exhibit lower downgrade rates?</t>
+          <t>Are there gender disparities in the rate at which insurance policies are downgraded? Variations in this indicator may be explored across customer type, gender, age, income, location, FSP type, type of insurance, and average premium. Do insurers with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside insurance lapse rates to explore whether policy downgrades serve as a step before full lapse for vulnerable policyholders, and whether customer groups with higher downgrade rates subsequently show higher lapse rates.</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -9019,7 +9020,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>What percentage of unpaid matured longer-term investments is attributable to each gender? Are unpaid amounts disproportionately concentrated in any gender? How do FSPs rank in terms of unpaid proportions of matured longer-term investments by gender?</t>
+          <t>Are there gender disparities in the share of unpaid matured long-term investments? Variations in this indicator may be explored across customer gender, age, income, location, customer type, product type, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside net rate of return on investments to explore whether FSPs with higher rates of unpaid matured investments also deliver lower net returns to customers, and whether some customer groups are disproportionately exposed to both risks.</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -9079,7 +9080,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>How do transfers of pension fund balances to a different pension fund administrator vary by gender? Does this vary according to the level of FSP gender diversity? What percentage of contributors transferred funds compared to all customers, and are there gender disparities in this proportion? Are certain customer segments, such as women, women-owned MSMEs owners, and low-value accounts, more likely to make high-to-low transfers (switching to a fund administrator that has been paying lower returns)? Are FSPs with higher levels of gender diversity less likely to receive savers coming from an administrator that previously paid higher returns?</t>
+          <t>Are there gender disparities in pension fund switching rates? Variations in this indicator may be explored across customer type, gender, age, income, location, FSP type, and pension type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside net pension replacement rate to explore whether pension fund switching behavior leads to better or worse replacement rate outcomes across customer groups.</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -9139,7 +9140,7 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>Do genders differ in how long they hold their transaction accounts? Are some genders disproportionately represented in longer, medium, or shorter account tenures? Which genders show higher account loyalty across different FSPs/types, and which tend to close accounts sooner?</t>
+          <t>Are there gender disparities in account tenure (loyalty)? Variations in this indicator may be explored across customer gender, age, income, location, customer type, product type and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside depositors who actively close deposit accounts to explore customer groups with shorter average tenure are also more likely to actively close accounts, helping distinguish between voluntary exit and gradual disengagement.</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -9200,7 +9201,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>What proportion of balances held in inactive/dormant/suspense accounts is attributable to each gender? Are these balances disproportionately skewed by gender? Which FSPs have notable skews (higher than market averages) in balances held in inactive/dormant/suspense accounts by gender?</t>
+          <t>Are there gender disparities in the share of total balances held in inactive or dormant accounts? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, and product type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -9260,7 +9261,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>How does the average revenue earned from inactive and dormant accounts compare by gender? Are there gender disparities in the charges applied to these accounts compared to the overall market average? How do relevant FSPs rank in terms of the average revenue earned from these accounts, and does this ranking change when analyzed by gender?</t>
+          <t>Are there gender disparities in the average revenue earned from inactive or dormant accounts which could reflect discrimination via pricing? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, and product type. This indicator can be analyzed alongside the inactive and dormant accounts (number and balance) indicators. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -9320,7 +9321,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>How do take-up rates vary by gender? Do any genders have higher take-up rates than the overall market average? How do FSPs compare in terms of take-up rates by gender?</t>
+          <t>Are there gender disparities in take-up rates for approved financial products? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, and product type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside rejections of product applications to explore whether customer groups with lower application rejection rates also show higher take-up of approved products.</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -9380,7 +9381,7 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>How do relevant FSPs rank in terms of closing costs (from highest to lowest), and does this ranking change when the average is computed by gender? Are women and men equally likely to incur account closure fees, or are there gendered patterns in the types of financial service providers (FSPs) they use that influence the likelihood or amount of such fees? How might account closure costs act as a barrier to financial flexibility or mobility? Are women more likely to avoid formal financial services due to concerns over the cost of exiting the system? Additionally, are FSPs that charge lower or no closure fees more accessible to certain gender groups, and does this vary by geography or provider type?</t>
+          <t>Are there gender disparities in account closure costs? Variations in this indicator may be explored across customer gender, age, income, location, customer type, product type, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside product portability requests and rejected product portability requests to explore whether high closure costs suppress FSP-switching requests from certain customer groups.</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
@@ -9440,7 +9441,7 @@
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the volume of Suspiciou transaction reports (STRs) generated, including for MSMEs by the owner's gender? Is there a correlation between the volume of these reports and the composition of the FSP customer base by gender? For example, do FSPs with a higher proportion of women in their customer base report a lower volume of STR? Are there disparities in STR statistics across FSPs with different levels of gender diversity?</t>
+          <t>Are there gender patterns in the customer segments most often associated with suspicious transaction reports? Variations in this indicator may be explored across FSP type and transaction type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -9490,7 +9491,7 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>Are there customer gender disparities in the volume of systematic transaction reports (transactions that are not suspicious but reach regulatory thresholds for reporting) to the FIU, including for MSMEs by the owner's gender? Is there a correlation between the volume of these reports and the composition of the FSP customer base by gender? For example, do FSPs with a higher proportion of women in their customer base report a lower volume of systematic transaction reports, including those involving women? How do FSPs with different levels of gender diversity differ in the patterns of systematic reporting to the FIU?</t>
+          <t>Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? Variations in this indicator may be explored across FSP type.</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -9540,7 +9541,7 @@
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the representation of loan guarantors? What types of loans and borrowers, across different FSP types, are more likely to show gender disparities in the use of guarantors? Are there disparities in loan performance (NPLs, delinquency, interest income) depending on the gender of the guarantor?</t>
+          <t>Are there gender disparities in the representation of loan guarantors? Variations in this indicator may be explored across customer type, gender, income, location, FSP type, product type, and loan term and size. Do female borrowers disproportionately require male guarantors compared to the reverse? Is there a relationship between the gender pairing of borrower and guarantor and loan performance (delinquency, NPL)? Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside borrowers whose collateral was seized to explore whether loan portfolios relying more heavily on guarantors of a particular customer group show different collateral seizure rates, and what this implies about risk allocation by customer groups.</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -9600,7 +9601,7 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>Are there gender disparities (including for MSMEs based on the gender of ownership) in delinquency rates (also considering the number of unpaid installments) for loans of different types, terms and sizes? Do smaller loans have lower delinquency rates and how does this vary across genders? Do FSPs with higher levels of gender diversity present lower delinquency rates?</t>
+          <t>Are there gender disparities in delinquency rates? Variations in this indicator may be explored across customer type, gender, age, income, location, FSP type, product type, and loan size and term. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside loan loss provisions to explore whether FSPs provisioning more heavily against certain loan segments also show higher delinquency rates in those segments, and whether socio-demographic disparities in provisioning reflects actual differences in credit risk.</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -9660,7 +9661,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the rates of non-performing loans (NPL) within retail/MSME portfolios, and how do these differences vary by age, income levels, geographic location, and types of financial service providers? Do women or WMSME exhibit different patterns of loan repayment and default compared to men, and what factors might explain these variations? How do NPL rates differ across loan types, and are portfolios with higher female borrower participation associated with lower or higher NPL ratios? Are financial service providers with greater gender diversity in their workforce or leadership more effective at managing NPLs equitably across genders? What insights do gender-disaggregated NPL data provide regarding credit risk, financial resilience, and inclusion of vulnerable or underserved gender groups?</t>
+          <t>Are there gender disparities in NPL rates? Variations in this indicator may be explored across customer gender, customer type, FSP type, product type, loan size, and loan term. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside delinquency rates in the retail loan portfolio to explore whether socio-demographic patterns in early-stage delinquency are a reliable leading indicator of NPL outcomes by customer grouop.</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -9720,7 +9721,7 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the share of restructured loans within retail/MSME loan portfolios, and how do these differences vary by age, income levels, and geographic location? Are women or other gender groups more likely to have loans restructured, potentially reflecting differences in financial vulnerability or repayment capacity? How do patterns of loan restructuring differ across loan types and sectors by gender? Do financial service providers with greater gender diversity in their workforce or leadership demonstrate more equitable practices in loan restructuring across gender groups? What do gender-disaggregated data on restructured loans reveal about the resilience and support available to borrowers facing financial stress?</t>
+          <t>Are there gender disparities in the share of restructured loans? Variations in this indicator may be explored across customer gender, customer type, customer income, FSP type, credit type, loan size, and loan term. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside delinquency rates and NPLs to explore whether customer groups with higher restructuring rates also show elevated delinquency or NPL ratios, or whether restructuring successfully prevents default.</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
@@ -9780,7 +9781,7 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>Are higher levels of gender diversity at FSPs and in their customer base correlated with lower levels of large exposures in loan operations? How are large exposures distributed across different products, gender, and locations? Do large exposures show different delinquency and NPL levels based on gender?</t>
+          <t>How are large exposures distributed by product type and customer socio-demographics? This indicator may be analyzed alongside NPLs and delinquency indicators. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? Variations in this indicator may be explored across FSP type, product type, customer gender, age, income, and location.</t>
         </is>
       </c>
       <c r="J172" t="inlineStr">
@@ -9835,7 +9836,7 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the incidence of loan write-offs among retail/MSME borrowers? How do these disparities shift when further disaggregated by age, income, loan size, and geographic location? Do women or other gender groups experience higher or lower write-off rates compared to men, and what factors might explain these patterns? When analyzed in relation to the gender diversity of financial service providers’ leadership or top management, is higher gender diversity associated with more equitable write-off rates across customer genders? What insights do gender-disaggregated write-off data provide about risk assessment, financial inclusion, and borrower resilience?</t>
+          <t>Are there gender disparities in loan write-off rates? Variations in this indicator may be explored across customer gender, customer type, FSP type, credit type, loan size, and loan term. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside NPLs in the retail portfolio to explore whether socio-demographic patterns in non-performing loans translate predictably into write-offs.</t>
         </is>
       </c>
       <c r="J173" t="inlineStr">
@@ -9890,7 +9891,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the provisioning level allocated to customers? When disaggregated by other demographics such as age and location, do the observed gender-based differences change? Do vulnerable customers tend to have loans with higher provisioning levels, and are there gender differences in these patterns? When analyzed in relation to the gender diversity of FSPs' top management, is a higher level of gender diversity associated with differences in provisioning levels? And how does this relationship compare when considering gender diversity across other staff levels?</t>
+          <t>Are there gender disparities in provisioning levels? Variations in this indicator may be explored across customer gender, age, income and location, FSP type, product type, and average loan size and loan term. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside write-offs ratio to explore whether customer groups with higher provisioning levels also experience higher write-off rates, helping assess whether provisioning accurately anticipates credit losses by customer segment.</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
@@ -9948,6 +9949,11 @@
           <t>This indicator quantifies how much of the loan book is exposed to climate-related physical risks, specifically. These risks materialize through direct damage to assets, disruptions in business operations, or negative impacts on local economies, all of which can lead to higher rates of loan defaults and losses for the lender. This indicator should complement the all-encompassing indicator that measures climate-related risks (both physical and transition risks). Definitions and concepts of climate-related risks vary across countries. The Basel Committee has defined climate-related financial risks, including physical risks, while the NGFS provides a range of additional defintions, including nature-related financial risks.</t>
         </is>
       </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>Are there gender disparities in customer exposure to climate-related physical risks, particularly for women-led MSMEs in vulnerable sectors or regions? Variations in this indicator may be explored across customer gender, customer type, FSP type, and product type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside physical risk in the insurance portfolio to explore whether FSPs operating across both lending and insurance lines show consistent socio-demographic patterns in their exposure to climate-related physical risks.</t>
+        </is>
+      </c>
       <c r="I175" t="inlineStr">
         <is>
           <t>For analyses with a primary focus on financial inclusion, for this indicator it is recommended that only retail customers and/or financial products held by retail customers are considered. Where data permits, this indicator can be examined separately for MSMEs.</t>
@@ -9995,7 +10001,7 @@
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>How are FSP gender diversity and the gender composition of the customer base correlated with liquidity risk?</t>
+          <t>Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside liquid asset ratio to explore whether disparities are consistent across both flow-based and stock-based measures of liquidity. Variations in this indicator may be explored across FSP type.</t>
         </is>
       </c>
       <c r="L176" t="inlineStr">
@@ -10040,7 +10046,7 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>Is there a correlation between higher levels of gender diversity in FSPs and lower risk levels?</t>
+          <t>Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? Variations in this indicator may be explored across FSP type and product type.</t>
         </is>
       </c>
       <c r="L177" t="inlineStr">
@@ -10085,7 +10091,7 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the average amount of funds in suspense accounts, including for low-income customers and MSMEs based on the ownership gender? Are there gender disparities in the distribution of low-income customers with suspense accounts (and for which types of accounts?) compared to the whole customer base? Comparing this indicator with failed transactions and customer losses (if available), are there gender disparities in financial losses after funds remain in suspense or temporary accounts, which could indicate potential internal frauds? Comparing this indicator with FSP gender diversity, does higher gender diversity correlate with lower amounts in suspense accounts or customer losses after funds are temporarily placed in suspense accounts?</t>
+          <t>Are there gender disparities in the average amount of funds held in suspense accounts? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type. This indicator can be compared with failed transaction rates by gender. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="J178" t="inlineStr">
@@ -10140,7 +10146,7 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>Do incomplete/failed transactions impact different genders differently, including low-income customers and MSMEs based on the ownership gender? Comparing this indicator with the amount of losses suffered by customers (if available), are there gender disparities in financial losses due to failed transactions? How does this indicator compare with indicators on values maintained in suspense accounts and their variation by gender? Do different types of FSPs and accounts perform differently across the gender in terms of failed transactions? Comparing this indicator with gender diversity, does higher gender diversity correlate with a lower prevalence of failed transactions?</t>
+          <t>Are there gender disparities in the impact of failed transactions? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, transaction type and average size. This indicator can be analyzed alonside the indicator on financial loss due to failed transaction, and be compared with the indicator on balances in suspense accounts. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="J179" t="inlineStr">
@@ -10197,7 +10203,7 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>How are FSP gender diversity and gender composition of customer base correlated with the frequency of operational disruption incidents?</t>
+          <t>Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside successful cyber attacks to explore whether FSPs with higher rates of one type of operational failure also tend to show higher rates of the other, and whether this varies by customer groups. Variations in this indicator may be explored across FSP type and types of incidents.</t>
         </is>
       </c>
       <c r="J180" t="inlineStr">
@@ -10252,7 +10258,7 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>Are higher levels of gender diversity at FSPs correlated with the frequency of successful cyber attacks?</t>
+          <t>Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? Variations in this indicator may be explored across FSP type and type of cyber attacks.</t>
         </is>
       </c>
       <c r="J181" t="inlineStr">
@@ -10307,7 +10313,7 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>How do FSPs’ gender diversity and the gender composition of their customer base correlate with the costs incurred from reinsurance? Are there gendered patterns in how reinsurance expenses impact insurers and their customers?</t>
+          <t>Do insurers with greater gender diversity in their workforce, management, or board, incur different reinsurance costs? Do insurers with different levels of gender balance in their customer base, show different performance in this indicator? Variations in this indicator may be explored across insurer type, and type of reinsurance.</t>
         </is>
       </c>
       <c r="J182" t="inlineStr">
@@ -10362,7 +10368,7 @@
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>Are there gender disparities in claims ratios for insurance products, including for MSMEs based on the owner's gender? Are excessively low claims ratios correlated with low premiums (a proxy for targeting lower-income segments)? Are women more likely to be targeted by products with low claims ratios, potentially indicating lower-value offerings? Are FSPs with higher levels of gender diversity less likely to have excessively low claims ratios for insurance sold to vulnerable segments, such as women and women-owned MSMEs? When comparing with coverage ratios (amount of claims paid relative to the claim value), how do gender disparities in coverage ratios compare with claims paid?</t>
+          <t>Are there gender differences in loss ratios? Do insurers with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do insurers with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside insurance claims settlement ratio to explore whether insurers with higher loss ratios also show lower settlement ratios. Variations in this indicator may be explored across customer type, gender, income, age, location, FSP type, ype of insurance and average premium.</t>
         </is>
       </c>
       <c r="J183" t="inlineStr">
@@ -10417,7 +10423,7 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>How has the participation of different genders in incurred insurance claims evolved over time, both for individuals and MSMEs by owner’s gender? Are there gender differences in the types of claims incurred? How does the level of gender diversity within FSPs relate to these patterns?</t>
+          <t>Are there gender disparities in the volume or value of claims incurred? Variations in this indicator may be explored across customer type, gender, age, income, location, FSP type, type of insurance, and average premium. Do insurers with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do insurers with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside insurance claims paid to explore whether socio-demographic disparities in claims incurred translate into equivalent disparities in claims paid.</t>
         </is>
       </c>
       <c r="J184" t="inlineStr">
@@ -10473,7 +10479,7 @@
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>Are there gender disparities in insurance policy renewal rates, including among MSMEs by owner gender? Do certain policy types have lower renewal rates among specific gender groups? Could these differences signal mismatches between products and customer needs, posing strategic risks for insurers?</t>
+          <t>Are there gender disparities in insurance policy renewal rates? Variations in this indicator may be explored across customer type, gender, age, income, location, FSP type, and type of insurance and average premium. Do insurers with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do insurers with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside insurance lapse rates to explore whether socio-demographic patterns in renewal and lapse are mirror images of each other.</t>
         </is>
       </c>
       <c r="J185" t="inlineStr">
@@ -10528,7 +10534,7 @@
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>What is the relationship between FSP gender diversity, customer gender composition, and the degree of dependency on reinsurance? Are there gender-based patterns in insurers’ risk retention strategies?</t>
+          <t>Do insurers with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do insurers with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside cost of reinsurance to explore whether insurers with lower risk retention also face higher reinsurance costs, and whether the gender composition of the portfolio influences both. Variations in this indicator may be explored across product type, customer type, and insurer type.</t>
         </is>
       </c>
       <c r="L186" t="inlineStr">
@@ -10573,7 +10579,7 @@
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the adequacy of technical provisions maintained by FSPs? How do FSPs with higher gender diversity in management and governance compare in maintaining technical provisions that fairly reflect risks associated with serving diverse gender groups? Are provisions sufficiently accounting for potential differences in claims or defaults related to gender segments in the portfolio?</t>
+          <t>Do insurers with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do insurers with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside the insurance claims (loss) ratio to explore whether insurers that maintain higher technical provisions also show lower or more stable loss ratios, and whether this relationship varies across customer groups. Variations in this indicator may be explored across insurer type.</t>
         </is>
       </c>
       <c r="L187" t="inlineStr">
@@ -10618,7 +10624,7 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>How do FSP gender diversity and customer gender composition correlate with exposure to climate-related physical risks in insurance portfolios? Are there gender disparities in financial risk exposure due to climate impacts, including among MSMEs by owner gender?</t>
+          <t>Are there gender disparities in financial risk exposure to climate-related physical risks? Variations in this indicator may be explored across customer gender, customer type, age, income, location, and insurer type. Do insurers with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="L188" t="inlineStr">
@@ -10663,7 +10669,7 @@
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>How are FSP gender diversity and the gender composition of the customer base correlated with CAR levels?</t>
+          <t>Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside Tier 1 capital ratio to explore whether any differences by FSP gender diversity are consistent across both measures. Variations in this indicator may be explored across FSP type.</t>
         </is>
       </c>
       <c r="L189" t="inlineStr">
@@ -10708,7 +10714,7 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>Do FSPs with greater gender diversity in leadership and customer base tend to maintain stronger Tier 1 capital ratios? Is there any evidence that gender-inclusive governance correlates with improved capital adequacy and financial resilience? How might gender-related risk factors influence the calculation or management of Tier 1 capital?</t>
+          <t>Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? Variations in this indicator may be explored across FSP type.</t>
         </is>
       </c>
       <c r="L190" t="inlineStr">
@@ -10753,7 +10759,7 @@
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>Do financial service providers (FSPs) with higher gender diversity in leadership or governance report different interest margin ratios compared to less gender‑diverse peers? Are there associations between the gender composition of the customer base (e.g. share of women borrowers/depositors) and margin outcomes? Could gendered pricing—such as differential rates offered to male vs. female clients—impact FSP interest margins? Over time, do changes in margin ratios correlate with shifts in gender inclusion (e.g. more women customers or staff)?</t>
+          <t>Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside indicators of costs faced by borrowers, to explore correlations between gender disparities in pricing and performance in interest margin ratios. Variations in this indicator may be explored across FSP type.</t>
         </is>
       </c>
       <c r="L191" t="inlineStr">
@@ -10798,7 +10804,7 @@
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>How do insurance premiums written vary by gender of the policyholder, including for individuals and MSMEs based on owner gender? Are there gender disparities in the types and values of insurance products purchased, reflected in premiums collected? Do women or other gender groups pay systematically higher or lower premiums, and what might this indicate about risk assessment or product suitability? How do FSPs with higher gender diversity compare in the total premiums written to different gender segments? Are trends in premiums written by gender evolving over time, and do these trends vary by product type or geographic region?</t>
+          <t>Are there gender disparities in the volume or value of premiums written? Variations in this indicator may be explored across customer type, gender, age, income, location, FSP type, type of insurance, and average premium. Do insurers with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside insurance claims incurred to explore whether socio-demographic disparities in the volume or value of premiums written are mirrored by corresponding disparities in claims incurred.</t>
         </is>
       </c>
       <c r="J192" t="inlineStr">
@@ -10853,7 +10859,7 @@
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>Are there gender-related differences in the efficiency of FSP operations, for example, in cost-to-income ratios? Do FSPs with more gender-diverse teams or client bases demonstrate better operational efficiency? How do gender dynamics in product design, customer service, and outreach impact overall institutional efficiency?</t>
+          <t>Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside personnel expenses per customer/contract to explore whether disparities are driven in part by differences in the cost of serving different customer segments. Variations in this indicator may be explored across FSP type.</t>
         </is>
       </c>
       <c r="L193" t="inlineStr">
@@ -10898,7 +10904,7 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>Is there a gender dimension in personnel cost efficiency—that is, do FSPs with more balanced or female‑inclusive staff structures show lower personnel expenses per customer or contract? Are personnel expense ratios correlated with the gender composition of staff and how services are delivered to different gender groups? Do FSPs serving a higher proportion of women customers incur different per-customer personnel costs (e.g. due to agent outreach, financial literacy support)? How does this metric evolve over time in relation to efforts to promote gender inclusion in staffing and service models?</t>
+          <t>Do FSPs serving a higher proportion of women customers incur different per-customer personnel costs? Do FSPs with greater gender diversity at board, management, and staff levels show better performance on this indicator? This indicator can be analyzed alongside efficiency ratio to explore whether FSPs with higher per-customer personnel costs also show weaker overall efficiency ratios, and whether serving a more gender-diverse customer base correlates with different cost structures. Variations in this indicator may be explored across FSP type.</t>
         </is>
       </c>
       <c r="L194" t="inlineStr">
@@ -10943,7 +10949,7 @@
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>Do FSPs with greater gender diversity in their workforce, management, or boards tend to achieve higher or more stable ROA? Is there evidence that the gender composition of the customer base (e.g. more female clients) affects asset returns, for instance through differences in risk, lending, or deposit behaviors? When comparing across FSPs, does ROA differ systematically in institutions with stronger gender inclusion strategies? How have ROA trends shifted over time relative to changes in gender diversity (staffing or customer composition)?</t>
+          <t>Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside efficiency ratio and NPLs to explore whether FSPs with stronger risk management and operational efficiency also show higher asset returns, and whether these relationships are consistent across FSPs with different gender diversity profiles. Variations in this indicator may be explored across FSP type.</t>
         </is>
       </c>
       <c r="L195" t="inlineStr">
@@ -10988,7 +10994,7 @@
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>Is there a relationship between gender diversity in leadership or equity ownership and ROE performance across FSPs? Are FSPs that prioritize gender inclusion more likely to achieve higher equity returns, possibly through broader market reach or more balanced risk management? How does the gender mix of customers, especially depositors and borrowers, relate to ROE outcomes? Over time, do improvements in gender inclusion (in staffing or customer base) precede or follow changes in ROE?</t>
+          <t>Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside ROA to explore whether disparities in ROE reflect differences in leverage as well as asset returns, helping distinguish between financial strategy and operational performance. Variations in this indicator may be explored across FSP type.</t>
         </is>
       </c>
       <c r="L196" t="inlineStr">
@@ -11033,7 +11039,7 @@
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>How does the gender composition of borrowers in the total financial sector credit portfolio compare across the number and value of outstanding credit operations? Are there gender disparities in both the frequency (number) of credit operations and the total credit amounts extended? How do these disparities vary by loan type, sector, or borrower demographics such as age, income, and location? Are women or other gender groups underrepresented in certain types of credit or regions within the overall portfolio? How do FSPs with higher levels of gender diversity compare in terms of the balance and number of credit operations granted to different genders? Are portfolios with more balanced gender representation associated with differences in credit performance, such as lower default rates or more stable repayment patterns?</t>
+          <t>Are there gender disparities in the distribution of credit operations? Variations in this indicator may be explored across customer type, gender, FSP type, and product type.</t>
         </is>
       </c>
       <c r="J197" t="inlineStr">
@@ -11089,7 +11095,7 @@
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>Are there gender disparities in deposit stability or volatility, and do accounts held by different gender groups show distinct patterns in the frequency or magnitude of balance fluctuations? Could these differences reflect varying income regularity, saving habits, or financial resilience? How do these patterns vary across age, income level, or geographic location? Are there notable differences in deposit stability between FSPs with higher or lower levels of gender diversity in their customer base? Do FSPs with greater gender diversity among their clients tend to experience greater deposit stickiness overall?</t>
+          <t>Do accounts held by different gender groups show distinct patterns in deposit stability or volatility? Variations in this indicator may be explored across FSP type, product type, customer type, customer gender, age, income, location. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside net savings account flows to explore whether accounts with more volatile balances also show lower average net savings, and whether socio-demographic disparities in savings volatility are consistent with patterns in net savings behavior.</t>
         </is>
       </c>
       <c r="L198" t="inlineStr">
@@ -11210,7 +11216,7 @@
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>Are there gender disparities in participation in the rural credit portfolio, when measured by number of loans and disaggregated by loan type and type of borrower (individual or MSME)? Are these disparities more pronounced in certain types of financial service providers or geographic regions? Do FSPs with higher levels of gender diversity tend to allocate a greater share of loan volume to rural women or women-led MSMEs? Does the proportion of rural credit within the total number of loans granted to women differ significantly from that of men, and what does this reveal about access to credit by gender and location?</t>
+          <t>Are there gender disparities in access to rural credit by volume? Variations in this indicator may be explored across customer type, gender, age, location, income, FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
@@ -11270,7 +11276,7 @@
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>How is FSP gender diversity and the gender composition of the customer base correlated with climate-related financial risks (physical and transition) and other environmental risks?</t>
+          <t>Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? Variations in this indicator may be explored across FSP type, product type, customer type and gender.</t>
         </is>
       </c>
       <c r="J202" t="inlineStr">
@@ -11325,7 +11331,7 @@
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>How is FSP gender diversity correlated with lending to high polluters?</t>
+          <t>Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside financed emissions to explore whether FSPs with high polluting-sector exposures also show higher overall financed emissions, and whether both indicators are correlated with FSP gender diversity. Variations in this indicator may be explored across FSP type.</t>
         </is>
       </c>
       <c r="J203" t="inlineStr">
@@ -11380,7 +11386,7 @@
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>How is FSP gender diversity correlated with financed emissions of the loan and securities portfolio?</t>
+          <t>Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside green/sustainable loans to explore whether FSPs with a higher share of green lending also show lower financed emissions overall, and whether gender-diverse FSPs lead on both dimensions. Variations in this indicator may be explored across FSP type, customer type, gender, and product type.</t>
         </is>
       </c>
       <c r="J204" t="inlineStr">
@@ -11435,7 +11441,7 @@
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>Are there gender, location, and income disparities in access to green and sustainable loans, including those aimed at climate adaptation and resilience? How do these disparities intersect with factors such as age and sector of activity? Are women or other gender groups underrepresented among borrowers of green loans, and what barriers might contribute to this? Do financial service providers with higher levels of gender diversity tend to have relatively larger and more inclusive green/sustainable loan portfolios? How do repayment patterns and loan terms for green loans differ by gender, and what implications do these have for promoting equitable access to climate finance?</t>
+          <t>Are there gender disparities in access to green or sustainable loans? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, credit type, loan size, and loan term. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="J205" t="inlineStr">
@@ -11490,7 +11496,7 @@
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the share of the outstanding retail loan portfolio held by rural borrowers, disaggregated by gender and type of borrower? Are these disparities more significant in specific regions or FSP types? Do rural women hold a lower share of outstanding balances, and could this reflect differences in loan size, duration, or repayment behavior? How does the share of rural credit within the total outstanding credit held by women compare to that of men, and what does it suggest about the gendered distribution of long-term credit in rural areas?</t>
+          <t>Are there gender disparities in access to rural credit by outstanding balance? Variations in this indicator may be explored across customer type, gender, age, location, income, FSP type. This indicator can be analyzed alongside green/sustainable loans to explore the intersection of gender, climate, and rural finance. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
@@ -11550,7 +11556,7 @@
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the value of new rural credit disbursed to borrowers, disaggregated by gender and borrower type? Are these disparities more evident in certain regions or financial service providers, particularly among those with less gender diversity? Do women in rural areas systematically receive smaller disbursements compared to men in similar loan categories or activities? Does the share of rural credit within the total disbursed credit to women differ significantly from that of men, and what does it indicate about access to productive credit for rural women? Has the share of credit disbursed to rural women changed over time in proportion to their role in the rural economy?</t>
+          <t>Are there gender disparities in access to rural credit by principal disbursed? Variations in this indicator may be explored across customer gender, age, type, location, income, FSP type. This indicator can be analyzed alongside green/sustainable loans to explore the intersection of gender, climate, and rural finance. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
@@ -11610,7 +11616,7 @@
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>Are there disparities by gender, income, and location in the likelihood of acquiring green or sustainable insurance products, including climate resilience coverage? Are certain gender groups underserved in this market? Do financial service providers (FSPs) with higher levels of gender diversity tend to maintain larger or more diverse green/sustainable insurance portfolios?</t>
+          <t>Are there gender disparities in access to and uptake of green or sustainable insurance products? Variations in this indicator may be explored across customer type, gender, age, income, location, FSP type, type of insurance, and average premium. Do insurers with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside green/sustainable loans to explore whether customer groups with lower access to green credit also show lower uptake of green insurance products.</t>
         </is>
       </c>
       <c r="J208" t="inlineStr">
@@ -11665,7 +11671,7 @@
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the acquisition/holding of green/sustainable bonds? Are FSPs with higher levels of gender diversity more likely to distribute sustainable or green bonds to a more diverse investor base?  Comparing this with gender diversity at FSPs, are institutions with higher levels of gender diversity more likely to have larger green/sustainable portfolios?</t>
+          <t>Are there gender disparities in access to and participation in holding green or sustainable bonds? Variations in this indicator may be explored across customer type, gender, age, income, location. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? FSP type, and main activity.</t>
         </is>
       </c>
       <c r="L209" t="inlineStr">
@@ -11710,7 +11716,7 @@
       </c>
       <c r="H210" t="inlineStr">
         <is>
-          <t>Do companies with higher levels of gender diversity issue more green bonds? Are FSPs with higher levels of gender diversity more likely to distribute sustainable or green bonds?</t>
+          <t>Are there gender disparities in access to and participation in issuing green or sustainable bonds? Variations in this indicator may be explored across customer type, gender, FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside holdings of green/sustainable bonds to explore whether socio-demographic disparities in green bond issuance participation are mirrored by disparities in holding.</t>
         </is>
       </c>
       <c r="J210" t="inlineStr">
@@ -11765,7 +11771,7 @@
       </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>How is FSP gender diversity correlated with climate-related financial risks and other environmental risks arising from the investment portfolio of insurers and banks?</t>
+          <t>Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? This indicator can be analyzed alongside climate and other environmental risk in the credit portfolio to explore whether FSPs show consistent socio-demographic patterns in environmental risk exposure across both their lending and investment activities. Variations in this indicator may be explored across FSP type.</t>
         </is>
       </c>
       <c r="J211" t="inlineStr">
@@ -11820,7 +11826,7 @@
       </c>
       <c r="H212" t="inlineStr">
         <is>
-          <t>Are there gender disparities in workforce participation across different types of FSPs? At what responsibility levels? How does gender diversity in FSP management correlate with key financial indicators (e.g., Stability, Financial Inclusion, Customer Protection, Sustainability)? Do more gender-diverse FSPs serve more women or women-owned MSMEs, at better terms, with lower risk? Comparing with climate-related financial data (e.g., green loan portfolios, green insurance), does gender diversity in FSPs correlate with the growth of these portfolios? If legal or regulatory gender equity requirements exist for FSPs, are they being met? Does gender diversity correlate with risk metrics and supervisory risk scores? How does gender diversity correlate with enforcement and other supervisory actions?</t>
+          <t>Are there gender disparities in FSP workforce participation across different levels of responsibility (board, management, staff)? Variations in this indicator may be explored across FSP type. By analyzing gender diversity with performance indicators and prudential rartios, how does gender diversity in FSP leadership correlate with key indicators such as ROE, ROA, capital adequacy ratio, efficiency ratio, liquidity ratio, interest margin ratio (for lenders), technical provisions (for insurers)? If gender equity requirements exist for FSPs, are they being met? Does gender diversity correlate with overall supervisory risk scores of risk-based prudential and conduct superivision, or enforcement actions?</t>
         </is>
       </c>
       <c r="L212" t="inlineStr">
@@ -11865,7 +11871,7 @@
       </c>
       <c r="H213" t="inlineStr">
         <is>
-          <t>Are there significant gender disparities in the customer base across different types of financial service providers (FSPs)? What share of each FSP's customers are women or women-owned MSMEs? How does the gender diversity of the FSP customer base vary by institution size, sector, and geographic region? What correlations exist between the gender diversity of the customer base and key financial inclusion metrics mesauring account ownership, loan uptake, insurance coverage and financial health? How does greater gender diversity among customers relate to customer protection outcomes, including complaint resolution and fair treatment? Are FSPs with more gender-diverse customer bases also demonstrating stronger prudential performance and sustainability indicators? How do gender disparities in the customer base influence financial outcomes such as Financial Health? And broader social and economic outcomes, such as women's economic empowerment, MSME growth, climate change, jobs creation or poverty reduction?</t>
+          <t>What is the gender composition of each FSP's customer base across product types, and how has it evolved over time? Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Variations in this indicator may be explored across FSP type, FSP location, product type, customer gender, age, income, and location. This indicator can be analyzed alongside gender diversity at FSP (by reference workforce group) to explore whether FSPs with greater internal gender diversity in their workforce also tend to serve a more gender-balanced customer base.</t>
         </is>
       </c>
       <c r="L213" t="inlineStr">
@@ -11910,7 +11916,7 @@
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>Are there gender disparities in compensation for similar positions or responsibilities (Board, management, staff)? How does this compare with other macro indicators related to financial stability and portfolio performance across FSPs (credit, insurance, investment funds, pensions)? Are FSPs with greater gender diversity in the Board more likely to present lower gender pay gap?</t>
+          <t>Are there gender pay gaps for similar roles and responsibility levels (board, management, staff) at FSPs? Variations in this indicator may be explored across FSP type. Do FSPs with greater board-level gender diversity tend to have smaller gender pay gaps? How do pay gap levels correlate with FSP performance indicators such as ROW, ROE, efficiency ratio, NPL, and delinquency? This indicator can be analyzed alongside the Human Resources Gender Index (HRGI) to explore whether FSPs with better overall gender HR policies, as captured in the HRGI, also show smaller gender pay gaps.</t>
         </is>
       </c>
       <c r="L214" t="inlineStr">
@@ -11956,7 +11962,7 @@
       </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t>How do financial service providers (FSPs) compare in their Human Resources Gender Index (HRGI) scores? Are FSPs with higher levels of gender diversity in their workforce more likely to perform better across the various HRGI dimensions, such as recruitment, retention, promotion, and leadership representation? When comparing HRGI scores with key performance indicators (e.g., capital and liquidity, profitability, efficiency, customer satisfaction, innovation), is there evidence of a positive correlation? How do HRGI scores vary by FSP type, size, or region, and what best practices can be identified from top performers? How does HRGI performance relate to gender-related outcomes, such as gender-balanced customer bases or inclusive product offerings?</t>
+          <t>How do FSPs compare in their HRGI scores across dimensions of representation, pay equity, recruitment, promotion, and retention? Do FSPs with higher HRGI scores tend to perform better on key financial indicators (capital adequacy, profitability, NPL rates, consumer protection outcomes)? How do HRGI scores vary by FSP type and region?</t>
         </is>
       </c>
       <c r="L215" t="inlineStr">
@@ -12001,7 +12007,7 @@
       </c>
       <c r="H216" t="inlineStr">
         <is>
-          <t>To what extent does the gender of individuals in leadership or control positions within the proposed FSPs influence the likelihood of obtaining a license from the regulatory authority?</t>
+          <t>Do applications by FSPs with greater gender diversity in their management or board show different probably of being approved? This indicator can be analyzed alongside new licenses granted to diverse FSPs to explore whether the overall volume of licenses granted to gender-diverse FSPs reflects a higher application success rate, or simply more applications. Variations in this indicator may be explored across FSP type.</t>
         </is>
       </c>
       <c r="L216" t="inlineStr">
@@ -12046,7 +12052,7 @@
       </c>
       <c r="H217" t="inlineStr">
         <is>
-          <t>Are there differences in the rates of return for crowdfunding projects depending on the gender assigned to the MSME seeking funding?</t>
+          <t>Are there gender disparities in crowdfunding differential rate of return (equity)? Variations in this indicator may be explored across customer type, gender, age, income, location, FSP type, and product type. Do crowdfunding platforms with more gender-diverse management show more equitable outcomes for female campaign sponsors?</t>
         </is>
       </c>
       <c r="J217" t="inlineStr">
@@ -12101,7 +12107,7 @@
       </c>
       <c r="H218" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the rejection rates and the reasons for rejection of crowdfunding projects presented for authorization by the securities regulator?</t>
+          <t>Are there gender disparities in crowdfunding authorization rejection rate? Variations in this indicator may be explored across customer type, gender, age, income, location, FSP type, and product type. Do crowdfunding platforms with more gender-diverse management show more equitable outcomes for female campaign sponsors?This indicator can be analyzed alongside crowdfunding – success rate to explore whether customer groups facing higher authorization rejection rates also show lower overall success rates.</t>
         </is>
       </c>
       <c r="L218" t="inlineStr">
@@ -12146,7 +12152,7 @@
       </c>
       <c r="H219" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the success rates of crowdfunding projects? Are smaller or younger MSMEs headed by women more likely to face challenges in crowdfunding?</t>
+          <t>Are there gender disparities in crowdfunding success rate, and do women-led ventures face different rates or outcomes compared to men? Variations in this indicator may be explored across customer type, gender, income, age, location, FSP type, and product type. Do crowdfunding platforms with more gender-diverse management show more equitable outcomes for female campaign sponsors?</t>
         </is>
       </c>
       <c r="J219" t="inlineStr">
@@ -12201,7 +12207,7 @@
       </c>
       <c r="H220" t="inlineStr">
         <is>
-          <t>Are there disparities in crowdfunding volumes and values raised, according to the gender of the MSMEs asking for funds? Are there disparities in terms of funding periods? Among women-owned MSMEs, which types and ages (years in operation) are driving growth in crowdfunding transactions? Are crowdfunding platforms operated by diverse management more likely to attract women-owned MSMEs, and young MSMEs headed by women?</t>
+          <t>Are there gender disparities in crowdfunding transactions, and do women-led ventures face different rates or outcomes compared to men? Variations in this indicator may be explored across customer type, gender, age, income, location, FSP type, and product type. Do crowdfunding platforms with more gender-diverse management show more equitable outcomes for female campaign sponsors? This indicator can be analyzed alongside crowdfunding – success rate to explore whether socio-demographic disparities in the volume of crowdfunding campaigns are compounded by disparities in success rates.</t>
         </is>
       </c>
       <c r="L220" t="inlineStr">
@@ -12246,7 +12252,7 @@
       </c>
       <c r="H221" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the growth of reatil investors in P2P lending platforms? How do invested amounts and types vary by investor gender and other demographics? For example, do women prefer to invest in women-led MSMEs, smaller projects, or younger enterprises? Do P2P platforms operated by diverse management more likely to attract a more diverse investor base?</t>
+          <t>Are there gender disparities across P2P investors? Variations in this indicator may be explored across customer type, gender, age, income, location, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside P2P – credit operations to explore whether socio-demographic disparities on the investor side of P2P markets are mirrored by disparities on the borrower side.</t>
         </is>
       </c>
       <c r="L221" t="inlineStr">
@@ -12291,7 +12297,7 @@
       </c>
       <c r="H222" t="inlineStr">
         <is>
-          <t>How has participation in investment funds evolved by gender, both for individuals and MSMEs considering the gender of their owners? What types of investment funds show growing participation by women?</t>
+          <t>Are there gender disparities in the ownership of investment fund shares? Variations in this indicator may be explored across customer type, gender, age, income, location, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? This indicator can be analyzed alongside investment accounts (outstanding balance) to explore whether socio-demographic disparities in fund share ownership are proportional to disparities in total investment account balances.</t>
         </is>
       </c>
       <c r="J222" t="inlineStr">
@@ -12346,7 +12352,7 @@
       </c>
       <c r="H223" t="inlineStr">
         <is>
-          <t>Are there gender disparities in interest rate spreads offered to borrowers, and how do these differences vary across regions, income levels, and types of financial service providers? Do women or other gender groups consistently face higher lending rates relative to reference rates compared to men, potentially indicating unequal credit costs? How do interest rate spreads differ by loan type or sector, and are there gender patterns in these variations? Are financial service providers with higher gender diversity more likely to offer more equitable interest rate spreads across gender groups? How do differences in interest rate spreads impact borrowing behavior and access to credit for different gender groups?</t>
+          <t>Are there gender disparities in the interest rate spreads faced by borrowers? Variations in this indicator may be explored across customer gender, customer type, age, income, location, FSP type, credit type, loan size, and loan term. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside annual percentage rate (APR) for retail credit to explore whether customer groups facing higher APRs are concentrated in loan types or FSPs that also show wider spreads over reference rates.</t>
         </is>
       </c>
       <c r="I223" t="inlineStr">
@@ -12406,7 +12412,7 @@
       </c>
       <c r="H224" t="inlineStr">
         <is>
-          <t>Are there gender disparities in data-sharing consent within the open finance scheme, including for MSMEs based on the ownership gender and low-value accounts? What types of accounts are more commonly subject to data-sharing consents? Which types of FSPs have a higher percentage of customers who have given data-sharing consent, and do these percentages vary by gender? If the information is available, what are the most common types and terms for these consents?</t>
+          <t>Are there gender disparities in data sharing consent rates for open finance? Variations in this indicator may be explored across customer type, gender, age, income, location, and FSP type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside consents for sharing data with third parties to explore whether customer groups consenting to data sharing within open finance schemes are also more likely to share data with third parties.</t>
         </is>
       </c>
       <c r="I224" t="inlineStr">
@@ -12466,7 +12472,7 @@
       </c>
       <c r="H225" t="inlineStr">
         <is>
-          <t>Open finance performance will vary across FSPs for a range of reasons such as their current data architecture and other firm-specific aspects. The objective of looking into this indicator from a gender perspective is to identify whether FSPs that concentrate underserved, low-income women and women-led MSMEs also present poor open finance performance. This indicator can be analyzed together with other open finance performance indicators (Unsuccessful API calls, API response time), and open finance adoption indicators (% customer that have given consent, payment initiation transactions)</t>
+          <t>Does API infrastructure for open finance show performance differences across FSPs that could disproportionately affect digital-first FSPs serving gender-diverse or underserved customer bases? Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside open finance – API error rate and open finance – API response time to explore whether FSPs with lower API availability also show higher error rates and slower response times. Variations in this indicator may be explored across FSP type and API type.</t>
         </is>
       </c>
       <c r="I225" t="inlineStr">
@@ -12526,7 +12532,7 @@
       </c>
       <c r="H226" t="inlineStr">
         <is>
-          <t>Open finance performance will vary across FSPs for a range of reasons such as their current data architecture and other firm-specific aspects. The objective of looking into this indicator from a gender perspective is to identify whether FSPs that concentrate underserved, low-income women and women-led MSMEs also present poor open finance performance. This indicator can be analyzed together with other open finance performance indicators (Unsuccessful API calls, API response time), and open finance adoption indicators (% customer that have given consent, payment initiation transactions)</t>
+          <t>Does API error rate show performance differences that could disproportionately affect digital-first FSPs serving gender-diverse and underserved customer bases? Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? Variations in this indicator may be explored across FSP type and API type.</t>
         </is>
       </c>
       <c r="I226" t="inlineStr">
@@ -12586,7 +12592,7 @@
       </c>
       <c r="H227" t="inlineStr">
         <is>
-          <t>Open finance performance will vary across FSPs for a range of reasons such as their current data architecture and other firm-specific aspects. The objective of looking into this indicator from a gender perspective is to identify whether FSPs that concentrate underserved, low-income women and women-led MSMEs also present poor open finance performance. This indicator can be analyzed together with other open finance performance indicators (Unsuccessful API calls, API response time), and open finance adoption indicators (% customer that have given consent, payment initiation transactions)</t>
+          <t>Does API call response time show performance differences that could disproportionately affect digital-first FSPs serving gender-diverse or underserved customer bases? Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? Variations in this indicator may be explored across FSP type, and API type.</t>
         </is>
       </c>
       <c r="I227" t="inlineStr">
@@ -12646,7 +12652,7 @@
       </c>
       <c r="H228" t="inlineStr">
         <is>
-          <t>Are there gender disparities in the adoption of payment initiation transactions within the open finance scheme, including for MSMEs by the owner's gender? Do FSPs with higher levels of gender diversity tend to have a larger share of diverse customers conducting payment initiation transactions?</t>
+          <t>Are there gender disparities in the use of payment initiation services through open finance channels? Variations in this indicator may be explored across customer type, gender, age, income, location, and FSP type. Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside access to the instant/fast payment system to explore whether socio-demographic gaps in payment initiation through open finance channels are related to gaps in registration in the instant payment system.</t>
         </is>
       </c>
       <c r="I228" t="inlineStr">
@@ -12697,7 +12703,7 @@
       </c>
       <c r="H229" t="inlineStr">
         <is>
-          <t>How many products does each gender take up on average during the onboarding stage, and how do these numbers compare? What are the gender disparities in the likelihood of adopting multiple products? Which FSPs stand out in multi-product onboarding, and does their ranking change when analyzed by gender? Note: Active usage of products should also be assessed for multiple products taken up during onboarding.</t>
+          <t>Are there gender disparities in the average number of products taken up during onboarding? Variations in this indicator may be explored across customer gender, age, income, location, customer type, product type and FSP type. this indicator can be analyzed alongisde the active usage of products taken up during onboarding. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside product take-up ratio to explore whether disparities in bundled product uptake at onboarding persist into actual product activation and usage.</t>
         </is>
       </c>
       <c r="I229" t="inlineStr">
@@ -12757,7 +12763,7 @@
       </c>
       <c r="H230" t="inlineStr">
         <is>
-          <t>Are there customer gender, income and location disparities in account and loan portability or FSP switching requests? Are FSPs with higher levels of gender diversity more likely to receive portability or switching requests or be the destination FSP (rather than the origin) for such requests?</t>
+          <t>Are there gender disparities in account and loan portability or FSP switching requests? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, and product type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator? This indicator can be analyzed alongside rejected product portability requests to explore whether customer groups submitting more portability requests also face higher rejection rates.</t>
         </is>
       </c>
       <c r="I230" t="inlineStr">
@@ -12817,7 +12823,7 @@
       </c>
       <c r="H231" t="inlineStr">
         <is>
-          <t>Are there customer gender, income, and location disparities in the approval of portability requests? Are FSPs with higher levels of gender diversity more likely to approve portability requests?</t>
+          <t>Are there gender disparities in the rate of rejected portability requests? Variations in this indicator may be explored across customer gender, age, income, location, customer type, FSP type, and product type. Do FSPs with greater gender diversity in their workforce, management, or board, show different performance in this indicator? Do FSPs with different levels of gender balance in their customer base, show different performance in this indicator?</t>
         </is>
       </c>
       <c r="I231" t="inlineStr">

</xml_diff>